<commit_message>
wip: fill family members and documents lists
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="108">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -331,7 +331,13 @@
     <t xml:space="preserve">Поле з актуальною інформацією</t>
   </si>
   <si>
+    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
     <t xml:space="preserve">Основна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
   </si>
   <si>
     <t xml:space="preserve">Адреси Контакти</t>
@@ -350,13 +356,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy;@"/>
     <numFmt numFmtId="166" formatCode="&quot;Да&quot;;&quot;Да&quot;;&quot;Нет&quot;"/>
     <numFmt numFmtId="167" formatCode="@"/>
+    <numFmt numFmtId="168" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -430,6 +437,14 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -542,7 +557,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -727,12 +742,24 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2172,7 +2199,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1048576"/>
+  <dimension ref="A1:M1048576"/>
   <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="43" width="23.16"/>
@@ -2194,143 +2221,372 @@
       <c r="D1" s="45" t="s">
         <v>100</v>
       </c>
+      <c r="F1" s="2"/>
+      <c r="G1" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="46" t="s">
-        <v>101</v>
+      <c r="A2" s="47" t="s">
+        <v>102</v>
       </c>
       <c r="B2" s="42" t="str">
         <f aca="false">Основна!A9</f>
         <v>Прізвище</v>
       </c>
-      <c r="C2" s="47" t="str">
+      <c r="C2" s="48" t="str">
         <f aca="false">IF(Основна!B9 = 0, "",  Основна!B9)</f>
         <v/>
       </c>
       <c r="D2" s="42"/>
+      <c r="G2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M2" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="46"/>
+      <c r="A3" s="47"/>
       <c r="B3" s="42" t="str">
         <f aca="false">Основна!A10</f>
         <v>Ім’я</v>
       </c>
-      <c r="C3" s="47" t="str">
+      <c r="C3" s="48" t="str">
         <f aca="false">IF(Основна!B10 = 0, "",  Основна!B10)</f>
         <v/>
       </c>
       <c r="D3" s="42"/>
+      <c r="G3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M3" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46"/>
+      <c r="A4" s="47"/>
       <c r="B4" s="42" t="str">
         <f aca="false">Основна!A11</f>
         <v>По батькові </v>
       </c>
-      <c r="C4" s="47" t="str">
+      <c r="C4" s="48" t="str">
         <f aca="false">IF(Основна!B11 = 0, "",  Основна!B11)</f>
         <v/>
       </c>
       <c r="D4" s="42"/>
+      <c r="G4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="46"/>
+      <c r="A5" s="47"/>
       <c r="B5" s="42" t="str">
         <f aca="false">Основна!A12</f>
         <v>Дата народження </v>
       </c>
-      <c r="C5" s="47" t="str">
+      <c r="C5" s="48" t="str">
         <f aca="false">IF(Основна!B12 = 0, "",  Основна!B12)</f>
         <v/>
       </c>
       <c r="D5" s="42"/>
+      <c r="G5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="49" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="46"/>
+      <c r="A6" s="47"/>
       <c r="B6" s="42" t="str">
         <f aca="false">Основна!A13</f>
         <v>Громадянство</v>
       </c>
-      <c r="C6" s="47" t="str">
+      <c r="C6" s="48" t="str">
         <f aca="false">IF(Основна!B13 = 0, "",  Основна!B13)</f>
         <v>Україна</v>
       </c>
       <c r="D6" s="42"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46"/>
+      <c r="A7" s="47"/>
       <c r="B7" s="42" t="str">
         <f aca="false">Основна!A14</f>
         <v>Освіта </v>
       </c>
-      <c r="C7" s="47" t="str">
+      <c r="C7" s="48" t="str">
         <f aca="false">IF(Основна!B14 = 0, "",  Основна!B14)</f>
         <v/>
       </c>
       <c r="D7" s="42"/>
+      <c r="G7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="46"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46"/>
+      <c r="A8" s="47"/>
       <c r="B8" s="42" t="str">
         <f aca="false">Основна!A15</f>
         <v>ППС чи ІТС</v>
       </c>
-      <c r="C8" s="47" t="str">
+      <c r="C8" s="48" t="str">
         <f aca="false">IF(Основна!B15 = 0, "",  Основна!B15)</f>
         <v>ППС</v>
       </c>
       <c r="D8" s="42"/>
+      <c r="G8" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="46"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="42" t="str">
         <f aca="false">Основна!A16</f>
         <v>Науковий ступінь</v>
       </c>
-      <c r="C9" s="47" t="str">
+      <c r="C9" s="48" t="str">
         <f aca="false">IF(Основна!B16 = 0, "",  Основна!B16)</f>
         <v/>
       </c>
       <c r="D9" s="42"/>
+      <c r="G9" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="46"/>
+      <c r="A10" s="47"/>
       <c r="B10" s="42" t="str">
         <f aca="false">Основна!A17</f>
         <v>Вчене звання</v>
       </c>
-      <c r="C10" s="47" t="str">
+      <c r="C10" s="48" t="str">
         <f aca="false">IF(Основна!B17 = 0, "",  Основна!B17)</f>
         <v/>
       </c>
       <c r="D10" s="42"/>
+      <c r="G10" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46"/>
+      <c r="A11" s="47"/>
       <c r="B11" s="42" t="str">
         <f aca="false">Основна!A18</f>
         <v>Сімейний стан</v>
       </c>
-      <c r="C11" s="47" t="str">
+      <c r="C11" s="48" t="str">
         <f aca="false">IF(Основна!B18 = 0, "",  Основна!B18)</f>
         <v/>
       </c>
       <c r="D11" s="42"/>
+      <c r="G11" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="46"/>
+      <c r="A12" s="47"/>
       <c r="B12" s="42" t="str">
         <f aca="false">Основна!A21</f>
         <v>Інститут</v>
       </c>
-      <c r="C12" s="47" t="str">
+      <c r="C12" s="48" t="str">
         <f aca="false">IF(Основна!B21 = 0, "",  Основна!B21)</f>
         <v/>
       </c>
       <c r="D12" s="42"/>
+      <c r="G12" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46"/>
+      <c r="A13" s="47"/>
       <c r="B13" s="42" t="str">
         <f aca="false">Основна!A22</f>
         <v>Кафедра (відділ)</v>
@@ -2340,9 +2596,29 @@
         <v/>
       </c>
       <c r="D13" s="42"/>
+      <c r="G13" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="25" t="n">
+        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="46"/>
+      <c r="A14" s="47"/>
       <c r="B14" s="42" t="str">
         <f aca="false">Основна!A23</f>
         <v>Посада</v>
@@ -2354,7 +2630,7 @@
       <c r="D14" s="42"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="46"/>
+      <c r="A15" s="47"/>
       <c r="B15" s="42" t="str">
         <f aca="false">Основна!A24</f>
         <v>Номер наказу про призначення</v>
@@ -2364,9 +2640,14 @@
         <v/>
       </c>
       <c r="D15" s="42"/>
+      <c r="G15" s="46" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="46"/>
+      <c r="A16" s="47"/>
       <c r="B16" s="42" t="str">
         <f aca="false">Основна!A25</f>
         <v>Дата наказу про призначення</v>
@@ -2376,9 +2657,21 @@
         <v/>
       </c>
       <c r="D16" s="42"/>
+      <c r="G16" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="46"/>
+      <c r="A17" s="47"/>
       <c r="B17" s="42" t="str">
         <f aca="false">Основна!A28</f>
         <v>Група обліку</v>
@@ -2388,9 +2681,21 @@
         <v/>
       </c>
       <c r="D17" s="42"/>
+      <c r="G17" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46"/>
+      <c r="A18" s="47"/>
       <c r="B18" s="42" t="str">
         <f aca="false">Основна!A29</f>
         <v>Категорія обліку</v>
@@ -2400,9 +2705,21 @@
         <v/>
       </c>
       <c r="D18" s="42"/>
+      <c r="G18" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="46"/>
+      <c r="A19" s="47"/>
       <c r="B19" s="42" t="str">
         <f aca="false">Основна!A30</f>
         <v>Склад</v>
@@ -2412,9 +2729,21 @@
         <v/>
       </c>
       <c r="D19" s="42"/>
+      <c r="G19" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="46"/>
+      <c r="A20" s="47"/>
       <c r="B20" s="42" t="str">
         <f aca="false">Основна!A31</f>
         <v>Військове звання</v>
@@ -2424,9 +2753,21 @@
         <v/>
       </c>
       <c r="D20" s="42"/>
+      <c r="G20" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="46"/>
+      <c r="A21" s="47"/>
       <c r="B21" s="42" t="str">
         <f aca="false">Основна!A32</f>
         <v>Військово-облікова спеціальність</v>
@@ -2436,9 +2777,21 @@
         <v/>
       </c>
       <c r="D21" s="42"/>
+      <c r="G21" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="50" t="n">
+        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46"/>
+      <c r="A22" s="47"/>
       <c r="B22" s="42" t="str">
         <f aca="false">Основна!A33</f>
         <v> Придатність до військової служби</v>
@@ -2450,7 +2803,7 @@
       <c r="D22" s="42"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="46"/>
+      <c r="A23" s="47"/>
       <c r="B23" s="42" t="str">
         <f aca="false">Основна!A34</f>
         <v>Териториальний центр комплектування та соціальної підтримки</v>
@@ -2462,7 +2815,7 @@
       <c r="D23" s="42"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="46"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="42" t="str">
         <f aca="false">Основна!A35</f>
         <v>Перебування на спеціальному обліку</v>
@@ -2474,8 +2827,8 @@
       <c r="D24" s="42"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="46" t="s">
-        <v>102</v>
+      <c r="A25" s="47" t="s">
+        <v>104</v>
       </c>
       <c r="B25" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A4</f>
@@ -2488,7 +2841,7 @@
       <c r="D25" s="42"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="46"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A5</f>
         <v>Область</v>
@@ -2500,7 +2853,7 @@
       <c r="D26" s="42"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="46"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A6</f>
         <v>Місто</v>
@@ -2512,7 +2865,7 @@
       <c r="D27" s="42"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="46"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A7</f>
         <v>Район (міста)</v>
@@ -2524,7 +2877,7 @@
       <c r="D28" s="42"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="46"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A8</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
@@ -2536,7 +2889,7 @@
       <c r="D29" s="42"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="46"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A9</f>
         <v>Індекс</v>
@@ -2548,7 +2901,7 @@
       <c r="D30" s="42"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="46"/>
+      <c r="A31" s="47"/>
       <c r="B31" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A12</f>
         <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
@@ -2560,7 +2913,7 @@
       <c r="D31" s="42"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="46"/>
+      <c r="A32" s="47"/>
       <c r="B32" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A13</f>
         <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
@@ -2572,7 +2925,7 @@
       <c r="D32" s="42"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="46"/>
+      <c r="A33" s="47"/>
       <c r="B33" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A16</f>
         <v>Співпадає із адресою фактичного проживання</v>
@@ -2584,7 +2937,7 @@
       <c r="D33" s="42"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="46"/>
+      <c r="A34" s="47"/>
       <c r="B34" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A18</f>
         <v>Країна</v>
@@ -2596,7 +2949,7 @@
       <c r="D34" s="42"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="46"/>
+      <c r="A35" s="47"/>
       <c r="B35" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A19</f>
         <v>Область</v>
@@ -2608,7 +2961,7 @@
       <c r="D35" s="42"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="46"/>
+      <c r="A36" s="47"/>
       <c r="B36" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A20</f>
         <v>Місто</v>
@@ -2620,7 +2973,7 @@
       <c r="D36" s="42"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="46"/>
+      <c r="A37" s="47"/>
       <c r="B37" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A21</f>
         <v>Район (міста)</v>
@@ -2632,7 +2985,7 @@
       <c r="D37" s="42"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="46"/>
+      <c r="A38" s="47"/>
       <c r="B38" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A22</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
@@ -2644,7 +2997,7 @@
       <c r="D38" s="42"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="46"/>
+      <c r="A39" s="47"/>
       <c r="B39" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A23</f>
         <v>Індекс</v>
@@ -2656,937 +3009,937 @@
       <c r="D39" s="42"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="46" t="s">
-        <v>103</v>
+      <c r="A40" s="47" t="s">
+        <v>105</v>
       </c>
       <c r="B40" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C40" s="48" t="str">
+      <c r="C40" s="51" t="str">
         <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
         <v/>
       </c>
-      <c r="D40" s="49"/>
+      <c r="D40" s="52"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="46"/>
+      <c r="A41" s="47"/>
       <c r="B41" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C41" s="48" t="str">
+      <c r="C41" s="51" t="str">
         <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
         <v/>
       </c>
-      <c r="D41" s="49"/>
+      <c r="D41" s="52"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="46"/>
+      <c r="A42" s="47"/>
       <c r="B42" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C42" s="48" t="str">
+      <c r="C42" s="51" t="str">
         <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
-      <c r="D42" s="49"/>
+      <c r="D42" s="52"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="46"/>
+      <c r="A43" s="47"/>
       <c r="B43" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C43" s="48" t="str">
+      <c r="C43" s="51" t="str">
         <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
-      <c r="D43" s="49"/>
+      <c r="D43" s="52"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="46"/>
+      <c r="A44" s="47"/>
       <c r="B44" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C44" s="48" t="str">
+      <c r="C44" s="51" t="str">
         <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
-      <c r="D44" s="49"/>
+      <c r="D44" s="52"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="46"/>
+      <c r="A45" s="47"/>
       <c r="B45" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C45" s="48" t="str">
+      <c r="C45" s="51" t="str">
         <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
-      <c r="D45" s="49"/>
+      <c r="D45" s="52"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="46"/>
+      <c r="A46" s="47"/>
       <c r="B46" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C46" s="48" t="str">
+      <c r="C46" s="51" t="str">
         <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
-      <c r="D46" s="49"/>
+      <c r="D46" s="52"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="46"/>
+      <c r="A47" s="47"/>
       <c r="B47" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C47" s="48" t="str">
+      <c r="C47" s="51" t="str">
         <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
-      <c r="D47" s="49"/>
+      <c r="D47" s="52"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="46"/>
+      <c r="A48" s="47"/>
       <c r="B48" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C48" s="48" t="str">
+      <c r="C48" s="51" t="str">
         <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
-      <c r="D48" s="49"/>
+      <c r="D48" s="52"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="46"/>
+      <c r="A49" s="47"/>
       <c r="B49" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C49" s="48" t="str">
+      <c r="C49" s="51" t="str">
         <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
-      <c r="D49" s="49"/>
+      <c r="D49" s="52"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="46"/>
+      <c r="A50" s="47"/>
       <c r="B50" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C50" s="48" t="str">
+      <c r="C50" s="51" t="str">
         <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
-      <c r="D50" s="49"/>
+      <c r="D50" s="52"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="46"/>
+      <c r="A51" s="47"/>
       <c r="B51" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C51" s="48" t="str">
+      <c r="C51" s="51" t="str">
         <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
-      <c r="D51" s="49"/>
+      <c r="D51" s="52"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="46"/>
+      <c r="A52" s="47"/>
       <c r="B52" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C52" s="48" t="str">
+      <c r="C52" s="51" t="str">
         <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
-      <c r="D52" s="49"/>
+      <c r="D52" s="52"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="46"/>
+      <c r="A53" s="47"/>
       <c r="B53" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C53" s="48" t="str">
+      <c r="C53" s="51" t="str">
         <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
-      <c r="D53" s="49"/>
+      <c r="D53" s="52"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="46"/>
+      <c r="A54" s="47"/>
       <c r="B54" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C54" s="48" t="str">
+      <c r="C54" s="51" t="str">
         <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
-      <c r="D54" s="49"/>
+      <c r="D54" s="52"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="46"/>
+      <c r="A55" s="47"/>
       <c r="B55" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C55" s="48" t="str">
+      <c r="C55" s="51" t="str">
         <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
-      <c r="D55" s="49"/>
+      <c r="D55" s="52"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="46"/>
+      <c r="A56" s="47"/>
       <c r="B56" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C56" s="48" t="str">
+      <c r="C56" s="51" t="str">
         <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
-      <c r="D56" s="49"/>
+      <c r="D56" s="52"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="46"/>
+      <c r="A57" s="47"/>
       <c r="B57" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C57" s="48" t="str">
+      <c r="C57" s="51" t="str">
         <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
-      <c r="D57" s="49"/>
+      <c r="D57" s="52"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="46"/>
+      <c r="A58" s="47"/>
       <c r="B58" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C58" s="48" t="str">
+      <c r="C58" s="51" t="str">
         <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
-      <c r="D58" s="49"/>
+      <c r="D58" s="52"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="46"/>
+      <c r="A59" s="47"/>
       <c r="B59" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C59" s="48" t="str">
+      <c r="C59" s="51" t="str">
         <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
-      <c r="D59" s="49"/>
+      <c r="D59" s="52"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="46"/>
+      <c r="A60" s="47"/>
       <c r="B60" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C60" s="48" t="str">
+      <c r="C60" s="51" t="str">
         <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
-      <c r="D60" s="49"/>
+      <c r="D60" s="52"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="46"/>
+      <c r="A61" s="47"/>
       <c r="B61" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C61" s="48" t="str">
+      <c r="C61" s="51" t="str">
         <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
-      <c r="D61" s="49"/>
+      <c r="D61" s="52"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="46"/>
+      <c r="A62" s="47"/>
       <c r="B62" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C62" s="48" t="str">
+      <c r="C62" s="51" t="str">
         <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
-      <c r="D62" s="49"/>
+      <c r="D62" s="52"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="46"/>
+      <c r="A63" s="47"/>
       <c r="B63" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C63" s="48" t="str">
+      <c r="C63" s="51" t="str">
         <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
-      <c r="D63" s="49"/>
+      <c r="D63" s="52"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="46"/>
+      <c r="A64" s="47"/>
       <c r="B64" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C64" s="48" t="str">
+      <c r="C64" s="51" t="str">
         <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
-      <c r="D64" s="49"/>
+      <c r="D64" s="52"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="46"/>
+      <c r="A65" s="47"/>
       <c r="B65" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C65" s="48" t="str">
+      <c r="C65" s="51" t="str">
         <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
-      <c r="D65" s="49"/>
+      <c r="D65" s="52"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="46"/>
+      <c r="A66" s="47"/>
       <c r="B66" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C66" s="48" t="str">
+      <c r="C66" s="51" t="str">
         <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
-      <c r="D66" s="49"/>
+      <c r="D66" s="52"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="46"/>
+      <c r="A67" s="47"/>
       <c r="B67" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C67" s="48" t="str">
+      <c r="C67" s="51" t="str">
         <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
-      <c r="D67" s="49"/>
+      <c r="D67" s="52"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="46"/>
+      <c r="A68" s="47"/>
       <c r="B68" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C68" s="48" t="str">
+      <c r="C68" s="51" t="str">
         <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
-      <c r="D68" s="49"/>
+      <c r="D68" s="52"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="46"/>
+      <c r="A69" s="47"/>
       <c r="B69" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C69" s="48" t="str">
+      <c r="C69" s="51" t="str">
         <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
-      <c r="D69" s="49"/>
+      <c r="D69" s="52"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="46"/>
+      <c r="A70" s="47"/>
       <c r="B70" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C70" s="48" t="str">
+      <c r="C70" s="51" t="str">
         <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
         <v/>
       </c>
-      <c r="D70" s="49"/>
+      <c r="D70" s="52"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="46"/>
+      <c r="A71" s="47"/>
       <c r="B71" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C71" s="48" t="str">
+      <c r="C71" s="51" t="str">
         <f aca="false">IF(Освіта!D13 = 0, "", Освіта!D13)</f>
         <v/>
       </c>
-      <c r="D71" s="49"/>
+      <c r="D71" s="52"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="46"/>
+      <c r="A72" s="47"/>
       <c r="B72" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C72" s="48" t="str">
+      <c r="C72" s="51" t="str">
         <f aca="false">IF(Освіта!E13 = 0, "", Освіта!E13)</f>
         <v/>
       </c>
-      <c r="D72" s="49"/>
+      <c r="D72" s="52"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="46"/>
+      <c r="A73" s="47"/>
       <c r="B73" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C73" s="48" t="str">
+      <c r="C73" s="51" t="str">
         <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
         <v/>
       </c>
-      <c r="D73" s="49"/>
+      <c r="D73" s="52"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="46"/>
+      <c r="A74" s="47"/>
       <c r="B74" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C74" s="48" t="str">
+      <c r="C74" s="51" t="str">
         <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
         <v/>
       </c>
-      <c r="D74" s="49"/>
+      <c r="D74" s="52"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="46"/>
+      <c r="A75" s="47"/>
       <c r="B75" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C75" s="48" t="str">
+      <c r="C75" s="51" t="str">
         <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
         <v/>
       </c>
-      <c r="D75" s="49"/>
+      <c r="D75" s="52"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="46"/>
+      <c r="A76" s="47"/>
       <c r="B76" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C76" s="48" t="str">
+      <c r="C76" s="51" t="str">
         <f aca="false">IF(Освіта!D14 = 0, "", Освіта!D14)</f>
         <v/>
       </c>
-      <c r="D76" s="49"/>
+      <c r="D76" s="52"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="46"/>
+      <c r="A77" s="47"/>
       <c r="B77" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C77" s="48" t="str">
+      <c r="C77" s="51" t="str">
         <f aca="false">IF(Освіта!E14 = 0, "", Освіта!E14)</f>
         <v/>
       </c>
-      <c r="D77" s="49"/>
+      <c r="D77" s="52"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="46"/>
+      <c r="A78" s="47"/>
       <c r="B78" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C78" s="48" t="str">
+      <c r="C78" s="51" t="str">
         <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
         <v/>
       </c>
-      <c r="D78" s="49"/>
+      <c r="D78" s="52"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="46"/>
+      <c r="A79" s="47"/>
       <c r="B79" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C79" s="48" t="str">
+      <c r="C79" s="51" t="str">
         <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
         <v/>
       </c>
-      <c r="D79" s="49"/>
+      <c r="D79" s="52"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="46"/>
+      <c r="A80" s="47"/>
       <c r="B80" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C80" s="48" t="str">
+      <c r="C80" s="51" t="str">
         <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
         <v/>
       </c>
-      <c r="D80" s="49"/>
+      <c r="D80" s="52"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="46"/>
+      <c r="A81" s="47"/>
       <c r="B81" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C81" s="48" t="str">
+      <c r="C81" s="51" t="str">
         <f aca="false">IF(Освіта!D15 = 0, "", Освіта!D15)</f>
         <v/>
       </c>
-      <c r="D81" s="49"/>
+      <c r="D81" s="52"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="46"/>
+      <c r="A82" s="47"/>
       <c r="B82" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C82" s="48" t="str">
+      <c r="C82" s="51" t="str">
         <f aca="false">IF(Освіта!E15 = 0, "", Освіта!E15)</f>
         <v/>
       </c>
-      <c r="D82" s="49"/>
+      <c r="D82" s="52"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="46"/>
+      <c r="A83" s="47"/>
       <c r="B83" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C83" s="48" t="str">
+      <c r="C83" s="51" t="str">
         <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
         <v/>
       </c>
-      <c r="D83" s="49"/>
+      <c r="D83" s="52"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="46"/>
+      <c r="A84" s="47"/>
       <c r="B84" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C84" s="48" t="str">
+      <c r="C84" s="51" t="str">
         <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
         <v/>
       </c>
-      <c r="D84" s="49"/>
+      <c r="D84" s="52"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="46"/>
+      <c r="A85" s="47"/>
       <c r="B85" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C85" s="48" t="str">
+      <c r="C85" s="51" t="str">
         <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
         <v/>
       </c>
-      <c r="D85" s="49"/>
+      <c r="D85" s="52"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="46"/>
+      <c r="A86" s="47"/>
       <c r="B86" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C86" s="48" t="str">
+      <c r="C86" s="51" t="str">
         <f aca="false">IF(Освіта!D16 = 0, "", Освіта!D16)</f>
         <v/>
       </c>
-      <c r="D86" s="49"/>
+      <c r="D86" s="52"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="46"/>
+      <c r="A87" s="47"/>
       <c r="B87" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C87" s="48" t="str">
+      <c r="C87" s="51" t="str">
         <f aca="false">IF(Освіта!E16 = 0, "", Освіта!E16)</f>
         <v/>
       </c>
-      <c r="D87" s="49"/>
+      <c r="D87" s="52"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="46"/>
+      <c r="A88" s="47"/>
       <c r="B88" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C88" s="48" t="str">
+      <c r="C88" s="51" t="str">
         <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
         <v/>
       </c>
-      <c r="D88" s="49"/>
+      <c r="D88" s="52"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="46"/>
+      <c r="A89" s="47"/>
       <c r="B89" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C89" s="48" t="str">
+      <c r="C89" s="51" t="str">
         <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
         <v/>
       </c>
-      <c r="D89" s="49"/>
+      <c r="D89" s="52"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="46"/>
+      <c r="A90" s="47"/>
       <c r="B90" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C90" s="48" t="str">
+      <c r="C90" s="51" t="str">
         <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
         <v/>
       </c>
-      <c r="D90" s="49"/>
+      <c r="D90" s="52"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="46"/>
+      <c r="A91" s="47"/>
       <c r="B91" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C91" s="48" t="str">
+      <c r="C91" s="51" t="str">
         <f aca="false">IF(Освіта!D17 = 0, "", Освіта!D17)</f>
         <v/>
       </c>
-      <c r="D91" s="49"/>
+      <c r="D91" s="52"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="46"/>
+      <c r="A92" s="47"/>
       <c r="B92" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C92" s="48" t="str">
+      <c r="C92" s="51" t="str">
         <f aca="false">IF(Освіта!E17 = 0, "", Освіта!E17)</f>
         <v/>
       </c>
-      <c r="D92" s="49"/>
+      <c r="D92" s="52"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="46"/>
+      <c r="A93" s="47"/>
       <c r="B93" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C93" s="48" t="str">
+      <c r="C93" s="51" t="str">
         <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
         <v/>
       </c>
-      <c r="D93" s="49"/>
+      <c r="D93" s="52"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="46"/>
+      <c r="A94" s="47"/>
       <c r="B94" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C94" s="48" t="str">
+      <c r="C94" s="51" t="str">
         <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
         <v/>
       </c>
-      <c r="D94" s="49"/>
+      <c r="D94" s="52"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="46"/>
+      <c r="A95" s="47"/>
       <c r="B95" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C95" s="48" t="str">
+      <c r="C95" s="51" t="str">
         <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
-      <c r="D95" s="49"/>
+      <c r="D95" s="52"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="46"/>
+      <c r="A96" s="47"/>
       <c r="B96" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C96" s="48" t="str">
+      <c r="C96" s="51" t="str">
         <f aca="false">IF(Освіта!D18 = 0, "", Освіта!D18)</f>
         <v/>
       </c>
-      <c r="D96" s="49"/>
+      <c r="D96" s="52"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="46"/>
+      <c r="A97" s="47"/>
       <c r="B97" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C97" s="48" t="str">
+      <c r="C97" s="51" t="str">
         <f aca="false">IF(Освіта!E18 = 0, "", Освіта!E18)</f>
         <v/>
       </c>
-      <c r="D97" s="49"/>
+      <c r="D97" s="52"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="46" t="s">
-        <v>104</v>
+      <c r="A98" s="47" t="s">
+        <v>106</v>
       </c>
       <c r="B98" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C98" s="48" t="str">
+      <c r="C98" s="51" t="str">
         <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
         <v/>
       </c>
-      <c r="D98" s="49"/>
+      <c r="D98" s="52"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="46"/>
+      <c r="A99" s="47"/>
       <c r="B99" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C99" s="48" t="str">
+      <c r="C99" s="51" t="str">
         <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
         <v/>
       </c>
-      <c r="D99" s="49"/>
+      <c r="D99" s="52"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="46"/>
+      <c r="A100" s="47"/>
       <c r="B100" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C100" s="48" t="str">
+      <c r="C100" s="51" t="str">
         <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
         <v/>
       </c>
-      <c r="D100" s="49"/>
+      <c r="D100" s="52"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="46"/>
+      <c r="A101" s="47"/>
       <c r="B101" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C101" s="48" t="str">
+      <c r="C101" s="51" t="str">
         <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
         <v/>
       </c>
-      <c r="D101" s="49"/>
+      <c r="D101" s="52"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="46"/>
+      <c r="A102" s="47"/>
       <c r="B102" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C102" s="48" t="str">
+      <c r="C102" s="51" t="str">
         <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
         <v/>
       </c>
-      <c r="D102" s="49"/>
+      <c r="D102" s="52"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="46"/>
+      <c r="A103" s="47"/>
       <c r="B103" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C103" s="48" t="str">
+      <c r="C103" s="51" t="str">
         <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
         <v/>
       </c>
-      <c r="D103" s="49"/>
+      <c r="D103" s="52"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="46"/>
+      <c r="A104" s="47"/>
       <c r="B104" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C104" s="48" t="str">
+      <c r="C104" s="51" t="str">
         <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
         <v/>
       </c>
-      <c r="D104" s="49"/>
+      <c r="D104" s="52"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="46"/>
+      <c r="A105" s="47"/>
       <c r="B105" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C105" s="48" t="str">
+      <c r="C105" s="51" t="str">
         <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
         <v/>
       </c>
-      <c r="D105" s="49"/>
+      <c r="D105" s="52"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="46"/>
+      <c r="A106" s="47"/>
       <c r="B106" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C106" s="48" t="str">
+      <c r="C106" s="51" t="str">
         <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
         <v/>
       </c>
-      <c r="D106" s="49"/>
+      <c r="D106" s="52"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="46"/>
+      <c r="A107" s="47"/>
       <c r="B107" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C107" s="48" t="str">
+      <c r="C107" s="51" t="str">
         <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
         <v/>
       </c>
-      <c r="D107" s="49"/>
+      <c r="D107" s="52"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="46"/>
+      <c r="A108" s="47"/>
       <c r="B108" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C108" s="48" t="str">
+      <c r="C108" s="51" t="str">
         <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
         <v/>
       </c>
-      <c r="D108" s="49"/>
+      <c r="D108" s="52"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="46"/>
+      <c r="A109" s="47"/>
       <c r="B109" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C109" s="48" t="str">
+      <c r="C109" s="51" t="str">
         <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
         <v/>
       </c>
-      <c r="D109" s="49"/>
+      <c r="D109" s="52"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="46"/>
+      <c r="A110" s="47"/>
       <c r="B110" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C110" s="48" t="str">
+      <c r="C110" s="51" t="str">
         <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
         <v/>
       </c>
-      <c r="D110" s="49"/>
+      <c r="D110" s="52"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="46"/>
+      <c r="A111" s="47"/>
       <c r="B111" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C111" s="48" t="str">
+      <c r="C111" s="51" t="str">
         <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
         <v/>
       </c>
-      <c r="D111" s="49"/>
+      <c r="D111" s="52"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="46"/>
+      <c r="A112" s="47"/>
       <c r="B112" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C112" s="48" t="str">
+      <c r="C112" s="51" t="str">
         <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
         <v/>
       </c>
-      <c r="D112" s="49"/>
+      <c r="D112" s="52"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="46"/>
+      <c r="A113" s="47"/>
       <c r="B113" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C113" s="48" t="str">
+      <c r="C113" s="51" t="str">
         <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
         <v/>
       </c>
-      <c r="D113" s="49"/>
+      <c r="D113" s="52"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="46"/>
+      <c r="A114" s="47"/>
       <c r="B114" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C114" s="48" t="str">
+      <c r="C114" s="51" t="str">
         <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
         <v/>
       </c>
-      <c r="D114" s="49"/>
+      <c r="D114" s="52"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="46"/>
+      <c r="A115" s="47"/>
       <c r="B115" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C115" s="48" t="str">
+      <c r="C115" s="51" t="str">
         <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
         <v/>
       </c>
-      <c r="D115" s="49"/>
+      <c r="D115" s="52"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="46" t="s">
-        <v>105</v>
+      <c r="A116" s="47" t="s">
+        <v>107</v>
       </c>
       <c r="B116" s="42" t="str">
         <f aca="false">Документи!A4</f>
         <v>Тип документу</v>
       </c>
-      <c r="C116" s="47" t="str">
+      <c r="C116" s="48" t="str">
         <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
         <v/>
       </c>
       <c r="D116" s="42"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="46"/>
+      <c r="A117" s="47"/>
       <c r="B117" s="42" t="str">
         <f aca="false">Документи!A5</f>
         <v>Серія та номер </v>
@@ -3598,7 +3951,7 @@
       <c r="D117" s="42"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="46"/>
+      <c r="A118" s="47"/>
       <c r="B118" s="42" t="str">
         <f aca="false">Документи!A6</f>
         <v>Ким виданий</v>
@@ -3610,7 +3963,7 @@
       <c r="D118" s="42"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="46"/>
+      <c r="A119" s="47"/>
       <c r="B119" s="42" t="str">
         <f aca="false">Документи!A7</f>
         <v>Дата видачі</v>
@@ -3622,19 +3975,19 @@
       <c r="D119" s="42"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="46"/>
+      <c r="A120" s="47"/>
       <c r="B120" s="42" t="str">
         <f aca="false">Документи!A10</f>
         <v>Тип документу</v>
       </c>
-      <c r="C120" s="47" t="str">
+      <c r="C120" s="48" t="str">
         <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
         <v/>
       </c>
       <c r="D120" s="42"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="46"/>
+      <c r="A121" s="47"/>
       <c r="B121" s="42" t="str">
         <f aca="false">Документи!A11</f>
         <v>Серія та номер </v>
@@ -3646,7 +3999,7 @@
       <c r="D121" s="42"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="46"/>
+      <c r="A122" s="47"/>
       <c r="B122" s="42" t="str">
         <f aca="false">Документи!A12</f>
         <v>Ким виданий</v>
@@ -3658,7 +4011,7 @@
       <c r="D122" s="42"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="46"/>
+      <c r="A123" s="47"/>
       <c r="B123" s="42" t="str">
         <f aca="false">Документи!A13</f>
         <v>Дата видачі</v>
@@ -3670,19 +4023,19 @@
       <c r="D123" s="42"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="46"/>
+      <c r="A124" s="47"/>
       <c r="B124" s="42" t="str">
         <f aca="false">Документи!A16</f>
         <v>Серія та номер </v>
       </c>
-      <c r="C124" s="47" t="str">
+      <c r="C124" s="48" t="str">
         <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
         <v/>
       </c>
       <c r="D124" s="42"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="46"/>
+      <c r="A125" s="47"/>
       <c r="B125" s="42" t="str">
         <f aca="false">Документи!A17</f>
         <v>Ким виданий</v>
@@ -3694,7 +4047,7 @@
       <c r="D125" s="42"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="46"/>
+      <c r="A126" s="47"/>
       <c r="B126" s="42" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
@@ -3706,7 +4059,70 @@
       <c r="D126" s="42"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B127" s="0"/>
+      <c r="D127" s="48"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D128" s="48"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D129" s="48"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D130" s="48"/>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D131" s="48"/>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D132" s="48"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D133" s="48"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D134" s="48"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D135" s="48"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D136" s="48"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D137" s="48"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D138" s="48"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D139" s="48"/>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D140" s="48"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D141" s="48"/>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D142" s="48"/>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D143" s="48"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D144" s="48"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D145" s="48"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D146" s="48"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D147" s="48"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D148" s="48"/>
     </row>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3719,13 +4135,22 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
+    <mergeCell ref="G1:M1"/>
     <mergeCell ref="A2:A24"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="G15:I15"/>
     <mergeCell ref="A25:A39"/>
     <mergeCell ref="A40:A97"/>
     <mergeCell ref="A98:A115"/>
     <mergeCell ref="A116:A126"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:I21" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
wip: excel drop-down lists | refactor: ElDataPreparer arrays filling
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="162">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -334,10 +334,172 @@
     <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
   </si>
   <si>
+    <t xml:space="preserve">Тип заповнення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва списку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значення</t>
+  </si>
+  <si>
     <t xml:space="preserve">Основна</t>
   </si>
   <si>
+    <t xml:space="preserve">Визначений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професійно-технічна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неповна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ІТС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">одружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неодружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">незаміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучена</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдова</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдівець</t>
+  </si>
+  <si>
+    <t xml:space="preserve">військовозобов'язаний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">призовник</t>
+  </si>
+  <si>
     <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">обмежено-придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">непридатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не перебуває</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТАК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">НІ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">денна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вечірня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заочна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">спеціаліст</t>
+  </si>
+  <si>
+    <t xml:space="preserve">бакалавр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">магістр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">кандидат наук</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PhD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">доцент</t>
+  </si>
+  <si>
+    <t xml:space="preserve">доктор наук</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">аспірантура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ад'юнктура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">докторантура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">дружина</t>
+  </si>
+  <si>
+    <t xml:space="preserve">чоловік</t>
+  </si>
+  <si>
+    <t xml:space="preserve">донька</t>
+  </si>
+  <si>
+    <t xml:space="preserve">син</t>
+  </si>
+  <si>
+    <t xml:space="preserve">донька подружжя</t>
+  </si>
+  <si>
+    <t xml:space="preserve">син подружжя</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу (паспорт)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паперовий паспорт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID картка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу (Військовий квіток)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квиток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Посвідчення особи офіцера</t>
+  </si>
+  <si>
+    <t xml:space="preserve">З бази даних</t>
   </si>
   <si>
     <t xml:space="preserve">Адреси Контакти</t>
@@ -557,7 +719,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="60">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -734,6 +896,10 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -746,6 +912,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -756,6 +930,22 @@
     </xf>
     <xf numFmtId="168" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2199,239 +2389,348 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M1048576"/>
+  <dimension ref="A1:X148"/>
   <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="43" width="23.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="53.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="29.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="31.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="19.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="44" width="37.54"/>
   </cols>
   <sheetData>
-    <row r="1" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" s="46" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="45" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="45" t="s">
+      <c r="B1" s="46" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="45" t="s">
+      <c r="C1" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="45" t="s">
+      <c r="D1" s="46" t="s">
         <v>100</v>
       </c>
       <c r="F1" s="2"/>
-      <c r="G1" s="46" t="s">
+      <c r="G1" s="47" t="s">
         <v>101</v>
       </c>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="O1" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="P1" s="49" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q1" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="47" t="s">
-        <v>102</v>
+      <c r="A2" s="50" t="s">
+        <v>105</v>
       </c>
       <c r="B2" s="42" t="str">
         <f aca="false">Основна!A9</f>
         <v>Прізвище</v>
       </c>
-      <c r="C2" s="48" t="str">
+      <c r="C2" s="51" t="str">
         <f aca="false">IF(Основна!B9 = 0, "",  Основна!B9)</f>
         <v/>
       </c>
       <c r="D2" s="42"/>
-      <c r="G2" s="49" t="n">
+      <c r="G2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="H2" s="49" t="n">
+      <c r="H2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="I2" s="49" t="n">
+      <c r="I2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="J2" s="49" t="n">
+      <c r="J2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="K2" s="49" t="n">
+      <c r="K2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="L2" s="49" t="n">
+      <c r="L2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="M2" s="49" t="n">
+      <c r="M2" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
+      <c r="O2" s="53" t="s">
+        <v>106</v>
+      </c>
+      <c r="P2" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="47"/>
+      <c r="A3" s="50"/>
       <c r="B3" s="42" t="str">
         <f aca="false">Основна!A10</f>
         <v>Ім’я</v>
       </c>
-      <c r="C3" s="48" t="str">
+      <c r="C3" s="51" t="str">
         <f aca="false">IF(Основна!B10 = 0, "",  Основна!B10)</f>
         <v/>
       </c>
       <c r="D3" s="42"/>
-      <c r="G3" s="49" t="n">
+      <c r="G3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="49" t="n">
+      <c r="H3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="I3" s="49" t="n">
+      <c r="I3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="J3" s="49" t="n">
+      <c r="J3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="K3" s="49" t="n">
+      <c r="K3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="L3" s="49" t="n">
+      <c r="L3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="M3" s="49" t="n">
+      <c r="M3" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
+      <c r="O3" s="53"/>
+      <c r="P3" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="47"/>
+      <c r="A4" s="50"/>
       <c r="B4" s="42" t="str">
         <f aca="false">Основна!A11</f>
         <v>По батькові </v>
       </c>
-      <c r="C4" s="48" t="str">
+      <c r="C4" s="51" t="str">
         <f aca="false">IF(Основна!B11 = 0, "",  Основна!B11)</f>
         <v/>
       </c>
       <c r="D4" s="42"/>
-      <c r="G4" s="49" t="n">
+      <c r="G4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="49" t="n">
+      <c r="H4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="I4" s="49" t="n">
+      <c r="I4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="49" t="n">
+      <c r="J4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="49" t="n">
+      <c r="K4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="L4" s="49" t="n">
+      <c r="L4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="M4" s="49" t="n">
+      <c r="M4" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
+      <c r="O4" s="53"/>
+      <c r="P4" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="47"/>
+      <c r="A5" s="50"/>
       <c r="B5" s="42" t="str">
         <f aca="false">Основна!A12</f>
         <v>Дата народження </v>
       </c>
-      <c r="C5" s="48" t="str">
+      <c r="C5" s="51" t="str">
         <f aca="false">IF(Основна!B12 = 0, "",  Основна!B12)</f>
         <v/>
       </c>
       <c r="D5" s="42"/>
-      <c r="G5" s="49" t="n">
+      <c r="G5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="49" t="n">
+      <c r="H5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="49" t="n">
+      <c r="I5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="49" t="n">
+      <c r="J5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="49" t="n">
+      <c r="K5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="49" t="n">
+      <c r="L5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="M5" s="49" t="n">
+      <c r="M5" s="52" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
+      <c r="O5" s="53"/>
+      <c r="P5" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="47"/>
+      <c r="A6" s="50"/>
       <c r="B6" s="42" t="str">
         <f aca="false">Основна!A13</f>
         <v>Громадянство</v>
       </c>
-      <c r="C6" s="48" t="str">
+      <c r="C6" s="51" t="str">
         <f aca="false">IF(Основна!B13 = 0, "",  Основна!B13)</f>
         <v>Україна</v>
       </c>
       <c r="D6" s="42"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="47"/>
+      <c r="A7" s="50"/>
       <c r="B7" s="42" t="str">
         <f aca="false">Основна!A14</f>
         <v>Освіта </v>
       </c>
-      <c r="C7" s="48" t="str">
+      <c r="C7" s="51" t="str">
         <f aca="false">IF(Основна!B14 = 0, "",  Основна!B14)</f>
         <v/>
       </c>
       <c r="D7" s="42"/>
-      <c r="G7" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="H7" s="46"/>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="G7" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="O7" s="53"/>
+      <c r="P7" s="54" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="47"/>
+      <c r="A8" s="50"/>
       <c r="B8" s="42" t="str">
         <f aca="false">Основна!A15</f>
         <v>ППС чи ІТС</v>
       </c>
-      <c r="C8" s="48" t="str">
+      <c r="C8" s="51" t="str">
         <f aca="false">IF(Основна!B15 = 0, "",  Основна!B15)</f>
         <v>ППС</v>
       </c>
@@ -2456,14 +2755,21 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="47"/>
+      <c r="O8" s="53"/>
+      <c r="P8" s="54" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="50"/>
       <c r="B9" s="42" t="str">
         <f aca="false">Основна!A16</f>
         <v>Науковий ступінь</v>
       </c>
-      <c r="C9" s="48" t="str">
+      <c r="C9" s="51" t="str">
         <f aca="false">IF(Основна!B16 = 0, "",  Основна!B16)</f>
         <v/>
       </c>
@@ -2488,14 +2794,24 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="47"/>
+      <c r="O9" s="53"/>
+      <c r="P9" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="50"/>
       <c r="B10" s="42" t="str">
         <f aca="false">Основна!A17</f>
         <v>Вчене звання</v>
       </c>
-      <c r="C10" s="48" t="str">
+      <c r="C10" s="51" t="str">
         <f aca="false">IF(Основна!B17 = 0, "",  Основна!B17)</f>
         <v/>
       </c>
@@ -2520,14 +2836,27 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
+      <c r="O10" s="53"/>
+      <c r="P10" s="54" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="47"/>
+      <c r="A11" s="50"/>
       <c r="B11" s="42" t="str">
         <f aca="false">Основна!A18</f>
         <v>Сімейний стан</v>
       </c>
-      <c r="C11" s="48" t="str">
+      <c r="C11" s="51" t="str">
         <f aca="false">IF(Основна!B18 = 0, "",  Основна!B18)</f>
         <v/>
       </c>
@@ -2552,14 +2881,27 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
+      <c r="O11" s="53"/>
+      <c r="P11" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="47"/>
+      <c r="A12" s="50"/>
       <c r="B12" s="42" t="str">
         <f aca="false">Основна!A21</f>
         <v>Інститут</v>
       </c>
-      <c r="C12" s="48" t="str">
+      <c r="C12" s="51" t="str">
         <f aca="false">IF(Основна!B21 = 0, "",  Основна!B21)</f>
         <v/>
       </c>
@@ -2584,9 +2926,28 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
+      <c r="O12" s="53"/>
+      <c r="P12" s="54" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="U12" s="2" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="47"/>
+      <c r="A13" s="50"/>
       <c r="B13" s="42" t="str">
         <f aca="false">Основна!A22</f>
         <v>Кафедра (відділ)</v>
@@ -2616,9 +2977,22 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
+      <c r="O13" s="53"/>
+      <c r="P13" s="54" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="47"/>
+      <c r="A14" s="50"/>
       <c r="B14" s="42" t="str">
         <f aca="false">Основна!A23</f>
         <v>Посада</v>
@@ -2628,9 +3002,31 @@
         <v/>
       </c>
       <c r="D14" s="42"/>
+      <c r="O14" s="53"/>
+      <c r="P14" s="54" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="U14" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="47"/>
+      <c r="A15" s="50"/>
       <c r="B15" s="42" t="str">
         <f aca="false">Основна!A24</f>
         <v>Номер наказу про призначення</v>
@@ -2640,14 +3036,24 @@
         <v/>
       </c>
       <c r="D15" s="42"/>
-      <c r="G15" s="46" t="s">
+      <c r="G15" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="O15" s="53"/>
+      <c r="P15" s="55" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q15" s="56" t="s">
+        <v>152</v>
+      </c>
+      <c r="R15" s="56" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="47"/>
+      <c r="A16" s="50"/>
       <c r="B16" s="42" t="str">
         <f aca="false">Основна!A25</f>
         <v>Дата наказу про призначення</v>
@@ -2657,21 +3063,31 @@
         <v/>
       </c>
       <c r="D16" s="42"/>
-      <c r="G16" s="50" t="n">
+      <c r="G16" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="50" t="n">
+      <c r="H16" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="50" t="n">
+      <c r="I16" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
+      <c r="O16" s="53"/>
+      <c r="P16" s="55" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q16" s="56" t="s">
+        <v>155</v>
+      </c>
+      <c r="R16" s="56" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="47"/>
+      <c r="A17" s="50"/>
       <c r="B17" s="42" t="str">
         <f aca="false">Основна!A28</f>
         <v>Група обліку</v>
@@ -2681,21 +3097,27 @@
         <v/>
       </c>
       <c r="D17" s="42"/>
-      <c r="G17" s="50" t="n">
+      <c r="G17" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="50" t="n">
+      <c r="H17" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
-      <c r="I17" s="50" t="n">
+      <c r="I17" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
+      <c r="O17" s="53" t="s">
+        <v>157</v>
+      </c>
+      <c r="P17" s="18" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47"/>
+      <c r="A18" s="50"/>
       <c r="B18" s="42" t="str">
         <f aca="false">Основна!A29</f>
         <v>Категорія обліку</v>
@@ -2705,21 +3127,25 @@
         <v/>
       </c>
       <c r="D18" s="42"/>
-      <c r="G18" s="50" t="n">
+      <c r="G18" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="50" t="n">
+      <c r="H18" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="50" t="n">
+      <c r="I18" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
+      <c r="O18" s="53"/>
+      <c r="P18" s="18" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47"/>
+      <c r="A19" s="50"/>
       <c r="B19" s="42" t="str">
         <f aca="false">Основна!A30</f>
         <v>Склад</v>
@@ -2729,21 +3155,25 @@
         <v/>
       </c>
       <c r="D19" s="42"/>
-      <c r="G19" s="50" t="n">
+      <c r="G19" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="50" t="n">
+      <c r="H19" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
-      <c r="I19" s="50" t="n">
+      <c r="I19" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
+      <c r="O19" s="53"/>
+      <c r="P19" s="18" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="47"/>
+      <c r="A20" s="50"/>
       <c r="B20" s="42" t="str">
         <f aca="false">Основна!A31</f>
         <v>Військове звання</v>
@@ -2753,21 +3183,25 @@
         <v/>
       </c>
       <c r="D20" s="42"/>
-      <c r="G20" s="50" t="n">
+      <c r="G20" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
-      <c r="H20" s="50" t="n">
+      <c r="H20" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
-      <c r="I20" s="50" t="n">
+      <c r="I20" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
+      <c r="O20" s="53"/>
+      <c r="P20" s="18" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="47"/>
+      <c r="A21" s="50"/>
       <c r="B21" s="42" t="str">
         <f aca="false">Основна!A32</f>
         <v>Військово-облікова спеціальність</v>
@@ -2777,21 +3211,25 @@
         <v/>
       </c>
       <c r="D21" s="42"/>
-      <c r="G21" s="50" t="n">
+      <c r="G21" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
-      <c r="H21" s="50" t="n">
+      <c r="H21" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
-      <c r="I21" s="50" t="n">
+      <c r="I21" s="57" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
+      <c r="O21" s="53"/>
+      <c r="P21" s="18" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="47"/>
+      <c r="A22" s="50"/>
       <c r="B22" s="42" t="str">
         <f aca="false">Основна!A33</f>
         <v> Придатність до військової служби</v>
@@ -2801,9 +3239,13 @@
         <v/>
       </c>
       <c r="D22" s="42"/>
+      <c r="O22" s="53"/>
+      <c r="P22" s="18" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="47"/>
+      <c r="A23" s="50"/>
       <c r="B23" s="42" t="str">
         <f aca="false">Основна!A34</f>
         <v>Териториальний центр комплектування та соціальної підтримки</v>
@@ -2813,9 +3255,13 @@
         <v/>
       </c>
       <c r="D23" s="42"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="47"/>
+      <c r="O23" s="53"/>
+      <c r="P23" s="18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="50"/>
       <c r="B24" s="42" t="str">
         <f aca="false">Основна!A35</f>
         <v>Перебування на спеціальному обліку</v>
@@ -2825,10 +3271,14 @@
         <v/>
       </c>
       <c r="D24" s="42"/>
+      <c r="O24" s="53"/>
+      <c r="P24" s="54" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="47" t="s">
-        <v>104</v>
+      <c r="A25" s="50" t="s">
+        <v>158</v>
       </c>
       <c r="B25" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A4</f>
@@ -2839,9 +3289,13 @@
         <v/>
       </c>
       <c r="D25" s="42"/>
+      <c r="O25" s="53"/>
+      <c r="P25" s="31" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="47"/>
+      <c r="A26" s="50"/>
       <c r="B26" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A5</f>
         <v>Область</v>
@@ -2851,9 +3305,13 @@
         <v/>
       </c>
       <c r="D26" s="42"/>
+      <c r="O26" s="53"/>
+      <c r="P26" s="28" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="47"/>
+      <c r="A27" s="50"/>
       <c r="B27" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A6</f>
         <v>Місто</v>
@@ -2863,9 +3321,13 @@
         <v/>
       </c>
       <c r="D27" s="42"/>
+      <c r="O27" s="53"/>
+      <c r="P27" s="28" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="47"/>
+      <c r="A28" s="50"/>
       <c r="B28" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A7</f>
         <v>Район (міста)</v>
@@ -2875,9 +3337,13 @@
         <v/>
       </c>
       <c r="D28" s="42"/>
+      <c r="O28" s="53"/>
+      <c r="P28" s="54" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="47"/>
+      <c r="A29" s="50"/>
       <c r="B29" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A8</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
@@ -2889,7 +3355,7 @@
       <c r="D29" s="42"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="47"/>
+      <c r="A30" s="50"/>
       <c r="B30" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A9</f>
         <v>Індекс</v>
@@ -2901,7 +3367,7 @@
       <c r="D30" s="42"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="47"/>
+      <c r="A31" s="50"/>
       <c r="B31" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A12</f>
         <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
@@ -2913,7 +3379,7 @@
       <c r="D31" s="42"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="47"/>
+      <c r="A32" s="50"/>
       <c r="B32" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A13</f>
         <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
@@ -2925,7 +3391,7 @@
       <c r="D32" s="42"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47"/>
+      <c r="A33" s="50"/>
       <c r="B33" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A16</f>
         <v>Співпадає із адресою фактичного проживання</v>
@@ -2937,7 +3403,7 @@
       <c r="D33" s="42"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47"/>
+      <c r="A34" s="50"/>
       <c r="B34" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A18</f>
         <v>Країна</v>
@@ -2949,7 +3415,7 @@
       <c r="D34" s="42"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="47"/>
+      <c r="A35" s="50"/>
       <c r="B35" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A19</f>
         <v>Область</v>
@@ -2961,7 +3427,7 @@
       <c r="D35" s="42"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="47"/>
+      <c r="A36" s="50"/>
       <c r="B36" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A20</f>
         <v>Місто</v>
@@ -2973,7 +3439,7 @@
       <c r="D36" s="42"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="47"/>
+      <c r="A37" s="50"/>
       <c r="B37" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A21</f>
         <v>Район (міста)</v>
@@ -2985,7 +3451,7 @@
       <c r="D37" s="42"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="47"/>
+      <c r="A38" s="50"/>
       <c r="B38" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A22</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
@@ -2997,7 +3463,7 @@
       <c r="D38" s="42"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="47"/>
+      <c r="A39" s="50"/>
       <c r="B39" s="42" t="str">
         <f aca="false">'Адреси Контакти'!A23</f>
         <v>Індекс</v>
@@ -3009,937 +3475,937 @@
       <c r="D39" s="42"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="47" t="s">
-        <v>105</v>
+      <c r="A40" s="50" t="s">
+        <v>159</v>
       </c>
       <c r="B40" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C40" s="51" t="str">
+      <c r="C40" s="58" t="str">
         <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
         <v/>
       </c>
-      <c r="D40" s="52"/>
+      <c r="D40" s="59"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="47"/>
+      <c r="A41" s="50"/>
       <c r="B41" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C41" s="51" t="str">
+      <c r="C41" s="58" t="str">
         <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
         <v/>
       </c>
-      <c r="D41" s="52"/>
+      <c r="D41" s="59"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="47"/>
+      <c r="A42" s="50"/>
       <c r="B42" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C42" s="51" t="str">
+      <c r="C42" s="58" t="str">
         <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
-      <c r="D42" s="52"/>
+      <c r="D42" s="59"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="47"/>
+      <c r="A43" s="50"/>
       <c r="B43" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C43" s="51" t="str">
+      <c r="C43" s="58" t="str">
         <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
-      <c r="D43" s="52"/>
+      <c r="D43" s="59"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="47"/>
+      <c r="A44" s="50"/>
       <c r="B44" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C44" s="51" t="str">
+      <c r="C44" s="58" t="str">
         <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
-      <c r="D44" s="52"/>
+      <c r="D44" s="59"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47"/>
+      <c r="A45" s="50"/>
       <c r="B45" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C45" s="51" t="str">
+      <c r="C45" s="58" t="str">
         <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
-      <c r="D45" s="52"/>
+      <c r="D45" s="59"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47"/>
+      <c r="A46" s="50"/>
       <c r="B46" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C46" s="51" t="str">
+      <c r="C46" s="58" t="str">
         <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
-      <c r="D46" s="52"/>
+      <c r="D46" s="59"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="47"/>
+      <c r="A47" s="50"/>
       <c r="B47" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C47" s="51" t="str">
+      <c r="C47" s="58" t="str">
         <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
-      <c r="D47" s="52"/>
+      <c r="D47" s="59"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="47"/>
+      <c r="A48" s="50"/>
       <c r="B48" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C48" s="51" t="str">
+      <c r="C48" s="58" t="str">
         <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
-      <c r="D48" s="52"/>
+      <c r="D48" s="59"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="47"/>
+      <c r="A49" s="50"/>
       <c r="B49" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C49" s="51" t="str">
+      <c r="C49" s="58" t="str">
         <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
-      <c r="D49" s="52"/>
+      <c r="D49" s="59"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="47"/>
+      <c r="A50" s="50"/>
       <c r="B50" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C50" s="51" t="str">
+      <c r="C50" s="58" t="str">
         <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
-      <c r="D50" s="52"/>
+      <c r="D50" s="59"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47"/>
+      <c r="A51" s="50"/>
       <c r="B51" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C51" s="51" t="str">
+      <c r="C51" s="58" t="str">
         <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
-      <c r="D51" s="52"/>
+      <c r="D51" s="59"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47"/>
+      <c r="A52" s="50"/>
       <c r="B52" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C52" s="51" t="str">
+      <c r="C52" s="58" t="str">
         <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
-      <c r="D52" s="52"/>
+      <c r="D52" s="59"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="47"/>
+      <c r="A53" s="50"/>
       <c r="B53" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C53" s="51" t="str">
+      <c r="C53" s="58" t="str">
         <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
-      <c r="D53" s="52"/>
+      <c r="D53" s="59"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="47"/>
+      <c r="A54" s="50"/>
       <c r="B54" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C54" s="51" t="str">
+      <c r="C54" s="58" t="str">
         <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
-      <c r="D54" s="52"/>
+      <c r="D54" s="59"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="47"/>
+      <c r="A55" s="50"/>
       <c r="B55" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C55" s="51" t="str">
+      <c r="C55" s="58" t="str">
         <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
-      <c r="D55" s="52"/>
+      <c r="D55" s="59"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="47"/>
+      <c r="A56" s="50"/>
       <c r="B56" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C56" s="51" t="str">
+      <c r="C56" s="58" t="str">
         <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
-      <c r="D56" s="52"/>
+      <c r="D56" s="59"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47"/>
+      <c r="A57" s="50"/>
       <c r="B57" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C57" s="51" t="str">
+      <c r="C57" s="58" t="str">
         <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
-      <c r="D57" s="52"/>
+      <c r="D57" s="59"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47"/>
+      <c r="A58" s="50"/>
       <c r="B58" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C58" s="51" t="str">
+      <c r="C58" s="58" t="str">
         <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
-      <c r="D58" s="52"/>
+      <c r="D58" s="59"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="47"/>
+      <c r="A59" s="50"/>
       <c r="B59" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C59" s="51" t="str">
+      <c r="C59" s="58" t="str">
         <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
-      <c r="D59" s="52"/>
+      <c r="D59" s="59"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="47"/>
+      <c r="A60" s="50"/>
       <c r="B60" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C60" s="51" t="str">
+      <c r="C60" s="58" t="str">
         <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
-      <c r="D60" s="52"/>
+      <c r="D60" s="59"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="47"/>
+      <c r="A61" s="50"/>
       <c r="B61" s="42" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C61" s="51" t="str">
+      <c r="C61" s="58" t="str">
         <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
-      <c r="D61" s="52"/>
+      <c r="D61" s="59"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="47"/>
+      <c r="A62" s="50"/>
       <c r="B62" s="42" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C62" s="51" t="str">
+      <c r="C62" s="58" t="str">
         <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
-      <c r="D62" s="52"/>
+      <c r="D62" s="59"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="47"/>
+      <c r="A63" s="50"/>
       <c r="B63" s="42" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C63" s="51" t="str">
+      <c r="C63" s="58" t="str">
         <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
-      <c r="D63" s="52"/>
+      <c r="D63" s="59"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="47"/>
+      <c r="A64" s="50"/>
       <c r="B64" s="42" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C64" s="51" t="str">
+      <c r="C64" s="58" t="str">
         <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
-      <c r="D64" s="52"/>
+      <c r="D64" s="59"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="47"/>
+      <c r="A65" s="50"/>
       <c r="B65" s="42" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C65" s="51" t="str">
+      <c r="C65" s="58" t="str">
         <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
-      <c r="D65" s="52"/>
+      <c r="D65" s="59"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="47"/>
+      <c r="A66" s="50"/>
       <c r="B66" s="42" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C66" s="51" t="str">
+      <c r="C66" s="58" t="str">
         <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
-      <c r="D66" s="52"/>
+      <c r="D66" s="59"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="47"/>
+      <c r="A67" s="50"/>
       <c r="B67" s="42" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C67" s="51" t="str">
+      <c r="C67" s="58" t="str">
         <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
-      <c r="D67" s="52"/>
+      <c r="D67" s="59"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="47"/>
+      <c r="A68" s="50"/>
       <c r="B68" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C68" s="51" t="str">
+      <c r="C68" s="58" t="str">
         <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
-      <c r="D68" s="52"/>
+      <c r="D68" s="59"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="47"/>
+      <c r="A69" s="50"/>
       <c r="B69" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C69" s="51" t="str">
+      <c r="C69" s="58" t="str">
         <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
-      <c r="D69" s="52"/>
+      <c r="D69" s="59"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="47"/>
+      <c r="A70" s="50"/>
       <c r="B70" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C70" s="51" t="str">
+      <c r="C70" s="58" t="str">
         <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
         <v/>
       </c>
-      <c r="D70" s="52"/>
+      <c r="D70" s="59"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="47"/>
+      <c r="A71" s="50"/>
       <c r="B71" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C71" s="51" t="str">
+      <c r="C71" s="58" t="str">
         <f aca="false">IF(Освіта!D13 = 0, "", Освіта!D13)</f>
         <v/>
       </c>
-      <c r="D71" s="52"/>
+      <c r="D71" s="59"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="47"/>
+      <c r="A72" s="50"/>
       <c r="B72" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C72" s="51" t="str">
+      <c r="C72" s="58" t="str">
         <f aca="false">IF(Освіта!E13 = 0, "", Освіта!E13)</f>
         <v/>
       </c>
-      <c r="D72" s="52"/>
+      <c r="D72" s="59"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="47"/>
+      <c r="A73" s="50"/>
       <c r="B73" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C73" s="51" t="str">
+      <c r="C73" s="58" t="str">
         <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
         <v/>
       </c>
-      <c r="D73" s="52"/>
+      <c r="D73" s="59"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="47"/>
+      <c r="A74" s="50"/>
       <c r="B74" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C74" s="51" t="str">
+      <c r="C74" s="58" t="str">
         <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
         <v/>
       </c>
-      <c r="D74" s="52"/>
+      <c r="D74" s="59"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="47"/>
+      <c r="A75" s="50"/>
       <c r="B75" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C75" s="51" t="str">
+      <c r="C75" s="58" t="str">
         <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
         <v/>
       </c>
-      <c r="D75" s="52"/>
+      <c r="D75" s="59"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="47"/>
+      <c r="A76" s="50"/>
       <c r="B76" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C76" s="51" t="str">
+      <c r="C76" s="58" t="str">
         <f aca="false">IF(Освіта!D14 = 0, "", Освіта!D14)</f>
         <v/>
       </c>
-      <c r="D76" s="52"/>
+      <c r="D76" s="59"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="47"/>
+      <c r="A77" s="50"/>
       <c r="B77" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C77" s="51" t="str">
+      <c r="C77" s="58" t="str">
         <f aca="false">IF(Освіта!E14 = 0, "", Освіта!E14)</f>
         <v/>
       </c>
-      <c r="D77" s="52"/>
+      <c r="D77" s="59"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="47"/>
+      <c r="A78" s="50"/>
       <c r="B78" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C78" s="51" t="str">
+      <c r="C78" s="58" t="str">
         <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
         <v/>
       </c>
-      <c r="D78" s="52"/>
+      <c r="D78" s="59"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="47"/>
+      <c r="A79" s="50"/>
       <c r="B79" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C79" s="51" t="str">
+      <c r="C79" s="58" t="str">
         <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
         <v/>
       </c>
-      <c r="D79" s="52"/>
+      <c r="D79" s="59"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="47"/>
+      <c r="A80" s="50"/>
       <c r="B80" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C80" s="51" t="str">
+      <c r="C80" s="58" t="str">
         <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
         <v/>
       </c>
-      <c r="D80" s="52"/>
+      <c r="D80" s="59"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="47"/>
+      <c r="A81" s="50"/>
       <c r="B81" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C81" s="51" t="str">
+      <c r="C81" s="58" t="str">
         <f aca="false">IF(Освіта!D15 = 0, "", Освіта!D15)</f>
         <v/>
       </c>
-      <c r="D81" s="52"/>
+      <c r="D81" s="59"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="47"/>
+      <c r="A82" s="50"/>
       <c r="B82" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C82" s="51" t="str">
+      <c r="C82" s="58" t="str">
         <f aca="false">IF(Освіта!E15 = 0, "", Освіта!E15)</f>
         <v/>
       </c>
-      <c r="D82" s="52"/>
+      <c r="D82" s="59"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="47"/>
+      <c r="A83" s="50"/>
       <c r="B83" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C83" s="51" t="str">
+      <c r="C83" s="58" t="str">
         <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
         <v/>
       </c>
-      <c r="D83" s="52"/>
+      <c r="D83" s="59"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="47"/>
+      <c r="A84" s="50"/>
       <c r="B84" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C84" s="51" t="str">
+      <c r="C84" s="58" t="str">
         <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
         <v/>
       </c>
-      <c r="D84" s="52"/>
+      <c r="D84" s="59"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="47"/>
+      <c r="A85" s="50"/>
       <c r="B85" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C85" s="51" t="str">
+      <c r="C85" s="58" t="str">
         <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
         <v/>
       </c>
-      <c r="D85" s="52"/>
+      <c r="D85" s="59"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="47"/>
+      <c r="A86" s="50"/>
       <c r="B86" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C86" s="51" t="str">
+      <c r="C86" s="58" t="str">
         <f aca="false">IF(Освіта!D16 = 0, "", Освіта!D16)</f>
         <v/>
       </c>
-      <c r="D86" s="52"/>
+      <c r="D86" s="59"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="47"/>
+      <c r="A87" s="50"/>
       <c r="B87" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C87" s="51" t="str">
+      <c r="C87" s="58" t="str">
         <f aca="false">IF(Освіта!E16 = 0, "", Освіта!E16)</f>
         <v/>
       </c>
-      <c r="D87" s="52"/>
+      <c r="D87" s="59"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="47"/>
+      <c r="A88" s="50"/>
       <c r="B88" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C88" s="51" t="str">
+      <c r="C88" s="58" t="str">
         <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
         <v/>
       </c>
-      <c r="D88" s="52"/>
+      <c r="D88" s="59"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="47"/>
+      <c r="A89" s="50"/>
       <c r="B89" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C89" s="51" t="str">
+      <c r="C89" s="58" t="str">
         <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
         <v/>
       </c>
-      <c r="D89" s="52"/>
+      <c r="D89" s="59"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="47"/>
+      <c r="A90" s="50"/>
       <c r="B90" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C90" s="51" t="str">
+      <c r="C90" s="58" t="str">
         <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
         <v/>
       </c>
-      <c r="D90" s="52"/>
+      <c r="D90" s="59"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="47"/>
+      <c r="A91" s="50"/>
       <c r="B91" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C91" s="51" t="str">
+      <c r="C91" s="58" t="str">
         <f aca="false">IF(Освіта!D17 = 0, "", Освіта!D17)</f>
         <v/>
       </c>
-      <c r="D91" s="52"/>
+      <c r="D91" s="59"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="47"/>
+      <c r="A92" s="50"/>
       <c r="B92" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C92" s="51" t="str">
+      <c r="C92" s="58" t="str">
         <f aca="false">IF(Освіта!E17 = 0, "", Освіта!E17)</f>
         <v/>
       </c>
-      <c r="D92" s="52"/>
+      <c r="D92" s="59"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="47"/>
+      <c r="A93" s="50"/>
       <c r="B93" s="42" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C93" s="51" t="str">
+      <c r="C93" s="58" t="str">
         <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
         <v/>
       </c>
-      <c r="D93" s="52"/>
+      <c r="D93" s="59"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="47"/>
+      <c r="A94" s="50"/>
       <c r="B94" s="42" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C94" s="51" t="str">
+      <c r="C94" s="58" t="str">
         <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
         <v/>
       </c>
-      <c r="D94" s="52"/>
+      <c r="D94" s="59"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="47"/>
+      <c r="A95" s="50"/>
       <c r="B95" s="42" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C95" s="51" t="str">
+      <c r="C95" s="58" t="str">
         <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
-      <c r="D95" s="52"/>
+      <c r="D95" s="59"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="47"/>
+      <c r="A96" s="50"/>
       <c r="B96" s="42" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C96" s="51" t="str">
+      <c r="C96" s="58" t="str">
         <f aca="false">IF(Освіта!D18 = 0, "", Освіта!D18)</f>
         <v/>
       </c>
-      <c r="D96" s="52"/>
+      <c r="D96" s="59"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="47"/>
+      <c r="A97" s="50"/>
       <c r="B97" s="42" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C97" s="51" t="str">
+      <c r="C97" s="58" t="str">
         <f aca="false">IF(Освіта!E18 = 0, "", Освіта!E18)</f>
         <v/>
       </c>
-      <c r="D97" s="52"/>
+      <c r="D97" s="59"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="47" t="s">
-        <v>106</v>
+      <c r="A98" s="50" t="s">
+        <v>160</v>
       </c>
       <c r="B98" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C98" s="51" t="str">
+      <c r="C98" s="58" t="str">
         <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
         <v/>
       </c>
-      <c r="D98" s="52"/>
+      <c r="D98" s="59"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="47"/>
+      <c r="A99" s="50"/>
       <c r="B99" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C99" s="51" t="str">
+      <c r="C99" s="58" t="str">
         <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
         <v/>
       </c>
-      <c r="D99" s="52"/>
+      <c r="D99" s="59"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="47"/>
+      <c r="A100" s="50"/>
       <c r="B100" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C100" s="51" t="str">
+      <c r="C100" s="58" t="str">
         <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
         <v/>
       </c>
-      <c r="D100" s="52"/>
+      <c r="D100" s="59"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="47"/>
+      <c r="A101" s="50"/>
       <c r="B101" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C101" s="51" t="str">
+      <c r="C101" s="58" t="str">
         <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
         <v/>
       </c>
-      <c r="D101" s="52"/>
+      <c r="D101" s="59"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="47"/>
+      <c r="A102" s="50"/>
       <c r="B102" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C102" s="51" t="str">
+      <c r="C102" s="58" t="str">
         <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
         <v/>
       </c>
-      <c r="D102" s="52"/>
+      <c r="D102" s="59"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="47"/>
+      <c r="A103" s="50"/>
       <c r="B103" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C103" s="51" t="str">
+      <c r="C103" s="58" t="str">
         <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
         <v/>
       </c>
-      <c r="D103" s="52"/>
+      <c r="D103" s="59"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="47"/>
+      <c r="A104" s="50"/>
       <c r="B104" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C104" s="51" t="str">
+      <c r="C104" s="58" t="str">
         <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
         <v/>
       </c>
-      <c r="D104" s="52"/>
+      <c r="D104" s="59"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="47"/>
+      <c r="A105" s="50"/>
       <c r="B105" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C105" s="51" t="str">
+      <c r="C105" s="58" t="str">
         <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
         <v/>
       </c>
-      <c r="D105" s="52"/>
+      <c r="D105" s="59"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="47"/>
+      <c r="A106" s="50"/>
       <c r="B106" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C106" s="51" t="str">
+      <c r="C106" s="58" t="str">
         <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
         <v/>
       </c>
-      <c r="D106" s="52"/>
+      <c r="D106" s="59"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="47"/>
+      <c r="A107" s="50"/>
       <c r="B107" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C107" s="51" t="str">
+      <c r="C107" s="58" t="str">
         <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
         <v/>
       </c>
-      <c r="D107" s="52"/>
+      <c r="D107" s="59"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="47"/>
+      <c r="A108" s="50"/>
       <c r="B108" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C108" s="51" t="str">
+      <c r="C108" s="58" t="str">
         <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
         <v/>
       </c>
-      <c r="D108" s="52"/>
+      <c r="D108" s="59"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="47"/>
+      <c r="A109" s="50"/>
       <c r="B109" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C109" s="51" t="str">
+      <c r="C109" s="58" t="str">
         <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
         <v/>
       </c>
-      <c r="D109" s="52"/>
+      <c r="D109" s="59"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="47"/>
+      <c r="A110" s="50"/>
       <c r="B110" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C110" s="51" t="str">
+      <c r="C110" s="58" t="str">
         <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
         <v/>
       </c>
-      <c r="D110" s="52"/>
+      <c r="D110" s="59"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="47"/>
+      <c r="A111" s="50"/>
       <c r="B111" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C111" s="51" t="str">
+      <c r="C111" s="58" t="str">
         <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
         <v/>
       </c>
-      <c r="D111" s="52"/>
+      <c r="D111" s="59"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="47"/>
+      <c r="A112" s="50"/>
       <c r="B112" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C112" s="51" t="str">
+      <c r="C112" s="58" t="str">
         <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
         <v/>
       </c>
-      <c r="D112" s="52"/>
+      <c r="D112" s="59"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="47"/>
+      <c r="A113" s="50"/>
       <c r="B113" s="42" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C113" s="51" t="str">
+      <c r="C113" s="58" t="str">
         <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
         <v/>
       </c>
-      <c r="D113" s="52"/>
+      <c r="D113" s="59"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="47"/>
+      <c r="A114" s="50"/>
       <c r="B114" s="42" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C114" s="51" t="str">
+      <c r="C114" s="58" t="str">
         <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
         <v/>
       </c>
-      <c r="D114" s="52"/>
+      <c r="D114" s="59"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="47"/>
+      <c r="A115" s="50"/>
       <c r="B115" s="42" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C115" s="51" t="str">
+      <c r="C115" s="58" t="str">
         <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
         <v/>
       </c>
-      <c r="D115" s="52"/>
+      <c r="D115" s="59"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="47" t="s">
-        <v>107</v>
+      <c r="A116" s="50" t="s">
+        <v>161</v>
       </c>
       <c r="B116" s="42" t="str">
         <f aca="false">Документи!A4</f>
         <v>Тип документу</v>
       </c>
-      <c r="C116" s="48" t="str">
+      <c r="C116" s="51" t="str">
         <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
         <v/>
       </c>
       <c r="D116" s="42"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="47"/>
+      <c r="A117" s="50"/>
       <c r="B117" s="42" t="str">
         <f aca="false">Документи!A5</f>
         <v>Серія та номер </v>
@@ -3951,7 +4417,7 @@
       <c r="D117" s="42"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="47"/>
+      <c r="A118" s="50"/>
       <c r="B118" s="42" t="str">
         <f aca="false">Документи!A6</f>
         <v>Ким виданий</v>
@@ -3963,7 +4429,7 @@
       <c r="D118" s="42"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="47"/>
+      <c r="A119" s="50"/>
       <c r="B119" s="42" t="str">
         <f aca="false">Документи!A7</f>
         <v>Дата видачі</v>
@@ -3975,19 +4441,19 @@
       <c r="D119" s="42"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="47"/>
+      <c r="A120" s="50"/>
       <c r="B120" s="42" t="str">
         <f aca="false">Документи!A10</f>
         <v>Тип документу</v>
       </c>
-      <c r="C120" s="48" t="str">
+      <c r="C120" s="51" t="str">
         <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
         <v/>
       </c>
       <c r="D120" s="42"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="47"/>
+      <c r="A121" s="50"/>
       <c r="B121" s="42" t="str">
         <f aca="false">Документи!A11</f>
         <v>Серія та номер </v>
@@ -3999,7 +4465,7 @@
       <c r="D121" s="42"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="47"/>
+      <c r="A122" s="50"/>
       <c r="B122" s="42" t="str">
         <f aca="false">Документи!A12</f>
         <v>Ким виданий</v>
@@ -4011,7 +4477,7 @@
       <c r="D122" s="42"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="47"/>
+      <c r="A123" s="50"/>
       <c r="B123" s="42" t="str">
         <f aca="false">Документи!A13</f>
         <v>Дата видачі</v>
@@ -4023,19 +4489,19 @@
       <c r="D123" s="42"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="47"/>
+      <c r="A124" s="50"/>
       <c r="B124" s="42" t="str">
         <f aca="false">Документи!A16</f>
         <v>Серія та номер </v>
       </c>
-      <c r="C124" s="48" t="str">
+      <c r="C124" s="51" t="str">
         <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
         <v/>
       </c>
       <c r="D124" s="42"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="47"/>
+      <c r="A125" s="50"/>
       <c r="B125" s="42" t="str">
         <f aca="false">Документи!A17</f>
         <v>Ким виданий</v>
@@ -4047,7 +4513,7 @@
       <c r="D125" s="42"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="47"/>
+      <c r="A126" s="50"/>
       <c r="B126" s="42" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
@@ -4059,87 +4525,80 @@
       <c r="D126" s="42"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D127" s="48"/>
+      <c r="D127" s="51"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D128" s="48"/>
+      <c r="D128" s="51"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D129" s="48"/>
+      <c r="D129" s="51"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D130" s="48"/>
+      <c r="D130" s="51"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D131" s="48"/>
+      <c r="D131" s="51"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D132" s="48"/>
+      <c r="D132" s="51"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D133" s="48"/>
+      <c r="D133" s="51"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D134" s="48"/>
+      <c r="D134" s="51"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D135" s="48"/>
+      <c r="D135" s="51"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D136" s="48"/>
+      <c r="D136" s="51"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D137" s="48"/>
+      <c r="D137" s="51"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D138" s="48"/>
+      <c r="D138" s="51"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D139" s="48"/>
+      <c r="D139" s="51"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D140" s="48"/>
+      <c r="D140" s="51"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D141" s="48"/>
+      <c r="D141" s="51"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D142" s="48"/>
+      <c r="D142" s="51"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D143" s="48"/>
+      <c r="D143" s="51"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D144" s="48"/>
+      <c r="D144" s="51"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D145" s="48"/>
+      <c r="D145" s="51"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D146" s="48"/>
+      <c r="D146" s="51"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D147" s="48"/>
+      <c r="D147" s="51"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D148" s="48"/>
-    </row>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="D148" s="51"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="11">
     <mergeCell ref="G1:M1"/>
+    <mergeCell ref="Q1:T1"/>
     <mergeCell ref="A2:A24"/>
+    <mergeCell ref="O2:O16"/>
     <mergeCell ref="G7:K7"/>
     <mergeCell ref="G15:I15"/>
+    <mergeCell ref="O17:O28"/>
     <mergeCell ref="A25:A39"/>
     <mergeCell ref="A40:A97"/>
     <mergeCell ref="A98:A115"/>

</xml_diff>

<commit_message>
feat: copy tables from global sheet to destination (education, posteducation, family)
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Довідка по заповненню" sheetId="1" state="visible" r:id="rId3"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="162">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -73,298 +73,298 @@
     <t xml:space="preserve">ППС чи ІТС</t>
   </si>
   <si>
+    <t xml:space="preserve">Науковий ступінь</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Stepen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вчене звання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Zvanie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сімейний стан</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПОСАДА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Інститут</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Fakultet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кафедра (відділ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Kafedra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Посада</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Dolghnost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Номер наказу про призначення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата наказу про призначення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВІДОМОСТІ ПРО ВІЙСЬКОВИЙ ОБЛІК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Група обліку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Категорія обліку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Склад</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (VSklad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військове звання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Vzvanie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військово-облікова спеціальність</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 цифр</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Придатність до військової служби</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Териториальний центр комплектування та соціальної підтримки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Voenkomat) із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Перебування на спеціальному обліку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">АДРЕСИ ТА КОНТАКТИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11. Місце фактичного проживання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Країна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Country)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Область</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (RegionUkraine) із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Місто</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Район (міста)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (RegionKharkiv) із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Адреса (вулиця, № будинку, квартири)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Індекс</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 цифр, не обовязкове</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Телефони</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (основний)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 цифр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12. Місце проживання за державною реєстрацією </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Співпадає із адресою фактичного проживання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва освітнього закладу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія та номер дисплома (свідоцтва)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік закінчення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Спеціальність (професія) за дипломом (свідоцтвом) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кваліфікація за дипломом (свідоцтвом)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Форма навчання (денна, вечірня, заочна)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівень освіти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Диплом, номер, дата видачі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Науковий ступінь, учене звання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівень підготовки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Склад родини</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПІБ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік народження</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри!!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ДОКУМЕНТИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія та номер </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ким виданий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата видачі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квіток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК224345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закордоний паспорт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: FF453210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва сторінки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва поля</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле для оновлення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле з актуальною інформацією</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип заповнення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва списку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Основна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Визначений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професійно-технічна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неповна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна вища</t>
+  </si>
+  <si>
     <t xml:space="preserve">ППС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Науковий ступінь</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Stepen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вчене звання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Zvanie)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сімейний стан</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПОСАДА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Інститут</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Fakultet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кафедра (відділ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Kafedra)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Посада</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Dolghnost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Номер наказу про призначення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата наказу про призначення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ВІДОМОСТІ ПРО ВІЙСЬКОВИЙ ОБЛІК</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Група обліку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Категорія обліку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Склад</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (VSklad)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військове звання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Vzvanie)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військово-облікова спеціальність</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 цифр</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Придатність до військової служби</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Териториальний центр комплектування та соціальної підтримки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Voenkomat) із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Перебування на спеціальному обліку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">АДРЕСИ ТА КОНТАКТИ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11. Місце фактичного проживання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Країна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Country)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Область</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (RegionUkraine) із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Місто</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Район (міста)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (RegionKharkiv) із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адреса (вулиця, № будинку, квартири)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Індекс</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 цифр, не обовязкове</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Телефони</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (основний)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 цифр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12. Місце проживання за державною реєстрацією </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Співпадає із адресою фактичного проживання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва освітнього закладу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія та номер дисплома (свідоцтва)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік закінчення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Спеціальність (професія) за дипломом (свідоцтвом) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кваліфікація за дипломом (свідоцтвом)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Форма навчання (денна, вечірня, заочна)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рівень освіти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Диплом, номер, дата видачі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Науковий ступінь, учене звання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рівень підготовки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Склад родини</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПІБ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік народження</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри!!!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДОКУМЕНТИ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип документу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія та номер </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ким виданий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата видачі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військовий квіток</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК224345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закордоний паспорт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: FF453210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва сторінки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва поля</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле для оновлення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле з актуальною інформацією</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип заповнення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва списку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Значення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Основна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Визначений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">професійно-технічна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неповна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна вища</t>
   </si>
   <si>
     <t xml:space="preserve">ІТС</t>
@@ -719,7 +719,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -864,18 +864,14 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -896,10 +892,6 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -928,7 +920,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -952,11 +944,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1230,7 +1222,7 @@
   <dimension ref="A2:D1048576"/>
   <sheetFormatPr defaultColWidth="8.62890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="31.08"/>
   </cols>
@@ -1341,9 +1333,7 @@
       <c r="A15" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>15</v>
-      </c>
+      <c r="B15" s="13"/>
       <c r="C15" s="2" t="str">
         <f aca="false">IF('Системна інформація'!D8 = 0, "", 'Системна інформація'!D8)</f>
         <v/>
@@ -1354,7 +1344,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" s="12"/>
       <c r="C16" s="2" t="str">
@@ -1362,12 +1352,12 @@
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="2" t="str">
@@ -1375,12 +1365,12 @@
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="2" t="str">
@@ -1397,13 +1387,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="2" t="str">
@@ -1411,12 +1401,12 @@
         <v/>
       </c>
       <c r="D21" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="2" t="str">
@@ -1424,12 +1414,12 @@
         <v/>
       </c>
       <c r="D22" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="2" t="str">
@@ -1437,12 +1427,12 @@
         <v/>
       </c>
       <c r="D23" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="2" t="str">
@@ -1450,12 +1440,12 @@
         <v/>
       </c>
       <c r="D24" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="2" t="str">
@@ -1471,13 +1461,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="2" t="str">
@@ -1490,7 +1480,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="2" t="str">
@@ -1503,7 +1493,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B30" s="12"/>
       <c r="C30" s="2" t="str">
@@ -1511,12 +1501,12 @@
         <v/>
       </c>
       <c r="D30" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="2" t="str">
@@ -1524,12 +1514,12 @@
         <v/>
       </c>
       <c r="D31" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B32" s="19"/>
       <c r="C32" s="2" t="str">
@@ -1537,12 +1527,12 @@
         <v/>
       </c>
       <c r="D32" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B33" s="12"/>
       <c r="C33" s="2" t="str">
@@ -1550,12 +1540,12 @@
         <v/>
       </c>
       <c r="D33" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="2" t="str">
@@ -1563,12 +1553,12 @@
         <v/>
       </c>
       <c r="D34" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="2" t="str">
@@ -1576,42 +1566,74 @@
         <v/>
       </c>
       <c r="D35" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B15" type="list">
-      <formula1>"ППС,ІТС"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B31" type="list">
-      <formula1>"полковник,підполковник,майор,капітан,ст.лейтенант,лейтенант,мол.лейтенант"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B14" type="list">
-      <formula1>"базова загальна середня,повна загальна середня,професійно-технічна,неповна вища,базова вища,повна вища"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B18" type="list">
-      <formula1>"одружений,неодружений,заміжня,незаміжня,розлучений,розлучена,вдова,вдівець"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
+  <dataValidations count="16">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B29" type="list">
       <formula1>"1,2"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="B35" type="list">
-      <formula1>"Не перебуває"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B22" type="list">
+      <formula1>'Системна інформація'!$Q$20:$ZA$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="B33" type="list">
-      <formula1>"придатний,обмежено-придатний,непридатний"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B14" type="list">
+      <formula1>'Системна інформація'!$Q$2:$ZA$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B28" type="list">
-      <formula1>"військовозобов'язаний,призовник"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B15" type="list">
+      <formula1>'Системна інформація'!$Q$3:$ZA$3</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B16" type="list">
+      <formula1>'Системна інформація'!$Q$17:$ZA$17</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B17" type="list">
+      <formula1>'Системна інформація'!$Q$18:$ZA$18</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B18" type="list">
+      <formula1>'Системна інформація'!$Q$4:$ZA$4</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B24" type="list">
+      <formula1>'Системна інформація'!$Q$21:$ZA$21</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B28" type="list">
+      <formula1>'Системна інформація'!$Q$5:$ZA$5</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність свого інституту в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого інституту ще не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B21" type="list">
+      <formula1>'Системна інформація'!$Q$19:$ZA$19</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність своєї посади в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такої посади поки не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B23" type="list">
+      <formula1>'Системна інформація'!$Q$21:$ZA$21</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B30" type="list">
+      <formula1>'Системна інформація'!$Q$22:$ZA$22</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B31" type="list">
+      <formula1>'Системна інформація'!$Q$23:$ZA$23</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="B33" type="list">
+      <formula1>'Системна інформація'!$Q$7:$ZA$7</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність свого ТЦК в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого ТЦК поки не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B34" type="list">
+      <formula1>'Системна інформація'!$Q$24:$ZA$24</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="B35" type="list">
+      <formula1>'Системна інформація'!$Q$8:$ZA$8</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1641,12 +1663,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="22"/>
@@ -1654,7 +1676,7 @@
     </row>
     <row r="4" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="25"/>
       <c r="C4" s="22" t="str">
@@ -1662,12 +1684,12 @@
         <v/>
       </c>
       <c r="D4" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="27"/>
       <c r="C5" s="22" t="str">
@@ -1675,12 +1697,12 @@
         <v/>
       </c>
       <c r="D5" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="22" t="str">
@@ -1688,12 +1710,12 @@
         <v/>
       </c>
       <c r="D6" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="27"/>
       <c r="C7" s="22" t="str">
@@ -1701,12 +1723,12 @@
         <v/>
       </c>
       <c r="D7" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" s="27"/>
       <c r="C8" s="22" t="str">
@@ -1716,7 +1738,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B9" s="27"/>
       <c r="C9" s="22" t="str">
@@ -1724,7 +1746,7 @@
         <v/>
       </c>
       <c r="D9" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1734,7 +1756,7 @@
     </row>
     <row r="11" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="2"/>
@@ -1742,7 +1764,7 @@
     </row>
     <row r="12" s="23" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B12" s="27"/>
       <c r="C12" s="22" t="str">
@@ -1750,12 +1772,12 @@
         <v/>
       </c>
       <c r="D12" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" s="23" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="22" t="str">
@@ -1763,7 +1785,7 @@
         <v/>
       </c>
       <c r="D13" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,7 +1796,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="2"/>
@@ -1782,7 +1804,7 @@
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" s="25"/>
       <c r="C16" s="22" t="str">
@@ -1801,7 +1823,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B18" s="25"/>
       <c r="C18" s="22" t="str">
@@ -1809,12 +1831,12 @@
         <v/>
       </c>
       <c r="D18" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="22" t="str">
@@ -1822,12 +1844,12 @@
         <v/>
       </c>
       <c r="D19" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="22" t="str">
@@ -1835,12 +1857,12 @@
         <v/>
       </c>
       <c r="D20" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="22" t="str">
@@ -1848,12 +1870,12 @@
         <v/>
       </c>
       <c r="D21" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="22" t="str">
@@ -1863,7 +1885,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B23" s="27"/>
       <c r="C23" s="22" t="str">
@@ -1871,7 +1893,7 @@
         <v/>
       </c>
       <c r="D23" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1915,76 +1937,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="C4" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="D4" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="E4" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="F4" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="G4" s="34" t="s">
         <v>70</v>
-      </c>
-      <c r="G4" s="34" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="35"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="35"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="35"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>13</v>
@@ -1995,71 +2017,71 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="C12" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12" s="34" t="s">
+      <c r="E12" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="33" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="38"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
+      <c r="A13" s="36"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="38"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
+      <c r="A14" s="36"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38"/>
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
+      <c r="A16" s="36"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>13</v>
@@ -2069,15 +2091,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F5:F8" type="list">
-      <formula1>"денна,вечірня,заочна"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G5:G8" type="list">
-      <formula1>"спеціаліст,бакалавр,магістр"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E13:E18" type="list">
       <formula1>"аспірантура,ад'юнктура,докторантура"</formula1>
       <formula2>0</formula2>
@@ -2112,63 +2126,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="38" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="C4" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="34" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="38"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="38"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
+      <c r="A6" s="36"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="38"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="A8" s="36"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="38"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
+      <c r="A9" s="36"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="38"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
+      <c r="A10" s="36"/>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2205,17 +2219,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="40" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="41" t="s">
-        <v>86</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="2" t="str">
@@ -2227,8 +2241,8 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="42" t="s">
-        <v>87</v>
+      <c r="A5" s="41" t="s">
+        <v>86</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="2" t="str">
@@ -2236,12 +2250,12 @@
         <v/>
       </c>
       <c r="D5" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="41" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="42" t="s">
-        <v>89</v>
       </c>
       <c r="B6" s="14"/>
       <c r="C6" s="2" t="str">
@@ -2249,12 +2263,12 @@
         <v/>
       </c>
       <c r="D6" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="41" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="42" t="s">
-        <v>91</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="2" t="str">
@@ -2267,12 +2281,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="41" t="s">
-        <v>86</v>
+      <c r="A10" s="40" t="s">
+        <v>85</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="2" t="str">
@@ -2284,8 +2298,8 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="42" t="s">
-        <v>87</v>
+      <c r="A11" s="41" t="s">
+        <v>86</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="2" t="str">
@@ -2293,12 +2307,12 @@
         <v/>
       </c>
       <c r="D11" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="42" t="s">
-        <v>89</v>
+      <c r="A12" s="41" t="s">
+        <v>88</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="2" t="str">
@@ -2307,8 +2321,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="42" t="s">
-        <v>91</v>
+      <c r="A13" s="41" t="s">
+        <v>90</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="2" t="str">
@@ -2321,12 +2335,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="42" t="s">
-        <v>87</v>
+      <c r="A16" s="41" t="s">
+        <v>86</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="2" t="str">
@@ -2334,12 +2348,12 @@
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="42" t="s">
-        <v>89</v>
+      <c r="A17" s="41" t="s">
+        <v>88</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="2" t="str">
@@ -2347,12 +2361,12 @@
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="42" t="s">
-        <v>91</v>
+      <c r="A18" s="41" t="s">
+        <v>90</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="2" t="str">
@@ -2392,208 +2406,208 @@
   <dimension ref="A1:X148"/>
   <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="43" width="23.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="42" width="23.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="53.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="29.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="31.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="19.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="44" width="37.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="19.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="37.54"/>
   </cols>
   <sheetData>
-    <row r="1" s="46" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="45" t="s">
+    <row r="1" s="44" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="44" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="C1" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="D1" s="44" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="45" t="s">
         <v>100</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="47" t="s">
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="O1" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="O1" s="48" t="s">
+      <c r="P1" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="P1" s="49" t="s">
+      <c r="Q1" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="Q1" s="48" t="s">
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="50" t="s">
-        <v>105</v>
-      </c>
-      <c r="B2" s="42" t="str">
+      <c r="B2" s="41" t="str">
         <f aca="false">Основна!A9</f>
         <v>Прізвище</v>
       </c>
-      <c r="C2" s="51" t="str">
+      <c r="C2" s="49" t="str">
         <f aca="false">IF(Основна!B9 = 0, "",  Основна!B9)</f>
         <v/>
       </c>
-      <c r="D2" s="42"/>
-      <c r="G2" s="52" t="n">
+      <c r="D2" s="41"/>
+      <c r="G2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="H2" s="52" t="n">
+      <c r="H2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="I2" s="52" t="n">
+      <c r="I2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="J2" s="52" t="n">
+      <c r="J2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="K2" s="52" t="n">
+      <c r="K2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="L2" s="52" t="n">
+      <c r="L2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="M2" s="52" t="n">
+      <c r="M2" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
-      <c r="O2" s="53" t="s">
-        <v>106</v>
+      <c r="O2" s="51" t="s">
+        <v>105</v>
       </c>
       <c r="P2" s="18" t="s">
         <v>12</v>
       </c>
       <c r="Q2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="V2" s="2" t="s">
-        <v>112</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="50"/>
-      <c r="B3" s="42" t="str">
+      <c r="A3" s="48"/>
+      <c r="B3" s="41" t="str">
         <f aca="false">Основна!A10</f>
         <v>Ім’я</v>
       </c>
-      <c r="C3" s="51" t="str">
+      <c r="C3" s="49" t="str">
         <f aca="false">IF(Основна!B10 = 0, "",  Основна!B10)</f>
         <v/>
       </c>
-      <c r="D3" s="42"/>
-      <c r="G3" s="52" t="n">
+      <c r="D3" s="41"/>
+      <c r="G3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="52" t="n">
+      <c r="H3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="I3" s="52" t="n">
+      <c r="I3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="J3" s="52" t="n">
+      <c r="J3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="K3" s="52" t="n">
+      <c r="K3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="L3" s="52" t="n">
+      <c r="L3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="M3" s="52" t="n">
+      <c r="M3" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
-      <c r="O3" s="53"/>
+      <c r="O3" s="51"/>
       <c r="P3" s="18" t="s">
         <v>14</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>15</v>
+        <v>112</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="50"/>
-      <c r="B4" s="42" t="str">
+      <c r="A4" s="48"/>
+      <c r="B4" s="41" t="str">
         <f aca="false">Основна!A11</f>
         <v>По батькові </v>
       </c>
-      <c r="C4" s="51" t="str">
+      <c r="C4" s="49" t="str">
         <f aca="false">IF(Основна!B11 = 0, "",  Основна!B11)</f>
         <v/>
       </c>
-      <c r="D4" s="42"/>
-      <c r="G4" s="52" t="n">
+      <c r="D4" s="41"/>
+      <c r="G4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="52" t="n">
+      <c r="H4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="I4" s="52" t="n">
+      <c r="I4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="52" t="n">
+      <c r="J4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="52" t="n">
+      <c r="K4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="L4" s="52" t="n">
+      <c r="L4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="M4" s="52" t="n">
+      <c r="M4" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
-      <c r="O4" s="53"/>
+      <c r="O4" s="51"/>
       <c r="P4" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>114</v>
@@ -2621,47 +2635,47 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="50"/>
-      <c r="B5" s="42" t="str">
+      <c r="A5" s="48"/>
+      <c r="B5" s="41" t="str">
         <f aca="false">Основна!A12</f>
         <v>Дата народження </v>
       </c>
-      <c r="C5" s="51" t="str">
+      <c r="C5" s="49" t="str">
         <f aca="false">IF(Основна!B12 = 0, "",  Основна!B12)</f>
         <v/>
       </c>
-      <c r="D5" s="42"/>
-      <c r="G5" s="52" t="n">
+      <c r="D5" s="41"/>
+      <c r="G5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="52" t="n">
+      <c r="H5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="52" t="n">
+      <c r="I5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="52" t="n">
+      <c r="J5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="52" t="n">
+      <c r="K5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="52" t="n">
+      <c r="L5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="M5" s="52" t="n">
+      <c r="M5" s="50" t="n">
         <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="53"/>
+      <c r="O5" s="51"/>
       <c r="P5" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>122</v>
@@ -2671,19 +2685,19 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="50"/>
-      <c r="B6" s="42" t="str">
+      <c r="A6" s="48"/>
+      <c r="B6" s="41" t="str">
         <f aca="false">Основна!A13</f>
         <v>Громадянство</v>
       </c>
-      <c r="C6" s="51" t="str">
+      <c r="C6" s="49" t="str">
         <f aca="false">IF(Основна!B13 = 0, "",  Основна!B13)</f>
         <v>Україна</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="O6" s="53"/>
+      <c r="D6" s="41"/>
+      <c r="O6" s="51"/>
       <c r="P6" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>1</v>
@@ -2693,26 +2707,26 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="50"/>
-      <c r="B7" s="42" t="str">
+      <c r="A7" s="48"/>
+      <c r="B7" s="41" t="str">
         <f aca="false">Основна!A14</f>
         <v>Освіта </v>
       </c>
-      <c r="C7" s="51" t="str">
+      <c r="C7" s="49" t="str">
         <f aca="false">IF(Основна!B14 = 0, "",  Основна!B14)</f>
         <v/>
       </c>
-      <c r="D7" s="42"/>
-      <c r="G7" s="47" t="s">
+      <c r="D7" s="41"/>
+      <c r="G7" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="H7" s="47"/>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
-      <c r="K7" s="47"/>
-      <c r="O7" s="53"/>
-      <c r="P7" s="54" t="s">
-        <v>40</v>
+      <c r="H7" s="45"/>
+      <c r="I7" s="45"/>
+      <c r="J7" s="45"/>
+      <c r="K7" s="45"/>
+      <c r="O7" s="51"/>
+      <c r="P7" s="52" t="s">
+        <v>39</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>125</v>
@@ -2725,16 +2739,16 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="50"/>
-      <c r="B8" s="42" t="str">
+      <c r="A8" s="48"/>
+      <c r="B8" s="41" t="str">
         <f aca="false">Основна!A15</f>
         <v>ППС чи ІТС</v>
       </c>
-      <c r="C8" s="51" t="str">
+      <c r="C8" s="49" t="str">
         <f aca="false">IF(Основна!B15 = 0, "",  Основна!B15)</f>
-        <v>ППС</v>
-      </c>
-      <c r="D8" s="42"/>
+        <v/>
+      </c>
+      <c r="D8" s="41"/>
       <c r="G8" s="25" t="n">
         <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
@@ -2755,25 +2769,25 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
-      <c r="O8" s="53"/>
-      <c r="P8" s="54" t="s">
-        <v>44</v>
+      <c r="O8" s="51"/>
+      <c r="P8" s="52" t="s">
+        <v>43</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="50"/>
-      <c r="B9" s="42" t="str">
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="48"/>
+      <c r="B9" s="41" t="str">
         <f aca="false">Основна!A16</f>
         <v>Науковий ступінь</v>
       </c>
-      <c r="C9" s="51" t="str">
+      <c r="C9" s="49" t="str">
         <f aca="false">IF(Основна!B16 = 0, "",  Основна!B16)</f>
         <v/>
       </c>
-      <c r="D9" s="42"/>
+      <c r="D9" s="41"/>
       <c r="G9" s="25" t="n">
         <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
@@ -2794,9 +2808,9 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
-      <c r="O9" s="53"/>
+      <c r="O9" s="51"/>
       <c r="P9" s="31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>129</v>
@@ -2805,17 +2819,17 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="50"/>
-      <c r="B10" s="42" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="48"/>
+      <c r="B10" s="41" t="str">
         <f aca="false">Основна!A17</f>
         <v>Вчене звання</v>
       </c>
-      <c r="C10" s="51" t="str">
+      <c r="C10" s="49" t="str">
         <f aca="false">IF(Основна!B17 = 0, "",  Основна!B17)</f>
         <v/>
       </c>
-      <c r="D10" s="42"/>
+      <c r="D10" s="41"/>
       <c r="G10" s="25" t="n">
         <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
@@ -2836,9 +2850,9 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="53"/>
-      <c r="P10" s="54" t="s">
-        <v>70</v>
+      <c r="O10" s="51"/>
+      <c r="P10" s="52" t="s">
+        <v>69</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>131</v>
@@ -2851,16 +2865,16 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="50"/>
-      <c r="B11" s="42" t="str">
+      <c r="A11" s="48"/>
+      <c r="B11" s="41" t="str">
         <f aca="false">Основна!A18</f>
         <v>Сімейний стан</v>
       </c>
-      <c r="C11" s="51" t="str">
+      <c r="C11" s="49" t="str">
         <f aca="false">IF(Основна!B18 = 0, "",  Основна!B18)</f>
         <v/>
       </c>
-      <c r="D11" s="42"/>
+      <c r="D11" s="41"/>
       <c r="G11" s="25" t="n">
         <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
@@ -2881,9 +2895,9 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
-      <c r="O11" s="53"/>
-      <c r="P11" s="54" t="s">
-        <v>71</v>
+      <c r="O11" s="51"/>
+      <c r="P11" s="52" t="s">
+        <v>70</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>134</v>
@@ -2896,16 +2910,16 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="50"/>
-      <c r="B12" s="42" t="str">
+      <c r="A12" s="48"/>
+      <c r="B12" s="41" t="str">
         <f aca="false">Основна!A21</f>
         <v>Інститут</v>
       </c>
-      <c r="C12" s="51" t="str">
+      <c r="C12" s="49" t="str">
         <f aca="false">IF(Основна!B21 = 0, "",  Основна!B21)</f>
         <v/>
       </c>
-      <c r="D12" s="42"/>
+      <c r="D12" s="41"/>
       <c r="G12" s="25" t="n">
         <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
@@ -2926,9 +2940,9 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
-      <c r="O12" s="53"/>
-      <c r="P12" s="54" t="s">
-        <v>76</v>
+      <c r="O12" s="51"/>
+      <c r="P12" s="52" t="s">
+        <v>75</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>137</v>
@@ -2947,16 +2961,16 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="50"/>
-      <c r="B13" s="42" t="str">
+      <c r="A13" s="48"/>
+      <c r="B13" s="41" t="str">
         <f aca="false">Основна!A22</f>
         <v>Кафедра (відділ)</v>
       </c>
-      <c r="C13" s="42" t="str">
+      <c r="C13" s="41" t="str">
         <f aca="false">IF(Основна!B22 = 0, "",  Основна!B22)</f>
         <v/>
       </c>
-      <c r="D13" s="42"/>
+      <c r="D13" s="41"/>
       <c r="G13" s="25" t="n">
         <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
@@ -2977,9 +2991,9 @@
         <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
-      <c r="O13" s="53"/>
-      <c r="P13" s="54" t="s">
-        <v>77</v>
+      <c r="O13" s="51"/>
+      <c r="P13" s="52" t="s">
+        <v>76</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>142</v>
@@ -2992,19 +3006,19 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="50"/>
-      <c r="B14" s="42" t="str">
+      <c r="A14" s="48"/>
+      <c r="B14" s="41" t="str">
         <f aca="false">Основна!A23</f>
         <v>Посада</v>
       </c>
-      <c r="C14" s="42" t="str">
+      <c r="C14" s="41" t="str">
         <f aca="false">IF(Основна!B23 = 0, "",  Основна!B23)</f>
         <v/>
       </c>
-      <c r="D14" s="42"/>
-      <c r="O14" s="53"/>
-      <c r="P14" s="54" t="s">
-        <v>80</v>
+      <c r="D14" s="41"/>
+      <c r="O14" s="51"/>
+      <c r="P14" s="52" t="s">
+        <v>79</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>145</v>
@@ -3026,1569 +3040,1569 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="50"/>
-      <c r="B15" s="42" t="str">
+      <c r="A15" s="48"/>
+      <c r="B15" s="41" t="str">
         <f aca="false">Основна!A24</f>
         <v>Номер наказу про призначення</v>
       </c>
-      <c r="C15" s="42" t="str">
+      <c r="C15" s="41" t="str">
         <f aca="false">IF(Основна!B24 = 0, "",  Основна!B24)</f>
         <v/>
       </c>
-      <c r="D15" s="42"/>
-      <c r="G15" s="47" t="s">
-        <v>79</v>
-      </c>
-      <c r="H15" s="47"/>
-      <c r="I15" s="47"/>
-      <c r="O15" s="53"/>
-      <c r="P15" s="55" t="s">
+      <c r="D15" s="41"/>
+      <c r="G15" s="45" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="O15" s="51"/>
+      <c r="P15" s="53" t="s">
         <v>151</v>
       </c>
-      <c r="Q15" s="56" t="s">
+      <c r="Q15" s="54" t="s">
         <v>152</v>
       </c>
-      <c r="R15" s="56" t="s">
+      <c r="R15" s="54" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="50"/>
-      <c r="B16" s="42" t="str">
+      <c r="A16" s="48"/>
+      <c r="B16" s="41" t="str">
         <f aca="false">Основна!A25</f>
         <v>Дата наказу про призначення</v>
       </c>
-      <c r="C16" s="42" t="str">
+      <c r="C16" s="41" t="str">
         <f aca="false">IF(Основна!B25 = 0, "",  Основна!B25)</f>
         <v/>
       </c>
-      <c r="D16" s="42"/>
-      <c r="G16" s="57" t="n">
+      <c r="D16" s="41"/>
+      <c r="G16" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="57" t="n">
+      <c r="H16" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="57" t="n">
+      <c r="I16" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
-      <c r="O16" s="53"/>
-      <c r="P16" s="55" t="s">
+      <c r="O16" s="51"/>
+      <c r="P16" s="53" t="s">
         <v>154</v>
       </c>
-      <c r="Q16" s="56" t="s">
+      <c r="Q16" s="54" t="s">
         <v>155</v>
       </c>
-      <c r="R16" s="56" t="s">
+      <c r="R16" s="54" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="50"/>
-      <c r="B17" s="42" t="str">
+      <c r="A17" s="48"/>
+      <c r="B17" s="41" t="str">
         <f aca="false">Основна!A28</f>
         <v>Група обліку</v>
       </c>
-      <c r="C17" s="42" t="str">
+      <c r="C17" s="41" t="str">
         <f aca="false">IF(Основна!B28 = 0, "",  Основна!B28)</f>
         <v/>
       </c>
-      <c r="D17" s="42"/>
-      <c r="G17" s="57" t="n">
+      <c r="D17" s="41"/>
+      <c r="G17" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="57" t="n">
+      <c r="H17" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
-      <c r="I17" s="57" t="n">
+      <c r="I17" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
-      <c r="O17" s="53" t="s">
+      <c r="O17" s="51" t="s">
         <v>157</v>
       </c>
       <c r="P17" s="18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="50"/>
-      <c r="B18" s="42" t="str">
+      <c r="A18" s="48"/>
+      <c r="B18" s="41" t="str">
         <f aca="false">Основна!A29</f>
         <v>Категорія обліку</v>
       </c>
-      <c r="C18" s="42" t="str">
+      <c r="C18" s="41" t="str">
         <f aca="false">IF(Основна!B29 = 0, "",  Основна!B29)</f>
         <v/>
       </c>
-      <c r="D18" s="42"/>
-      <c r="G18" s="57" t="n">
+      <c r="D18" s="41"/>
+      <c r="G18" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="57" t="n">
+      <c r="H18" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="57" t="n">
+      <c r="I18" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
-      <c r="O18" s="53"/>
+      <c r="O18" s="51"/>
       <c r="P18" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="50"/>
-      <c r="B19" s="42" t="str">
+      <c r="A19" s="48"/>
+      <c r="B19" s="41" t="str">
         <f aca="false">Основна!A30</f>
         <v>Склад</v>
       </c>
-      <c r="C19" s="42" t="str">
+      <c r="C19" s="41" t="str">
         <f aca="false">IF(Основна!B30 = 0, "",  Основна!B30)</f>
         <v/>
       </c>
-      <c r="D19" s="42"/>
-      <c r="G19" s="57" t="n">
+      <c r="D19" s="41"/>
+      <c r="G19" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="57" t="n">
+      <c r="H19" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
-      <c r="I19" s="57" t="n">
+      <c r="I19" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
-      <c r="O19" s="53"/>
+      <c r="O19" s="51"/>
       <c r="P19" s="18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="50"/>
-      <c r="B20" s="42" t="str">
+      <c r="A20" s="48"/>
+      <c r="B20" s="41" t="str">
         <f aca="false">Основна!A31</f>
         <v>Військове звання</v>
       </c>
-      <c r="C20" s="42" t="str">
+      <c r="C20" s="41" t="str">
         <f aca="false">IF(Основна!B31 = 0, "",  Основна!B31)</f>
         <v/>
       </c>
-      <c r="D20" s="42"/>
-      <c r="G20" s="57" t="n">
+      <c r="D20" s="41"/>
+      <c r="G20" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
-      <c r="H20" s="57" t="n">
+      <c r="H20" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
-      <c r="I20" s="57" t="n">
+      <c r="I20" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
-      <c r="O20" s="53"/>
+      <c r="O20" s="51"/>
       <c r="P20" s="18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="50"/>
-      <c r="B21" s="42" t="str">
+      <c r="A21" s="48"/>
+      <c r="B21" s="41" t="str">
         <f aca="false">Основна!A32</f>
         <v>Військово-облікова спеціальність</v>
       </c>
-      <c r="C21" s="42" t="str">
+      <c r="C21" s="41" t="str">
         <f aca="false">IF(Основна!B32 = 0, "",  Основна!B32)</f>
         <v/>
       </c>
-      <c r="D21" s="42"/>
-      <c r="G21" s="57" t="n">
+      <c r="D21" s="41"/>
+      <c r="G21" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
-      <c r="H21" s="57" t="n">
+      <c r="H21" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
-      <c r="I21" s="57" t="n">
+      <c r="I21" s="55" t="n">
         <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
-      <c r="O21" s="53"/>
+      <c r="O21" s="51"/>
       <c r="P21" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50"/>
-      <c r="B22" s="42" t="str">
+      <c r="A22" s="48"/>
+      <c r="B22" s="41" t="str">
         <f aca="false">Основна!A33</f>
         <v> Придатність до військової служби</v>
       </c>
-      <c r="C22" s="42" t="str">
+      <c r="C22" s="41" t="str">
         <f aca="false">IF(Основна!B33 = 0, "",  Основна!B33)</f>
         <v/>
       </c>
-      <c r="D22" s="42"/>
-      <c r="O22" s="53"/>
+      <c r="D22" s="41"/>
+      <c r="O22" s="51"/>
       <c r="P22" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50"/>
-      <c r="B23" s="42" t="str">
+      <c r="A23" s="48"/>
+      <c r="B23" s="41" t="str">
         <f aca="false">Основна!A34</f>
         <v>Териториальний центр комплектування та соціальної підтримки</v>
       </c>
-      <c r="C23" s="42" t="str">
+      <c r="C23" s="41" t="str">
         <f aca="false">IF(Основна!B34 = 0, "",  Основна!B34)</f>
         <v/>
       </c>
-      <c r="D23" s="42"/>
-      <c r="O23" s="53"/>
+      <c r="D23" s="41"/>
+      <c r="O23" s="51"/>
       <c r="P23" s="18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50"/>
-      <c r="B24" s="42" t="str">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="48"/>
+      <c r="B24" s="41" t="str">
         <f aca="false">Основна!A35</f>
         <v>Перебування на спеціальному обліку</v>
       </c>
-      <c r="C24" s="42" t="str">
+      <c r="C24" s="41" t="str">
         <f aca="false">IF(Основна!B35 = 0, "",  Основна!B35)</f>
         <v/>
       </c>
-      <c r="D24" s="42"/>
-      <c r="O24" s="53"/>
-      <c r="P24" s="54" t="s">
-        <v>42</v>
+      <c r="D24" s="41"/>
+      <c r="O24" s="51"/>
+      <c r="P24" s="52" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="48" t="s">
         <v>158</v>
       </c>
-      <c r="B25" s="42" t="str">
+      <c r="B25" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A4</f>
         <v>Країна</v>
       </c>
-      <c r="C25" s="42" t="str">
+      <c r="C25" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B4 = 0, "", 'Адреси Контакти'!B4)</f>
         <v/>
       </c>
-      <c r="D25" s="42"/>
-      <c r="O25" s="53"/>
+      <c r="D25" s="41"/>
+      <c r="O25" s="51"/>
       <c r="P25" s="31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="50"/>
-      <c r="B26" s="42" t="str">
+      <c r="A26" s="48"/>
+      <c r="B26" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A5</f>
         <v>Область</v>
       </c>
-      <c r="C26" s="42" t="str">
+      <c r="C26" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B5 = 0, "", 'Адреси Контакти'!B5)</f>
         <v/>
       </c>
-      <c r="D26" s="42"/>
-      <c r="O26" s="53"/>
+      <c r="D26" s="41"/>
+      <c r="O26" s="51"/>
       <c r="P26" s="28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="50"/>
-      <c r="B27" s="42" t="str">
+      <c r="A27" s="48"/>
+      <c r="B27" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A6</f>
         <v>Місто</v>
       </c>
-      <c r="C27" s="42" t="str">
+      <c r="C27" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B6 = 0, "", 'Адреси Контакти'!B6)</f>
         <v/>
       </c>
-      <c r="D27" s="42"/>
-      <c r="O27" s="53"/>
+      <c r="D27" s="41"/>
+      <c r="O27" s="51"/>
       <c r="P27" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="50"/>
-      <c r="B28" s="42" t="str">
+      <c r="A28" s="48"/>
+      <c r="B28" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A7</f>
         <v>Район (міста)</v>
       </c>
-      <c r="C28" s="42" t="str">
+      <c r="C28" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B7 = 0, "", 'Адреси Контакти'!B7)</f>
         <v/>
       </c>
-      <c r="D28" s="42"/>
-      <c r="O28" s="53"/>
-      <c r="P28" s="54" t="s">
-        <v>65</v>
+      <c r="D28" s="41"/>
+      <c r="O28" s="51"/>
+      <c r="P28" s="52" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="50"/>
-      <c r="B29" s="42" t="str">
+      <c r="A29" s="48"/>
+      <c r="B29" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A8</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
       </c>
-      <c r="C29" s="42" t="str">
+      <c r="C29" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B8 = 0, "", 'Адреси Контакти'!B8)</f>
         <v/>
       </c>
-      <c r="D29" s="42"/>
+      <c r="D29" s="41"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="50"/>
-      <c r="B30" s="42" t="str">
+      <c r="A30" s="48"/>
+      <c r="B30" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A9</f>
         <v>Індекс</v>
       </c>
-      <c r="C30" s="42" t="str">
+      <c r="C30" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B9 = 0, "", 'Адреси Контакти'!B9)</f>
         <v/>
       </c>
-      <c r="D30" s="42"/>
+      <c r="D30" s="41"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="50"/>
-      <c r="B31" s="42" t="str">
+      <c r="A31" s="48"/>
+      <c r="B31" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A12</f>
         <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
       </c>
-      <c r="C31" s="42" t="str">
+      <c r="C31" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B12 = 0, "", 'Адреси Контакти'!B12)</f>
         <v/>
       </c>
-      <c r="D31" s="42"/>
+      <c r="D31" s="41"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="50"/>
-      <c r="B32" s="42" t="str">
+      <c r="A32" s="48"/>
+      <c r="B32" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A13</f>
         <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
       </c>
-      <c r="C32" s="42" t="str">
+      <c r="C32" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B13 = 0, "", 'Адреси Контакти'!B13)</f>
         <v/>
       </c>
-      <c r="D32" s="42"/>
+      <c r="D32" s="41"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="50"/>
-      <c r="B33" s="42" t="str">
+      <c r="A33" s="48"/>
+      <c r="B33" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A16</f>
         <v>Співпадає із адресою фактичного проживання</v>
       </c>
-      <c r="C33" s="42" t="str">
+      <c r="C33" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B16 = 0, "", 'Адреси Контакти'!B16)</f>
         <v/>
       </c>
-      <c r="D33" s="42"/>
+      <c r="D33" s="41"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="50"/>
-      <c r="B34" s="42" t="str">
+      <c r="A34" s="48"/>
+      <c r="B34" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A18</f>
         <v>Країна</v>
       </c>
-      <c r="C34" s="42" t="str">
+      <c r="C34" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B18 = 0, "", 'Адреси Контакти'!B18)</f>
         <v/>
       </c>
-      <c r="D34" s="42"/>
+      <c r="D34" s="41"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="50"/>
-      <c r="B35" s="42" t="str">
+      <c r="A35" s="48"/>
+      <c r="B35" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A19</f>
         <v>Область</v>
       </c>
-      <c r="C35" s="42" t="str">
+      <c r="C35" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B19 = 0, "", 'Адреси Контакти'!B19)</f>
         <v/>
       </c>
-      <c r="D35" s="42"/>
+      <c r="D35" s="41"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="50"/>
-      <c r="B36" s="42" t="str">
+      <c r="A36" s="48"/>
+      <c r="B36" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A20</f>
         <v>Місто</v>
       </c>
-      <c r="C36" s="42" t="str">
+      <c r="C36" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B20 = 0, "", 'Адреси Контакти'!B20)</f>
         <v/>
       </c>
-      <c r="D36" s="42"/>
+      <c r="D36" s="41"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="50"/>
-      <c r="B37" s="42" t="str">
+      <c r="A37" s="48"/>
+      <c r="B37" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A21</f>
         <v>Район (міста)</v>
       </c>
-      <c r="C37" s="42" t="str">
+      <c r="C37" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B21 = 0, "", 'Адреси Контакти'!B21)</f>
         <v/>
       </c>
-      <c r="D37" s="42"/>
+      <c r="D37" s="41"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="50"/>
-      <c r="B38" s="42" t="str">
+      <c r="A38" s="48"/>
+      <c r="B38" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A22</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
       </c>
-      <c r="C38" s="42" t="str">
+      <c r="C38" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B22 = 0, "", 'Адреси Контакти'!B22)</f>
         <v/>
       </c>
-      <c r="D38" s="42"/>
+      <c r="D38" s="41"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="50"/>
-      <c r="B39" s="42" t="str">
+      <c r="A39" s="48"/>
+      <c r="B39" s="41" t="str">
         <f aca="false">'Адреси Контакти'!A23</f>
         <v>Індекс</v>
       </c>
-      <c r="C39" s="42" t="str">
+      <c r="C39" s="41" t="str">
         <f aca="false">IF('Адреси Контакти'!B23 = 0, "", 'Адреси Контакти'!B23)</f>
         <v/>
       </c>
-      <c r="D39" s="42"/>
+      <c r="D39" s="41"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="50" t="s">
+      <c r="A40" s="48" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="42" t="str">
+      <c r="B40" s="41" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C40" s="58" t="str">
+      <c r="C40" s="56" t="str">
         <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
         <v/>
       </c>
-      <c r="D40" s="59"/>
+      <c r="D40" s="57"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="50"/>
-      <c r="B41" s="42" t="str">
+      <c r="A41" s="48"/>
+      <c r="B41" s="41" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C41" s="58" t="str">
+      <c r="C41" s="56" t="str">
         <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
         <v/>
       </c>
-      <c r="D41" s="59"/>
+      <c r="D41" s="57"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="50"/>
-      <c r="B42" s="42" t="str">
+      <c r="A42" s="48"/>
+      <c r="B42" s="41" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C42" s="58" t="str">
+      <c r="C42" s="56" t="str">
         <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
-      <c r="D42" s="59"/>
+      <c r="D42" s="57"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="50"/>
-      <c r="B43" s="42" t="str">
+      <c r="A43" s="48"/>
+      <c r="B43" s="41" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C43" s="58" t="str">
+      <c r="C43" s="56" t="str">
         <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
-      <c r="D43" s="59"/>
+      <c r="D43" s="57"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="50"/>
-      <c r="B44" s="42" t="str">
+      <c r="A44" s="48"/>
+      <c r="B44" s="41" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C44" s="58" t="str">
+      <c r="C44" s="56" t="str">
         <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
-      <c r="D44" s="59"/>
+      <c r="D44" s="57"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="50"/>
-      <c r="B45" s="42" t="str">
+      <c r="A45" s="48"/>
+      <c r="B45" s="41" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C45" s="58" t="str">
+      <c r="C45" s="56" t="str">
         <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
-      <c r="D45" s="59"/>
+      <c r="D45" s="57"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="50"/>
-      <c r="B46" s="42" t="str">
+      <c r="A46" s="48"/>
+      <c r="B46" s="41" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C46" s="58" t="str">
+      <c r="C46" s="56" t="str">
         <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
-      <c r="D46" s="59"/>
+      <c r="D46" s="57"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="50"/>
-      <c r="B47" s="42" t="str">
+      <c r="A47" s="48"/>
+      <c r="B47" s="41" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C47" s="58" t="str">
+      <c r="C47" s="56" t="str">
         <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
-      <c r="D47" s="59"/>
+      <c r="D47" s="57"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="50"/>
-      <c r="B48" s="42" t="str">
+      <c r="A48" s="48"/>
+      <c r="B48" s="41" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C48" s="58" t="str">
+      <c r="C48" s="56" t="str">
         <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
-      <c r="D48" s="59"/>
+      <c r="D48" s="57"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="50"/>
-      <c r="B49" s="42" t="str">
+      <c r="A49" s="48"/>
+      <c r="B49" s="41" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C49" s="58" t="str">
+      <c r="C49" s="56" t="str">
         <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
-      <c r="D49" s="59"/>
+      <c r="D49" s="57"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="50"/>
-      <c r="B50" s="42" t="str">
+      <c r="A50" s="48"/>
+      <c r="B50" s="41" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C50" s="58" t="str">
+      <c r="C50" s="56" t="str">
         <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
-      <c r="D50" s="59"/>
+      <c r="D50" s="57"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="50"/>
-      <c r="B51" s="42" t="str">
+      <c r="A51" s="48"/>
+      <c r="B51" s="41" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C51" s="58" t="str">
+      <c r="C51" s="56" t="str">
         <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
-      <c r="D51" s="59"/>
+      <c r="D51" s="57"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="50"/>
-      <c r="B52" s="42" t="str">
+      <c r="A52" s="48"/>
+      <c r="B52" s="41" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C52" s="58" t="str">
+      <c r="C52" s="56" t="str">
         <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
-      <c r="D52" s="59"/>
+      <c r="D52" s="57"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="50"/>
-      <c r="B53" s="42" t="str">
+      <c r="A53" s="48"/>
+      <c r="B53" s="41" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C53" s="58" t="str">
+      <c r="C53" s="56" t="str">
         <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
-      <c r="D53" s="59"/>
+      <c r="D53" s="57"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="50"/>
-      <c r="B54" s="42" t="str">
+      <c r="A54" s="48"/>
+      <c r="B54" s="41" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C54" s="58" t="str">
+      <c r="C54" s="56" t="str">
         <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
-      <c r="D54" s="59"/>
+      <c r="D54" s="57"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="50"/>
-      <c r="B55" s="42" t="str">
+      <c r="A55" s="48"/>
+      <c r="B55" s="41" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C55" s="58" t="str">
+      <c r="C55" s="56" t="str">
         <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
-      <c r="D55" s="59"/>
+      <c r="D55" s="57"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="50"/>
-      <c r="B56" s="42" t="str">
+      <c r="A56" s="48"/>
+      <c r="B56" s="41" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C56" s="58" t="str">
+      <c r="C56" s="56" t="str">
         <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
-      <c r="D56" s="59"/>
+      <c r="D56" s="57"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="50"/>
-      <c r="B57" s="42" t="str">
+      <c r="A57" s="48"/>
+      <c r="B57" s="41" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C57" s="58" t="str">
+      <c r="C57" s="56" t="str">
         <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
-      <c r="D57" s="59"/>
+      <c r="D57" s="57"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="50"/>
-      <c r="B58" s="42" t="str">
+      <c r="A58" s="48"/>
+      <c r="B58" s="41" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C58" s="58" t="str">
+      <c r="C58" s="56" t="str">
         <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
-      <c r="D58" s="59"/>
+      <c r="D58" s="57"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="50"/>
-      <c r="B59" s="42" t="str">
+      <c r="A59" s="48"/>
+      <c r="B59" s="41" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C59" s="58" t="str">
+      <c r="C59" s="56" t="str">
         <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
-      <c r="D59" s="59"/>
+      <c r="D59" s="57"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="50"/>
-      <c r="B60" s="42" t="str">
+      <c r="A60" s="48"/>
+      <c r="B60" s="41" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C60" s="58" t="str">
+      <c r="C60" s="56" t="str">
         <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
-      <c r="D60" s="59"/>
+      <c r="D60" s="57"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="50"/>
-      <c r="B61" s="42" t="str">
+      <c r="A61" s="48"/>
+      <c r="B61" s="41" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C61" s="58" t="str">
+      <c r="C61" s="56" t="str">
         <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
-      <c r="D61" s="59"/>
+      <c r="D61" s="57"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="50"/>
-      <c r="B62" s="42" t="str">
+      <c r="A62" s="48"/>
+      <c r="B62" s="41" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C62" s="58" t="str">
+      <c r="C62" s="56" t="str">
         <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
-      <c r="D62" s="59"/>
+      <c r="D62" s="57"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="50"/>
-      <c r="B63" s="42" t="str">
+      <c r="A63" s="48"/>
+      <c r="B63" s="41" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C63" s="58" t="str">
+      <c r="C63" s="56" t="str">
         <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
-      <c r="D63" s="59"/>
+      <c r="D63" s="57"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="50"/>
-      <c r="B64" s="42" t="str">
+      <c r="A64" s="48"/>
+      <c r="B64" s="41" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C64" s="58" t="str">
+      <c r="C64" s="56" t="str">
         <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
-      <c r="D64" s="59"/>
+      <c r="D64" s="57"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="50"/>
-      <c r="B65" s="42" t="str">
+      <c r="A65" s="48"/>
+      <c r="B65" s="41" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C65" s="58" t="str">
+      <c r="C65" s="56" t="str">
         <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
-      <c r="D65" s="59"/>
+      <c r="D65" s="57"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="50"/>
-      <c r="B66" s="42" t="str">
+      <c r="A66" s="48"/>
+      <c r="B66" s="41" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C66" s="58" t="str">
+      <c r="C66" s="56" t="str">
         <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
-      <c r="D66" s="59"/>
+      <c r="D66" s="57"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="50"/>
-      <c r="B67" s="42" t="str">
+      <c r="A67" s="48"/>
+      <c r="B67" s="41" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C67" s="58" t="str">
+      <c r="C67" s="56" t="str">
         <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
-      <c r="D67" s="59"/>
+      <c r="D67" s="57"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="50"/>
-      <c r="B68" s="42" t="str">
+      <c r="A68" s="48"/>
+      <c r="B68" s="41" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C68" s="58" t="str">
+      <c r="C68" s="56" t="str">
         <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
-      <c r="D68" s="59"/>
+      <c r="D68" s="57"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="50"/>
-      <c r="B69" s="42" t="str">
+      <c r="A69" s="48"/>
+      <c r="B69" s="41" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C69" s="58" t="str">
+      <c r="C69" s="56" t="str">
         <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
-      <c r="D69" s="59"/>
+      <c r="D69" s="57"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="50"/>
-      <c r="B70" s="42" t="str">
+      <c r="A70" s="48"/>
+      <c r="B70" s="41" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C70" s="58" t="str">
+      <c r="C70" s="56" t="str">
         <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
         <v/>
       </c>
-      <c r="D70" s="59"/>
+      <c r="D70" s="57"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="50"/>
-      <c r="B71" s="42" t="str">
+      <c r="A71" s="48"/>
+      <c r="B71" s="41" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C71" s="58" t="str">
+      <c r="C71" s="56" t="str">
         <f aca="false">IF(Освіта!D13 = 0, "", Освіта!D13)</f>
         <v/>
       </c>
-      <c r="D71" s="59"/>
+      <c r="D71" s="57"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="50"/>
-      <c r="B72" s="42" t="str">
+      <c r="A72" s="48"/>
+      <c r="B72" s="41" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C72" s="58" t="str">
+      <c r="C72" s="56" t="str">
         <f aca="false">IF(Освіта!E13 = 0, "", Освіта!E13)</f>
         <v/>
       </c>
-      <c r="D72" s="59"/>
+      <c r="D72" s="57"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="50"/>
-      <c r="B73" s="42" t="str">
+      <c r="A73" s="48"/>
+      <c r="B73" s="41" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C73" s="58" t="str">
+      <c r="C73" s="56" t="str">
         <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
         <v/>
       </c>
-      <c r="D73" s="59"/>
+      <c r="D73" s="57"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="50"/>
-      <c r="B74" s="42" t="str">
+      <c r="A74" s="48"/>
+      <c r="B74" s="41" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C74" s="58" t="str">
+      <c r="C74" s="56" t="str">
         <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
         <v/>
       </c>
-      <c r="D74" s="59"/>
+      <c r="D74" s="57"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="50"/>
-      <c r="B75" s="42" t="str">
+      <c r="A75" s="48"/>
+      <c r="B75" s="41" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C75" s="58" t="str">
+      <c r="C75" s="56" t="str">
         <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
         <v/>
       </c>
-      <c r="D75" s="59"/>
+      <c r="D75" s="57"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="50"/>
-      <c r="B76" s="42" t="str">
+      <c r="A76" s="48"/>
+      <c r="B76" s="41" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C76" s="58" t="str">
+      <c r="C76" s="56" t="str">
         <f aca="false">IF(Освіта!D14 = 0, "", Освіта!D14)</f>
         <v/>
       </c>
-      <c r="D76" s="59"/>
+      <c r="D76" s="57"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="50"/>
-      <c r="B77" s="42" t="str">
+      <c r="A77" s="48"/>
+      <c r="B77" s="41" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C77" s="58" t="str">
+      <c r="C77" s="56" t="str">
         <f aca="false">IF(Освіта!E14 = 0, "", Освіта!E14)</f>
         <v/>
       </c>
-      <c r="D77" s="59"/>
+      <c r="D77" s="57"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="50"/>
-      <c r="B78" s="42" t="str">
+      <c r="A78" s="48"/>
+      <c r="B78" s="41" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C78" s="58" t="str">
+      <c r="C78" s="56" t="str">
         <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
         <v/>
       </c>
-      <c r="D78" s="59"/>
+      <c r="D78" s="57"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="50"/>
-      <c r="B79" s="42" t="str">
+      <c r="A79" s="48"/>
+      <c r="B79" s="41" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C79" s="58" t="str">
+      <c r="C79" s="56" t="str">
         <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
         <v/>
       </c>
-      <c r="D79" s="59"/>
+      <c r="D79" s="57"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="50"/>
-      <c r="B80" s="42" t="str">
+      <c r="A80" s="48"/>
+      <c r="B80" s="41" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C80" s="58" t="str">
+      <c r="C80" s="56" t="str">
         <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
         <v/>
       </c>
-      <c r="D80" s="59"/>
+      <c r="D80" s="57"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="50"/>
-      <c r="B81" s="42" t="str">
+      <c r="A81" s="48"/>
+      <c r="B81" s="41" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C81" s="58" t="str">
+      <c r="C81" s="56" t="str">
         <f aca="false">IF(Освіта!D15 = 0, "", Освіта!D15)</f>
         <v/>
       </c>
-      <c r="D81" s="59"/>
+      <c r="D81" s="57"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="50"/>
-      <c r="B82" s="42" t="str">
+      <c r="A82" s="48"/>
+      <c r="B82" s="41" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C82" s="58" t="str">
+      <c r="C82" s="56" t="str">
         <f aca="false">IF(Освіта!E15 = 0, "", Освіта!E15)</f>
         <v/>
       </c>
-      <c r="D82" s="59"/>
+      <c r="D82" s="57"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="50"/>
-      <c r="B83" s="42" t="str">
+      <c r="A83" s="48"/>
+      <c r="B83" s="41" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C83" s="58" t="str">
+      <c r="C83" s="56" t="str">
         <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
         <v/>
       </c>
-      <c r="D83" s="59"/>
+      <c r="D83" s="57"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="50"/>
-      <c r="B84" s="42" t="str">
+      <c r="A84" s="48"/>
+      <c r="B84" s="41" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C84" s="58" t="str">
+      <c r="C84" s="56" t="str">
         <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
         <v/>
       </c>
-      <c r="D84" s="59"/>
+      <c r="D84" s="57"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="50"/>
-      <c r="B85" s="42" t="str">
+      <c r="A85" s="48"/>
+      <c r="B85" s="41" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C85" s="58" t="str">
+      <c r="C85" s="56" t="str">
         <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
         <v/>
       </c>
-      <c r="D85" s="59"/>
+      <c r="D85" s="57"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="50"/>
-      <c r="B86" s="42" t="str">
+      <c r="A86" s="48"/>
+      <c r="B86" s="41" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C86" s="58" t="str">
+      <c r="C86" s="56" t="str">
         <f aca="false">IF(Освіта!D16 = 0, "", Освіта!D16)</f>
         <v/>
       </c>
-      <c r="D86" s="59"/>
+      <c r="D86" s="57"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="50"/>
-      <c r="B87" s="42" t="str">
+      <c r="A87" s="48"/>
+      <c r="B87" s="41" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C87" s="58" t="str">
+      <c r="C87" s="56" t="str">
         <f aca="false">IF(Освіта!E16 = 0, "", Освіта!E16)</f>
         <v/>
       </c>
-      <c r="D87" s="59"/>
+      <c r="D87" s="57"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="50"/>
-      <c r="B88" s="42" t="str">
+      <c r="A88" s="48"/>
+      <c r="B88" s="41" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C88" s="58" t="str">
+      <c r="C88" s="56" t="str">
         <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
         <v/>
       </c>
-      <c r="D88" s="59"/>
+      <c r="D88" s="57"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="50"/>
-      <c r="B89" s="42" t="str">
+      <c r="A89" s="48"/>
+      <c r="B89" s="41" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C89" s="58" t="str">
+      <c r="C89" s="56" t="str">
         <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
         <v/>
       </c>
-      <c r="D89" s="59"/>
+      <c r="D89" s="57"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="50"/>
-      <c r="B90" s="42" t="str">
+      <c r="A90" s="48"/>
+      <c r="B90" s="41" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C90" s="58" t="str">
+      <c r="C90" s="56" t="str">
         <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
         <v/>
       </c>
-      <c r="D90" s="59"/>
+      <c r="D90" s="57"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="50"/>
-      <c r="B91" s="42" t="str">
+      <c r="A91" s="48"/>
+      <c r="B91" s="41" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C91" s="58" t="str">
+      <c r="C91" s="56" t="str">
         <f aca="false">IF(Освіта!D17 = 0, "", Освіта!D17)</f>
         <v/>
       </c>
-      <c r="D91" s="59"/>
+      <c r="D91" s="57"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="50"/>
-      <c r="B92" s="42" t="str">
+      <c r="A92" s="48"/>
+      <c r="B92" s="41" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C92" s="58" t="str">
+      <c r="C92" s="56" t="str">
         <f aca="false">IF(Освіта!E17 = 0, "", Освіта!E17)</f>
         <v/>
       </c>
-      <c r="D92" s="59"/>
+      <c r="D92" s="57"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="50"/>
-      <c r="B93" s="42" t="str">
+      <c r="A93" s="48"/>
+      <c r="B93" s="41" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C93" s="58" t="str">
+      <c r="C93" s="56" t="str">
         <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
         <v/>
       </c>
-      <c r="D93" s="59"/>
+      <c r="D93" s="57"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="50"/>
-      <c r="B94" s="42" t="str">
+      <c r="A94" s="48"/>
+      <c r="B94" s="41" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Диплом, номер, дата видачі</v>
       </c>
-      <c r="C94" s="58" t="str">
+      <c r="C94" s="56" t="str">
         <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
         <v/>
       </c>
-      <c r="D94" s="59"/>
+      <c r="D94" s="57"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="50"/>
-      <c r="B95" s="42" t="str">
+      <c r="A95" s="48"/>
+      <c r="B95" s="41" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C95" s="58" t="str">
+      <c r="C95" s="56" t="str">
         <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
-      <c r="D95" s="59"/>
+      <c r="D95" s="57"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="50"/>
-      <c r="B96" s="42" t="str">
+      <c r="A96" s="48"/>
+      <c r="B96" s="41" t="str">
         <f aca="false">Освіта!$D$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C96" s="58" t="str">
+      <c r="C96" s="56" t="str">
         <f aca="false">IF(Освіта!D18 = 0, "", Освіта!D18)</f>
         <v/>
       </c>
-      <c r="D96" s="59"/>
+      <c r="D96" s="57"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="50"/>
-      <c r="B97" s="42" t="str">
+      <c r="A97" s="48"/>
+      <c r="B97" s="41" t="str">
         <f aca="false">Освіта!$E$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C97" s="58" t="str">
+      <c r="C97" s="56" t="str">
         <f aca="false">IF(Освіта!E18 = 0, "", Освіта!E18)</f>
         <v/>
       </c>
-      <c r="D97" s="59"/>
+      <c r="D97" s="57"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="50" t="s">
+      <c r="A98" s="48" t="s">
         <v>160</v>
       </c>
-      <c r="B98" s="42" t="str">
+      <c r="B98" s="41" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C98" s="58" t="str">
+      <c r="C98" s="56" t="str">
         <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
         <v/>
       </c>
-      <c r="D98" s="59"/>
+      <c r="D98" s="57"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="50"/>
-      <c r="B99" s="42" t="str">
+      <c r="A99" s="48"/>
+      <c r="B99" s="41" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C99" s="58" t="str">
+      <c r="C99" s="56" t="str">
         <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
         <v/>
       </c>
-      <c r="D99" s="59"/>
+      <c r="D99" s="57"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="50"/>
-      <c r="B100" s="42" t="str">
+      <c r="A100" s="48"/>
+      <c r="B100" s="41" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C100" s="58" t="str">
+      <c r="C100" s="56" t="str">
         <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
         <v/>
       </c>
-      <c r="D100" s="59"/>
+      <c r="D100" s="57"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="50"/>
-      <c r="B101" s="42" t="str">
+      <c r="A101" s="48"/>
+      <c r="B101" s="41" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C101" s="58" t="str">
+      <c r="C101" s="56" t="str">
         <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
         <v/>
       </c>
-      <c r="D101" s="59"/>
+      <c r="D101" s="57"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="50"/>
-      <c r="B102" s="42" t="str">
+      <c r="A102" s="48"/>
+      <c r="B102" s="41" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C102" s="58" t="str">
+      <c r="C102" s="56" t="str">
         <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
         <v/>
       </c>
-      <c r="D102" s="59"/>
+      <c r="D102" s="57"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="50"/>
-      <c r="B103" s="42" t="str">
+      <c r="A103" s="48"/>
+      <c r="B103" s="41" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C103" s="58" t="str">
+      <c r="C103" s="56" t="str">
         <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
         <v/>
       </c>
-      <c r="D103" s="59"/>
+      <c r="D103" s="57"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="50"/>
-      <c r="B104" s="42" t="str">
+      <c r="A104" s="48"/>
+      <c r="B104" s="41" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C104" s="58" t="str">
+      <c r="C104" s="56" t="str">
         <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
         <v/>
       </c>
-      <c r="D104" s="59"/>
+      <c r="D104" s="57"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="50"/>
-      <c r="B105" s="42" t="str">
+      <c r="A105" s="48"/>
+      <c r="B105" s="41" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C105" s="58" t="str">
+      <c r="C105" s="56" t="str">
         <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
         <v/>
       </c>
-      <c r="D105" s="59"/>
+      <c r="D105" s="57"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="50"/>
-      <c r="B106" s="42" t="str">
+      <c r="A106" s="48"/>
+      <c r="B106" s="41" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C106" s="58" t="str">
+      <c r="C106" s="56" t="str">
         <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
         <v/>
       </c>
-      <c r="D106" s="59"/>
+      <c r="D106" s="57"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="50"/>
-      <c r="B107" s="42" t="str">
+      <c r="A107" s="48"/>
+      <c r="B107" s="41" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C107" s="58" t="str">
+      <c r="C107" s="56" t="str">
         <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
         <v/>
       </c>
-      <c r="D107" s="59"/>
+      <c r="D107" s="57"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="50"/>
-      <c r="B108" s="42" t="str">
+      <c r="A108" s="48"/>
+      <c r="B108" s="41" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C108" s="58" t="str">
+      <c r="C108" s="56" t="str">
         <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
         <v/>
       </c>
-      <c r="D108" s="59"/>
+      <c r="D108" s="57"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="50"/>
-      <c r="B109" s="42" t="str">
+      <c r="A109" s="48"/>
+      <c r="B109" s="41" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C109" s="58" t="str">
+      <c r="C109" s="56" t="str">
         <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
         <v/>
       </c>
-      <c r="D109" s="59"/>
+      <c r="D109" s="57"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="50"/>
-      <c r="B110" s="42" t="str">
+      <c r="A110" s="48"/>
+      <c r="B110" s="41" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C110" s="58" t="str">
+      <c r="C110" s="56" t="str">
         <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
         <v/>
       </c>
-      <c r="D110" s="59"/>
+      <c r="D110" s="57"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="50"/>
-      <c r="B111" s="42" t="str">
+      <c r="A111" s="48"/>
+      <c r="B111" s="41" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C111" s="58" t="str">
+      <c r="C111" s="56" t="str">
         <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
         <v/>
       </c>
-      <c r="D111" s="59"/>
+      <c r="D111" s="57"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="50"/>
-      <c r="B112" s="42" t="str">
+      <c r="A112" s="48"/>
+      <c r="B112" s="41" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C112" s="58" t="str">
+      <c r="C112" s="56" t="str">
         <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
         <v/>
       </c>
-      <c r="D112" s="59"/>
+      <c r="D112" s="57"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="50"/>
-      <c r="B113" s="42" t="str">
+      <c r="A113" s="48"/>
+      <c r="B113" s="41" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C113" s="58" t="str">
+      <c r="C113" s="56" t="str">
         <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
         <v/>
       </c>
-      <c r="D113" s="59"/>
+      <c r="D113" s="57"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="50"/>
-      <c r="B114" s="42" t="str">
+      <c r="A114" s="48"/>
+      <c r="B114" s="41" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>ПІБ</v>
       </c>
-      <c r="C114" s="58" t="str">
+      <c r="C114" s="56" t="str">
         <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
         <v/>
       </c>
-      <c r="D114" s="59"/>
+      <c r="D114" s="57"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="50"/>
-      <c r="B115" s="42" t="str">
+      <c r="A115" s="48"/>
+      <c r="B115" s="41" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C115" s="58" t="str">
+      <c r="C115" s="56" t="str">
         <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
         <v/>
       </c>
-      <c r="D115" s="59"/>
+      <c r="D115" s="57"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="50" t="s">
+      <c r="A116" s="48" t="s">
         <v>161</v>
       </c>
-      <c r="B116" s="42" t="str">
+      <c r="B116" s="41" t="str">
         <f aca="false">Документи!A4</f>
         <v>Тип документу</v>
       </c>
-      <c r="C116" s="51" t="str">
+      <c r="C116" s="49" t="str">
         <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
         <v/>
       </c>
-      <c r="D116" s="42"/>
+      <c r="D116" s="41"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="50"/>
-      <c r="B117" s="42" t="str">
+      <c r="A117" s="48"/>
+      <c r="B117" s="41" t="str">
         <f aca="false">Документи!A5</f>
         <v>Серія та номер </v>
       </c>
-      <c r="C117" s="42" t="str">
+      <c r="C117" s="41" t="str">
         <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
         <v/>
       </c>
-      <c r="D117" s="42"/>
+      <c r="D117" s="41"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="50"/>
-      <c r="B118" s="42" t="str">
+      <c r="A118" s="48"/>
+      <c r="B118" s="41" t="str">
         <f aca="false">Документи!A6</f>
         <v>Ким виданий</v>
       </c>
-      <c r="C118" s="42" t="str">
+      <c r="C118" s="41" t="str">
         <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
         <v/>
       </c>
-      <c r="D118" s="42"/>
+      <c r="D118" s="41"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="50"/>
-      <c r="B119" s="42" t="str">
+      <c r="A119" s="48"/>
+      <c r="B119" s="41" t="str">
         <f aca="false">Документи!A7</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C119" s="42" t="str">
+      <c r="C119" s="41" t="str">
         <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
         <v/>
       </c>
-      <c r="D119" s="42"/>
+      <c r="D119" s="41"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="50"/>
-      <c r="B120" s="42" t="str">
+      <c r="A120" s="48"/>
+      <c r="B120" s="41" t="str">
         <f aca="false">Документи!A10</f>
         <v>Тип документу</v>
       </c>
-      <c r="C120" s="51" t="str">
+      <c r="C120" s="49" t="str">
         <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
         <v/>
       </c>
-      <c r="D120" s="42"/>
+      <c r="D120" s="41"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="50"/>
-      <c r="B121" s="42" t="str">
+      <c r="A121" s="48"/>
+      <c r="B121" s="41" t="str">
         <f aca="false">Документи!A11</f>
         <v>Серія та номер </v>
       </c>
-      <c r="C121" s="42" t="str">
+      <c r="C121" s="41" t="str">
         <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
         <v/>
       </c>
-      <c r="D121" s="42"/>
+      <c r="D121" s="41"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="50"/>
-      <c r="B122" s="42" t="str">
+      <c r="A122" s="48"/>
+      <c r="B122" s="41" t="str">
         <f aca="false">Документи!A12</f>
         <v>Ким виданий</v>
       </c>
-      <c r="C122" s="42" t="str">
+      <c r="C122" s="41" t="str">
         <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
         <v/>
       </c>
-      <c r="D122" s="42"/>
+      <c r="D122" s="41"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="50"/>
-      <c r="B123" s="42" t="str">
+      <c r="A123" s="48"/>
+      <c r="B123" s="41" t="str">
         <f aca="false">Документи!A13</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C123" s="42" t="str">
+      <c r="C123" s="41" t="str">
         <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
         <v/>
       </c>
-      <c r="D123" s="42"/>
+      <c r="D123" s="41"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="50"/>
-      <c r="B124" s="42" t="str">
+      <c r="A124" s="48"/>
+      <c r="B124" s="41" t="str">
         <f aca="false">Документи!A16</f>
         <v>Серія та номер </v>
       </c>
-      <c r="C124" s="51" t="str">
+      <c r="C124" s="49" t="str">
         <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
         <v/>
       </c>
-      <c r="D124" s="42"/>
+      <c r="D124" s="41"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="50"/>
-      <c r="B125" s="42" t="str">
+      <c r="A125" s="48"/>
+      <c r="B125" s="41" t="str">
         <f aca="false">Документи!A17</f>
         <v>Ким виданий</v>
       </c>
-      <c r="C125" s="42" t="str">
+      <c r="C125" s="41" t="str">
         <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
         <v/>
       </c>
-      <c r="D125" s="42"/>
+      <c r="D125" s="41"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="50"/>
-      <c r="B126" s="42" t="str">
+      <c r="A126" s="48"/>
+      <c r="B126" s="41" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C126" s="42" t="str">
+      <c r="C126" s="41" t="str">
         <f aca="false">IF(Документи!B18 = 0, "", Документи!B18)</f>
         <v/>
       </c>
-      <c r="D126" s="42"/>
+      <c r="D126" s="41"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D127" s="51"/>
+      <c r="D127" s="49"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D128" s="51"/>
+      <c r="D128" s="49"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D129" s="51"/>
+      <c r="D129" s="49"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D130" s="51"/>
+      <c r="D130" s="49"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D131" s="51"/>
+      <c r="D131" s="49"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D132" s="51"/>
+      <c r="D132" s="49"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D133" s="51"/>
+      <c r="D133" s="49"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D134" s="51"/>
+      <c r="D134" s="49"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D135" s="51"/>
+      <c r="D135" s="49"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D136" s="51"/>
+      <c r="D136" s="49"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D137" s="51"/>
+      <c r="D137" s="49"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D138" s="51"/>
+      <c r="D138" s="49"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D139" s="51"/>
+      <c r="D139" s="49"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D140" s="51"/>
+      <c r="D140" s="49"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D141" s="51"/>
+      <c r="D141" s="49"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D142" s="51"/>
+      <c r="D142" s="49"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D143" s="51"/>
+      <c r="D143" s="49"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D144" s="51"/>
+      <c r="D144" s="49"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D145" s="51"/>
+      <c r="D145" s="49"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D146" s="51"/>
+      <c r="D146" s="49"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D147" s="51"/>
+      <c r="D147" s="49"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D148" s="51"/>
+      <c r="D148" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>

<commit_message>
feat: add dedicated buttons for import/export | fix: button position
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Довідка по заповненню" sheetId="1" state="visible" r:id="rId3"/>
@@ -982,7 +982,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1520,7 +1520,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="41.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
         <v>41</v>
       </c>
@@ -11539,8 +11539,8 @@
         <v>Назва освітнього закладу</v>
       </c>
       <c r="C40" s="65" t="str">
-        <f aca="false">IF(Освіта!A4 = 0, "", Освіта!A4)</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
+        <v/>
       </c>
       <c r="D40" s="66"/>
     </row>
@@ -11551,8 +11551,8 @@
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
       <c r="C41" s="65" t="str">
-        <f aca="false">IF(Освіта!B4 = 0, "", Освіта!B4)</f>
-        <v>Серія та номер дисплома (свідоцтва)</v>
+        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
+        <v/>
       </c>
       <c r="D41" s="66"/>
     </row>
@@ -11563,8 +11563,8 @@
         <v>Рік закінчення</v>
       </c>
       <c r="C42" s="65" t="str">
-        <f aca="false">IF(Освіта!C4 = 0, "", Освіта!C4)</f>
-        <v>Рік закінчення</v>
+        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
+        <v/>
       </c>
       <c r="D42" s="66"/>
     </row>
@@ -11575,8 +11575,8 @@
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C43" s="65" t="str">
-        <f aca="false">IF(Освіта!D4 = 0, "", Освіта!D4)</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
+        <v/>
       </c>
       <c r="D43" s="66"/>
     </row>
@@ -11587,8 +11587,8 @@
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C44" s="65" t="str">
-        <f aca="false">IF(Освіта!E4 = 0, "", Освіта!E4)</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
+        <v/>
       </c>
       <c r="D44" s="66"/>
     </row>
@@ -11599,8 +11599,8 @@
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C45" s="65" t="str">
-        <f aca="false">IF(Освіта!F4 = 0, "", Освіта!F4)</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
+        <v/>
       </c>
       <c r="D45" s="66"/>
     </row>
@@ -11611,8 +11611,8 @@
         <v>Рівень освіти</v>
       </c>
       <c r="C46" s="65" t="str">
-        <f aca="false">IF(Освіта!G4 = 0, "", Освіта!G4)</f>
-        <v>Рівень освіти</v>
+        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
+        <v/>
       </c>
       <c r="D46" s="66"/>
     </row>
@@ -11623,7 +11623,7 @@
         <v>Назва освітнього закладу</v>
       </c>
       <c r="C47" s="65" t="str">
-        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
+        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
       <c r="D47" s="66"/>
@@ -11635,7 +11635,7 @@
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
       <c r="C48" s="65" t="str">
-        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
+        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
       <c r="D48" s="66"/>
@@ -11647,7 +11647,7 @@
         <v>Рік закінчення</v>
       </c>
       <c r="C49" s="65" t="str">
-        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
+        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
       <c r="D49" s="66"/>
@@ -11659,7 +11659,7 @@
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C50" s="65" t="str">
-        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
+        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
       <c r="D50" s="66"/>
@@ -11671,7 +11671,7 @@
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C51" s="65" t="str">
-        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
+        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
       <c r="D51" s="66"/>
@@ -11683,7 +11683,7 @@
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C52" s="65" t="str">
-        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
+        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
       <c r="D52" s="66"/>
@@ -11695,7 +11695,7 @@
         <v>Рівень освіти</v>
       </c>
       <c r="C53" s="65" t="str">
-        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
+        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
       <c r="D53" s="66"/>
@@ -11707,7 +11707,7 @@
         <v>Назва освітнього закладу</v>
       </c>
       <c r="C54" s="65" t="str">
-        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
+        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
       <c r="D54" s="66"/>
@@ -11719,7 +11719,7 @@
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
       <c r="C55" s="65" t="str">
-        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
+        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
       <c r="D55" s="66"/>
@@ -11731,7 +11731,7 @@
         <v>Рік закінчення</v>
       </c>
       <c r="C56" s="65" t="str">
-        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
+        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
       <c r="D56" s="66"/>
@@ -11743,7 +11743,7 @@
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C57" s="65" t="str">
-        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
+        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
       <c r="D57" s="66"/>
@@ -11755,7 +11755,7 @@
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C58" s="65" t="str">
-        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
+        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
       <c r="D58" s="66"/>
@@ -11767,7 +11767,7 @@
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C59" s="65" t="str">
-        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
+        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
       <c r="D59" s="66"/>
@@ -11779,7 +11779,7 @@
         <v>Рівень освіти</v>
       </c>
       <c r="C60" s="65" t="str">
-        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
+        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
       <c r="D60" s="66"/>
@@ -11791,7 +11791,7 @@
         <v>Назва освітнього закладу</v>
       </c>
       <c r="C61" s="65" t="str">
-        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
+        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
       <c r="D61" s="66"/>
@@ -11803,7 +11803,7 @@
         <v>Серія та номер дисплома (свідоцтва)</v>
       </c>
       <c r="C62" s="65" t="str">
-        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
+        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
       <c r="D62" s="66"/>
@@ -11815,7 +11815,7 @@
         <v>Рік закінчення</v>
       </c>
       <c r="C63" s="65" t="str">
-        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
+        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
       <c r="D63" s="66"/>
@@ -11827,7 +11827,7 @@
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C64" s="65" t="str">
-        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
+        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
       <c r="D64" s="66"/>
@@ -11839,7 +11839,7 @@
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C65" s="65" t="str">
-        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
+        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
       <c r="D65" s="66"/>
@@ -11851,7 +11851,7 @@
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C66" s="65" t="str">
-        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
+        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
       <c r="D66" s="66"/>
@@ -11863,7 +11863,7 @@
         <v>Рівень освіти</v>
       </c>
       <c r="C67" s="65" t="str">
-        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
+        <f aca="false">IF(Освіта!G8 = 0, "", $освіта.g)</f>
         <v/>
       </c>
       <c r="D67" s="66"/>

</xml_diff>

<commit_message>
fix: separate PIB in excel | fix: separate diploma series and number in education and posteducation
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="165">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -220,7 +220,10 @@
     <t xml:space="preserve">Назва освітнього закладу</t>
   </si>
   <si>
-    <t xml:space="preserve">Серія та номер дисплома (свідоцтва)</t>
+    <t xml:space="preserve">Серія дисплома (свідоцтва)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Номер дисплома (свідоцтва)</t>
   </si>
   <si>
     <t xml:space="preserve">Рік закінчення</t>
@@ -247,7 +250,13 @@
     <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
   </si>
   <si>
-    <t xml:space="preserve">Диплом, номер, дата видачі</t>
+    <t xml:space="preserve">Серія дисплома</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Номер диплома</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата видачі диплома</t>
   </si>
   <si>
     <t xml:space="preserve">Науковий ступінь, учене звання</t>
@@ -265,7 +274,7 @@
     <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
   </si>
   <si>
-    <t xml:space="preserve">ПІБ</t>
+    <t xml:space="preserve">По-батькові</t>
   </si>
   <si>
     <t xml:space="preserve">Рік народження</t>
@@ -602,7 +611,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -625,6 +634,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFCCCCCC"/>
         <bgColor rgb="FFD0CECE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB2B2B2"/>
+        <bgColor rgb="FFCCCCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -721,7 +736,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -978,11 +993,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1045,7 +1068,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FFB2B2B2"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -1905,7 +1928,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="28.46"/>
@@ -1955,17 +1978,20 @@
       <c r="C4" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="36" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="35" t="s">
         <v>68</v>
       </c>
       <c r="G4" s="36" t="s">
         <v>69</v>
+      </c>
+      <c r="H4" s="36" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1976,6 +2002,7 @@
       <c r="E5" s="38"/>
       <c r="F5" s="38"/>
       <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="37"/>
@@ -1985,6 +2012,7 @@
       <c r="E6" s="38"/>
       <c r="F6" s="38"/>
       <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37"/>
@@ -1994,6 +2022,7 @@
       <c r="E7" s="38"/>
       <c r="F7" s="38"/>
       <c r="G7" s="38"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37"/>
@@ -2003,19 +2032,20 @@
       <c r="E8" s="38"/>
       <c r="F8" s="38"/>
       <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33"/>
       <c r="B9" s="33"/>
-      <c r="C9" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" s="33"/>
+      <c r="D9" s="39" t="s">
+        <v>71</v>
+      </c>
       <c r="E9" s="33"/>
-      <c r="F9" s="39" t="s">
+      <c r="F9" s="33"/>
+      <c r="G9" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="39" t="s">
+      <c r="H9" s="39" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2030,7 +2060,7 @@
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="33"/>
@@ -2039,24 +2069,28 @@
       <c r="F11" s="33"/>
       <c r="G11" s="33"/>
     </row>
-    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>74</v>
+        <v>75</v>
+      </c>
+      <c r="D12" s="35" t="s">
+        <v>76</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
+        <v>66</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="35" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
@@ -2064,8 +2098,8 @@
       <c r="C13" s="40"/>
       <c r="D13" s="40"/>
       <c r="E13" s="40"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="33"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
@@ -2073,8 +2107,8 @@
       <c r="C14" s="40"/>
       <c r="D14" s="40"/>
       <c r="E14" s="40"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="33"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
@@ -2082,8 +2116,8 @@
       <c r="C15" s="40"/>
       <c r="D15" s="40"/>
       <c r="E15" s="40"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
@@ -2091,8 +2125,8 @@
       <c r="C16" s="40"/>
       <c r="D16" s="40"/>
       <c r="E16" s="40"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="37"/>
@@ -2100,8 +2134,8 @@
       <c r="C17" s="40"/>
       <c r="D17" s="40"/>
       <c r="E17" s="40"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37"/>
@@ -2109,44 +2143,46 @@
       <c r="C18" s="40"/>
       <c r="D18" s="40"/>
       <c r="E18" s="40"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33"/>
       <c r="B19" s="33"/>
-      <c r="C19" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="39" t="s">
+      <c r="E19" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="F19" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="G19" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F5:F8" type="list">
+  <dataValidations count="6">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F13:F18" type="list">
+      <formula1>'Системна інформація'!$Q$12:$ZA$12</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G13:G18" type="list">
+      <formula1>'Системна інформація'!$Q$13:$ZA$13</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність свого ВНЗ в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого ВНЗ наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A13:A18" type="list">
+      <formula1>'Системна інформація'!$Q$28:$ZA$28</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність свого ВНЗ в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого ВНЗ наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A5:A8" type="list">
+      <formula1>'Системна інформація'!$Q$28:$ZA$28</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:G8" type="list">
       <formula1>'Системна інформація'!$Q$10:$ZA$10</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:G8" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H5:H8" type="list">
       <formula1>'Системна інформація'!$Q$11:$ZA$11</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D13:D18" type="list">
-      <formula1>'Системна інформація'!$Q$12:$ZA$12</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E13:E18" type="list">
-      <formula1>'Системна інформація'!$Q$13:$ZA$13</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" error="Перевірте наявність свого ВНЗ в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого ВНЗ наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A5:A8 A13:A18" type="list">
-      <formula1>'Системна інформація'!$Q$28:$ZA$28</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2165,78 +2201,98 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.62890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="18.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="40.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="2" width="28.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="14.6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="42" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>79</v>
+        <v>5</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>80</v>
+        <v>6</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="45"/>
       <c r="B5" s="46"/>
       <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="45"/>
       <c r="B6" s="46"/>
       <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="45"/>
       <c r="B7" s="46"/>
       <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="45"/>
       <c r="B8" s="46"/>
       <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="45"/>
       <c r="B9" s="46"/>
       <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="45"/>
       <c r="B10" s="46"/>
       <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>81</v>
+      <c r="E11" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A5:A10" type="list">
@@ -2268,21 +2324,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="41" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="47" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D116 = 0, "", 'Системна інформація'!D116)</f>
+        <f aca="false">IF('Системна інформація'!D144 = 0, "", 'Системна інформація'!D144)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="s">
@@ -2291,37 +2347,37 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="48" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D117 = 0, "", 'Системна інформація'!D117)</f>
+        <f aca="false">IF('Системна інформація'!D145 = 0, "", 'Системна інформація'!D145)</f>
         <v/>
       </c>
       <c r="D5" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D118 = 0, "", 'Системна інформація'!D118)</f>
+        <f aca="false">IF('Системна інформація'!D146 = 0, "", 'Системна інформація'!D146)</f>
         <v/>
       </c>
       <c r="D6" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D119 = 0, "", 'Системна інформація'!D119)</f>
+        <f aca="false">IF('Системна інформація'!D147 = 0, "", 'Системна інформація'!D147)</f>
         <v/>
       </c>
       <c r="D7" s="2" t="s">
@@ -2330,16 +2386,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="47" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
+        <f aca="false">IF('Системна інформація'!D148 = 0, "", 'Системна інформація'!D148)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="s">
@@ -2348,34 +2404,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
+        <f aca="false">IF('Системна інформація'!D149 = 0, "", 'Системна інформація'!D149)</f>
         <v/>
       </c>
       <c r="D11" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
+        <f aca="false">IF('Системна інформація'!D150 = 0, "", 'Системна інформація'!D150)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
+        <f aca="false">IF('Системна інформація'!D151 = 0, "", 'Системна інформація'!D151)</f>
         <v/>
       </c>
       <c r="D13" s="2" t="s">
@@ -2384,42 +2440,42 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="41" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
+        <f aca="false">IF('Системна інформація'!D153 = 0, "", 'Системна інформація'!D153)</f>
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="48" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D126 = 0, "", 'Системна інформація'!D126)</f>
+        <f aca="false">IF('Системна інформація'!D154 = 0, "", 'Системна інформація'!D154)</f>
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="48" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
+        <f aca="false">IF('Системна інформація'!D155 = 0, "", 'Системна інформація'!D155)</f>
         <v/>
       </c>
       <c r="D18" s="2" t="s">
@@ -2465,20 +2521,20 @@
   <sheetData>
     <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B1" s="51" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C1" s="51" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D1" s="51" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="52" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H1" s="52"/>
       <c r="I1" s="52"/>
@@ -2486,14 +2542,15 @@
       <c r="K1" s="52"/>
       <c r="L1" s="52"/>
       <c r="M1" s="52"/>
+      <c r="N1" s="52"/>
       <c r="O1" s="53" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P1" s="54" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="Q1" s="53" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="R1" s="53"/>
       <c r="S1" s="53"/>
@@ -2501,7 +2558,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="55" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B2" s="48" t="str">
         <f aca="false">Основна!A9</f>
@@ -2513,56 +2570,60 @@
       </c>
       <c r="D2" s="48"/>
       <c r="G2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="H2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="I2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="J2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="K2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="L2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="M2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
+      <c r="N2" s="57" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O2" s="58" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>11</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2577,31 +2638,35 @@
       </c>
       <c r="D3" s="48"/>
       <c r="G3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="H3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="I3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="J3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="K3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="L3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="M3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="57" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="O3" s="58"/>
@@ -2609,10 +2674,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2627,31 +2692,35 @@
       </c>
       <c r="D4" s="48"/>
       <c r="G4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="H4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="I4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="J4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="K4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="L4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="M4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" s="57" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="O4" s="58"/>
@@ -2659,28 +2728,28 @@
         <v>18</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2695,31 +2764,35 @@
       </c>
       <c r="D5" s="48"/>
       <c r="G5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="I5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="K5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="L5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="M5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*7+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="57" t="n">
+        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="O5" s="58"/>
@@ -2727,10 +2800,10 @@
         <v>30</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2774,26 +2847,26 @@
       </c>
       <c r="D7" s="48"/>
       <c r="G7" s="59" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H7" s="59"/>
       <c r="I7" s="59"/>
       <c r="J7" s="59"/>
       <c r="K7" s="59"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
+      <c r="L7" s="59"/>
+      <c r="M7" s="59"/>
       <c r="O7" s="58"/>
       <c r="P7" s="60" t="s">
         <v>38</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2808,33 +2881,39 @@
       </c>
       <c r="D8" s="48"/>
       <c r="G8" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="J8" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="K8" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="L8" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O8" s="58"/>
       <c r="P8" s="60" t="s">
         <v>42</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2849,36 +2928,42 @@
       </c>
       <c r="D9" s="48"/>
       <c r="G9" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="I9" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="J9" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="K9" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="L9" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O9" s="58"/>
       <c r="P9" s="31" t="s">
         <v>60</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2893,39 +2978,45 @@
       </c>
       <c r="D10" s="48"/>
       <c r="G10" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="H10" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="I10" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="J10" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="K10" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="L10" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O10" s="58"/>
       <c r="P10" s="60" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2940,39 +3031,45 @@
       </c>
       <c r="D11" s="48"/>
       <c r="G11" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="H11" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="I11" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="J11" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="K11" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
+      <c r="L11" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O11" s="58"/>
       <c r="P11" s="60" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2987,45 +3084,51 @@
       </c>
       <c r="D12" s="48"/>
       <c r="G12" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="I12" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="J12" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="K12" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="L12" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O12" s="58"/>
       <c r="P12" s="60" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3040,39 +3143,45 @@
       </c>
       <c r="D13" s="48"/>
       <c r="G13" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(G$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="H13" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(H$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(I$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="J13" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(J$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="K13" s="61" t="n">
-        <f aca="true">OFFSET($D$68,(ROW()-ROW(K$8))*5+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+      <c r="L13" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="61" t="n">
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
+        <v>0</v>
+      </c>
       <c r="O13" s="58"/>
       <c r="P13" s="60" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3095,25 +3204,25 @@
       <c r="M14" s="2"/>
       <c r="O14" s="58"/>
       <c r="P14" s="60" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="U14" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3128,23 +3237,23 @@
       </c>
       <c r="D15" s="48"/>
       <c r="G15" s="59" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H15" s="59"/>
       <c r="I15" s="59"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="J15" s="59"/>
+      <c r="K15" s="59"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="O15" s="58"/>
       <c r="P15" s="62" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="Q15" s="63" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="R15" s="63" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3159,30 +3268,36 @@
       </c>
       <c r="D16" s="48"/>
       <c r="G16" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="H16" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="I16" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="J16" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <v>0</v>
+      </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="O16" s="58"/>
       <c r="P16" s="62" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="Q16" s="63" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="R16" s="63" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3197,23 +3312,29 @@
       </c>
       <c r="D17" s="48"/>
       <c r="G17" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="I17" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="J17" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <v>0</v>
+      </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="O17" s="58" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>14</v>
@@ -3892,19 +4013,25 @@
       </c>
       <c r="D18" s="48"/>
       <c r="G18" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="I18" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="J18" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <v>0</v>
+      </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="O18" s="58"/>
@@ -4585,19 +4712,25 @@
       </c>
       <c r="D19" s="48"/>
       <c r="G19" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="H19" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="I19" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+      <c r="J19" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <v>0</v>
+      </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="O19" s="58"/>
@@ -5278,19 +5411,25 @@
       </c>
       <c r="D20" s="48"/>
       <c r="G20" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
+      <c r="J20" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <v>0</v>
+      </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="O20" s="58"/>
@@ -5971,19 +6110,25 @@
       </c>
       <c r="D21" s="48"/>
       <c r="G21" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(G$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(H$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="I21" s="61" t="n">
-        <f aca="true">OFFSET($D$98,(ROW()-ROW(I$16))*3+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="J21" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="61" t="n">
+        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <v>0</v>
+      </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="O21" s="58"/>
@@ -8685,7 +8830,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="55" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B25" s="48" t="str">
         <f aca="false">'Адреси Контакти'!A4</f>
@@ -11527,7 +11672,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="55" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B40" s="48" t="str">
         <f aca="false">Освіта!$A$4</f>
@@ -11543,7 +11688,7 @@
       <c r="A41" s="55"/>
       <c r="B41" s="48" t="str">
         <f aca="false">Освіта!$B$4</f>
-        <v>Серія та номер дисплома (свідоцтва)</v>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C41" s="64" t="str">
         <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
@@ -11555,7 +11700,7 @@
       <c r="A42" s="55"/>
       <c r="B42" s="48" t="str">
         <f aca="false">Освіта!$C$4</f>
-        <v>Рік закінчення</v>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C42" s="64" t="str">
         <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
@@ -11567,7 +11712,7 @@
       <c r="A43" s="55"/>
       <c r="B43" s="48" t="str">
         <f aca="false">Освіта!$D$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <v>Рік закінчення</v>
       </c>
       <c r="C43" s="64" t="str">
         <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
@@ -11579,7 +11724,7 @@
       <c r="A44" s="55"/>
       <c r="B44" s="48" t="str">
         <f aca="false">Освіта!$E$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C44" s="64" t="str">
         <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
@@ -11591,7 +11736,7 @@
       <c r="A45" s="55"/>
       <c r="B45" s="48" t="str">
         <f aca="false">Освіта!$F$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C45" s="64" t="str">
         <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
@@ -11603,7 +11748,7 @@
       <c r="A46" s="55"/>
       <c r="B46" s="48" t="str">
         <f aca="false">Освіта!$G$4</f>
-        <v>Рівень освіти</v>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C46" s="64" t="str">
         <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
@@ -11614,11 +11759,11 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="55"/>
       <c r="B47" s="48" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C47" s="64" t="str">
-        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
+        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
         <v/>
       </c>
       <c r="D47" s="65"/>
@@ -11626,11 +11771,11 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="55"/>
       <c r="B48" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія та номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C48" s="64" t="str">
-        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
+        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
       <c r="D48" s="65"/>
@@ -11638,11 +11783,11 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="55"/>
       <c r="B49" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C49" s="64" t="str">
-        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
+        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
       <c r="D49" s="65"/>
@@ -11650,11 +11795,11 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="55"/>
       <c r="B50" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C50" s="64" t="str">
-        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
+        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
       <c r="D50" s="65"/>
@@ -11662,11 +11807,11 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="55"/>
       <c r="B51" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C51" s="64" t="str">
-        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
+        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
       <c r="D51" s="65"/>
@@ -11674,11 +11819,11 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="55"/>
       <c r="B52" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C52" s="64" t="str">
-        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
+        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
       <c r="D52" s="65"/>
@@ -11686,11 +11831,11 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="55"/>
       <c r="B53" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C53" s="64" t="str">
-        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
+        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
       <c r="D53" s="65"/>
@@ -11698,11 +11843,11 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="55"/>
       <c r="B54" s="48" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C54" s="64" t="str">
-        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
+        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
       <c r="D54" s="65"/>
@@ -11710,11 +11855,11 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="55"/>
       <c r="B55" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія та номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C55" s="64" t="str">
-        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
+        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
         <v/>
       </c>
       <c r="D55" s="65"/>
@@ -11722,11 +11867,11 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="55"/>
       <c r="B56" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C56" s="64" t="str">
-        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
+        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
       <c r="D56" s="65"/>
@@ -11734,11 +11879,11 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="55"/>
       <c r="B57" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C57" s="64" t="str">
-        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
+        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
       <c r="D57" s="65"/>
@@ -11746,11 +11891,11 @@
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="55"/>
       <c r="B58" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C58" s="64" t="str">
-        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
+        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
       <c r="D58" s="65"/>
@@ -11758,11 +11903,11 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="55"/>
       <c r="B59" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C59" s="64" t="str">
-        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
+        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
       <c r="D59" s="65"/>
@@ -11770,11 +11915,11 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="55"/>
       <c r="B60" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C60" s="64" t="str">
-        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
+        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
       <c r="D60" s="65"/>
@@ -11782,11 +11927,11 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="55"/>
       <c r="B61" s="48" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C61" s="64" t="str">
-        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
+        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
       <c r="D61" s="65"/>
@@ -11794,11 +11939,11 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="55"/>
       <c r="B62" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія та номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C62" s="64" t="str">
-        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
+        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
       <c r="D62" s="65"/>
@@ -11806,11 +11951,11 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="55"/>
       <c r="B63" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C63" s="64" t="str">
-        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
+        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
         <v/>
       </c>
       <c r="D63" s="65"/>
@@ -11818,11 +11963,11 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="55"/>
       <c r="B64" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C64" s="64" t="str">
-        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
+        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
       <c r="D64" s="65"/>
@@ -11830,11 +11975,11 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="55"/>
       <c r="B65" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C65" s="64" t="str">
-        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
+        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
       <c r="D65" s="65"/>
@@ -11842,11 +11987,11 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="55"/>
       <c r="B66" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C66" s="64" t="str">
-        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
+        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
       <c r="D66" s="65"/>
@@ -11854,11 +11999,11 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="55"/>
       <c r="B67" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C67" s="64" t="str">
-        <f aca="false">IF(Освіта!G8 = 0, "", $освіта.g)</f>
+        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
       <c r="D67" s="65"/>
@@ -11866,11 +12011,11 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="55"/>
       <c r="B68" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C68" s="64" t="str">
-        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
+        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
       <c r="D68" s="65"/>
@@ -11878,11 +12023,11 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="55"/>
       <c r="B69" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Диплом, номер, дата видачі</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C69" s="64" t="str">
-        <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
+        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
       <c r="D69" s="65"/>
@@ -11890,11 +12035,11 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="55"/>
       <c r="B70" s="48" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C70" s="64" t="str">
-        <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
+        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
       <c r="D70" s="65"/>
@@ -11902,11 +12047,11 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="55"/>
       <c r="B71" s="48" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Науковий ступінь, учене звання</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C71" s="64" t="str">
-        <f aca="false">IF(Освіта!D13 = 0, "", Освіта!D13)</f>
+        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
         <v/>
       </c>
       <c r="D71" s="65"/>
@@ -11914,11 +12059,11 @@
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="55"/>
       <c r="B72" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C72" s="64" t="str">
-        <f aca="false">IF(Освіта!E13 = 0, "", Освіта!E13)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C72" s="66" t="str">
+        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
       <c r="D72" s="65"/>
@@ -11926,35 +12071,35 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="55"/>
       <c r="B73" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C73" s="64" t="str">
-        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Серія дисплома</v>
+      </c>
+      <c r="C73" s="66" t="str">
+        <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
       <c r="D73" s="65"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="55"/>
-      <c r="B74" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Диплом, номер, дата видачі</v>
-      </c>
-      <c r="C74" s="64" t="str">
-        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
+      <c r="B74" s="0" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Номер диплома</v>
+      </c>
+      <c r="C74" s="66" t="str">
+        <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
         <v/>
       </c>
       <c r="D74" s="65"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="55"/>
-      <c r="B75" s="48" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C75" s="64" t="str">
-        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
+      <c r="B75" s="0" t="str">
+        <f aca="false">Освіта!$D$12</f>
+        <v>Дата видачі диплома</v>
+      </c>
+      <c r="C75" s="66" t="str">
+        <f aca="false">IF(Освіта!D13 = 0, "", Освіта!D13)</f>
         <v/>
       </c>
       <c r="D75" s="65"/>
@@ -11962,11 +12107,11 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="55"/>
       <c r="B76" s="48" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C76" s="64" t="str">
-        <f aca="false">IF(Освіта!D14 = 0, "", Освіта!D14)</f>
+        <f aca="false">Освіта!$E$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C76" s="66" t="str">
+        <f aca="false">IF(Освіта!E13 = 0, "", Освіта!E13)</f>
         <v/>
       </c>
       <c r="D76" s="65"/>
@@ -11974,11 +12119,11 @@
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="55"/>
       <c r="B77" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C77" s="64" t="str">
-        <f aca="false">IF(Освіта!E14 = 0, "", Освіта!E14)</f>
+        <f aca="false">Освіта!$F$12</f>
+        <v>Науковий ступінь, учене звання</v>
+      </c>
+      <c r="C77" s="66" t="str">
+        <f aca="false">IF(Освіта!F13 = 0, "", Освіта!F13)</f>
         <v/>
       </c>
       <c r="D77" s="65"/>
@@ -11986,95 +12131,102 @@
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="55"/>
       <c r="B78" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C78" s="64" t="str">
-        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
+        <f aca="false">Освіта!$G$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C78" s="66" t="str">
+        <f aca="false">IF(Освіта!G13 = 0, "", Освіта!G13)</f>
         <v/>
       </c>
       <c r="D78" s="65"/>
+      <c r="O78" s="0"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="55"/>
       <c r="B79" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Диплом, номер, дата видачі</v>
-      </c>
-      <c r="C79" s="64" t="str">
-        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C79" s="66" t="str">
+        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
         <v/>
       </c>
       <c r="D79" s="65"/>
+      <c r="O79" s="0"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="55"/>
       <c r="B80" s="48" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C80" s="64" t="str">
-        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Серія дисплома</v>
+      </c>
+      <c r="C80" s="66" t="str">
+        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
         <v/>
       </c>
       <c r="D80" s="65"/>
+      <c r="O80" s="0"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="55"/>
-      <c r="B81" s="48" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C81" s="64" t="str">
-        <f aca="false">IF(Освіта!D15 = 0, "", Освіта!D15)</f>
+      <c r="B81" s="0" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Номер диплома</v>
+      </c>
+      <c r="C81" s="66" t="str">
+        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
         <v/>
       </c>
       <c r="D81" s="65"/>
+      <c r="O81" s="0"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="55"/>
-      <c r="B82" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C82" s="64" t="str">
-        <f aca="false">IF(Освіта!E15 = 0, "", Освіта!E15)</f>
+      <c r="B82" s="0" t="str">
+        <f aca="false">Освіта!$D$12</f>
+        <v>Дата видачі диплома</v>
+      </c>
+      <c r="C82" s="66" t="str">
+        <f aca="false">IF(Освіта!D14 = 0, "", Освіта!D14)</f>
         <v/>
       </c>
       <c r="D82" s="65"/>
+      <c r="O82" s="0"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="55"/>
       <c r="B83" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C83" s="64" t="str">
-        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
+        <f aca="false">Освіта!$E$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C83" s="66" t="str">
+        <f aca="false">IF(Освіта!E14 = 0, "", Освіта!E14)</f>
         <v/>
       </c>
       <c r="D83" s="65"/>
+      <c r="O83" s="0"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="55"/>
       <c r="B84" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Диплом, номер, дата видачі</v>
-      </c>
-      <c r="C84" s="64" t="str">
-        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
+        <f aca="false">Освіта!$F$12</f>
+        <v>Науковий ступінь, учене звання</v>
+      </c>
+      <c r="C84" s="66" t="str">
+        <f aca="false">IF(Освіта!F14 = 0, "", Освіта!F14)</f>
         <v/>
       </c>
       <c r="D84" s="65"/>
+      <c r="O84" s="0"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="55"/>
       <c r="B85" s="48" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C85" s="64" t="str">
-        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
+        <f aca="false">Освіта!$G$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C85" s="66" t="str">
+        <f aca="false">IF(Освіта!G14 = 0, "", Освіта!G14)</f>
         <v/>
       </c>
       <c r="D85" s="65"/>
@@ -12082,11 +12234,11 @@
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="55"/>
       <c r="B86" s="48" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C86" s="64" t="str">
-        <f aca="false">IF(Освіта!D16 = 0, "", Освіта!D16)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C86" s="66" t="str">
+        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
         <v/>
       </c>
       <c r="D86" s="65"/>
@@ -12094,35 +12246,35 @@
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="55"/>
       <c r="B87" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C87" s="64" t="str">
-        <f aca="false">IF(Освіта!E16 = 0, "", Освіта!E16)</f>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Серія дисплома</v>
+      </c>
+      <c r="C87" s="66" t="str">
+        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
         <v/>
       </c>
       <c r="D87" s="65"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="55"/>
-      <c r="B88" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C88" s="64" t="str">
-        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
+      <c r="B88" s="0" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Номер диплома</v>
+      </c>
+      <c r="C88" s="66" t="str">
+        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
         <v/>
       </c>
       <c r="D88" s="65"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="55"/>
-      <c r="B89" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Диплом, номер, дата видачі</v>
-      </c>
-      <c r="C89" s="64" t="str">
-        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
+      <c r="B89" s="0" t="str">
+        <f aca="false">Освіта!$D$12</f>
+        <v>Дата видачі диплома</v>
+      </c>
+      <c r="C89" s="66" t="str">
+        <f aca="false">IF(Освіта!D15 = 0, "", Освіта!D15)</f>
         <v/>
       </c>
       <c r="D89" s="65"/>
@@ -12130,11 +12282,11 @@
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="55"/>
       <c r="B90" s="48" t="str">
-        <f aca="false">Освіта!$C$12</f>
+        <f aca="false">Освіта!$E$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C90" s="64" t="str">
-        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
+      <c r="C90" s="66" t="str">
+        <f aca="false">IF(Освіта!E15 = 0, "", Освіта!E15)</f>
         <v/>
       </c>
       <c r="D90" s="65"/>
@@ -12142,11 +12294,11 @@
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="55"/>
       <c r="B91" s="48" t="str">
-        <f aca="false">Освіта!$D$12</f>
+        <f aca="false">Освіта!$F$12</f>
         <v>Науковий ступінь, учене звання</v>
       </c>
-      <c r="C91" s="64" t="str">
-        <f aca="false">IF(Освіта!D17 = 0, "", Освіта!D17)</f>
+      <c r="C91" s="66" t="str">
+        <f aca="false">IF(Освіта!F15 = 0, "", Освіта!F15)</f>
         <v/>
       </c>
       <c r="D91" s="65"/>
@@ -12154,11 +12306,11 @@
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="55"/>
       <c r="B92" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
+        <f aca="false">Освіта!$G$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C92" s="64" t="str">
-        <f aca="false">IF(Освіта!E17 = 0, "", Освіта!E17)</f>
+      <c r="C92" s="66" t="str">
+        <f aca="false">IF(Освіта!G15 = 0, "", Освіта!G15)</f>
         <v/>
       </c>
       <c r="D92" s="65"/>
@@ -12169,8 +12321,8 @@
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C93" s="64" t="str">
-        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
+      <c r="C93" s="66" t="str">
+        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
         <v/>
       </c>
       <c r="D93" s="65"/>
@@ -12179,34 +12331,34 @@
       <c r="A94" s="55"/>
       <c r="B94" s="48" t="str">
         <f aca="false">Освіта!$B$12</f>
-        <v>Диплом, номер, дата видачі</v>
-      </c>
-      <c r="C94" s="64" t="str">
-        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
+        <v>Серія дисплома</v>
+      </c>
+      <c r="C94" s="66" t="str">
+        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
         <v/>
       </c>
       <c r="D94" s="65"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="55"/>
-      <c r="B95" s="48" t="str">
+      <c r="B95" s="0" t="str">
         <f aca="false">Освіта!$C$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C95" s="64" t="str">
-        <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
+        <v>Номер диплома</v>
+      </c>
+      <c r="C95" s="66" t="str">
+        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
         <v/>
       </c>
       <c r="D95" s="65"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="55"/>
-      <c r="B96" s="48" t="str">
+      <c r="B96" s="0" t="str">
         <f aca="false">Освіта!$D$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C96" s="64" t="str">
-        <f aca="false">IF(Освіта!D18 = 0, "", Освіта!D18)</f>
+        <v>Дата видачі диплома</v>
+      </c>
+      <c r="C96" s="66" t="str">
+        <f aca="false">IF(Освіта!D16 = 0, "", Освіта!D16)</f>
         <v/>
       </c>
       <c r="D96" s="65"/>
@@ -12215,24 +12367,22 @@
       <c r="A97" s="55"/>
       <c r="B97" s="48" t="str">
         <f aca="false">Освіта!$E$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C97" s="64" t="str">
-        <f aca="false">IF(Освіта!E18 = 0, "", Освіта!E18)</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C97" s="66" t="str">
+        <f aca="false">IF(Освіта!E16 = 0, "", Освіта!E16)</f>
         <v/>
       </c>
       <c r="D97" s="65"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="55" t="s">
-        <v>159</v>
-      </c>
+      <c r="A98" s="55"/>
       <c r="B98" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C98" s="64" t="str">
-        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
+        <f aca="false">Освіта!$F$12</f>
+        <v>Науковий ступінь, учене звання</v>
+      </c>
+      <c r="C98" s="66" t="str">
+        <f aca="false">IF(Освіта!F16 = 0, "", Освіта!F16)</f>
         <v/>
       </c>
       <c r="D98" s="65"/>
@@ -12240,11 +12390,11 @@
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="55"/>
       <c r="B99" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>ПІБ</v>
-      </c>
-      <c r="C99" s="64" t="str">
-        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
+        <f aca="false">Освіта!$G$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C99" s="66" t="str">
+        <f aca="false">IF(Освіта!G16 = 0, "", Освіта!G16)</f>
         <v/>
       </c>
       <c r="D99" s="65"/>
@@ -12252,11 +12402,11 @@
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="55"/>
       <c r="B100" s="48" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C100" s="64" t="str">
-        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C100" s="66" t="str">
+        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
         <v/>
       </c>
       <c r="D100" s="65"/>
@@ -12264,35 +12414,35 @@
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="55"/>
       <c r="B101" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C101" s="64" t="str">
-        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Серія дисплома</v>
+      </c>
+      <c r="C101" s="66" t="str">
+        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
         <v/>
       </c>
       <c r="D101" s="65"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="55"/>
-      <c r="B102" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>ПІБ</v>
-      </c>
-      <c r="C102" s="64" t="str">
-        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
+      <c r="B102" s="0" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Номер диплома</v>
+      </c>
+      <c r="C102" s="66" t="str">
+        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
         <v/>
       </c>
       <c r="D102" s="65"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="55"/>
-      <c r="B103" s="48" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C103" s="64" t="str">
-        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
+      <c r="B103" s="0" t="str">
+        <f aca="false">Освіта!$D$12</f>
+        <v>Дата видачі диплома</v>
+      </c>
+      <c r="C103" s="66" t="str">
+        <f aca="false">IF(Освіта!D17 = 0, "", Освіта!D17)</f>
         <v/>
       </c>
       <c r="D103" s="65"/>
@@ -12300,11 +12450,11 @@
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="55"/>
       <c r="B104" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C104" s="64" t="str">
-        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <f aca="false">Освіта!$E$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C104" s="66" t="str">
+        <f aca="false">IF(Освіта!E17 = 0, "", Освіта!E17)</f>
         <v/>
       </c>
       <c r="D104" s="65"/>
@@ -12312,11 +12462,11 @@
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="55"/>
       <c r="B105" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>ПІБ</v>
-      </c>
-      <c r="C105" s="64" t="str">
-        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
+        <f aca="false">Освіта!$F$12</f>
+        <v>Науковий ступінь, учене звання</v>
+      </c>
+      <c r="C105" s="66" t="str">
+        <f aca="false">IF(Освіта!F17 = 0, "", Освіта!F17)</f>
         <v/>
       </c>
       <c r="D105" s="65"/>
@@ -12324,11 +12474,11 @@
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="55"/>
       <c r="B106" s="48" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C106" s="64" t="str">
-        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
+        <f aca="false">Освіта!$G$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C106" s="66" t="str">
+        <f aca="false">IF(Освіта!G17 = 0, "", Освіта!G17)</f>
         <v/>
       </c>
       <c r="D106" s="65"/>
@@ -12336,11 +12486,11 @@
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="55"/>
       <c r="B107" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C107" s="64" t="str">
-        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C107" s="66" t="str">
+        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
         <v/>
       </c>
       <c r="D107" s="65"/>
@@ -12348,35 +12498,35 @@
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="55"/>
       <c r="B108" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>ПІБ</v>
-      </c>
-      <c r="C108" s="64" t="str">
-        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Серія дисплома</v>
+      </c>
+      <c r="C108" s="66" t="str">
+        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
         <v/>
       </c>
       <c r="D108" s="65"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="55"/>
-      <c r="B109" s="48" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C109" s="64" t="str">
-        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
+      <c r="B109" s="0" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Номер диплома</v>
+      </c>
+      <c r="C109" s="66" t="str">
+        <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
       <c r="D109" s="65"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="55"/>
-      <c r="B110" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C110" s="64" t="str">
-        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+      <c r="B110" s="0" t="str">
+        <f aca="false">Освіта!$D$12</f>
+        <v>Дата видачі диплома</v>
+      </c>
+      <c r="C110" s="66" t="str">
+        <f aca="false">IF(Освіта!D18 = 0, "", Освіта!D18)</f>
         <v/>
       </c>
       <c r="D110" s="65"/>
@@ -12384,11 +12534,11 @@
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="55"/>
       <c r="B111" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>ПІБ</v>
-      </c>
-      <c r="C111" s="64" t="str">
-        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
+        <f aca="false">Освіта!$E$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C111" s="66" t="str">
+        <f aca="false">IF(Освіта!E18 = 0, "", Освіта!E18)</f>
         <v/>
       </c>
       <c r="D111" s="65"/>
@@ -12396,11 +12546,11 @@
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="55"/>
       <c r="B112" s="48" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C112" s="64" t="str">
-        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
+        <f aca="false">Освіта!$F$12</f>
+        <v>Науковий ступінь, учене звання</v>
+      </c>
+      <c r="C112" s="66" t="str">
+        <f aca="false">IF(Освіта!F18 = 0, "", Освіта!F18)</f>
         <v/>
       </c>
       <c r="D112" s="65"/>
@@ -12408,23 +12558,25 @@
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="55"/>
       <c r="B113" s="48" t="str">
+        <f aca="false">Освіта!$G$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C113" s="66" t="str">
+        <f aca="false">IF(Освіта!G18 = 0, "", Освіта!G18)</f>
+        <v/>
+      </c>
+      <c r="D113" s="65"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="55" t="s">
+        <v>162</v>
+      </c>
+      <c r="B114" s="48" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C113" s="64" t="str">
-        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
-        <v/>
-      </c>
-      <c r="D113" s="65"/>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="55"/>
-      <c r="B114" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>ПІБ</v>
-      </c>
-      <c r="C114" s="64" t="str">
-        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
+      <c r="C114" s="67" t="str">
+        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
         <v/>
       </c>
       <c r="D114" s="65"/>
@@ -12432,182 +12584,526 @@
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="55"/>
       <c r="B115" s="48" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C115" s="67" t="str">
+        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
+        <v/>
+      </c>
+      <c r="D115" s="65"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="55"/>
+      <c r="B116" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C115" s="64" t="str">
-        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
-        <v/>
-      </c>
-      <c r="D115" s="65"/>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="55" t="s">
-        <v>160</v>
-      </c>
-      <c r="B116" s="48" t="str">
-        <f aca="false">Документи!A4</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C116" s="56" t="str">
-        <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
-        <v/>
-      </c>
-      <c r="D116" s="48"/>
+        <v>Ім’я</v>
+      </c>
+      <c r="C116" s="67" t="str">
+        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
+        <v/>
+      </c>
+      <c r="D116" s="65"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="55"/>
       <c r="B117" s="48" t="str">
-        <f aca="false">Документи!A5</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C117" s="48" t="str">
-        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
-        <v/>
-      </c>
-      <c r="D117" s="48"/>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C117" s="67" t="str">
+        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
+        <v/>
+      </c>
+      <c r="D117" s="65"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="55"/>
       <c r="B118" s="48" t="str">
-        <f aca="false">Документи!A6</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C118" s="48" t="str">
-        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
-        <v/>
-      </c>
-      <c r="D118" s="48"/>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C118" s="67" t="str">
+        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
+        <v/>
+      </c>
+      <c r="D118" s="65"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="55"/>
       <c r="B119" s="48" t="str">
-        <f aca="false">Документи!A7</f>
-        <v>Дата видачі</v>
-      </c>
-      <c r="C119" s="48" t="str">
-        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
-        <v/>
-      </c>
-      <c r="D119" s="48"/>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C119" s="67" t="str">
+        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <v/>
+      </c>
+      <c r="D119" s="65"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="55"/>
       <c r="B120" s="48" t="str">
-        <f aca="false">Документи!A10</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C120" s="56" t="str">
-        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
-        <v/>
-      </c>
-      <c r="D120" s="48"/>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C120" s="67" t="str">
+        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
+        <v/>
+      </c>
+      <c r="D120" s="65"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="55"/>
-      <c r="B121" s="48" t="str">
-        <f aca="false">Документи!A11</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C121" s="48" t="str">
-        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
-        <v/>
-      </c>
-      <c r="D121" s="48"/>
+      <c r="B121" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C121" s="67" t="str">
+        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
+        <v/>
+      </c>
+      <c r="D121" s="65"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="55"/>
       <c r="B122" s="48" t="str">
-        <f aca="false">Документи!A12</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C122" s="48" t="str">
-        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
-        <v/>
-      </c>
-      <c r="D122" s="48"/>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C122" s="67" t="str">
+        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
+        <v/>
+      </c>
+      <c r="D122" s="65"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="55"/>
       <c r="B123" s="48" t="str">
-        <f aca="false">Документи!A13</f>
-        <v>Дата видачі</v>
-      </c>
-      <c r="C123" s="48" t="str">
-        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
-        <v/>
-      </c>
-      <c r="D123" s="48"/>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C123" s="67" t="str">
+        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
+        <v/>
+      </c>
+      <c r="D123" s="65"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="55"/>
-      <c r="B124" s="48" t="s">
-        <v>161</v>
-      </c>
-      <c r="C124" s="48"/>
-      <c r="D124" s="48"/>
+      <c r="B124" s="48" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C124" s="67" t="str">
+        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <v/>
+      </c>
+      <c r="D124" s="65"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="55"/>
       <c r="B125" s="48" t="str">
-        <f aca="false">Документи!A16</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C125" s="56" t="str">
-        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
-        <v/>
-      </c>
-      <c r="D125" s="48"/>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C125" s="67" t="str">
+        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
+        <v/>
+      </c>
+      <c r="D125" s="65"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="55"/>
-      <c r="B126" s="48" t="str">
-        <f aca="false">Документи!A17</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C126" s="48" t="str">
-        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
-        <v/>
-      </c>
-      <c r="D126" s="48"/>
+      <c r="B126" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C126" s="67" t="str">
+        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
+        <v/>
+      </c>
+      <c r="D126" s="65"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="55"/>
       <c r="B127" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C127" s="67" t="str">
+        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
+        <v/>
+      </c>
+      <c r="D127" s="65"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="55"/>
+      <c r="B128" s="48" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C128" s="67" t="str">
+        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
+        <v/>
+      </c>
+      <c r="D128" s="65"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="55"/>
+      <c r="B129" s="48" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C129" s="67" t="str">
+        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <v/>
+      </c>
+      <c r="D129" s="65"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="55"/>
+      <c r="B130" s="48" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C130" s="67" t="str">
+        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
+        <v/>
+      </c>
+      <c r="D130" s="65"/>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="55"/>
+      <c r="B131" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C131" s="67" t="str">
+        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
+        <v/>
+      </c>
+      <c r="D131" s="65"/>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="55"/>
+      <c r="B132" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C132" s="67" t="str">
+        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
+        <v/>
+      </c>
+      <c r="D132" s="65"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="55"/>
+      <c r="B133" s="48" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C133" s="67" t="str">
+        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
+        <v/>
+      </c>
+      <c r="D133" s="65"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="55"/>
+      <c r="B134" s="48" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C134" s="67" t="str">
+        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+        <v/>
+      </c>
+      <c r="D134" s="65"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="55"/>
+      <c r="B135" s="48" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C135" s="67" t="str">
+        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
+        <v/>
+      </c>
+      <c r="D135" s="65"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="55"/>
+      <c r="B136" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C136" s="67" t="str">
+        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
+        <v/>
+      </c>
+      <c r="D136" s="65"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="55"/>
+      <c r="B137" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C137" s="67" t="str">
+        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
+        <v/>
+      </c>
+      <c r="D137" s="65"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="55"/>
+      <c r="B138" s="48" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C138" s="67" t="str">
+        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
+        <v/>
+      </c>
+      <c r="D138" s="65"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="55"/>
+      <c r="B139" s="48" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C139" s="67" t="str">
+        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
+        <v/>
+      </c>
+      <c r="D139" s="65"/>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="55"/>
+      <c r="B140" s="48" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C140" s="67" t="str">
+        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
+        <v/>
+      </c>
+      <c r="D140" s="65"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="55"/>
+      <c r="B141" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C141" s="67" t="str">
+        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
+        <v/>
+      </c>
+      <c r="D141" s="65"/>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="55"/>
+      <c r="B142" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C142" s="67" t="str">
+        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
+        <v/>
+      </c>
+      <c r="D142" s="65"/>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="55"/>
+      <c r="B143" s="48" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C143" s="67" t="str">
+        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
+        <v/>
+      </c>
+      <c r="D143" s="65"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="B144" s="48" t="str">
+        <f aca="false">Документи!A4</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C144" s="56" t="str">
+        <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
+        <v/>
+      </c>
+      <c r="D144" s="48"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="55"/>
+      <c r="B145" s="48" t="str">
+        <f aca="false">Документи!A5</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C145" s="48" t="str">
+        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
+        <v/>
+      </c>
+      <c r="D145" s="48"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="55"/>
+      <c r="B146" s="48" t="str">
+        <f aca="false">Документи!A6</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C146" s="48" t="str">
+        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
+        <v/>
+      </c>
+      <c r="D146" s="48"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="55"/>
+      <c r="B147" s="48" t="str">
+        <f aca="false">Документи!A7</f>
+        <v>Дата видачі</v>
+      </c>
+      <c r="C147" s="48" t="str">
+        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
+        <v/>
+      </c>
+      <c r="D147" s="48"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="55"/>
+      <c r="B148" s="48" t="str">
+        <f aca="false">Документи!A10</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C148" s="56" t="str">
+        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
+        <v/>
+      </c>
+      <c r="D148" s="48"/>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="55"/>
+      <c r="B149" s="48" t="str">
+        <f aca="false">Документи!A11</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C149" s="48" t="str">
+        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
+        <v/>
+      </c>
+      <c r="D149" s="48"/>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="55"/>
+      <c r="B150" s="48" t="str">
+        <f aca="false">Документи!A12</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C150" s="48" t="str">
+        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
+        <v/>
+      </c>
+      <c r="D150" s="48"/>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="55"/>
+      <c r="B151" s="48" t="str">
+        <f aca="false">Документи!A13</f>
+        <v>Дата видачі</v>
+      </c>
+      <c r="C151" s="48" t="str">
+        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
+        <v/>
+      </c>
+      <c r="D151" s="48"/>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="55"/>
+      <c r="B152" s="48" t="s">
+        <v>164</v>
+      </c>
+      <c r="C152" s="48"/>
+      <c r="D152" s="48"/>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="55"/>
+      <c r="B153" s="48" t="str">
+        <f aca="false">Документи!A16</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C153" s="56" t="str">
+        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
+        <v/>
+      </c>
+      <c r="D153" s="48"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="55"/>
+      <c r="B154" s="48" t="str">
+        <f aca="false">Документи!A17</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C154" s="48" t="str">
+        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
+        <v/>
+      </c>
+      <c r="D154" s="48"/>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="55"/>
+      <c r="B155" s="48" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C127" s="48" t="str">
+      <c r="C155" s="48" t="str">
         <f aca="false">IF(Документи!B18 = 0, "", Документи!B18)</f>
         <v/>
       </c>
-      <c r="D127" s="48"/>
-    </row>
+      <c r="D155" s="48"/>
+    </row>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="G1:N1"/>
     <mergeCell ref="Q1:T1"/>
     <mergeCell ref="A2:A24"/>
     <mergeCell ref="O2:O16"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G7:M7"/>
+    <mergeCell ref="G15:K15"/>
     <mergeCell ref="O17:O28"/>
     <mergeCell ref="A25:A39"/>
-    <mergeCell ref="A40:A97"/>
-    <mergeCell ref="A98:A115"/>
-    <mergeCell ref="A116:A127"/>
+    <mergeCell ref="A40:A113"/>
+    <mergeCell ref="A114:A143"/>
+    <mergeCell ref="A144:A155"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:I21" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:K21" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D40" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D40:D44" type="list">
       <formula1>'Системна інформація'!$Q$27:$ZA$27</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D42" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D46" type="list">
       <formula1>'Системна інформація'!$Q$11:$ZA$11</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
fix: delete unnecessary columns in Excel export template
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="162">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -250,201 +250,192 @@
     <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
   </si>
   <si>
-    <t xml:space="preserve">Серія дисплома</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Номер диплома</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата видачі диплома</t>
+    <t xml:space="preserve">Рівень підготовки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Склад родини</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По-батькові</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік народження</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри!!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ДОКУМЕНТИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія та номер </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ким виданий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата видачі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квіток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК224345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закордоний паспорт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: FF453210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва сторінки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва поля</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле для оновлення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле з актуальною інформацією</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип заповнення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва списку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Основна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Визначений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професійно-технічна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неповна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">НПП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ІТС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">одружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неодружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">незаміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучена</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдова</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдівець</t>
+  </si>
+  <si>
+    <t xml:space="preserve">військовозобов'язаний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">призовник</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">обмежено-придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">непридатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не перебуває</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТАК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">НІ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">денна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вечірня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заочна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">спеціаліст</t>
+  </si>
+  <si>
+    <t xml:space="preserve">бакалавр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">магістр</t>
   </si>
   <si>
     <t xml:space="preserve">Науковий ступінь, учене звання</t>
   </si>
   <si>
-    <t xml:space="preserve">Рівень підготовки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Склад родини</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">По-батькові</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік народження</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри!!!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДОКУМЕНТИ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип документу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія та номер </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ким виданий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата видачі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військовий квіток</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК224345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закордоний паспорт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: FF453210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва сторінки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва поля</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле для оновлення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле з актуальною інформацією</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип заповнення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва списку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Значення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Основна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Визначений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">професійно-технічна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неповна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ППС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ІТС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">одружений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неодружений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">заміжня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">незаміжня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">розлучений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">розлучена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вдова</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вдівець</t>
-  </si>
-  <si>
-    <t xml:space="preserve">військовозобов'язаний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">призовник</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">придатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">обмежено-придатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">непридатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не перебуває</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ТАК</t>
-  </si>
-  <si>
-    <t xml:space="preserve">НІ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">денна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вечірня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">заочна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">спеціаліст</t>
-  </si>
-  <si>
-    <t xml:space="preserve">бакалавр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">магістр</t>
-  </si>
-  <si>
     <t xml:space="preserve">кандидат наук</t>
   </si>
   <si>
@@ -502,7 +493,7 @@
     <t xml:space="preserve">Військовий квиток</t>
   </si>
   <si>
-    <t xml:space="preserve">Посвідчення особи офіцера</t>
+    <t xml:space="preserve">Військовий квиток офіцера запасу</t>
   </si>
   <si>
     <t xml:space="preserve">З бази даних</t>
@@ -736,7 +727,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -993,6 +984,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2074,98 +2069,85 @@
         <v>73</v>
       </c>
       <c r="B12" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" s="36" t="s">
-        <v>77</v>
-      </c>
-      <c r="G12" s="35" t="s">
-        <v>78</v>
-      </c>
+      <c r="D12" s="0"/>
+      <c r="E12" s="0"/>
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
       <c r="B13" s="40"/>
       <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
+      <c r="D13" s="0"/>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="40"/>
       <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
+      <c r="D14" s="0"/>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
       <c r="B15" s="40"/>
       <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
+      <c r="D15" s="0"/>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
       <c r="B16" s="40"/>
       <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
+      <c r="D16" s="0"/>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="37"/>
       <c r="B17" s="40"/>
       <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
+      <c r="D17" s="0"/>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37"/>
       <c r="B18" s="40"/>
       <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33"/>
-      <c r="B19" s="33"/>
-      <c r="E19" s="39" t="s">
+      <c r="B19" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="F19" s="39" t="s">
+      <c r="C19" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="39" t="s">
-        <v>12</v>
-      </c>
+      <c r="E19" s="0"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="0"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F13:F18" type="list">
-      <formula1>'Системна інформація'!$Q$12:$ZA$12</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G13:G18" type="list">
+  <dataValidations count="5">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C13:C18" type="list">
       <formula1>'Системна інформація'!$Q$13:$ZA$13</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2211,12 +2193,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="42" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
@@ -2225,7 +2207,7 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B4" s="44" t="s">
         <v>5</v>
@@ -2234,10 +2216,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2287,7 +2269,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2324,21 +2306,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="41" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="47" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D144 = 0, "", 'Системна інформація'!D144)</f>
+        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="s">
@@ -2347,37 +2329,37 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="48" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D145 = 0, "", 'Системна інформація'!D145)</f>
+        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
         <v/>
       </c>
       <c r="D5" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D146 = 0, "", 'Системна інформація'!D146)</f>
+        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
         <v/>
       </c>
       <c r="D6" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D147 = 0, "", 'Системна інформація'!D147)</f>
+        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
         <v/>
       </c>
       <c r="D7" s="2" t="s">
@@ -2386,16 +2368,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="47" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D148 = 0, "", 'Системна інформація'!D148)</f>
+        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="s">
@@ -2404,34 +2386,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D149 = 0, "", 'Системна інформація'!D149)</f>
+        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
         <v/>
       </c>
       <c r="D11" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D150 = 0, "", 'Системна інформація'!D150)</f>
+        <f aca="false">IF('Системна інформація'!D126 = 0, "", 'Системна інформація'!D126)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D151 = 0, "", 'Системна інформація'!D151)</f>
+        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
         <v/>
       </c>
       <c r="D13" s="2" t="s">
@@ -2440,42 +2422,42 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="41" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D153 = 0, "", 'Системна інформація'!D153)</f>
+        <f aca="false">IF('Системна інформація'!D129 = 0, "", 'Системна інформація'!D129)</f>
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="48" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D154 = 0, "", 'Системна інформація'!D154)</f>
+        <f aca="false">IF('Системна інформація'!D130 = 0, "", 'Системна інформація'!D130)</f>
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="48" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D155 = 0, "", 'Системна інформація'!D155)</f>
+        <f aca="false">IF('Системна інформація'!D131 = 0, "", 'Системна інформація'!D131)</f>
         <v/>
       </c>
       <c r="D18" s="2" t="s">
@@ -2521,20 +2503,20 @@
   <sheetData>
     <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B1" s="51" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C1" s="51" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D1" s="51" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="52" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H1" s="52"/>
       <c r="I1" s="52"/>
@@ -2544,13 +2526,13 @@
       <c r="M1" s="52"/>
       <c r="N1" s="52"/>
       <c r="O1" s="53" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="P1" s="54" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="Q1" s="53" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="R1" s="53"/>
       <c r="S1" s="53"/>
@@ -2558,7 +2540,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="55" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B2" s="48" t="str">
         <f aca="false">Основна!A9</f>
@@ -2602,28 +2584,28 @@
         <v>0</v>
       </c>
       <c r="O2" s="58" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>11</v>
       </c>
       <c r="Q2" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2674,10 +2656,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2728,28 +2710,28 @@
         <v>18</v>
       </c>
       <c r="Q4" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="U4" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="X4" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2800,10 +2782,10 @@
         <v>30</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2847,26 +2829,22 @@
       </c>
       <c r="D7" s="48"/>
       <c r="G7" s="59" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H7" s="59"/>
       <c r="I7" s="59"/>
-      <c r="J7" s="59"/>
-      <c r="K7" s="59"/>
-      <c r="L7" s="59"/>
-      <c r="M7" s="59"/>
       <c r="O7" s="58"/>
       <c r="P7" s="60" t="s">
         <v>38</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2881,31 +2859,15 @@
       </c>
       <c r="D8" s="48"/>
       <c r="G8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="M8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="O8" s="58"/>
@@ -2913,7 +2875,7 @@
         <v>42</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2928,31 +2890,15 @@
       </c>
       <c r="D9" s="48"/>
       <c r="G9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="I9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="M9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="O9" s="58"/>
@@ -2960,10 +2906,10 @@
         <v>60</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2978,31 +2924,15 @@
       </c>
       <c r="D10" s="48"/>
       <c r="G10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="H10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="I10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="M10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="O10" s="58"/>
@@ -3010,13 +2940,13 @@
         <v>69</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3031,31 +2961,15 @@
       </c>
       <c r="D11" s="48"/>
       <c r="G11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="H11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="I11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="O11" s="58"/>
@@ -3063,13 +2977,13 @@
         <v>70</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,51 +2998,35 @@
       </c>
       <c r="D12" s="48"/>
       <c r="G12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="I12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="M12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="O12" s="58"/>
       <c r="P12" s="60" t="s">
-        <v>77</v>
+        <v>135</v>
       </c>
       <c r="Q12" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="T12" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="R12" s="2" t="s">
+      <c r="U12" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="S12" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3143,45 +3041,29 @@
       </c>
       <c r="D13" s="48"/>
       <c r="G13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="H13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(J$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(K$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(L$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(M$8))*7+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="O13" s="58"/>
       <c r="P13" s="60" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3204,25 +3086,25 @@
       <c r="M14" s="2"/>
       <c r="O14" s="58"/>
       <c r="P14" s="60" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="Q14" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="T14" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="R14" s="2" t="s">
+      <c r="U14" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="S14" s="2" t="s">
+      <c r="V14" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="T14" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="U14" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="V14" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3237,7 +3119,7 @@
       </c>
       <c r="D15" s="48"/>
       <c r="G15" s="59" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H15" s="59"/>
       <c r="I15" s="59"/>
@@ -3247,13 +3129,13 @@
       <c r="M15" s="2"/>
       <c r="O15" s="58"/>
       <c r="P15" s="62" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Q15" s="63" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="R15" s="63" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3268,36 +3150,36 @@
       </c>
       <c r="D16" s="48"/>
       <c r="G16" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="H16" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="I16" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="J16" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="K16" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="O16" s="58"/>
       <c r="P16" s="62" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="Q16" s="63" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="R16" s="63" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3312,29 +3194,29 @@
       </c>
       <c r="D17" s="48"/>
       <c r="G17" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="I17" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="K17" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="O17" s="58" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>14</v>
@@ -4013,23 +3895,23 @@
       </c>
       <c r="D18" s="48"/>
       <c r="G18" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="I18" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="J18" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="K18" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="L18" s="2"/>
@@ -4712,23 +4594,23 @@
       </c>
       <c r="D19" s="48"/>
       <c r="G19" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="H19" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="I19" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="J19" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="K19" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="L19" s="2"/>
@@ -5411,23 +5293,23 @@
       </c>
       <c r="D20" s="48"/>
       <c r="G20" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="J20" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="K20" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="L20" s="2"/>
@@ -6110,23 +5992,23 @@
       </c>
       <c r="D21" s="48"/>
       <c r="G21" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="I21" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="K21" s="61" t="n">
-        <f aca="true">OFFSET($D$114,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="L21" s="2"/>
@@ -8830,7 +8712,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="55" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B25" s="48" t="str">
         <f aca="false">'Адреси Контакти'!A4</f>
@@ -11672,1405 +11554,1134 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="55" t="s">
-        <v>161</v>
-      </c>
-      <c r="B40" s="48" t="str">
+        <v>158</v>
+      </c>
+      <c r="B40" s="64" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C40" s="64" t="str">
+      <c r="C40" s="65" t="str">
         <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
         <v/>
       </c>
-      <c r="D40" s="65"/>
+      <c r="D40" s="66"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="55"/>
-      <c r="B41" s="48" t="str">
+      <c r="B41" s="64" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія дисплома (свідоцтва)</v>
       </c>
-      <c r="C41" s="64" t="str">
+      <c r="C41" s="65" t="str">
         <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
         <v/>
       </c>
-      <c r="D41" s="65"/>
+      <c r="D41" s="66"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="55"/>
-      <c r="B42" s="48" t="str">
+      <c r="B42" s="64" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C42" s="64" t="str">
+      <c r="C42" s="65" t="str">
         <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
-      <c r="D42" s="65"/>
+      <c r="D42" s="66"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="55"/>
-      <c r="B43" s="48" t="str">
+      <c r="B43" s="64" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C43" s="64" t="str">
+      <c r="C43" s="65" t="str">
         <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
-      <c r="D43" s="65"/>
+      <c r="D43" s="66"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="55"/>
-      <c r="B44" s="48" t="str">
+      <c r="B44" s="64" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C44" s="64" t="str">
+      <c r="C44" s="65" t="str">
         <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
-      <c r="D44" s="65"/>
+      <c r="D44" s="66"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="55"/>
-      <c r="B45" s="48" t="str">
+      <c r="B45" s="64" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C45" s="64" t="str">
+      <c r="C45" s="65" t="str">
         <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
-      <c r="D45" s="65"/>
+      <c r="D45" s="66"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="55"/>
-      <c r="B46" s="48" t="str">
+      <c r="B46" s="64" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C46" s="64" t="str">
+      <c r="C46" s="65" t="str">
         <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
-      <c r="D46" s="65"/>
+      <c r="D46" s="66"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="55"/>
-      <c r="B47" s="48" t="str">
+      <c r="B47" s="64" t="str">
         <f aca="false">Освіта!$H$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C47" s="64" t="str">
+      <c r="C47" s="65" t="str">
         <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
         <v/>
       </c>
-      <c r="D47" s="65"/>
+      <c r="D47" s="66"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="55"/>
-      <c r="B48" s="48" t="str">
+      <c r="B48" s="64" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C48" s="64" t="str">
+      <c r="C48" s="65" t="str">
         <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
-      <c r="D48" s="65"/>
+      <c r="D48" s="66"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="55"/>
-      <c r="B49" s="48" t="str">
+      <c r="B49" s="64" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія дисплома (свідоцтва)</v>
       </c>
-      <c r="C49" s="64" t="str">
+      <c r="C49" s="65" t="str">
         <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
-      <c r="D49" s="65"/>
+      <c r="D49" s="66"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="55"/>
-      <c r="B50" s="48" t="str">
+      <c r="B50" s="64" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C50" s="64" t="str">
+      <c r="C50" s="65" t="str">
         <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
-      <c r="D50" s="65"/>
+      <c r="D50" s="66"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="55"/>
-      <c r="B51" s="48" t="str">
+      <c r="B51" s="64" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C51" s="64" t="str">
+      <c r="C51" s="65" t="str">
         <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
-      <c r="D51" s="65"/>
+      <c r="D51" s="66"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="55"/>
-      <c r="B52" s="48" t="str">
+      <c r="B52" s="64" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C52" s="64" t="str">
+      <c r="C52" s="65" t="str">
         <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
-      <c r="D52" s="65"/>
+      <c r="D52" s="66"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="55"/>
-      <c r="B53" s="48" t="str">
+      <c r="B53" s="64" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C53" s="64" t="str">
+      <c r="C53" s="65" t="str">
         <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
-      <c r="D53" s="65"/>
+      <c r="D53" s="66"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="55"/>
-      <c r="B54" s="48" t="str">
+      <c r="B54" s="64" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C54" s="64" t="str">
+      <c r="C54" s="65" t="str">
         <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
-      <c r="D54" s="65"/>
+      <c r="D54" s="66"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="55"/>
-      <c r="B55" s="48" t="str">
+      <c r="B55" s="64" t="str">
         <f aca="false">Освіта!$H$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C55" s="64" t="str">
+      <c r="C55" s="65" t="str">
         <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
         <v/>
       </c>
-      <c r="D55" s="65"/>
+      <c r="D55" s="66"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="55"/>
-      <c r="B56" s="48" t="str">
+      <c r="B56" s="64" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C56" s="64" t="str">
+      <c r="C56" s="65" t="str">
         <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
-      <c r="D56" s="65"/>
+      <c r="D56" s="66"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="55"/>
-      <c r="B57" s="48" t="str">
+      <c r="B57" s="64" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія дисплома (свідоцтва)</v>
       </c>
-      <c r="C57" s="64" t="str">
+      <c r="C57" s="65" t="str">
         <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
-      <c r="D57" s="65"/>
+      <c r="D57" s="66"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="55"/>
-      <c r="B58" s="48" t="str">
+      <c r="B58" s="64" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C58" s="64" t="str">
+      <c r="C58" s="65" t="str">
         <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
-      <c r="D58" s="65"/>
+      <c r="D58" s="66"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="55"/>
-      <c r="B59" s="48" t="str">
+      <c r="B59" s="64" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C59" s="64" t="str">
+      <c r="C59" s="65" t="str">
         <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
-      <c r="D59" s="65"/>
+      <c r="D59" s="66"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="55"/>
-      <c r="B60" s="48" t="str">
+      <c r="B60" s="64" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C60" s="64" t="str">
+      <c r="C60" s="65" t="str">
         <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
-      <c r="D60" s="65"/>
+      <c r="D60" s="66"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="55"/>
-      <c r="B61" s="48" t="str">
+      <c r="B61" s="64" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C61" s="64" t="str">
+      <c r="C61" s="65" t="str">
         <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
-      <c r="D61" s="65"/>
+      <c r="D61" s="66"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="55"/>
-      <c r="B62" s="48" t="str">
+      <c r="B62" s="64" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C62" s="64" t="str">
+      <c r="C62" s="65" t="str">
         <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
-      <c r="D62" s="65"/>
+      <c r="D62" s="66"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="55"/>
-      <c r="B63" s="48" t="str">
+      <c r="B63" s="64" t="str">
         <f aca="false">Освіта!$H$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C63" s="64" t="str">
+      <c r="C63" s="65" t="str">
         <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
         <v/>
       </c>
-      <c r="D63" s="65"/>
+      <c r="D63" s="66"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="55"/>
-      <c r="B64" s="48" t="str">
+      <c r="B64" s="64" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
-      <c r="C64" s="64" t="str">
+      <c r="C64" s="65" t="str">
         <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
-      <c r="D64" s="65"/>
+      <c r="D64" s="66"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="55"/>
-      <c r="B65" s="48" t="str">
+      <c r="B65" s="64" t="str">
         <f aca="false">Освіта!$B$4</f>
         <v>Серія дисплома (свідоцтва)</v>
       </c>
-      <c r="C65" s="64" t="str">
+      <c r="C65" s="65" t="str">
         <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
-      <c r="D65" s="65"/>
+      <c r="D65" s="66"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="55"/>
-      <c r="B66" s="48" t="str">
+      <c r="B66" s="64" t="str">
         <f aca="false">Освіта!$C$4</f>
         <v>Номер дисплома (свідоцтва)</v>
       </c>
-      <c r="C66" s="64" t="str">
+      <c r="C66" s="65" t="str">
         <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
-      <c r="D66" s="65"/>
+      <c r="D66" s="66"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="55"/>
-      <c r="B67" s="48" t="str">
+      <c r="B67" s="64" t="str">
         <f aca="false">Освіта!$D$4</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C67" s="64" t="str">
+      <c r="C67" s="65" t="str">
         <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
-      <c r="D67" s="65"/>
+      <c r="D67" s="66"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="55"/>
-      <c r="B68" s="48" t="str">
+      <c r="B68" s="64" t="str">
         <f aca="false">Освіта!$E$4</f>
         <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
-      <c r="C68" s="64" t="str">
+      <c r="C68" s="65" t="str">
         <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
-      <c r="D68" s="65"/>
+      <c r="D68" s="66"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="55"/>
-      <c r="B69" s="48" t="str">
+      <c r="B69" s="64" t="str">
         <f aca="false">Освіта!$F$4</f>
         <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
-      <c r="C69" s="64" t="str">
+      <c r="C69" s="65" t="str">
         <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
-      <c r="D69" s="65"/>
+      <c r="D69" s="66"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="55"/>
-      <c r="B70" s="48" t="str">
+      <c r="B70" s="64" t="str">
         <f aca="false">Освіта!$G$4</f>
         <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
-      <c r="C70" s="64" t="str">
+      <c r="C70" s="65" t="str">
         <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
-      <c r="D70" s="65"/>
+      <c r="D70" s="66"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="55"/>
-      <c r="B71" s="48" t="str">
+      <c r="B71" s="64" t="str">
         <f aca="false">Освіта!$H$4</f>
         <v>Рівень освіти</v>
       </c>
-      <c r="C71" s="64" t="str">
+      <c r="C71" s="65" t="str">
         <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
         <v/>
       </c>
-      <c r="D71" s="65"/>
+      <c r="D71" s="66"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="55"/>
-      <c r="B72" s="48" t="str">
+      <c r="B72" s="64" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C72" s="66" t="str">
+      <c r="C72" s="67" t="str">
         <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
-      <c r="D72" s="65"/>
+      <c r="D72" s="66"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="55"/>
-      <c r="B73" s="48" t="str">
+      <c r="B73" s="64" t="str">
         <f aca="false">Освіта!$B$12</f>
-        <v>Серія дисплома</v>
-      </c>
-      <c r="C73" s="66" t="str">
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C73" s="67" t="str">
         <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
-      <c r="D73" s="65"/>
+      <c r="D73" s="66"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="55"/>
-      <c r="B74" s="0" t="str">
+      <c r="B74" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
-        <v>Номер диплома</v>
-      </c>
-      <c r="C74" s="66" t="str">
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C74" s="67" t="str">
         <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
         <v/>
       </c>
-      <c r="D74" s="65"/>
+      <c r="D74" s="66"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="55"/>
-      <c r="B75" s="0" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Дата видачі диплома</v>
-      </c>
-      <c r="C75" s="66" t="str">
-        <f aca="false">IF(Освіта!D13 = 0, "", Освіта!D13)</f>
-        <v/>
-      </c>
-      <c r="D75" s="65"/>
+      <c r="B75" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C75" s="67" t="str">
+        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
+        <v/>
+      </c>
+      <c r="D75" s="66"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="55"/>
-      <c r="B76" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
+      <c r="B76" s="64" t="str">
+        <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C76" s="66" t="str">
-        <f aca="false">IF(Освіта!E13 = 0, "", Освіта!E13)</f>
-        <v/>
-      </c>
-      <c r="D76" s="65"/>
+      <c r="C76" s="67" t="str">
+        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
+        <v/>
+      </c>
+      <c r="D76" s="66"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="55"/>
-      <c r="B77" s="48" t="str">
-        <f aca="false">Освіта!$F$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C77" s="66" t="str">
-        <f aca="false">IF(Освіта!F13 = 0, "", Освіта!F13)</f>
-        <v/>
-      </c>
-      <c r="D77" s="65"/>
+      <c r="B77" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C77" s="67" t="str">
+        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
+        <v/>
+      </c>
+      <c r="D77" s="66"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="55"/>
-      <c r="B78" s="48" t="str">
-        <f aca="false">Освіта!$G$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C78" s="66" t="str">
-        <f aca="false">IF(Освіта!G13 = 0, "", Освіта!G13)</f>
-        <v/>
-      </c>
-      <c r="D78" s="65"/>
-      <c r="O78" s="0"/>
+      <c r="B78" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C78" s="67" t="str">
+        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
+        <v/>
+      </c>
+      <c r="D78" s="66"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="55"/>
-      <c r="B79" s="48" t="str">
+      <c r="B79" s="64" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C79" s="67" t="str">
+        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
+        <v/>
+      </c>
+      <c r="D79" s="66"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="55"/>
+      <c r="B80" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C80" s="67" t="str">
+        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
+        <v/>
+      </c>
+      <c r="D80" s="66"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="55"/>
+      <c r="B81" s="64" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C79" s="66" t="str">
-        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
-        <v/>
-      </c>
-      <c r="D79" s="65"/>
-      <c r="O79" s="0"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="55"/>
-      <c r="B80" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Серія дисплома</v>
-      </c>
-      <c r="C80" s="66" t="str">
-        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
-        <v/>
-      </c>
-      <c r="D80" s="65"/>
-      <c r="O80" s="0"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="55"/>
-      <c r="B81" s="0" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Номер диплома</v>
-      </c>
-      <c r="C81" s="66" t="str">
-        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
-        <v/>
-      </c>
-      <c r="D81" s="65"/>
-      <c r="O81" s="0"/>
+      <c r="C81" s="67" t="str">
+        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
+        <v/>
+      </c>
+      <c r="D81" s="66"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="55"/>
-      <c r="B82" s="0" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Дата видачі диплома</v>
-      </c>
-      <c r="C82" s="66" t="str">
-        <f aca="false">IF(Освіта!D14 = 0, "", Освіта!D14)</f>
-        <v/>
-      </c>
-      <c r="D82" s="65"/>
-      <c r="O82" s="0"/>
+      <c r="B82" s="64" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C82" s="67" t="str">
+        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
+        <v/>
+      </c>
+      <c r="D82" s="66"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="55"/>
-      <c r="B83" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C83" s="66" t="str">
-        <f aca="false">IF(Освіта!E14 = 0, "", Освіта!E14)</f>
-        <v/>
-      </c>
-      <c r="D83" s="65"/>
-      <c r="O83" s="0"/>
+      <c r="B83" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C83" s="67" t="str">
+        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
+        <v/>
+      </c>
+      <c r="D83" s="66"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="55"/>
-      <c r="B84" s="48" t="str">
-        <f aca="false">Освіта!$F$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C84" s="66" t="str">
-        <f aca="false">IF(Освіта!F14 = 0, "", Освіта!F14)</f>
-        <v/>
-      </c>
-      <c r="D84" s="65"/>
-      <c r="O84" s="0"/>
+      <c r="B84" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C84" s="67" t="str">
+        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
+        <v/>
+      </c>
+      <c r="D84" s="66"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="55"/>
-      <c r="B85" s="48" t="str">
-        <f aca="false">Освіта!$G$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C85" s="66" t="str">
-        <f aca="false">IF(Освіта!G14 = 0, "", Освіта!G14)</f>
-        <v/>
-      </c>
-      <c r="D85" s="65"/>
+      <c r="B85" s="64" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C85" s="67" t="str">
+        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
+        <v/>
+      </c>
+      <c r="D85" s="66"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="55"/>
-      <c r="B86" s="48" t="str">
+      <c r="B86" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C86" s="67" t="str">
+        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
+        <v/>
+      </c>
+      <c r="D86" s="66"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="55"/>
+      <c r="B87" s="64" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C86" s="66" t="str">
-        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
-        <v/>
-      </c>
-      <c r="D86" s="65"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="55"/>
-      <c r="B87" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Серія дисплома</v>
-      </c>
-      <c r="C87" s="66" t="str">
-        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
-        <v/>
-      </c>
-      <c r="D87" s="65"/>
+      <c r="C87" s="67" t="str">
+        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
+        <v/>
+      </c>
+      <c r="D87" s="66"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="55"/>
-      <c r="B88" s="0" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Номер диплома</v>
-      </c>
-      <c r="C88" s="66" t="str">
-        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
-        <v/>
-      </c>
-      <c r="D88" s="65"/>
+      <c r="B88" s="64" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C88" s="67" t="str">
+        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
+        <v/>
+      </c>
+      <c r="D88" s="66"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="55"/>
-      <c r="B89" s="0" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Дата видачі диплома</v>
-      </c>
-      <c r="C89" s="66" t="str">
-        <f aca="false">IF(Освіта!D15 = 0, "", Освіта!D15)</f>
-        <v/>
-      </c>
-      <c r="D89" s="65"/>
+      <c r="B89" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C89" s="67" t="str">
+        <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
+        <v/>
+      </c>
+      <c r="D89" s="66"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="55"/>
-      <c r="B90" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C90" s="66" t="str">
-        <f aca="false">IF(Освіта!E15 = 0, "", Освіта!E15)</f>
-        <v/>
-      </c>
-      <c r="D90" s="65"/>
+      <c r="A90" s="55" t="s">
+        <v>159</v>
+      </c>
+      <c r="B90" s="64" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C90" s="68" t="str">
+        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
+        <v/>
+      </c>
+      <c r="D90" s="66"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="55"/>
-      <c r="B91" s="48" t="str">
-        <f aca="false">Освіта!$F$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C91" s="66" t="str">
-        <f aca="false">IF(Освіта!F15 = 0, "", Освіта!F15)</f>
-        <v/>
-      </c>
-      <c r="D91" s="65"/>
+      <c r="B91" s="64" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C91" s="68" t="str">
+        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
+        <v/>
+      </c>
+      <c r="D91" s="66"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="55"/>
-      <c r="B92" s="48" t="str">
-        <f aca="false">Освіта!$G$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C92" s="66" t="str">
-        <f aca="false">IF(Освіта!G15 = 0, "", Освіта!G15)</f>
-        <v/>
-      </c>
-      <c r="D92" s="65"/>
+      <c r="B92" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C92" s="68" t="str">
+        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
+        <v/>
+      </c>
+      <c r="D92" s="66"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="55"/>
-      <c r="B93" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C93" s="66" t="str">
-        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
-        <v/>
-      </c>
-      <c r="D93" s="65"/>
+      <c r="B93" s="64" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C93" s="68" t="str">
+        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
+        <v/>
+      </c>
+      <c r="D93" s="66"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="55"/>
-      <c r="B94" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Серія дисплома</v>
-      </c>
-      <c r="C94" s="66" t="str">
-        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
-        <v/>
-      </c>
-      <c r="D94" s="65"/>
+      <c r="B94" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C94" s="68" t="str">
+        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
+        <v/>
+      </c>
+      <c r="D94" s="66"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="55"/>
-      <c r="B95" s="0" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Номер диплома</v>
-      </c>
-      <c r="C95" s="66" t="str">
-        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
-        <v/>
-      </c>
-      <c r="D95" s="65"/>
+      <c r="B95" s="64" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C95" s="68" t="str">
+        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <v/>
+      </c>
+      <c r="D95" s="66"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="55"/>
-      <c r="B96" s="0" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Дата видачі диплома</v>
-      </c>
-      <c r="C96" s="66" t="str">
-        <f aca="false">IF(Освіта!D16 = 0, "", Освіта!D16)</f>
-        <v/>
-      </c>
-      <c r="D96" s="65"/>
+      <c r="B96" s="64" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C96" s="68" t="str">
+        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
+        <v/>
+      </c>
+      <c r="D96" s="66"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="55"/>
-      <c r="B97" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C97" s="66" t="str">
-        <f aca="false">IF(Освіта!E16 = 0, "", Освіта!E16)</f>
-        <v/>
-      </c>
-      <c r="D97" s="65"/>
+      <c r="B97" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C97" s="68" t="str">
+        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
+        <v/>
+      </c>
+      <c r="D97" s="66"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="55"/>
-      <c r="B98" s="48" t="str">
-        <f aca="false">Освіта!$F$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C98" s="66" t="str">
-        <f aca="false">IF(Освіта!F16 = 0, "", Освіта!F16)</f>
-        <v/>
-      </c>
-      <c r="D98" s="65"/>
+      <c r="B98" s="64" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C98" s="68" t="str">
+        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
+        <v/>
+      </c>
+      <c r="D98" s="66"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="55"/>
-      <c r="B99" s="48" t="str">
-        <f aca="false">Освіта!$G$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C99" s="66" t="str">
-        <f aca="false">IF(Освіта!G16 = 0, "", Освіта!G16)</f>
-        <v/>
-      </c>
-      <c r="D99" s="65"/>
+      <c r="B99" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C99" s="68" t="str">
+        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
+        <v/>
+      </c>
+      <c r="D99" s="66"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="55"/>
-      <c r="B100" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C100" s="66" t="str">
-        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
-        <v/>
-      </c>
-      <c r="D100" s="65"/>
+      <c r="B100" s="64" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C100" s="68" t="str">
+        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <v/>
+      </c>
+      <c r="D100" s="66"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="55"/>
-      <c r="B101" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Серія дисплома</v>
-      </c>
-      <c r="C101" s="66" t="str">
-        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
-        <v/>
-      </c>
-      <c r="D101" s="65"/>
+      <c r="B101" s="64" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C101" s="68" t="str">
+        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
+        <v/>
+      </c>
+      <c r="D101" s="66"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="55"/>
-      <c r="B102" s="0" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Номер диплома</v>
-      </c>
-      <c r="C102" s="66" t="str">
-        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
-        <v/>
-      </c>
-      <c r="D102" s="65"/>
+      <c r="B102" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C102" s="68" t="str">
+        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
+        <v/>
+      </c>
+      <c r="D102" s="66"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="55"/>
-      <c r="B103" s="0" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Дата видачі диплома</v>
-      </c>
-      <c r="C103" s="66" t="str">
-        <f aca="false">IF(Освіта!D17 = 0, "", Освіта!D17)</f>
-        <v/>
-      </c>
-      <c r="D103" s="65"/>
+      <c r="B103" s="64" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C103" s="68" t="str">
+        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
+        <v/>
+      </c>
+      <c r="D103" s="66"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="55"/>
-      <c r="B104" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C104" s="66" t="str">
-        <f aca="false">IF(Освіта!E17 = 0, "", Освіта!E17)</f>
-        <v/>
-      </c>
-      <c r="D104" s="65"/>
+      <c r="B104" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C104" s="68" t="str">
+        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
+        <v/>
+      </c>
+      <c r="D104" s="66"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="55"/>
-      <c r="B105" s="48" t="str">
-        <f aca="false">Освіта!$F$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C105" s="66" t="str">
-        <f aca="false">IF(Освіта!F17 = 0, "", Освіта!F17)</f>
-        <v/>
-      </c>
-      <c r="D105" s="65"/>
+      <c r="B105" s="64" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C105" s="68" t="str">
+        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <v/>
+      </c>
+      <c r="D105" s="66"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="55"/>
-      <c r="B106" s="48" t="str">
-        <f aca="false">Освіта!$G$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C106" s="66" t="str">
-        <f aca="false">IF(Освіта!G17 = 0, "", Освіта!G17)</f>
-        <v/>
-      </c>
-      <c r="D106" s="65"/>
+      <c r="B106" s="64" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C106" s="68" t="str">
+        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
+        <v/>
+      </c>
+      <c r="D106" s="66"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="55"/>
-      <c r="B107" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C107" s="66" t="str">
-        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
-        <v/>
-      </c>
-      <c r="D107" s="65"/>
+      <c r="B107" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C107" s="68" t="str">
+        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
+        <v/>
+      </c>
+      <c r="D107" s="66"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="55"/>
-      <c r="B108" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Серія дисплома</v>
-      </c>
-      <c r="C108" s="66" t="str">
-        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
-        <v/>
-      </c>
-      <c r="D108" s="65"/>
+      <c r="B108" s="64" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C108" s="68" t="str">
+        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
+        <v/>
+      </c>
+      <c r="D108" s="66"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="55"/>
-      <c r="B109" s="0" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Номер диплома</v>
-      </c>
-      <c r="C109" s="66" t="str">
-        <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
-        <v/>
-      </c>
-      <c r="D109" s="65"/>
+      <c r="B109" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C109" s="68" t="str">
+        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
+        <v/>
+      </c>
+      <c r="D109" s="66"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="55"/>
-      <c r="B110" s="0" t="str">
-        <f aca="false">Освіта!$D$12</f>
-        <v>Дата видачі диплома</v>
-      </c>
-      <c r="C110" s="66" t="str">
-        <f aca="false">IF(Освіта!D18 = 0, "", Освіта!D18)</f>
-        <v/>
-      </c>
-      <c r="D110" s="65"/>
+      <c r="B110" s="64" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C110" s="68" t="str">
+        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+        <v/>
+      </c>
+      <c r="D110" s="66"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="55"/>
-      <c r="B111" s="48" t="str">
-        <f aca="false">Освіта!$E$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C111" s="66" t="str">
-        <f aca="false">IF(Освіта!E18 = 0, "", Освіта!E18)</f>
-        <v/>
-      </c>
-      <c r="D111" s="65"/>
+      <c r="B111" s="64" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C111" s="68" t="str">
+        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
+        <v/>
+      </c>
+      <c r="D111" s="66"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="55"/>
-      <c r="B112" s="48" t="str">
-        <f aca="false">Освіта!$F$12</f>
-        <v>Науковий ступінь, учене звання</v>
-      </c>
-      <c r="C112" s="66" t="str">
-        <f aca="false">IF(Освіта!F18 = 0, "", Освіта!F18)</f>
-        <v/>
-      </c>
-      <c r="D112" s="65"/>
+      <c r="B112" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
+      </c>
+      <c r="C112" s="68" t="str">
+        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
+        <v/>
+      </c>
+      <c r="D112" s="66"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="55"/>
-      <c r="B113" s="48" t="str">
-        <f aca="false">Освіта!$G$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C113" s="66" t="str">
-        <f aca="false">IF(Освіта!G18 = 0, "", Освіта!G18)</f>
-        <v/>
-      </c>
-      <c r="D113" s="65"/>
+      <c r="B113" s="64" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
+      </c>
+      <c r="C113" s="68" t="str">
+        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
+        <v/>
+      </c>
+      <c r="D113" s="66"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="55" t="s">
-        <v>162</v>
-      </c>
-      <c r="B114" s="48" t="str">
+      <c r="A114" s="55"/>
+      <c r="B114" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C114" s="68" t="str">
+        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
+        <v/>
+      </c>
+      <c r="D114" s="66"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="55"/>
+      <c r="B115" s="64" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C114" s="67" t="str">
-        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
-        <v/>
-      </c>
-      <c r="D114" s="65"/>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="55"/>
-      <c r="B115" s="48" t="str">
+      <c r="C115" s="68" t="str">
+        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
+        <v/>
+      </c>
+      <c r="D115" s="66"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="55"/>
+      <c r="B116" s="64" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C115" s="67" t="str">
-        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
-        <v/>
-      </c>
-      <c r="D115" s="65"/>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="55"/>
-      <c r="B116" s="2" t="str">
+      <c r="C116" s="68" t="str">
+        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
+        <v/>
+      </c>
+      <c r="D116" s="66"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="55"/>
+      <c r="B117" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C116" s="67" t="str">
-        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
-        <v/>
-      </c>
-      <c r="D116" s="65"/>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="55"/>
-      <c r="B117" s="48" t="str">
+      <c r="C117" s="68" t="str">
+        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
+        <v/>
+      </c>
+      <c r="D117" s="66"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="55"/>
+      <c r="B118" s="64" t="str">
         <f aca="false">Родина!$D$4</f>
         <v>По-батькові</v>
       </c>
-      <c r="C117" s="67" t="str">
-        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
-        <v/>
-      </c>
-      <c r="D117" s="65"/>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="55"/>
-      <c r="B118" s="48" t="str">
+      <c r="C118" s="68" t="str">
+        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
+        <v/>
+      </c>
+      <c r="D118" s="66"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="55"/>
+      <c r="B119" s="64" t="str">
         <f aca="false">Родина!$E$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C118" s="67" t="str">
-        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
-        <v/>
-      </c>
-      <c r="D118" s="65"/>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="55"/>
-      <c r="B119" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C119" s="67" t="str">
-        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
-        <v/>
-      </c>
-      <c r="D119" s="65"/>
+      <c r="C119" s="68" t="str">
+        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
+        <v/>
+      </c>
+      <c r="D119" s="66"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="55"/>
-      <c r="B120" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
-      </c>
-      <c r="C120" s="67" t="str">
-        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
-        <v/>
-      </c>
-      <c r="D120" s="65"/>
+      <c r="A120" s="55" t="s">
+        <v>160</v>
+      </c>
+      <c r="B120" s="64" t="str">
+        <f aca="false">Документи!A4</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C120" s="56" t="str">
+        <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
+        <v/>
+      </c>
+      <c r="D120" s="64"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="55"/>
-      <c r="B121" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
-      </c>
-      <c r="C121" s="67" t="str">
-        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
-        <v/>
-      </c>
-      <c r="D121" s="65"/>
+      <c r="B121" s="64" t="str">
+        <f aca="false">Документи!A5</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C121" s="64" t="str">
+        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
+        <v/>
+      </c>
+      <c r="D121" s="64"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="55"/>
-      <c r="B122" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C122" s="67" t="str">
-        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
-        <v/>
-      </c>
-      <c r="D122" s="65"/>
+      <c r="B122" s="64" t="str">
+        <f aca="false">Документи!A6</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C122" s="64" t="str">
+        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
+        <v/>
+      </c>
+      <c r="D122" s="64"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="55"/>
-      <c r="B123" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C123" s="67" t="str">
-        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
-        <v/>
-      </c>
-      <c r="D123" s="65"/>
+      <c r="B123" s="64" t="str">
+        <f aca="false">Документи!A7</f>
+        <v>Дата видачі</v>
+      </c>
+      <c r="C123" s="64" t="str">
+        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
+        <v/>
+      </c>
+      <c r="D123" s="64"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="55"/>
-      <c r="B124" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C124" s="67" t="str">
-        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
-        <v/>
-      </c>
-      <c r="D124" s="65"/>
+      <c r="B124" s="64" t="str">
+        <f aca="false">Документи!A10</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C124" s="56" t="str">
+        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
+        <v/>
+      </c>
+      <c r="D124" s="64"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="55"/>
-      <c r="B125" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
-      </c>
-      <c r="C125" s="67" t="str">
-        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
-        <v/>
-      </c>
-      <c r="D125" s="65"/>
+      <c r="B125" s="64" t="str">
+        <f aca="false">Документи!A11</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C125" s="64" t="str">
+        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
+        <v/>
+      </c>
+      <c r="D125" s="64"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="55"/>
-      <c r="B126" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
-      </c>
-      <c r="C126" s="67" t="str">
-        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
-        <v/>
-      </c>
-      <c r="D126" s="65"/>
+      <c r="B126" s="64" t="str">
+        <f aca="false">Документи!A12</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C126" s="64" t="str">
+        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
+        <v/>
+      </c>
+      <c r="D126" s="64"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="55"/>
-      <c r="B127" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C127" s="67" t="str">
-        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
-        <v/>
-      </c>
-      <c r="D127" s="65"/>
+      <c r="B127" s="64" t="str">
+        <f aca="false">Документи!A13</f>
+        <v>Дата видачі</v>
+      </c>
+      <c r="C127" s="64" t="str">
+        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
+        <v/>
+      </c>
+      <c r="D127" s="64"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="55"/>
-      <c r="B128" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C128" s="67" t="str">
-        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
-        <v/>
-      </c>
-      <c r="D128" s="65"/>
+      <c r="B128" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="C128" s="64"/>
+      <c r="D128" s="64"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="55"/>
-      <c r="B129" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C129" s="67" t="str">
-        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
-        <v/>
-      </c>
-      <c r="D129" s="65"/>
+      <c r="B129" s="64" t="str">
+        <f aca="false">Документи!A16</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C129" s="56" t="str">
+        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
+        <v/>
+      </c>
+      <c r="D129" s="64"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="55"/>
-      <c r="B130" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
-      </c>
-      <c r="C130" s="67" t="str">
-        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
-        <v/>
-      </c>
-      <c r="D130" s="65"/>
+      <c r="B130" s="64" t="str">
+        <f aca="false">Документи!A17</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C130" s="64" t="str">
+        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
+        <v/>
+      </c>
+      <c r="D130" s="64"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="55"/>
-      <c r="B131" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
-      </c>
-      <c r="C131" s="67" t="str">
-        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
-        <v/>
-      </c>
-      <c r="D131" s="65"/>
-    </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="55"/>
-      <c r="B132" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C132" s="67" t="str">
-        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
-        <v/>
-      </c>
-      <c r="D132" s="65"/>
-    </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="55"/>
-      <c r="B133" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C133" s="67" t="str">
-        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
-        <v/>
-      </c>
-      <c r="D133" s="65"/>
-    </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="55"/>
-      <c r="B134" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C134" s="67" t="str">
-        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
-        <v/>
-      </c>
-      <c r="D134" s="65"/>
-    </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="55"/>
-      <c r="B135" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
-      </c>
-      <c r="C135" s="67" t="str">
-        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
-        <v/>
-      </c>
-      <c r="D135" s="65"/>
-    </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="55"/>
-      <c r="B136" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
-      </c>
-      <c r="C136" s="67" t="str">
-        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
-        <v/>
-      </c>
-      <c r="D136" s="65"/>
-    </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="55"/>
-      <c r="B137" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C137" s="67" t="str">
-        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
-        <v/>
-      </c>
-      <c r="D137" s="65"/>
-    </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="55"/>
-      <c r="B138" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C138" s="67" t="str">
-        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
-        <v/>
-      </c>
-      <c r="D138" s="65"/>
-    </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="55"/>
-      <c r="B139" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
-      </c>
-      <c r="C139" s="67" t="str">
-        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
-        <v/>
-      </c>
-      <c r="D139" s="65"/>
-    </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="55"/>
-      <c r="B140" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
-      </c>
-      <c r="C140" s="67" t="str">
-        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
-        <v/>
-      </c>
-      <c r="D140" s="65"/>
-    </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="55"/>
-      <c r="B141" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
-      </c>
-      <c r="C141" s="67" t="str">
-        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
-        <v/>
-      </c>
-      <c r="D141" s="65"/>
-    </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="55"/>
-      <c r="B142" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C142" s="67" t="str">
-        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
-        <v/>
-      </c>
-      <c r="D142" s="65"/>
-    </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="55"/>
-      <c r="B143" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C143" s="67" t="str">
-        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
-        <v/>
-      </c>
-      <c r="D143" s="65"/>
-    </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="55" t="s">
-        <v>163</v>
-      </c>
-      <c r="B144" s="48" t="str">
-        <f aca="false">Документи!A4</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C144" s="56" t="str">
-        <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
-        <v/>
-      </c>
-      <c r="D144" s="48"/>
-    </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="55"/>
-      <c r="B145" s="48" t="str">
-        <f aca="false">Документи!A5</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C145" s="48" t="str">
-        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
-        <v/>
-      </c>
-      <c r="D145" s="48"/>
-    </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="55"/>
-      <c r="B146" s="48" t="str">
-        <f aca="false">Документи!A6</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C146" s="48" t="str">
-        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
-        <v/>
-      </c>
-      <c r="D146" s="48"/>
-    </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="55"/>
-      <c r="B147" s="48" t="str">
-        <f aca="false">Документи!A7</f>
-        <v>Дата видачі</v>
-      </c>
-      <c r="C147" s="48" t="str">
-        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
-        <v/>
-      </c>
-      <c r="D147" s="48"/>
-    </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="55"/>
-      <c r="B148" s="48" t="str">
-        <f aca="false">Документи!A10</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C148" s="56" t="str">
-        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
-        <v/>
-      </c>
-      <c r="D148" s="48"/>
-    </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="55"/>
-      <c r="B149" s="48" t="str">
-        <f aca="false">Документи!A11</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C149" s="48" t="str">
-        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
-        <v/>
-      </c>
-      <c r="D149" s="48"/>
-    </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="55"/>
-      <c r="B150" s="48" t="str">
-        <f aca="false">Документи!A12</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C150" s="48" t="str">
-        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
-        <v/>
-      </c>
-      <c r="D150" s="48"/>
-    </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="55"/>
-      <c r="B151" s="48" t="str">
-        <f aca="false">Документи!A13</f>
-        <v>Дата видачі</v>
-      </c>
-      <c r="C151" s="48" t="str">
-        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
-        <v/>
-      </c>
-      <c r="D151" s="48"/>
-    </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="55"/>
-      <c r="B152" s="48" t="s">
-        <v>164</v>
-      </c>
-      <c r="C152" s="48"/>
-      <c r="D152" s="48"/>
-    </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="55"/>
-      <c r="B153" s="48" t="str">
-        <f aca="false">Документи!A16</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C153" s="56" t="str">
-        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
-        <v/>
-      </c>
-      <c r="D153" s="48"/>
-    </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="55"/>
-      <c r="B154" s="48" t="str">
-        <f aca="false">Документи!A17</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C154" s="48" t="str">
-        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
-        <v/>
-      </c>
-      <c r="D154" s="48"/>
-    </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="55"/>
-      <c r="B155" s="48" t="str">
+      <c r="B131" s="64" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C155" s="48" t="str">
+      <c r="C131" s="64" t="str">
         <f aca="false">IF(Документи!B18 = 0, "", Документи!B18)</f>
         <v/>
       </c>
-      <c r="D155" s="48"/>
-    </row>
+      <c r="D131" s="64"/>
+    </row>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -13086,13 +12697,13 @@
     <mergeCell ref="Q1:T1"/>
     <mergeCell ref="A2:A24"/>
     <mergeCell ref="O2:O16"/>
-    <mergeCell ref="G7:M7"/>
+    <mergeCell ref="G7:I7"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="O17:O28"/>
     <mergeCell ref="A25:A39"/>
-    <mergeCell ref="A40:A113"/>
-    <mergeCell ref="A114:A143"/>
-    <mergeCell ref="A144:A155"/>
+    <mergeCell ref="A40:A89"/>
+    <mergeCell ref="A90:A119"/>
+    <mergeCell ref="A120:A131"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:K21" type="none">

</xml_diff>

<commit_message>
fix: delete RegionKh from excel | style: rename ExportAdapter -> IOAdapter
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="162">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -169,337 +169,337 @@
     <t xml:space="preserve">Список на основі БД (Country)</t>
   </si>
   <si>
+    <t xml:space="preserve">Область (України)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (RegionUkraine) із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Місто</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Адреса (вулиця, № будинку, квартири)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Індекс</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 цифр, не обовязкове</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Телефони</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (основний)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 цифр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12. Місце проживання за державною реєстрацією </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Співпадає із адресою фактичного проживання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва освітнього закладу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія дисплома (свідоцтва)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Номер дисплома (свідоцтва)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік закінчення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Спеціальність (професія) за дипломом (свідоцтвом) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кваліфікація за дипломом (свідоцтвом)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Форма навчання (денна, вечірня, заочна)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівень освіти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівень підготовки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Склад родини</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По-батькові</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік народження</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри!!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ДОКУМЕНТИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія та номер </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ким виданий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата видачі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квіток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК224345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закордоний паспорт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: FF453210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва сторінки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва поля</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле для оновлення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле з актуальною інформацією</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип заповнення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва списку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Основна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Визначений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професійно-технічна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неповна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">НПП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ІТС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">одружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неодружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">незаміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучена</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдова</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдівець</t>
+  </si>
+  <si>
+    <t xml:space="preserve">військовозобов'язаний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">призовник</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">обмежено-придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">непридатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не перебуває</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТАК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">НІ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">денна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вечірня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заочна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">спеціаліст</t>
+  </si>
+  <si>
+    <t xml:space="preserve">бакалавр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">магістр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Науковий ступінь, учене звання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">кандидат наук</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PhD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">доцент</t>
+  </si>
+  <si>
+    <t xml:space="preserve">доктор наук</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">аспірантура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ад'юнктура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">докторантура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">дружина</t>
+  </si>
+  <si>
+    <t xml:space="preserve">чоловік</t>
+  </si>
+  <si>
+    <t xml:space="preserve">донька</t>
+  </si>
+  <si>
+    <t xml:space="preserve">син</t>
+  </si>
+  <si>
+    <t xml:space="preserve">донька подружжя</t>
+  </si>
+  <si>
+    <t xml:space="preserve">син подружжя</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу (паспорт)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паперовий паспорт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID картка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу (Військовий квіток)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квиток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квиток офіцера запасу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">З бази даних</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Адреси Контакти</t>
+  </si>
+  <si>
     <t xml:space="preserve">Область</t>
   </si>
   <si>
-    <t xml:space="preserve">Список на основі БД (RegionUkraine) із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Місто</t>
-  </si>
-  <si>
     <t xml:space="preserve">Район (міста)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (RegionKharkiv) із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адреса (вулиця, № будинку, квартири)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Індекс</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 цифр, не обовязкове</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Телефони</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (основний)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 цифр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12. Місце проживання за державною реєстрацією </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Співпадає із адресою фактичного проживання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва освітнього закладу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія дисплома (свідоцтва)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Номер дисплома (свідоцтва)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік закінчення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Спеціальність (професія) за дипломом (свідоцтвом) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кваліфікація за дипломом (свідоцтвом)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Форма навчання (денна, вечірня, заочна)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рівень освіти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рівень підготовки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Склад родини</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">По-батькові</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік народження</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри!!!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДОКУМЕНТИ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип документу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія та номер </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ким виданий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата видачі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військовий квіток</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК224345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закордоний паспорт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: FF453210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва сторінки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва поля</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле для оновлення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле з актуальною інформацією</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип заповнення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва списку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Значення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Основна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Визначений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">професійно-технічна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неповна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">НПП</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ІТС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">одружений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неодружений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">заміжня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">незаміжня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">розлучений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">розлучена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вдова</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вдівець</t>
-  </si>
-  <si>
-    <t xml:space="preserve">військовозобов'язаний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">призовник</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">придатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">обмежено-придатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">непридатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не перебуває</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ТАК</t>
-  </si>
-  <si>
-    <t xml:space="preserve">НІ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">денна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вечірня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">заочна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">спеціаліст</t>
-  </si>
-  <si>
-    <t xml:space="preserve">бакалавр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">магістр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Науковий ступінь, учене звання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">кандидат наук</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PhD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">доцент</t>
-  </si>
-  <si>
-    <t xml:space="preserve">доктор наук</t>
-  </si>
-  <si>
-    <t xml:space="preserve">професор</t>
-  </si>
-  <si>
-    <t xml:space="preserve">аспірантура</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ад'юнктура</t>
-  </si>
-  <si>
-    <t xml:space="preserve">докторантура</t>
-  </si>
-  <si>
-    <t xml:space="preserve">дружина</t>
-  </si>
-  <si>
-    <t xml:space="preserve">чоловік</t>
-  </si>
-  <si>
-    <t xml:space="preserve">донька</t>
-  </si>
-  <si>
-    <t xml:space="preserve">син</t>
-  </si>
-  <si>
-    <t xml:space="preserve">донька подружжя</t>
-  </si>
-  <si>
-    <t xml:space="preserve">син подружжя</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип документу (паспорт)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Паперовий паспорт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID картка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип документу (Військовий квіток)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військовий квиток</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військовий квиток офіцера запасу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">З бази даних</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адреси Контакти</t>
   </si>
   <si>
     <t xml:space="preserve">Освіта</t>
@@ -996,7 +996,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1519,7 +1519,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
         <v>38</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
         <v>42</v>
       </c>
@@ -1600,14 +1600,6 @@
       <formula1>'Системна інформація'!$Q$23:$ZA$23</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="B33" type="list">
-      <formula1>'Системна інформація'!$Q$7:$ZA$7</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="B35" type="list">
-      <formula1>'Системна інформація'!$Q$8:$ZA$8</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" error="Перевірте наявність своєї посади в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такої посади наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B23" type="list">
       <formula1>'Системна інформація'!$Q$21:$ZA$21</formula1>
       <formula2>0</formula2>
@@ -1622,6 +1614,14 @@
     </dataValidation>
     <dataValidation allowBlank="false" error="Перевірте наявність свого ТЦК в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого ТЦК наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B34" type="list">
       <formula1>'Системна інформація'!$Q$24:$ZA$24</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність свого типу придатності в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="information" errorTitle="Даного типу придатності не є в списку" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B33" type="list">
+      <formula1>'Системна інформація'!$Q$7:$ZA$7</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність типу перебування на спеціальному обліку в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="information" errorTitle="Даного типу перебування на спеціальному облік не є в списку" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B35" type="list">
+      <formula1>'Системна інформація'!$Q$8:$ZA$8</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1640,7 +1640,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D1048576"/>
   <sheetFormatPr defaultColWidth="8.62890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="20" width="24"/>
@@ -1701,8 +1701,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
+    <row r="7" s="25" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
         <v>50</v>
       </c>
       <c r="B7" s="27"/>
@@ -1710,47 +1710,47 @@
         <f aca="false">IF('Системна інформація'!D28 = 0, "", 'Системна інформація'!D28)</f>
         <v/>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="20"/>
+    </row>
+    <row r="8" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="8" s="25" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
-        <v>52</v>
       </c>
       <c r="B8" s="27"/>
       <c r="C8" s="22" t="str">
         <f aca="false">IF('Системна інформація'!D29 = 0, "", 'Системна інформація'!D29)</f>
         <v/>
       </c>
-      <c r="D8" s="20"/>
+      <c r="D8" s="20" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="9" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="29"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="20"/>
+    </row>
+    <row r="10" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D30 = 0, "", 'Системна інформація'!D30)</f>
-        <v/>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29"/>
-      <c r="B10" s="30"/>
+      <c r="B10" s="1"/>
       <c r="C10" s="2"/>
       <c r="D10" s="20"/>
     </row>
-    <row r="11" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="27"/>
+      <c r="C11" s="22" t="str">
+        <f aca="false">IF('Системна інформація'!D30 = 0, "", 'Системна інформація'!D30)</f>
+        <v/>
+      </c>
+      <c r="D11" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="20"/>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
@@ -1762,68 +1762,68 @@
         <v/>
       </c>
       <c r="D12" s="20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
+      <c r="B14" s="16"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="22"/>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="22" t="str">
+      <c r="B15" s="24"/>
+      <c r="C15" s="22" t="str">
         <f aca="false">IF('Системна інформація'!D32 = 0, "", 'Системна інформація'!D32)</f>
         <v/>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="22"/>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="22" t="str">
+      <c r="D15" s="22" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="22"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="24"/>
+      <c r="C17" s="22" t="str">
         <f aca="false">IF('Системна інформація'!D33 = 0, "", 'Системна інформація'!D33)</f>
         <v/>
       </c>
-      <c r="D16" s="22" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="22"/>
+      <c r="D17" s="25" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" s="24"/>
+      <c r="A18" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="27"/>
       <c r="C18" s="22" t="str">
         <f aca="false">IF('Системна інформація'!D34 = 0, "", 'Системна інформація'!D34)</f>
         <v/>
       </c>
-      <c r="D18" s="25" t="s">
-        <v>46</v>
+      <c r="D18" s="20" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="22" t="str">
@@ -1831,25 +1831,22 @@
         <v/>
       </c>
       <c r="D19" s="20" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="26" t="s">
-        <v>49</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="28" t="s">
+        <v>50</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="22" t="str">
         <f aca="false">IF('Системна інформація'!D36 = 0, "", 'Системна інформація'!D36)</f>
         <v/>
       </c>
-      <c r="D20" s="20" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="22" t="str">
@@ -1857,54 +1854,33 @@
         <v/>
       </c>
       <c r="D21" s="20" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="27"/>
-      <c r="C22" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D38 = 0, "", 'Системна інформація'!D38)</f>
-        <v/>
-      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D39 = 0, "", 'Системна інформація'!D39)</f>
-        <v/>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C24" s="22"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="22"/>
-    </row>
+      <c r="C23" s="22"/>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B4 B18" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B4 B17" type="list">
       <formula1>'Системна інформація'!$Q$25:$ZA$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5 B19" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B15" type="list">
+      <formula1>'Системна інформація'!$Q$9:$R$9</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність своєї області в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такої області наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5" type="list">
       <formula1>'Системна інформація'!$Q$26:$ZA$26</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B7 B21" type="list">
-      <formula1>'Системна інформація'!$Q$27:$ZA$27</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B16" type="list">
-      <formula1>'Системна інформація'!$Q$9:$R$9</formula1>
+    <dataValidation allowBlank="false" error="Перевірте наявність своєї області в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такої області наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B18" type="list">
+      <formula1>'Системна інформація'!$Q$26:$ZA$26</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1934,7 +1910,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
@@ -1954,7 +1930,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B3" s="34"/>
       <c r="C3" s="33"/>
@@ -1965,28 +1941,28 @@
     </row>
     <row r="4" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="D4" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="E4" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="F4" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="G4" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="H4" s="36" t="s">
         <v>68</v>
-      </c>
-      <c r="G4" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="H4" s="36" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2033,7 +2009,7 @@
       <c r="A9" s="33"/>
       <c r="B9" s="33"/>
       <c r="D9" s="39" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E9" s="33"/>
       <c r="F9" s="33"/>
@@ -2055,7 +2031,7 @@
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="33"/>
@@ -2066,84 +2042,54 @@
     </row>
     <row r="12" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="0"/>
-      <c r="E12" s="0"/>
-      <c r="F12" s="0"/>
-      <c r="G12" s="0"/>
+        <v>72</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
       <c r="B13" s="40"/>
       <c r="C13" s="40"/>
-      <c r="D13" s="0"/>
-      <c r="E13" s="0"/>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="40"/>
       <c r="C14" s="40"/>
-      <c r="D14" s="0"/>
-      <c r="E14" s="0"/>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
       <c r="B15" s="40"/>
       <c r="C15" s="40"/>
-      <c r="D15" s="0"/>
-      <c r="E15" s="0"/>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
       <c r="B16" s="40"/>
       <c r="C16" s="40"/>
-      <c r="D16" s="0"/>
-      <c r="E16" s="0"/>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="37"/>
       <c r="B17" s="40"/>
       <c r="C17" s="40"/>
-      <c r="D17" s="0"/>
-      <c r="E17" s="0"/>
-      <c r="F17" s="0"/>
-      <c r="G17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37"/>
       <c r="B18" s="40"/>
       <c r="C18" s="40"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33"/>
       <c r="B19" s="39" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C19" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="0"/>
       <c r="F19" s="39"/>
-      <c r="G19" s="0"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -2193,12 +2139,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="42" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
@@ -2207,7 +2153,7 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B4" s="44" t="s">
         <v>5</v>
@@ -2216,10 +2162,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2269,7 +2215,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2306,21 +2252,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="41" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="47" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
+        <f aca="false">IF('Системна інформація'!D118 = 0, "", 'Системна інформація'!D118)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="s">
@@ -2329,37 +2275,37 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
+        <f aca="false">IF('Системна інформація'!D119 = 0, "", 'Системна інформація'!D119)</f>
         <v/>
       </c>
       <c r="D5" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
+        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
         <v/>
       </c>
       <c r="D6" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
+        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
         <v/>
       </c>
       <c r="D7" s="2" t="s">
@@ -2368,16 +2314,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="47" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
+        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="s">
@@ -2386,34 +2332,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
+        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
         <v/>
       </c>
       <c r="D11" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D126 = 0, "", 'Системна інформація'!D126)</f>
+        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
+        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
         <v/>
       </c>
       <c r="D13" s="2" t="s">
@@ -2422,42 +2368,42 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="41" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D129 = 0, "", 'Системна інформація'!D129)</f>
+        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D130 = 0, "", 'Системна інформація'!D130)</f>
+        <f aca="false">IF('Системна інформація'!D128 = 0, "", 'Системна інформація'!D128)</f>
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="48" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D131 = 0, "", 'Системна інформація'!D131)</f>
+        <f aca="false">IF('Системна інформація'!D129 = 0, "", 'Системна інформація'!D129)</f>
         <v/>
       </c>
       <c r="D18" s="2" t="s">
@@ -2490,7 +2436,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:ZA1048576"/>
+  <dimension ref="A1:ZA130"/>
   <sheetFormatPr defaultColWidth="10.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="49" width="23.16"/>
@@ -2503,20 +2449,20 @@
   <sheetData>
     <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="D1" s="51" t="s">
         <v>95</v>
-      </c>
-      <c r="C1" s="51" t="s">
-        <v>96</v>
-      </c>
-      <c r="D1" s="51" t="s">
-        <v>97</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="52" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H1" s="52"/>
       <c r="I1" s="52"/>
@@ -2526,13 +2472,13 @@
       <c r="M1" s="52"/>
       <c r="N1" s="52"/>
       <c r="O1" s="53" t="s">
+        <v>97</v>
+      </c>
+      <c r="P1" s="54" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q1" s="53" t="s">
         <v>99</v>
-      </c>
-      <c r="P1" s="54" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q1" s="53" t="s">
-        <v>101</v>
       </c>
       <c r="R1" s="53"/>
       <c r="S1" s="53"/>
@@ -2540,7 +2486,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="55" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B2" s="48" t="str">
         <f aca="false">Основна!A9</f>
@@ -2552,60 +2498,60 @@
       </c>
       <c r="D2" s="48"/>
       <c r="G2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="H2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="I2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="J2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="K2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="L2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="M2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="N2" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="O2" s="58" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>11</v>
       </c>
       <c r="Q2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="S2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2620,35 +2566,35 @@
       </c>
       <c r="D3" s="48"/>
       <c r="G3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="H3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="I3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="J3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="K3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="L3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="M3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="N3" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="O3" s="58"/>
@@ -2656,10 +2602,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2674,35 +2620,35 @@
       </c>
       <c r="D4" s="48"/>
       <c r="G4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="H4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="I4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="J4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="K4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="L4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="M4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="N4" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="O4" s="58"/>
@@ -2710,28 +2656,28 @@
         <v>18</v>
       </c>
       <c r="Q4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="S4" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="X4" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2746,35 +2692,35 @@
       </c>
       <c r="D5" s="48"/>
       <c r="G5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="I5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="K5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="L5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="M5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="N5" s="57" t="n">
-        <f aca="true">OFFSET($D$40,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="O5" s="58"/>
@@ -2782,10 +2728,10 @@
         <v>30</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2829,7 +2775,7 @@
       </c>
       <c r="D7" s="48"/>
       <c r="G7" s="59" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H7" s="59"/>
       <c r="I7" s="59"/>
@@ -2838,13 +2784,13 @@
         <v>38</v>
       </c>
       <c r="Q7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="S7" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2859,15 +2805,15 @@
       </c>
       <c r="D8" s="48"/>
       <c r="G8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="O8" s="58"/>
@@ -2875,7 +2821,7 @@
         <v>42</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2890,26 +2836,26 @@
       </c>
       <c r="D9" s="48"/>
       <c r="G9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="I9" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="O9" s="58"/>
       <c r="P9" s="31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2924,29 +2870,29 @@
       </c>
       <c r="D10" s="48"/>
       <c r="G10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="H10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="I10" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="O10" s="58"/>
       <c r="P10" s="60" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="Q10" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="S10" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="R10" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="S10" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2961,29 +2907,29 @@
       </c>
       <c r="D11" s="48"/>
       <c r="G11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="H11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="I11" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="O11" s="58"/>
       <c r="P11" s="60" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="Q11" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="S11" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="R11" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2998,35 +2944,35 @@
       </c>
       <c r="D12" s="48"/>
       <c r="G12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="I12" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="O12" s="58"/>
       <c r="P12" s="60" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="R12" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="Q12" s="2" t="s">
+      <c r="S12" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="R12" s="2" t="s">
+      <c r="T12" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="S12" s="2" t="s">
+      <c r="U12" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3041,29 +2987,29 @@
       </c>
       <c r="D13" s="48"/>
       <c r="G13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="H13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="61" t="n">
-        <f aca="true">OFFSET($D$72,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="O13" s="58"/>
       <c r="P13" s="60" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="Q13" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="S13" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3086,25 +3032,25 @@
       <c r="M14" s="2"/>
       <c r="O14" s="58"/>
       <c r="P14" s="60" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="Q14" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="S14" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="R14" s="2" t="s">
+      <c r="T14" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="S14" s="2" t="s">
+      <c r="U14" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="T14" s="2" t="s">
+      <c r="V14" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="U14" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="V14" s="2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3119,7 +3065,7 @@
       </c>
       <c r="D15" s="48"/>
       <c r="G15" s="59" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H15" s="59"/>
       <c r="I15" s="59"/>
@@ -3129,13 +3075,13 @@
       <c r="M15" s="2"/>
       <c r="O15" s="58"/>
       <c r="P15" s="62" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q15" s="63" t="s">
+        <v>149</v>
+      </c>
+      <c r="R15" s="63" t="s">
         <v>150</v>
-      </c>
-      <c r="Q15" s="63" t="s">
-        <v>151</v>
-      </c>
-      <c r="R15" s="63" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3150,73 +3096,73 @@
       </c>
       <c r="D16" s="48"/>
       <c r="G16" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="H16" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="I16" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="J16" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="K16" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="O16" s="58"/>
       <c r="P16" s="62" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q16" s="63" t="s">
+        <v>152</v>
+      </c>
+      <c r="R16" s="63" t="s">
         <v>153</v>
-      </c>
-      <c r="Q16" s="63" t="s">
-        <v>154</v>
-      </c>
-      <c r="R16" s="63" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="55"/>
-      <c r="B17" s="48" t="str">
+      <c r="B17" s="64" t="str">
         <f aca="false">Основна!A28</f>
         <v>Група обліку</v>
       </c>
-      <c r="C17" s="48" t="str">
+      <c r="C17" s="64" t="str">
         <f aca="false">IF(Основна!B28 = 0, "",  Основна!B28)</f>
         <v/>
       </c>
-      <c r="D17" s="48"/>
+      <c r="D17" s="64"/>
       <c r="G17" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="I17" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="K17" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="O17" s="58" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>14</v>
@@ -3885,33 +3831,33 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="55"/>
-      <c r="B18" s="48" t="str">
+      <c r="B18" s="64" t="str">
         <f aca="false">Основна!A29</f>
         <v>Категорія обліку</v>
       </c>
-      <c r="C18" s="48" t="str">
+      <c r="C18" s="64" t="str">
         <f aca="false">IF(Основна!B29 = 0, "",  Основна!B29)</f>
         <v/>
       </c>
-      <c r="D18" s="48"/>
+      <c r="D18" s="64"/>
       <c r="G18" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="I18" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="J18" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="K18" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="L18" s="2"/>
@@ -4584,33 +4530,33 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="55"/>
-      <c r="B19" s="48" t="str">
+      <c r="B19" s="64" t="str">
         <f aca="false">Основна!A30</f>
         <v>Склад</v>
       </c>
-      <c r="C19" s="48" t="str">
+      <c r="C19" s="64" t="str">
         <f aca="false">IF(Основна!B30 = 0, "",  Основна!B30)</f>
         <v/>
       </c>
-      <c r="D19" s="48"/>
+      <c r="D19" s="64"/>
       <c r="G19" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="H19" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="I19" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="J19" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="K19" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="L19" s="2"/>
@@ -5283,33 +5229,33 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="55"/>
-      <c r="B20" s="48" t="str">
+      <c r="B20" s="64" t="str">
         <f aca="false">Основна!A31</f>
         <v>Військове звання</v>
       </c>
-      <c r="C20" s="48" t="str">
+      <c r="C20" s="64" t="str">
         <f aca="false">IF(Основна!B31 = 0, "",  Основна!B31)</f>
         <v/>
       </c>
-      <c r="D20" s="48"/>
+      <c r="D20" s="64"/>
       <c r="G20" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="J20" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="K20" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="L20" s="2"/>
@@ -5982,33 +5928,33 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="55"/>
-      <c r="B21" s="48" t="str">
+      <c r="B21" s="64" t="str">
         <f aca="false">Основна!A32</f>
         <v>Військово-облікова спеціальність</v>
       </c>
-      <c r="C21" s="48" t="str">
+      <c r="C21" s="64" t="str">
         <f aca="false">IF(Основна!B32 = 0, "",  Основна!B32)</f>
         <v/>
       </c>
-      <c r="D21" s="48"/>
+      <c r="D21" s="64"/>
       <c r="G21" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="I21" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="K21" s="61" t="n">
-        <f aca="true">OFFSET($D$90,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="L21" s="2"/>
@@ -6681,15 +6627,15 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="55"/>
-      <c r="B22" s="48" t="str">
+      <c r="B22" s="64" t="str">
         <f aca="false">Основна!A33</f>
         <v> Придатність до військової служби</v>
       </c>
-      <c r="C22" s="48" t="str">
+      <c r="C22" s="64" t="str">
         <f aca="false">IF(Основна!B33 = 0, "",  Основна!B33)</f>
         <v/>
       </c>
-      <c r="D22" s="48"/>
+      <c r="D22" s="64"/>
       <c r="O22" s="58"/>
       <c r="P22" s="9" t="s">
         <v>32</v>
@@ -7358,15 +7304,15 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="55"/>
-      <c r="B23" s="48" t="str">
+      <c r="B23" s="64" t="str">
         <f aca="false">Основна!A34</f>
         <v>Териториальний центр комплектування та соціальної підтримки</v>
       </c>
-      <c r="C23" s="48" t="str">
+      <c r="C23" s="64" t="str">
         <f aca="false">IF(Основна!B34 = 0, "",  Основна!B34)</f>
         <v/>
       </c>
-      <c r="D23" s="48"/>
+      <c r="D23" s="64"/>
       <c r="O23" s="58"/>
       <c r="P23" s="9" t="s">
         <v>34</v>
@@ -8035,15 +7981,15 @@
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="55"/>
-      <c r="B24" s="48" t="str">
+      <c r="B24" s="64" t="str">
         <f aca="false">Основна!A35</f>
         <v>Перебування на спеціальному обліку</v>
       </c>
-      <c r="C24" s="48" t="str">
+      <c r="C24" s="64" t="str">
         <f aca="false">IF(Основна!B35 = 0, "",  Основна!B35)</f>
         <v/>
       </c>
-      <c r="D24" s="48"/>
+      <c r="D24" s="64"/>
       <c r="O24" s="58"/>
       <c r="P24" s="60" t="s">
         <v>40</v>
@@ -8712,17 +8658,17 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="55" t="s">
-        <v>157</v>
-      </c>
-      <c r="B25" s="48" t="str">
+        <v>155</v>
+      </c>
+      <c r="B25" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A4</f>
         <v>Країна</v>
       </c>
-      <c r="C25" s="48" t="str">
+      <c r="C25" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B4 = 0, "", 'Адреси Контакти'!B4)</f>
         <v/>
       </c>
-      <c r="D25" s="48"/>
+      <c r="D25" s="64"/>
       <c r="O25" s="58"/>
       <c r="P25" s="31" t="s">
         <v>45</v>
@@ -9391,18 +9337,18 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="55"/>
-      <c r="B26" s="48" t="str">
+      <c r="B26" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A5</f>
-        <v>Область</v>
-      </c>
-      <c r="C26" s="48" t="str">
+        <v>Область (України)</v>
+      </c>
+      <c r="C26" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B5 = 0, "", 'Адреси Контакти'!B5)</f>
         <v/>
       </c>
-      <c r="D26" s="48"/>
+      <c r="D26" s="64"/>
       <c r="O26" s="58"/>
       <c r="P26" s="28" t="s">
-        <v>47</v>
+        <v>156</v>
       </c>
       <c r="Q26" s="56"/>
       <c r="R26" s="56"/>
@@ -10068,18 +10014,18 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="55"/>
-      <c r="B27" s="48" t="str">
+      <c r="B27" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A6</f>
         <v>Місто</v>
       </c>
-      <c r="C27" s="48" t="str">
+      <c r="C27" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B6 = 0, "", 'Адреси Контакти'!B6)</f>
         <v/>
       </c>
-      <c r="D27" s="48"/>
+      <c r="D27" s="64"/>
       <c r="O27" s="58"/>
       <c r="P27" s="28" t="s">
-        <v>50</v>
+        <v>157</v>
       </c>
       <c r="Q27" s="56"/>
       <c r="R27" s="56"/>
@@ -10745,18 +10691,18 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="55"/>
-      <c r="B28" s="48" t="str">
+      <c r="B28" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A7</f>
-        <v>Район (міста)</v>
-      </c>
-      <c r="C28" s="48" t="str">
+        <v>Адреса (вулиця, № будинку, квартири)</v>
+      </c>
+      <c r="C28" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B7 = 0, "", 'Адреси Контакти'!B7)</f>
         <v/>
       </c>
-      <c r="D28" s="48"/>
+      <c r="D28" s="64"/>
       <c r="O28" s="58"/>
       <c r="P28" s="60" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="Q28" s="56"/>
       <c r="R28" s="56"/>
@@ -11422,146 +11368,146 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="55"/>
-      <c r="B29" s="48" t="str">
+      <c r="B29" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A8</f>
-        <v>Адреса (вулиця, № будинку, квартири)</v>
-      </c>
-      <c r="C29" s="48" t="str">
+        <v>Індекс</v>
+      </c>
+      <c r="C29" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B8 = 0, "", 'Адреси Контакти'!B8)</f>
         <v/>
       </c>
-      <c r="D29" s="48"/>
+      <c r="D29" s="64"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="55"/>
-      <c r="B30" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A9</f>
-        <v>Індекс</v>
-      </c>
-      <c r="C30" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B9 = 0, "", 'Адреси Контакти'!B9)</f>
-        <v/>
-      </c>
-      <c r="D30" s="48"/>
+      <c r="B30" s="64" t="str">
+        <f aca="false">'Адреси Контакти'!A11</f>
+        <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
+      </c>
+      <c r="C30" s="64" t="str">
+        <f aca="false">IF('Адреси Контакти'!B11 = 0, "", 'Адреси Контакти'!B11)</f>
+        <v/>
+      </c>
+      <c r="D30" s="64"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="55"/>
-      <c r="B31" s="48" t="str">
+      <c r="B31" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A12</f>
-        <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
-      </c>
-      <c r="C31" s="48" t="str">
+        <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
+      </c>
+      <c r="C31" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B12 = 0, "", 'Адреси Контакти'!B12)</f>
         <v/>
       </c>
-      <c r="D31" s="48"/>
+      <c r="D31" s="64"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="55"/>
-      <c r="B32" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A13</f>
-        <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
-      </c>
-      <c r="C32" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B13 = 0, "", 'Адреси Контакти'!B13)</f>
-        <v/>
-      </c>
-      <c r="D32" s="48"/>
+      <c r="B32" s="64" t="str">
+        <f aca="false">'Адреси Контакти'!A15</f>
+        <v>Співпадає із адресою фактичного проживання</v>
+      </c>
+      <c r="C32" s="64" t="str">
+        <f aca="false">IF('Адреси Контакти'!B15 = 0, "", 'Адреси Контакти'!B15)</f>
+        <v/>
+      </c>
+      <c r="D32" s="64"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="55"/>
-      <c r="B33" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A16</f>
-        <v>Співпадає із адресою фактичного проживання</v>
-      </c>
-      <c r="C33" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B16 = 0, "", 'Адреси Контакти'!B16)</f>
-        <v/>
-      </c>
-      <c r="D33" s="48"/>
+      <c r="B33" s="64" t="str">
+        <f aca="false">'Адреси Контакти'!A17</f>
+        <v>Країна</v>
+      </c>
+      <c r="C33" s="64" t="str">
+        <f aca="false">IF('Адреси Контакти'!B17 = 0, "", 'Адреси Контакти'!B17)</f>
+        <v/>
+      </c>
+      <c r="D33" s="64"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="55"/>
-      <c r="B34" s="48" t="str">
+      <c r="B34" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A18</f>
-        <v>Країна</v>
-      </c>
-      <c r="C34" s="48" t="str">
+        <v>Область (України)</v>
+      </c>
+      <c r="C34" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B18 = 0, "", 'Адреси Контакти'!B18)</f>
         <v/>
       </c>
-      <c r="D34" s="48"/>
+      <c r="D34" s="64"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="55"/>
-      <c r="B35" s="48" t="str">
+      <c r="B35" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A19</f>
-        <v>Область</v>
-      </c>
-      <c r="C35" s="48" t="str">
+        <v>Місто</v>
+      </c>
+      <c r="C35" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B19 = 0, "", 'Адреси Контакти'!B19)</f>
         <v/>
       </c>
-      <c r="D35" s="48"/>
+      <c r="D35" s="64"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="55"/>
-      <c r="B36" s="48" t="str">
+      <c r="B36" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A20</f>
-        <v>Місто</v>
-      </c>
-      <c r="C36" s="48" t="str">
+        <v>Адреса (вулиця, № будинку, квартири)</v>
+      </c>
+      <c r="C36" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B20 = 0, "", 'Адреси Контакти'!B20)</f>
         <v/>
       </c>
-      <c r="D36" s="48"/>
+      <c r="D36" s="64"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="55"/>
-      <c r="B37" s="48" t="str">
+      <c r="B37" s="64" t="str">
         <f aca="false">'Адреси Контакти'!A21</f>
-        <v>Район (міста)</v>
-      </c>
-      <c r="C37" s="48" t="str">
+        <v>Індекс</v>
+      </c>
+      <c r="C37" s="64" t="str">
         <f aca="false">IF('Адреси Контакти'!B21 = 0, "", 'Адреси Контакти'!B21)</f>
         <v/>
       </c>
-      <c r="D37" s="48"/>
+      <c r="D37" s="64"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="55"/>
-      <c r="B38" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A22</f>
-        <v>Адреса (вулиця, № будинку, квартири)</v>
-      </c>
-      <c r="C38" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B22 = 0, "", 'Адреси Контакти'!B22)</f>
-        <v/>
-      </c>
-      <c r="D38" s="48"/>
+      <c r="A38" s="55" t="s">
+        <v>158</v>
+      </c>
+      <c r="B38" s="64" t="str">
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
+      </c>
+      <c r="C38" s="65" t="str">
+        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
+        <v/>
+      </c>
+      <c r="D38" s="66"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="55"/>
-      <c r="B39" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A23</f>
-        <v>Індекс</v>
-      </c>
-      <c r="C39" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B23 = 0, "", 'Адреси Контакти'!B23)</f>
-        <v/>
-      </c>
-      <c r="D39" s="48"/>
+      <c r="B39" s="64" t="str">
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
+      </c>
+      <c r="C39" s="65" t="str">
+        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
+        <v/>
+      </c>
+      <c r="D39" s="66"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="55" t="s">
-        <v>158</v>
-      </c>
+      <c r="A40" s="55"/>
       <c r="B40" s="64" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C40" s="65" t="str">
-        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
+        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
       <c r="D40" s="66"/>
@@ -11569,11 +11515,11 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="55"/>
       <c r="B41" s="64" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C41" s="65" t="str">
-        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
+        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
       <c r="D41" s="66"/>
@@ -11581,11 +11527,11 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="55"/>
       <c r="B42" s="64" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C42" s="65" t="str">
-        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
+        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
       <c r="D42" s="66"/>
@@ -11593,11 +11539,11 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="55"/>
       <c r="B43" s="64" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C43" s="65" t="str">
-        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
+        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
       <c r="D43" s="66"/>
@@ -11605,11 +11551,11 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="55"/>
       <c r="B44" s="64" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C44" s="65" t="str">
-        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
+        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
       <c r="D44" s="66"/>
@@ -11617,11 +11563,11 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="55"/>
       <c r="B45" s="64" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C45" s="65" t="str">
-        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
+        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
         <v/>
       </c>
       <c r="D45" s="66"/>
@@ -11629,11 +11575,11 @@
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="55"/>
       <c r="B46" s="64" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C46" s="65" t="str">
-        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
+        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
       <c r="D46" s="66"/>
@@ -11641,11 +11587,11 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="55"/>
       <c r="B47" s="64" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C47" s="65" t="str">
-        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
+        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
       <c r="D47" s="66"/>
@@ -11653,11 +11599,11 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="55"/>
       <c r="B48" s="64" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C48" s="65" t="str">
-        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
+        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
       <c r="D48" s="66"/>
@@ -11665,11 +11611,11 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="55"/>
       <c r="B49" s="64" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C49" s="65" t="str">
-        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
+        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
       <c r="D49" s="66"/>
@@ -11677,11 +11623,11 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="55"/>
       <c r="B50" s="64" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C50" s="65" t="str">
-        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
+        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
       <c r="D50" s="66"/>
@@ -11689,11 +11635,11 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="55"/>
       <c r="B51" s="64" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C51" s="65" t="str">
-        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
+        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
       <c r="D51" s="66"/>
@@ -11701,11 +11647,11 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="55"/>
       <c r="B52" s="64" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C52" s="65" t="str">
-        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
+        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
       <c r="D52" s="66"/>
@@ -11713,11 +11659,11 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="55"/>
       <c r="B53" s="64" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C53" s="65" t="str">
-        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
+        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
         <v/>
       </c>
       <c r="D53" s="66"/>
@@ -11725,11 +11671,11 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="55"/>
       <c r="B54" s="64" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C54" s="65" t="str">
-        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
+        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
       <c r="D54" s="66"/>
@@ -11737,11 +11683,11 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="55"/>
       <c r="B55" s="64" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C55" s="65" t="str">
-        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
+        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
       <c r="D55" s="66"/>
@@ -11749,11 +11695,11 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="55"/>
       <c r="B56" s="64" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C56" s="65" t="str">
-        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
+        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
       <c r="D56" s="66"/>
@@ -11761,11 +11707,11 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="55"/>
       <c r="B57" s="64" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C57" s="65" t="str">
-        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
+        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
       <c r="D57" s="66"/>
@@ -11773,11 +11719,11 @@
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="55"/>
       <c r="B58" s="64" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C58" s="65" t="str">
-        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
+        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
       <c r="D58" s="66"/>
@@ -11785,11 +11731,11 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="55"/>
       <c r="B59" s="64" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C59" s="65" t="str">
-        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
+        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
       <c r="D59" s="66"/>
@@ -11797,11 +11743,11 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="55"/>
       <c r="B60" s="64" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C60" s="65" t="str">
-        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
+        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
       <c r="D60" s="66"/>
@@ -11809,11 +11755,11 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="55"/>
       <c r="B61" s="64" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C61" s="65" t="str">
-        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
+        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
         <v/>
       </c>
       <c r="D61" s="66"/>
@@ -11821,11 +11767,11 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="55"/>
       <c r="B62" s="64" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C62" s="65" t="str">
-        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
+        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
       <c r="D62" s="66"/>
@@ -11833,11 +11779,11 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="55"/>
       <c r="B63" s="64" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C63" s="65" t="str">
-        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
+        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
       <c r="D63" s="66"/>
@@ -11845,11 +11791,11 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="55"/>
       <c r="B64" s="64" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C64" s="65" t="str">
-        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
+        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
       <c r="D64" s="66"/>
@@ -11857,11 +11803,11 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="55"/>
       <c r="B65" s="64" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C65" s="65" t="str">
-        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
+        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
       <c r="D65" s="66"/>
@@ -11869,11 +11815,11 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="55"/>
       <c r="B66" s="64" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C66" s="65" t="str">
-        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
+        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
       <c r="D66" s="66"/>
@@ -11881,11 +11827,11 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="55"/>
       <c r="B67" s="64" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C67" s="65" t="str">
-        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
+        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
       <c r="D67" s="66"/>
@@ -11893,11 +11839,11 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="55"/>
       <c r="B68" s="64" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C68" s="65" t="str">
-        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
+        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
       <c r="D68" s="66"/>
@@ -11905,11 +11851,11 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="55"/>
       <c r="B69" s="64" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C69" s="65" t="str">
-        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
+        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
         <v/>
       </c>
       <c r="D69" s="66"/>
@@ -11917,11 +11863,11 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="55"/>
       <c r="B70" s="64" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
-      </c>
-      <c r="C70" s="65" t="str">
-        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C70" s="67" t="str">
+        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
       <c r="D70" s="66"/>
@@ -11929,23 +11875,23 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="55"/>
       <c r="B71" s="64" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
-      </c>
-      <c r="C71" s="65" t="str">
-        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C71" s="67" t="str">
+        <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
       <c r="D71" s="66"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="55"/>
-      <c r="B72" s="64" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
+      <c r="B72" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
       </c>
       <c r="C72" s="67" t="str">
-        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
+        <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
         <v/>
       </c>
       <c r="D72" s="66"/>
@@ -11953,35 +11899,35 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="55"/>
       <c r="B73" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C73" s="67" t="str">
+        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
+        <v/>
+      </c>
+      <c r="D73" s="66"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="55"/>
+      <c r="B74" s="64" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C73" s="67" t="str">
-        <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
-        <v/>
-      </c>
-      <c r="D73" s="66"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="55"/>
-      <c r="B74" s="2" t="str">
+      <c r="C74" s="67" t="str">
+        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
+        <v/>
+      </c>
+      <c r="D74" s="66"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="55"/>
+      <c r="B75" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C74" s="67" t="str">
-        <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
-        <v/>
-      </c>
-      <c r="D74" s="66"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="55"/>
-      <c r="B75" s="64" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
       <c r="C75" s="67" t="str">
-        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
+        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
         <v/>
       </c>
       <c r="D75" s="66"/>
@@ -11989,35 +11935,35 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="55"/>
       <c r="B76" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C76" s="67" t="str">
+        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
+        <v/>
+      </c>
+      <c r="D76" s="66"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="55"/>
+      <c r="B77" s="64" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C76" s="67" t="str">
-        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
-        <v/>
-      </c>
-      <c r="D76" s="66"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="55"/>
-      <c r="B77" s="2" t="str">
+      <c r="C77" s="67" t="str">
+        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
+        <v/>
+      </c>
+      <c r="D77" s="66"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="55"/>
+      <c r="B78" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C77" s="67" t="str">
-        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
-        <v/>
-      </c>
-      <c r="D77" s="66"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="55"/>
-      <c r="B78" s="64" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
       <c r="C78" s="67" t="str">
-        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
+        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
         <v/>
       </c>
       <c r="D78" s="66"/>
@@ -12025,35 +11971,35 @@
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="55"/>
       <c r="B79" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C79" s="67" t="str">
+        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
+        <v/>
+      </c>
+      <c r="D79" s="66"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="55"/>
+      <c r="B80" s="64" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C79" s="67" t="str">
-        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
-        <v/>
-      </c>
-      <c r="D79" s="66"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="55"/>
-      <c r="B80" s="2" t="str">
+      <c r="C80" s="67" t="str">
+        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
+        <v/>
+      </c>
+      <c r="D80" s="66"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="55"/>
+      <c r="B81" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C80" s="67" t="str">
-        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
-        <v/>
-      </c>
-      <c r="D80" s="66"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="55"/>
-      <c r="B81" s="64" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
       <c r="C81" s="67" t="str">
-        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
+        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
         <v/>
       </c>
       <c r="D81" s="66"/>
@@ -12061,35 +12007,35 @@
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="55"/>
       <c r="B82" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C82" s="67" t="str">
+        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
+        <v/>
+      </c>
+      <c r="D82" s="66"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="55"/>
+      <c r="B83" s="64" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C82" s="67" t="str">
-        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
-        <v/>
-      </c>
-      <c r="D82" s="66"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="55"/>
-      <c r="B83" s="2" t="str">
+      <c r="C83" s="67" t="str">
+        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
+        <v/>
+      </c>
+      <c r="D83" s="66"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="55"/>
+      <c r="B84" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C83" s="67" t="str">
-        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
-        <v/>
-      </c>
-      <c r="D83" s="66"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="55"/>
-      <c r="B84" s="64" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
       <c r="C84" s="67" t="str">
-        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
+        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
         <v/>
       </c>
       <c r="D84" s="66"/>
@@ -12097,73 +12043,73 @@
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="55"/>
       <c r="B85" s="64" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C85" s="67" t="str">
+        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
+        <v/>
+      </c>
+      <c r="D85" s="66"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="55"/>
+      <c r="B86" s="64" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C85" s="67" t="str">
-        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
-        <v/>
-      </c>
-      <c r="D85" s="66"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="55"/>
-      <c r="B86" s="2" t="str">
+      <c r="C86" s="67" t="str">
+        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
+        <v/>
+      </c>
+      <c r="D86" s="66"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="55"/>
+      <c r="B87" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C86" s="67" t="str">
-        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
-        <v/>
-      </c>
-      <c r="D86" s="66"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="55"/>
-      <c r="B87" s="64" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
       <c r="C87" s="67" t="str">
-        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
+        <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
       <c r="D87" s="66"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="55"/>
+      <c r="A88" s="55" t="s">
+        <v>159</v>
+      </c>
       <c r="B88" s="64" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C88" s="67" t="str">
-        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C88" s="68" t="str">
+        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
         <v/>
       </c>
       <c r="D88" s="66"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="55"/>
-      <c r="B89" s="2" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рівень підготовки</v>
-      </c>
-      <c r="C89" s="67" t="str">
-        <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
+      <c r="B89" s="64" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
+      <c r="C89" s="68" t="str">
+        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
         <v/>
       </c>
       <c r="D89" s="66"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="55" t="s">
-        <v>159</v>
-      </c>
-      <c r="B90" s="64" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      <c r="A90" s="55"/>
+      <c r="B90" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C90" s="68" t="str">
-        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
+        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
         <v/>
       </c>
       <c r="D90" s="66"/>
@@ -12171,23 +12117,23 @@
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="55"/>
       <c r="B91" s="64" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C91" s="68" t="str">
-        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
+        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
         <v/>
       </c>
       <c r="D91" s="66"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="55"/>
-      <c r="B92" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B92" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C92" s="68" t="str">
-        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
+        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
         <v/>
       </c>
       <c r="D92" s="66"/>
@@ -12195,11 +12141,11 @@
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="55"/>
       <c r="B93" s="64" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C93" s="68" t="str">
-        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
+        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
         <v/>
       </c>
       <c r="D93" s="66"/>
@@ -12207,23 +12153,23 @@
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="55"/>
       <c r="B94" s="64" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C94" s="68" t="str">
-        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
+        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
         <v/>
       </c>
       <c r="D94" s="66"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="55"/>
-      <c r="B95" s="64" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      <c r="B95" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C95" s="68" t="str">
-        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
         <v/>
       </c>
       <c r="D95" s="66"/>
@@ -12231,23 +12177,23 @@
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="55"/>
       <c r="B96" s="64" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C96" s="68" t="str">
-        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
+        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
         <v/>
       </c>
       <c r="D96" s="66"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="55"/>
-      <c r="B97" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B97" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C97" s="68" t="str">
-        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
+        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
         <v/>
       </c>
       <c r="D97" s="66"/>
@@ -12255,11 +12201,11 @@
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="55"/>
       <c r="B98" s="64" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C98" s="68" t="str">
-        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
+        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
         <v/>
       </c>
       <c r="D98" s="66"/>
@@ -12267,23 +12213,23 @@
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="55"/>
       <c r="B99" s="64" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C99" s="68" t="str">
-        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
+        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
         <v/>
       </c>
       <c r="D99" s="66"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="55"/>
-      <c r="B100" s="64" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      <c r="B100" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C100" s="68" t="str">
-        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
         <v/>
       </c>
       <c r="D100" s="66"/>
@@ -12291,23 +12237,23 @@
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="55"/>
       <c r="B101" s="64" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C101" s="68" t="str">
-        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
+        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
         <v/>
       </c>
       <c r="D101" s="66"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="55"/>
-      <c r="B102" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B102" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C102" s="68" t="str">
-        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
+        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
         <v/>
       </c>
       <c r="D102" s="66"/>
@@ -12315,11 +12261,11 @@
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="55"/>
       <c r="B103" s="64" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C103" s="68" t="str">
-        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
+        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
         <v/>
       </c>
       <c r="D103" s="66"/>
@@ -12327,23 +12273,23 @@
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="55"/>
       <c r="B104" s="64" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C104" s="68" t="str">
-        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
+        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
         <v/>
       </c>
       <c r="D104" s="66"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="55"/>
-      <c r="B105" s="64" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      <c r="B105" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C105" s="68" t="str">
-        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
         <v/>
       </c>
       <c r="D105" s="66"/>
@@ -12351,23 +12297,23 @@
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="55"/>
       <c r="B106" s="64" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C106" s="68" t="str">
-        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
+        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
         <v/>
       </c>
       <c r="D106" s="66"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="55"/>
-      <c r="B107" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B107" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C107" s="68" t="str">
-        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
+        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
         <v/>
       </c>
       <c r="D107" s="66"/>
@@ -12375,11 +12321,11 @@
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="55"/>
       <c r="B108" s="64" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C108" s="68" t="str">
-        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
+        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
         <v/>
       </c>
       <c r="D108" s="66"/>
@@ -12387,23 +12333,23 @@
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="55"/>
       <c r="B109" s="64" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C109" s="68" t="str">
-        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
+        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
         <v/>
       </c>
       <c r="D109" s="66"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="55"/>
-      <c r="B110" s="64" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      <c r="B110" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C110" s="68" t="str">
-        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
         <v/>
       </c>
       <c r="D110" s="66"/>
@@ -12411,23 +12357,23 @@
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="55"/>
       <c r="B111" s="64" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C111" s="68" t="str">
-        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
+        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
         <v/>
       </c>
       <c r="D111" s="66"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="55"/>
-      <c r="B112" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B112" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C112" s="68" t="str">
-        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
+        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
         <v/>
       </c>
       <c r="D112" s="66"/>
@@ -12435,11 +12381,11 @@
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="55"/>
       <c r="B113" s="64" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C113" s="68" t="str">
-        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
+        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
         <v/>
       </c>
       <c r="D113" s="66"/>
@@ -12447,23 +12393,23 @@
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="55"/>
       <c r="B114" s="64" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C114" s="68" t="str">
-        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
+        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
         <v/>
       </c>
       <c r="D114" s="66"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="55"/>
-      <c r="B115" s="64" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      <c r="B115" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C115" s="68" t="str">
-        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
+        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
         <v/>
       </c>
       <c r="D115" s="66"/>
@@ -12471,61 +12417,61 @@
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="55"/>
       <c r="B116" s="64" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C116" s="68" t="str">
-        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
+        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
         <v/>
       </c>
       <c r="D116" s="66"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="55"/>
-      <c r="B117" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B117" s="64" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C117" s="68" t="str">
-        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
+        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
         <v/>
       </c>
       <c r="D117" s="66"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="55"/>
+      <c r="A118" s="55" t="s">
+        <v>160</v>
+      </c>
       <c r="B118" s="64" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C118" s="68" t="str">
-        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
-        <v/>
-      </c>
-      <c r="D118" s="66"/>
+        <f aca="false">Документи!A4</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C118" s="56" t="str">
+        <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
+        <v/>
+      </c>
+      <c r="D118" s="64"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="55"/>
       <c r="B119" s="64" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C119" s="68" t="str">
-        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
-        <v/>
-      </c>
-      <c r="D119" s="66"/>
+        <f aca="false">Документи!A5</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C119" s="64" t="str">
+        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
+        <v/>
+      </c>
+      <c r="D119" s="64"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="55" t="s">
-        <v>160</v>
-      </c>
+      <c r="A120" s="55"/>
       <c r="B120" s="64" t="str">
-        <f aca="false">Документи!A4</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C120" s="56" t="str">
-        <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
+        <f aca="false">Документи!A6</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C120" s="64" t="str">
+        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
         <v/>
       </c>
       <c r="D120" s="64"/>
@@ -12533,11 +12479,11 @@
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="55"/>
       <c r="B121" s="64" t="str">
-        <f aca="false">Документи!A5</f>
-        <v>Серія та номер </v>
+        <f aca="false">Документи!A7</f>
+        <v>Дата видачі</v>
       </c>
       <c r="C121" s="64" t="str">
-        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
+        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
         <v/>
       </c>
       <c r="D121" s="64"/>
@@ -12545,11 +12491,11 @@
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="55"/>
       <c r="B122" s="64" t="str">
-        <f aca="false">Документи!A6</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C122" s="64" t="str">
-        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
+        <f aca="false">Документи!A10</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C122" s="56" t="str">
+        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
         <v/>
       </c>
       <c r="D122" s="64"/>
@@ -12557,11 +12503,11 @@
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="55"/>
       <c r="B123" s="64" t="str">
-        <f aca="false">Документи!A7</f>
-        <v>Дата видачі</v>
+        <f aca="false">Документи!A11</f>
+        <v>Серія та номер </v>
       </c>
       <c r="C123" s="64" t="str">
-        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
+        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
         <v/>
       </c>
       <c r="D123" s="64"/>
@@ -12569,11 +12515,11 @@
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="55"/>
       <c r="B124" s="64" t="str">
-        <f aca="false">Документи!A10</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C124" s="56" t="str">
-        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
+        <f aca="false">Документи!A12</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C124" s="64" t="str">
+        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
         <v/>
       </c>
       <c r="D124" s="64"/>
@@ -12581,116 +12527,62 @@
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="55"/>
       <c r="B125" s="64" t="str">
-        <f aca="false">Документи!A11</f>
-        <v>Серія та номер </v>
+        <f aca="false">Документи!A13</f>
+        <v>Дата видачі</v>
       </c>
       <c r="C125" s="64" t="str">
-        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
+        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
         <v/>
       </c>
       <c r="D125" s="64"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="55"/>
-      <c r="B126" s="64" t="str">
-        <f aca="false">Документи!A12</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C126" s="64" t="str">
-        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
-        <v/>
-      </c>
+      <c r="B126" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="C126" s="64"/>
       <c r="D126" s="64"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="55"/>
       <c r="B127" s="64" t="str">
-        <f aca="false">Документи!A13</f>
-        <v>Дата видачі</v>
-      </c>
-      <c r="C127" s="64" t="str">
-        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
+        <f aca="false">Документи!A16</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C127" s="56" t="str">
+        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
         <v/>
       </c>
       <c r="D127" s="64"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="55"/>
-      <c r="B128" s="64" t="s">
-        <v>161</v>
-      </c>
-      <c r="C128" s="64"/>
+      <c r="B128" s="64" t="str">
+        <f aca="false">Документи!A17</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C128" s="64" t="str">
+        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
+        <v/>
+      </c>
       <c r="D128" s="64"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="55"/>
       <c r="B129" s="64" t="str">
-        <f aca="false">Документи!A16</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C129" s="56" t="str">
-        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
-        <v/>
-      </c>
-      <c r="D129" s="64"/>
-    </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="55"/>
-      <c r="B130" s="64" t="str">
-        <f aca="false">Документи!A17</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C130" s="64" t="str">
-        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
-        <v/>
-      </c>
-      <c r="D130" s="64"/>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="55"/>
-      <c r="B131" s="64" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C131" s="64" t="str">
+      <c r="C129" s="64" t="str">
         <f aca="false">IF(Документи!B18 = 0, "", Документи!B18)</f>
         <v/>
       </c>
-      <c r="D131" s="64"/>
-    </row>
-    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="D129" s="64"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="0"/>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="G1:N1"/>
@@ -12700,21 +12592,21 @@
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="O17:O28"/>
-    <mergeCell ref="A25:A39"/>
-    <mergeCell ref="A40:A89"/>
-    <mergeCell ref="A90:A119"/>
-    <mergeCell ref="A120:A131"/>
+    <mergeCell ref="A25:A37"/>
+    <mergeCell ref="A38:A87"/>
+    <mergeCell ref="A88:A117"/>
+    <mergeCell ref="A118:A129"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:K21" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D40:D44" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D38:D42" type="list">
       <formula1>'Системна інформація'!$Q$27:$ZA$27</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D46" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D44" type="list">
       <formula1>'Системна інформація'!$Q$11:$ZA$11</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
fix: delete reserv row in excel template | fix: style excel cells on export
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="162">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -154,250 +154,250 @@
     <t xml:space="preserve">Список на основі БД (Voenkomat) із додаванням</t>
   </si>
   <si>
+    <t xml:space="preserve">АДРЕСИ ТА КОНТАКТИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11. Місце фактичного проживання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Країна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (Country)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Область (України)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Список на основі БД (RegionUkraine) із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Місто</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Адреса (вулиця, № будинку, квартири)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Індекс</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 цифр, не обовязкове</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Телефони</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (основний)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 цифр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12. Місце проживання за державною реєстрацією </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Співпадає із адресою фактичного проживання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва освітнього закладу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія дисплома (свідоцтва)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Номер дисплома (свідоцтва)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік закінчення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Спеціальність (професія) за дипломом (свідоцтвом) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кваліфікація за дипломом (свідоцтвом)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Форма навчання (денна, вечірня, заочна)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівень освіти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рівень підготовки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Склад родини</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По-батькові</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рік народження</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 цифри!!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ДОКУМЕНТИ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип документу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Серія та номер </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ким виданий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата видачі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Військовий квіток</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: МК224345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закордоний паспорт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска: FF453210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва сторінки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва поля</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле для оновлення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поле з актуальною інформацією</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип заповнення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Назва списку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Основна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Визначений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна загальна середня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">професійно-технічна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неповна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">базова вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">повна вища</t>
+  </si>
+  <si>
+    <t xml:space="preserve">НПП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ІТС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">одружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">неодружений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">заміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">незаміжня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">розлучена</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдова</t>
+  </si>
+  <si>
+    <t xml:space="preserve">вдівець</t>
+  </si>
+  <si>
+    <t xml:space="preserve">військовозобов'язаний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">призовник</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">обмежено-придатний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">непридатний</t>
+  </si>
+  <si>
     <t xml:space="preserve">Перебування на спеціальному обліку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">АДРЕСИ ТА КОНТАКТИ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11. Місце фактичного проживання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Країна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (Country)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Область (України)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Список на основі БД (RegionUkraine) із додаванням</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Місто</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адреса (вулиця, № будинку, квартири)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Індекс</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 цифр, не обовязкове</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Телефони</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (основний)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 цифр</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12. Місце проживання за державною реєстрацією </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Співпадає із адресою фактичного проживання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва освітнього закладу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія дисплома (свідоцтва)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Номер дисплома (свідоцтва)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік закінчення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Спеціальність (професія) за дипломом (свідоцтвом) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кваліфікація за дипломом (свідоцтвом)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Форма навчання (денна, вечірня, заочна)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рівень освіти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва освітнього, наукового  закладу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рівень підготовки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. РОДИННИЙ СТАН</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Склад родини</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ступінь родинного зв’язку (склад сім'ї)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">По-батькові</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рік народження</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 цифри!!!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДОКУМЕНТИ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Паспорт (або ID-CARD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип документу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Серія та номер </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК229850 або 777111333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ким виданий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цирфи</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата видачі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Військовий квіток</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: МК224345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закордоний паспорт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска: FF453210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маска для ІД-картки: 4 цифри</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва сторінки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва поля</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле для оновлення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Поле з актуальною інформацією</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОСВІТА АКАДЕМІЧНА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тип заповнення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Назва списку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Значення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Основна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Визначений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна загальна середня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">професійно-технічна</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неповна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">базова вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">повна вища</t>
-  </si>
-  <si>
-    <t xml:space="preserve">НПП</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ІТС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">одружений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">неодружений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">заміжня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">незаміжня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">розлучений</t>
-  </si>
-  <si>
-    <t xml:space="preserve">розлучена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вдова</t>
-  </si>
-  <si>
-    <t xml:space="preserve">вдівець</t>
-  </si>
-  <si>
-    <t xml:space="preserve">військовозобов'язаний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">призовник</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ПІСЛЯДИПЛОМНА ПРОФЕСІЙНА ПІДГОТОВКА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">придатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">обмежено-придатний</t>
-  </si>
-  <si>
-    <t xml:space="preserve">непридатний</t>
   </si>
   <si>
     <t xml:space="preserve">Не перебуває</t>
@@ -1204,7 +1204,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:D35"/>
+  <dimension ref="A2:D1048576"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.37"/>
@@ -1541,21 +1541,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="26.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D24 = 0, "", 'Системна інформація'!D24)</f>
-        <v/>
-      </c>
-      <c r="D35" s="12" t="s">
-        <v>39</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <dataValidations count="16">
+  <dataValidations count="15">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B14" type="list">
       <formula1>'Системна інформація'!$Q$2:$ZA$2</formula1>
       <formula2>0</formula2>
@@ -1574,10 +1562,6 @@
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B18" type="list">
       <formula1>'Системна інформація'!$Q$4:$ZA$4</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B24" type="list">
-      <formula1>'Системна інформація'!$Q$21:$ZA$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B28" type="list">
@@ -1616,8 +1600,8 @@
       <formula1>'Системна інформація'!$Q$7:$ZA$7</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" error="Перевірте наявність типу перебування на спеціальному обліку в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="information" errorTitle="Даного типу перебування на спеціальному облік не є в списку" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B35" type="list">
-      <formula1>'Системна інформація'!$Q$8:$ZA$8</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B24" type="none">
+      <formula1>'Системна інформація'!$Q$21:$ZA$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1647,12 +1631,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="22"/>
@@ -1660,37 +1644,37 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" s="24"/>
       <c r="C4" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D25 = 0, "", 'Системна інформація'!D25)</f>
+        <f aca="false">IF('Системна інформація'!D24 = 0, "", 'Системна інформація'!D24)</f>
         <v/>
       </c>
       <c r="D4" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" s="27"/>
       <c r="C5" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D26 = 0, "", 'Системна інформація'!D26)</f>
+        <f aca="false">IF('Системна інформація'!D25 = 0, "", 'Системна інформація'!D25)</f>
         <v/>
       </c>
       <c r="D5" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D27 = 0, "", 'Системна інформація'!D27)</f>
+        <f aca="false">IF('Системна інформація'!D26 = 0, "", 'Системна інформація'!D26)</f>
         <v/>
       </c>
       <c r="D6" s="20" t="s">
@@ -1699,26 +1683,26 @@
     </row>
     <row r="7" s="25" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="27"/>
       <c r="C7" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D28 = 0, "", 'Системна інформація'!D28)</f>
+        <f aca="false">IF('Системна інформація'!D27 = 0, "", 'Системна інформація'!D27)</f>
         <v/>
       </c>
       <c r="D7" s="20"/>
     </row>
     <row r="8" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="27"/>
       <c r="C8" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D29 = 0, "", 'Системна інформація'!D29)</f>
+        <f aca="false">IF('Системна інформація'!D28 = 0, "", 'Системна інформація'!D28)</f>
         <v/>
       </c>
       <c r="D8" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1729,7 +1713,7 @@
     </row>
     <row r="10" s="25" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="2"/>
@@ -1737,28 +1721,28 @@
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="27"/>
       <c r="C11" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D30 = 0, "", 'Системна інформація'!D30)</f>
+        <f aca="false">IF('Системна інформація'!D29 = 0, "", 'Системна інформація'!D29)</f>
         <v/>
       </c>
       <c r="D11" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="27"/>
       <c r="C12" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D31 = 0, "", 'Системна інформація'!D31)</f>
+        <f aca="false">IF('Системна інформація'!D30 = 0, "", 'Системна інформація'!D30)</f>
         <v/>
       </c>
       <c r="D12" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1766,7 +1750,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="2"/>
@@ -1774,11 +1758,11 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" s="24"/>
       <c r="C15" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D32 = 0, "", 'Системна інформація'!D32)</f>
+        <f aca="false">IF('Системна інформація'!D31 = 0, "", 'Системна інформація'!D31)</f>
         <v/>
       </c>
       <c r="D15" s="22" t="s">
@@ -1793,37 +1777,37 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B17" s="24"/>
       <c r="C17" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D33 = 0, "", 'Системна інформація'!D33)</f>
+        <f aca="false">IF('Системна інформація'!D32 = 0, "", 'Системна інформація'!D32)</f>
         <v/>
       </c>
       <c r="D17" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D34 = 0, "", 'Системна інформація'!D34)</f>
+        <f aca="false">IF('Системна інформація'!D33 = 0, "", 'Системна інформація'!D33)</f>
         <v/>
       </c>
       <c r="D18" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B19" s="27"/>
       <c r="C19" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D35 = 0, "", 'Системна інформація'!D35)</f>
+        <f aca="false">IF('Системна інформація'!D34 = 0, "", 'Системна інформація'!D34)</f>
         <v/>
       </c>
       <c r="D19" s="20" t="s">
@@ -1832,25 +1816,25 @@
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D36 = 0, "", 'Системна інформація'!D36)</f>
+        <f aca="false">IF('Системна інформація'!D35 = 0, "", 'Системна інформація'!D35)</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="22" t="str">
-        <f aca="false">IF('Системна інформація'!D37 = 0, "", 'Системна інформація'!D37)</f>
+        <f aca="false">IF('Системна інформація'!D36 = 0, "", 'Системна інформація'!D36)</f>
         <v/>
       </c>
       <c r="D21" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1906,7 +1890,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
@@ -1926,7 +1910,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="34"/>
       <c r="C3" s="33"/>
@@ -1937,28 +1921,28 @@
     </row>
     <row r="4" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="C4" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="D4" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="E4" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="F4" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="G4" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="36" t="s">
+      <c r="H4" s="36" t="s">
         <v>67</v>
-      </c>
-      <c r="H4" s="36" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2005,7 +1989,7 @@
       <c r="A9" s="33"/>
       <c r="B9" s="33"/>
       <c r="D9" s="39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E9" s="33"/>
       <c r="F9" s="33"/>
@@ -2027,7 +2011,7 @@
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" s="33"/>
       <c r="C11" s="33"/>
@@ -2038,13 +2022,13 @@
     </row>
     <row r="12" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="35" t="s">
         <v>71</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2080,7 +2064,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33"/>
       <c r="B19" s="39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C19" s="39" t="s">
         <v>12</v>
@@ -2135,12 +2119,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
@@ -2149,7 +2133,7 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="43" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B4" s="44" t="s">
         <v>5</v>
@@ -2158,10 +2142,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" s="44" t="s">
         <v>76</v>
-      </c>
-      <c r="E4" s="44" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2211,7 +2195,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2248,21 +2232,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="47" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D118 = 0, "", 'Системна інформація'!D118)</f>
+        <f aca="false">IF('Системна інформація'!D117 = 0, "", 'Системна інформація'!D117)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="s">
@@ -2271,37 +2255,37 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D119 = 0, "", 'Системна інформація'!D119)</f>
+        <f aca="false">IF('Системна інформація'!D118 = 0, "", 'Системна інформація'!D118)</f>
         <v/>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
+        <f aca="false">IF('Системна інформація'!D119 = 0, "", 'Системна інформація'!D119)</f>
         <v/>
       </c>
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
+        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
         <v/>
       </c>
       <c r="D7" s="2" t="s">
@@ -2310,16 +2294,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="47" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
+        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="s">
@@ -2328,34 +2312,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
+        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
         <v/>
       </c>
       <c r="D11" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
+        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
+        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
         <v/>
       </c>
       <c r="D13" s="2" t="s">
@@ -2364,42 +2348,42 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
+        <f aca="false">IF('Системна інформація'!D126 = 0, "", 'Системна інформація'!D126)</f>
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D128 = 0, "", 'Системна інформація'!D128)</f>
+        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D129 = 0, "", 'Системна інформація'!D129)</f>
+        <f aca="false">IF('Системна інформація'!D128 = 0, "", 'Системна інформація'!D128)</f>
         <v/>
       </c>
       <c r="D18" s="2" t="s">
@@ -2445,20 +2429,20 @@
   <sheetData>
     <row r="1" s="51" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="C1" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="D1" s="51" t="s">
         <v>94</v>
-      </c>
-      <c r="D1" s="51" t="s">
-        <v>95</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="52" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H1" s="52"/>
       <c r="I1" s="52"/>
@@ -2468,13 +2452,13 @@
       <c r="M1" s="52"/>
       <c r="N1" s="52"/>
       <c r="O1" s="53" t="s">
+        <v>96</v>
+      </c>
+      <c r="P1" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="P1" s="54" t="s">
+      <c r="Q1" s="53" t="s">
         <v>98</v>
-      </c>
-      <c r="Q1" s="53" t="s">
-        <v>99</v>
       </c>
       <c r="R1" s="53"/>
       <c r="S1" s="53"/>
@@ -2482,7 +2466,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" s="48" t="str">
         <f aca="false">Основна!A9</f>
@@ -2494,60 +2478,60 @@
       </c>
       <c r="D2" s="48"/>
       <c r="G2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="H2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="I2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="J2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="K2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="L2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="M2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="N2" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="O2" s="58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>11</v>
       </c>
       <c r="Q2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2562,35 +2546,35 @@
       </c>
       <c r="D3" s="48"/>
       <c r="G3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="H3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="I3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="J3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="K3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="L3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="M3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="N3" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="O3" s="58"/>
@@ -2598,10 +2582,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="R3" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2616,35 +2600,35 @@
       </c>
       <c r="D4" s="48"/>
       <c r="G4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="H4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="I4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="J4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="K4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="L4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="M4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="N4" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="O4" s="58"/>
@@ -2652,28 +2636,28 @@
         <v>18</v>
       </c>
       <c r="Q4" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="R4" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="W4" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="X4" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2688,35 +2672,35 @@
       </c>
       <c r="D5" s="48"/>
       <c r="G5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="I5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="K5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="L5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="M5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="N5" s="57" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$37,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="O5" s="58"/>
@@ -2724,10 +2708,10 @@
         <v>30</v>
       </c>
       <c r="Q5" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="R5" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2771,7 +2755,7 @@
       </c>
       <c r="D7" s="48"/>
       <c r="G7" s="59" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H7" s="59"/>
       <c r="I7" s="59"/>
@@ -2780,13 +2764,13 @@
         <v>38</v>
       </c>
       <c r="Q7" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="R7" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="S7" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2801,26 +2785,26 @@
       </c>
       <c r="D8" s="48"/>
       <c r="G8" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="O8" s="58"/>
       <c r="P8" s="60" t="s">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="55"/>
       <c r="B9" s="48" t="str">
         <f aca="false">Основна!A16</f>
@@ -2832,20 +2816,20 @@
       </c>
       <c r="D9" s="48"/>
       <c r="G9" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="I9" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="O9" s="58"/>
       <c r="P9" s="31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>125</v>
@@ -2866,20 +2850,20 @@
       </c>
       <c r="D10" s="48"/>
       <c r="G10" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="H10" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="I10" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="O10" s="58"/>
       <c r="P10" s="60" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>127</v>
@@ -2903,20 +2887,20 @@
       </c>
       <c r="D11" s="48"/>
       <c r="G11" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="H11" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="I11" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="O11" s="58"/>
       <c r="P11" s="60" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>130</v>
@@ -2940,15 +2924,15 @@
       </c>
       <c r="D12" s="48"/>
       <c r="G12" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="I12" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="O12" s="58"/>
@@ -2983,20 +2967,20 @@
       </c>
       <c r="D13" s="48"/>
       <c r="G13" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="H13" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="61" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$69,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="O13" s="58"/>
       <c r="P13" s="60" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>139</v>
@@ -3028,7 +3012,7 @@
       <c r="M14" s="2"/>
       <c r="O14" s="58"/>
       <c r="P14" s="60" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>142</v>
@@ -3061,7 +3045,7 @@
       </c>
       <c r="D15" s="48"/>
       <c r="G15" s="59" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H15" s="59"/>
       <c r="I15" s="59"/>
@@ -3092,23 +3076,23 @@
       </c>
       <c r="D16" s="48"/>
       <c r="G16" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="H16" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="I16" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="J16" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="K16" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="L16" s="2"/>
@@ -3136,23 +3120,23 @@
       </c>
       <c r="D17" s="48"/>
       <c r="G17" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="I17" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="K17" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="L17" s="2"/>
@@ -3837,23 +3821,23 @@
       </c>
       <c r="D18" s="48"/>
       <c r="G18" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="I18" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="J18" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="K18" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="L18" s="2"/>
@@ -4536,23 +4520,23 @@
       </c>
       <c r="D19" s="48"/>
       <c r="G19" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="H19" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="I19" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="J19" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="K19" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="L19" s="2"/>
@@ -5235,23 +5219,23 @@
       </c>
       <c r="D20" s="48"/>
       <c r="G20" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="J20" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="K20" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="L20" s="2"/>
@@ -5934,23 +5918,23 @@
       </c>
       <c r="D21" s="48"/>
       <c r="G21" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="I21" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="K21" s="61" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$87,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="L21" s="2"/>
@@ -7976,13 +7960,15 @@
       <c r="ZA23" s="56"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="55"/>
+      <c r="A24" s="55" t="s">
+        <v>155</v>
+      </c>
       <c r="B24" s="48" t="str">
-        <f aca="false">Основна!A35</f>
-        <v>Перебування на спеціальному обліку</v>
+        <f aca="false">'Адреси Контакти'!A4</f>
+        <v>Країна</v>
       </c>
       <c r="C24" s="48" t="str">
-        <f aca="false">IF(Основна!B35 = 0, "",  Основна!B35)</f>
+        <f aca="false">IF('Адреси Контакти'!B4 = 0, "", 'Адреси Контакти'!B4)</f>
         <v/>
       </c>
       <c r="D24" s="48"/>
@@ -8653,21 +8639,19 @@
       <c r="ZA24" s="56"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="55" t="s">
-        <v>155</v>
-      </c>
+      <c r="A25" s="55"/>
       <c r="B25" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A4</f>
-        <v>Країна</v>
+        <f aca="false">'Адреси Контакти'!A5</f>
+        <v>Область (України)</v>
       </c>
       <c r="C25" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B4 = 0, "", 'Адреси Контакти'!B4)</f>
+        <f aca="false">IF('Адреси Контакти'!B5 = 0, "", 'Адреси Контакти'!B5)</f>
         <v/>
       </c>
       <c r="D25" s="48"/>
       <c r="O25" s="58"/>
       <c r="P25" s="31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q25" s="56"/>
       <c r="R25" s="56"/>
@@ -9334,11 +9318,11 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="55"/>
       <c r="B26" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A5</f>
-        <v>Область (України)</v>
+        <f aca="false">'Адреси Контакти'!A6</f>
+        <v>Місто</v>
       </c>
       <c r="C26" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B5 = 0, "", 'Адреси Контакти'!B5)</f>
+        <f aca="false">IF('Адреси Контакти'!B6 = 0, "", 'Адреси Контакти'!B6)</f>
         <v/>
       </c>
       <c r="D26" s="48"/>
@@ -10011,11 +9995,11 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="55"/>
       <c r="B27" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A6</f>
-        <v>Місто</v>
+        <f aca="false">'Адреси Контакти'!A7</f>
+        <v>Адреса (вулиця, № будинку, квартири)</v>
       </c>
       <c r="C27" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B6 = 0, "", 'Адреси Контакти'!B6)</f>
+        <f aca="false">IF('Адреси Контакти'!B7 = 0, "", 'Адреси Контакти'!B7)</f>
         <v/>
       </c>
       <c r="D27" s="48"/>
@@ -10688,17 +10672,17 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="55"/>
       <c r="B28" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A7</f>
-        <v>Адреса (вулиця, № будинку, квартири)</v>
+        <f aca="false">'Адреси Контакти'!A8</f>
+        <v>Індекс</v>
       </c>
       <c r="C28" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B7 = 0, "", 'Адреси Контакти'!B7)</f>
+        <f aca="false">IF('Адреси Контакти'!B8 = 0, "", 'Адреси Контакти'!B8)</f>
         <v/>
       </c>
       <c r="D28" s="48"/>
       <c r="O28" s="58"/>
       <c r="P28" s="60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q28" s="56"/>
       <c r="R28" s="56"/>
@@ -11365,11 +11349,11 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="55"/>
       <c r="B29" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A8</f>
-        <v>Індекс</v>
+        <f aca="false">'Адреси Контакти'!A11</f>
+        <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
       </c>
       <c r="C29" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B8 = 0, "", 'Адреси Контакти'!B8)</f>
+        <f aca="false">IF('Адреси Контакти'!B11 = 0, "", 'Адреси Контакти'!B11)</f>
         <v/>
       </c>
       <c r="D29" s="48"/>
@@ -11377,11 +11361,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="55"/>
       <c r="B30" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A11</f>
-        <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
+        <f aca="false">'Адреси Контакти'!A12</f>
+        <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
       </c>
       <c r="C30" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B11 = 0, "", 'Адреси Контакти'!B11)</f>
+        <f aca="false">IF('Адреси Контакти'!B12 = 0, "", 'Адреси Контакти'!B12)</f>
         <v/>
       </c>
       <c r="D30" s="48"/>
@@ -11389,11 +11373,11 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="55"/>
       <c r="B31" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A12</f>
-        <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
+        <f aca="false">'Адреси Контакти'!A15</f>
+        <v>Співпадає із адресою фактичного проживання</v>
       </c>
       <c r="C31" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B12 = 0, "", 'Адреси Контакти'!B12)</f>
+        <f aca="false">IF('Адреси Контакти'!B15 = 0, "", 'Адреси Контакти'!B15)</f>
         <v/>
       </c>
       <c r="D31" s="48"/>
@@ -11401,11 +11385,11 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="55"/>
       <c r="B32" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A15</f>
-        <v>Співпадає із адресою фактичного проживання</v>
+        <f aca="false">'Адреси Контакти'!A17</f>
+        <v>Країна</v>
       </c>
       <c r="C32" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B15 = 0, "", 'Адреси Контакти'!B15)</f>
+        <f aca="false">IF('Адреси Контакти'!B17 = 0, "", 'Адреси Контакти'!B17)</f>
         <v/>
       </c>
       <c r="D32" s="48"/>
@@ -11413,11 +11397,11 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="55"/>
       <c r="B33" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A17</f>
-        <v>Країна</v>
+        <f aca="false">'Адреси Контакти'!A18</f>
+        <v>Область (України)</v>
       </c>
       <c r="C33" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B17 = 0, "", 'Адреси Контакти'!B17)</f>
+        <f aca="false">IF('Адреси Контакти'!B18 = 0, "", 'Адреси Контакти'!B18)</f>
         <v/>
       </c>
       <c r="D33" s="48"/>
@@ -11425,11 +11409,11 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="55"/>
       <c r="B34" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A18</f>
-        <v>Область (України)</v>
+        <f aca="false">'Адреси Контакти'!A19</f>
+        <v>Місто</v>
       </c>
       <c r="C34" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B18 = 0, "", 'Адреси Контакти'!B18)</f>
+        <f aca="false">IF('Адреси Контакти'!B19 = 0, "", 'Адреси Контакти'!B19)</f>
         <v/>
       </c>
       <c r="D34" s="48"/>
@@ -11437,11 +11421,11 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="55"/>
       <c r="B35" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A19</f>
-        <v>Місто</v>
+        <f aca="false">'Адреси Контакти'!A20</f>
+        <v>Адреса (вулиця, № будинку, квартири)</v>
       </c>
       <c r="C35" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B19 = 0, "", 'Адреси Контакти'!B19)</f>
+        <f aca="false">IF('Адреси Контакти'!B20 = 0, "", 'Адреси Контакти'!B20)</f>
         <v/>
       </c>
       <c r="D35" s="48"/>
@@ -11449,37 +11433,37 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="55"/>
       <c r="B36" s="48" t="str">
-        <f aca="false">'Адреси Контакти'!A20</f>
-        <v>Адреса (вулиця, № будинку, квартири)</v>
-      </c>
-      <c r="C36" s="48" t="str">
-        <f aca="false">IF('Адреси Контакти'!B20 = 0, "", 'Адреси Контакти'!B20)</f>
-        <v/>
-      </c>
-      <c r="D36" s="48"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="55"/>
-      <c r="B37" s="48" t="str">
         <f aca="false">'Адреси Контакти'!A21</f>
         <v>Індекс</v>
       </c>
-      <c r="C37" s="48" t="str">
+      <c r="C36" s="48" t="str">
         <f aca="false">IF('Адреси Контакти'!B21 = 0, "", 'Адреси Контакти'!B21)</f>
         <v/>
       </c>
-      <c r="D37" s="48"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="55" t="s">
+      <c r="D36" s="48"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="B38" s="48" t="str">
+      <c r="B37" s="48" t="str">
         <f aca="false">Освіта!$A$4</f>
         <v>Назва освітнього закладу</v>
       </c>
+      <c r="C37" s="64" t="str">
+        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
+        <v/>
+      </c>
+      <c r="D37" s="65"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="55"/>
+      <c r="B38" s="48" t="str">
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
+      </c>
       <c r="C38" s="64" t="str">
-        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
+        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
         <v/>
       </c>
       <c r="D38" s="65"/>
@@ -11487,11 +11471,11 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="55"/>
       <c r="B39" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C39" s="64" t="str">
-        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
+        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
       <c r="D39" s="65"/>
@@ -11499,11 +11483,11 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="55"/>
       <c r="B40" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C40" s="64" t="str">
-        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
+        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
       <c r="D40" s="65"/>
@@ -11511,11 +11495,11 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="55"/>
       <c r="B41" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C41" s="64" t="str">
-        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
+        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
       <c r="D41" s="65"/>
@@ -11523,11 +11507,11 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="55"/>
       <c r="B42" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C42" s="64" t="str">
-        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
+        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
       <c r="D42" s="65"/>
@@ -11535,11 +11519,11 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="55"/>
       <c r="B43" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C43" s="64" t="str">
-        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
+        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
       <c r="D43" s="65"/>
@@ -11547,11 +11531,11 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="55"/>
       <c r="B44" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C44" s="64" t="str">
-        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
+        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
         <v/>
       </c>
       <c r="D44" s="65"/>
@@ -11559,11 +11543,11 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="55"/>
       <c r="B45" s="48" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C45" s="64" t="str">
-        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
+        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
       <c r="D45" s="65"/>
@@ -11571,11 +11555,11 @@
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="55"/>
       <c r="B46" s="48" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C46" s="64" t="str">
-        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
+        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
       <c r="D46" s="65"/>
@@ -11583,11 +11567,11 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="55"/>
       <c r="B47" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C47" s="64" t="str">
-        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
+        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
       <c r="D47" s="65"/>
@@ -11595,11 +11579,11 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="55"/>
       <c r="B48" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C48" s="64" t="str">
-        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
+        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
       <c r="D48" s="65"/>
@@ -11607,11 +11591,11 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="55"/>
       <c r="B49" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C49" s="64" t="str">
-        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
+        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
       <c r="D49" s="65"/>
@@ -11619,11 +11603,11 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="55"/>
       <c r="B50" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C50" s="64" t="str">
-        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
+        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
       <c r="D50" s="65"/>
@@ -11631,11 +11615,11 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="55"/>
       <c r="B51" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C51" s="64" t="str">
-        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
+        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
       <c r="D51" s="65"/>
@@ -11643,11 +11627,11 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="55"/>
       <c r="B52" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C52" s="64" t="str">
-        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
+        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
         <v/>
       </c>
       <c r="D52" s="65"/>
@@ -11655,11 +11639,11 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="55"/>
       <c r="B53" s="48" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C53" s="64" t="str">
-        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
+        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
       <c r="D53" s="65"/>
@@ -11667,11 +11651,11 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="55"/>
       <c r="B54" s="48" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C54" s="64" t="str">
-        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
+        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
       <c r="D54" s="65"/>
@@ -11679,11 +11663,11 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="55"/>
       <c r="B55" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C55" s="64" t="str">
-        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
+        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
       <c r="D55" s="65"/>
@@ -11691,11 +11675,11 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="55"/>
       <c r="B56" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C56" s="64" t="str">
-        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
+        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
       <c r="D56" s="65"/>
@@ -11703,11 +11687,11 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="55"/>
       <c r="B57" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C57" s="64" t="str">
-        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
+        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
       <c r="D57" s="65"/>
@@ -11715,11 +11699,11 @@
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="55"/>
       <c r="B58" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C58" s="64" t="str">
-        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
+        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
       <c r="D58" s="65"/>
@@ -11727,11 +11711,11 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="55"/>
       <c r="B59" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C59" s="64" t="str">
-        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
+        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
       <c r="D59" s="65"/>
@@ -11739,11 +11723,11 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="55"/>
       <c r="B60" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C60" s="64" t="str">
-        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
+        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
         <v/>
       </c>
       <c r="D60" s="65"/>
@@ -11751,11 +11735,11 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="55"/>
       <c r="B61" s="48" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C61" s="64" t="str">
-        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
+        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
       <c r="D61" s="65"/>
@@ -11763,11 +11747,11 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="55"/>
       <c r="B62" s="48" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C62" s="64" t="str">
-        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
+        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
       <c r="D62" s="65"/>
@@ -11775,11 +11759,11 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="55"/>
       <c r="B63" s="48" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C63" s="64" t="str">
-        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
+        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
       <c r="D63" s="65"/>
@@ -11787,11 +11771,11 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="55"/>
       <c r="B64" s="48" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C64" s="64" t="str">
-        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
+        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
       <c r="D64" s="65"/>
@@ -11799,11 +11783,11 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="55"/>
       <c r="B65" s="48" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C65" s="64" t="str">
-        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
+        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
       <c r="D65" s="65"/>
@@ -11811,11 +11795,11 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="55"/>
       <c r="B66" s="48" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C66" s="64" t="str">
-        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
+        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
       <c r="D66" s="65"/>
@@ -11823,11 +11807,11 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="55"/>
       <c r="B67" s="48" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C67" s="64" t="str">
-        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
+        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
       <c r="D67" s="65"/>
@@ -11835,11 +11819,11 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="55"/>
       <c r="B68" s="48" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C68" s="64" t="str">
-        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
+        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
         <v/>
       </c>
       <c r="D68" s="65"/>
@@ -11847,11 +11831,11 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="55"/>
       <c r="B69" s="48" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
-      </c>
-      <c r="C69" s="64" t="str">
-        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C69" s="66" t="str">
+        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
         <v/>
       </c>
       <c r="D69" s="65"/>
@@ -11859,35 +11843,35 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="55"/>
       <c r="B70" s="48" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C70" s="66" t="str">
+        <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
+        <v/>
+      </c>
+      <c r="D70" s="65"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="55"/>
+      <c r="B71" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C71" s="66" t="str">
+        <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
+        <v/>
+      </c>
+      <c r="D71" s="65"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="55"/>
+      <c r="B72" s="48" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C70" s="66" t="str">
-        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
-        <v/>
-      </c>
-      <c r="D70" s="65"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="55"/>
-      <c r="B71" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C71" s="66" t="str">
-        <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
-        <v/>
-      </c>
-      <c r="D71" s="65"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="55"/>
-      <c r="B72" s="2" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рівень підготовки</v>
-      </c>
       <c r="C72" s="66" t="str">
-        <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
+        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
         <v/>
       </c>
       <c r="D72" s="65"/>
@@ -11895,35 +11879,35 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="55"/>
       <c r="B73" s="48" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C73" s="66" t="str">
+        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
+        <v/>
+      </c>
+      <c r="D73" s="65"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="55"/>
+      <c r="B74" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C74" s="66" t="str">
+        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
+        <v/>
+      </c>
+      <c r="D74" s="65"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="55"/>
+      <c r="B75" s="48" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C73" s="66" t="str">
-        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
-        <v/>
-      </c>
-      <c r="D73" s="65"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="55"/>
-      <c r="B74" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C74" s="66" t="str">
-        <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
-        <v/>
-      </c>
-      <c r="D74" s="65"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="55"/>
-      <c r="B75" s="2" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рівень підготовки</v>
-      </c>
       <c r="C75" s="66" t="str">
-        <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
+        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
         <v/>
       </c>
       <c r="D75" s="65"/>
@@ -11931,35 +11915,35 @@
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="55"/>
       <c r="B76" s="48" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C76" s="66" t="str">
+        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
+        <v/>
+      </c>
+      <c r="D76" s="65"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="55"/>
+      <c r="B77" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C77" s="66" t="str">
+        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
+        <v/>
+      </c>
+      <c r="D77" s="65"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="55"/>
+      <c r="B78" s="48" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C76" s="66" t="str">
-        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
-        <v/>
-      </c>
-      <c r="D76" s="65"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="55"/>
-      <c r="B77" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C77" s="66" t="str">
-        <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
-        <v/>
-      </c>
-      <c r="D77" s="65"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="55"/>
-      <c r="B78" s="2" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рівень підготовки</v>
-      </c>
       <c r="C78" s="66" t="str">
-        <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
+        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
         <v/>
       </c>
       <c r="D78" s="65"/>
@@ -11967,35 +11951,35 @@
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="55"/>
       <c r="B79" s="48" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C79" s="66" t="str">
+        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
+        <v/>
+      </c>
+      <c r="D79" s="65"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="55"/>
+      <c r="B80" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C80" s="66" t="str">
+        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
+        <v/>
+      </c>
+      <c r="D80" s="65"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="55"/>
+      <c r="B81" s="48" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C79" s="66" t="str">
-        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
-        <v/>
-      </c>
-      <c r="D79" s="65"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="55"/>
-      <c r="B80" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C80" s="66" t="str">
-        <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
-        <v/>
-      </c>
-      <c r="D80" s="65"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="55"/>
-      <c r="B81" s="2" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рівень підготовки</v>
-      </c>
       <c r="C81" s="66" t="str">
-        <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
+        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
         <v/>
       </c>
       <c r="D81" s="65"/>
@@ -12003,35 +11987,35 @@
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="55"/>
       <c r="B82" s="48" t="str">
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
+      </c>
+      <c r="C82" s="66" t="str">
+        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
+        <v/>
+      </c>
+      <c r="D82" s="65"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="55"/>
+      <c r="B83" s="2" t="str">
+        <f aca="false">Освіта!$C$12</f>
+        <v>Рівень підготовки</v>
+      </c>
+      <c r="C83" s="66" t="str">
+        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
+        <v/>
+      </c>
+      <c r="D83" s="65"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="55"/>
+      <c r="B84" s="48" t="str">
         <f aca="false">Освіта!$A$12</f>
         <v>Назва освітнього, наукового  закладу</v>
       </c>
-      <c r="C82" s="66" t="str">
-        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
-        <v/>
-      </c>
-      <c r="D82" s="65"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="55"/>
-      <c r="B83" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C83" s="66" t="str">
-        <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
-        <v/>
-      </c>
-      <c r="D83" s="65"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="55"/>
-      <c r="B84" s="2" t="str">
-        <f aca="false">Освіта!$C$12</f>
-        <v>Рівень підготовки</v>
-      </c>
       <c r="C84" s="66" t="str">
-        <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
+        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
         <v/>
       </c>
       <c r="D84" s="65"/>
@@ -12039,73 +12023,73 @@
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="55"/>
       <c r="B85" s="48" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
+        <f aca="false">Освіта!$B$12</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C85" s="66" t="str">
-        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
+        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
         <v/>
       </c>
       <c r="D85" s="65"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="55"/>
-      <c r="B86" s="48" t="str">
-        <f aca="false">Освіта!$B$12</f>
-        <v>Рік закінчення</v>
-      </c>
-      <c r="C86" s="66" t="str">
-        <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
-        <v/>
-      </c>
-      <c r="D86" s="65"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="55"/>
-      <c r="B87" s="2" t="str">
+      <c r="B86" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C87" s="66" t="str">
+      <c r="C86" s="66" t="str">
         <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
-      <c r="D87" s="65"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="55" t="s">
+      <c r="D86" s="65"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="B88" s="48" t="str">
+      <c r="B87" s="48" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
+      <c r="C87" s="67" t="str">
+        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
+        <v/>
+      </c>
+      <c r="D87" s="65"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="55"/>
+      <c r="B88" s="48" t="str">
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
+      </c>
       <c r="C88" s="67" t="str">
-        <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
+        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
         <v/>
       </c>
       <c r="D88" s="65"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="55"/>
-      <c r="B89" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+      <c r="B89" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C89" s="67" t="str">
-        <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
+        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
         <v/>
       </c>
       <c r="D89" s="65"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="55"/>
-      <c r="B90" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B90" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C90" s="67" t="str">
-        <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
+        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
         <v/>
       </c>
       <c r="D90" s="65"/>
@@ -12113,11 +12097,11 @@
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="55"/>
       <c r="B91" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C91" s="67" t="str">
-        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
+        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
         <v/>
       </c>
       <c r="D91" s="65"/>
@@ -12125,11 +12109,11 @@
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="55"/>
       <c r="B92" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C92" s="67" t="str">
-        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
+        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
         <v/>
       </c>
       <c r="D92" s="65"/>
@@ -12137,35 +12121,35 @@
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="55"/>
       <c r="B93" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C93" s="67" t="str">
-        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
         <v/>
       </c>
       <c r="D93" s="65"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="55"/>
-      <c r="B94" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+      <c r="B94" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C94" s="67" t="str">
-        <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
+        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
         <v/>
       </c>
       <c r="D94" s="65"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="55"/>
-      <c r="B95" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B95" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C95" s="67" t="str">
-        <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
+        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
         <v/>
       </c>
       <c r="D95" s="65"/>
@@ -12173,11 +12157,11 @@
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="55"/>
       <c r="B96" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C96" s="67" t="str">
-        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
+        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
         <v/>
       </c>
       <c r="D96" s="65"/>
@@ -12185,11 +12169,11 @@
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="55"/>
       <c r="B97" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C97" s="67" t="str">
-        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
+        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
         <v/>
       </c>
       <c r="D97" s="65"/>
@@ -12197,35 +12181,35 @@
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="55"/>
       <c r="B98" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C98" s="67" t="str">
-        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
         <v/>
       </c>
       <c r="D98" s="65"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="55"/>
-      <c r="B99" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+      <c r="B99" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C99" s="67" t="str">
-        <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
+        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
         <v/>
       </c>
       <c r="D99" s="65"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="55"/>
-      <c r="B100" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B100" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C100" s="67" t="str">
-        <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
+        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
         <v/>
       </c>
       <c r="D100" s="65"/>
@@ -12233,11 +12217,11 @@
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="55"/>
       <c r="B101" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C101" s="67" t="str">
-        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
+        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
         <v/>
       </c>
       <c r="D101" s="65"/>
@@ -12245,11 +12229,11 @@
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="55"/>
       <c r="B102" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C102" s="67" t="str">
-        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
+        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
         <v/>
       </c>
       <c r="D102" s="65"/>
@@ -12257,35 +12241,35 @@
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="55"/>
       <c r="B103" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C103" s="67" t="str">
-        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
         <v/>
       </c>
       <c r="D103" s="65"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="55"/>
-      <c r="B104" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+      <c r="B104" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C104" s="67" t="str">
-        <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
+        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
         <v/>
       </c>
       <c r="D104" s="65"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="55"/>
-      <c r="B105" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B105" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C105" s="67" t="str">
-        <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
+        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
         <v/>
       </c>
       <c r="D105" s="65"/>
@@ -12293,11 +12277,11 @@
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="55"/>
       <c r="B106" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C106" s="67" t="str">
-        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
+        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
         <v/>
       </c>
       <c r="D106" s="65"/>
@@ -12305,11 +12289,11 @@
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="55"/>
       <c r="B107" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C107" s="67" t="str">
-        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
+        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
         <v/>
       </c>
       <c r="D107" s="65"/>
@@ -12317,35 +12301,35 @@
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="55"/>
       <c r="B108" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C108" s="67" t="str">
-        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
         <v/>
       </c>
       <c r="D108" s="65"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="55"/>
-      <c r="B109" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+      <c r="B109" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C109" s="67" t="str">
-        <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
+        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
         <v/>
       </c>
       <c r="D109" s="65"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="55"/>
-      <c r="B110" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B110" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C110" s="67" t="str">
-        <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
+        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
         <v/>
       </c>
       <c r="D110" s="65"/>
@@ -12353,11 +12337,11 @@
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="55"/>
       <c r="B111" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C111" s="67" t="str">
-        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
+        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
         <v/>
       </c>
       <c r="D111" s="65"/>
@@ -12365,11 +12349,11 @@
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="55"/>
       <c r="B112" s="48" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
       <c r="C112" s="67" t="str">
-        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
+        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
         <v/>
       </c>
       <c r="D112" s="65"/>
@@ -12377,35 +12361,35 @@
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="55"/>
       <c r="B113" s="48" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$B$4</f>
+        <v>Прізвище</v>
       </c>
       <c r="C113" s="67" t="str">
-        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
+        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
         <v/>
       </c>
       <c r="D113" s="65"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="55"/>
-      <c r="B114" s="48" t="str">
-        <f aca="false">Родина!$B$4</f>
-        <v>Прізвище</v>
+      <c r="B114" s="2" t="str">
+        <f aca="false">Родина!$C$4</f>
+        <v>Ім’я</v>
       </c>
       <c r="C114" s="67" t="str">
-        <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
+        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
         <v/>
       </c>
       <c r="D114" s="65"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="55"/>
-      <c r="B115" s="2" t="str">
-        <f aca="false">Родина!$C$4</f>
-        <v>Ім’я</v>
+      <c r="B115" s="48" t="str">
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C115" s="67" t="str">
-        <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
+        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
         <v/>
       </c>
       <c r="D115" s="65"/>
@@ -12413,37 +12397,37 @@
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="55"/>
       <c r="B116" s="48" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C116" s="67" t="str">
-        <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
-        <v/>
-      </c>
-      <c r="D116" s="65"/>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="55"/>
-      <c r="B117" s="48" t="str">
         <f aca="false">Родина!$E$4</f>
         <v>Рік народження</v>
       </c>
-      <c r="C117" s="67" t="str">
+      <c r="C116" s="67" t="str">
         <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
         <v/>
       </c>
-      <c r="D117" s="65"/>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="55" t="s">
+      <c r="D116" s="65"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="55" t="s">
         <v>160</v>
       </c>
-      <c r="B118" s="48" t="str">
+      <c r="B117" s="48" t="str">
         <f aca="false">Документи!A4</f>
         <v>Тип документу</v>
       </c>
-      <c r="C118" s="56" t="str">
+      <c r="C117" s="56" t="str">
         <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
+        <v/>
+      </c>
+      <c r="D117" s="48"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="55"/>
+      <c r="B118" s="48" t="str">
+        <f aca="false">Документи!A5</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C118" s="48" t="str">
+        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
         <v/>
       </c>
       <c r="D118" s="48"/>
@@ -12451,11 +12435,11 @@
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="55"/>
       <c r="B119" s="48" t="str">
-        <f aca="false">Документи!A5</f>
-        <v>Серія та номер </v>
+        <f aca="false">Документи!A6</f>
+        <v>Ким виданий</v>
       </c>
       <c r="C119" s="48" t="str">
-        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
+        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
         <v/>
       </c>
       <c r="D119" s="48"/>
@@ -12463,11 +12447,11 @@
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="55"/>
       <c r="B120" s="48" t="str">
-        <f aca="false">Документи!A6</f>
-        <v>Ким виданий</v>
+        <f aca="false">Документи!A7</f>
+        <v>Дата видачі</v>
       </c>
       <c r="C120" s="48" t="str">
-        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
+        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
         <v/>
       </c>
       <c r="D120" s="48"/>
@@ -12475,11 +12459,11 @@
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="55"/>
       <c r="B121" s="48" t="str">
-        <f aca="false">Документи!A7</f>
-        <v>Дата видачі</v>
-      </c>
-      <c r="C121" s="48" t="str">
-        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
+        <f aca="false">Документи!A10</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C121" s="56" t="str">
+        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
         <v/>
       </c>
       <c r="D121" s="48"/>
@@ -12487,11 +12471,11 @@
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="55"/>
       <c r="B122" s="48" t="str">
-        <f aca="false">Документи!A10</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C122" s="56" t="str">
-        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
+        <f aca="false">Документи!A11</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C122" s="48" t="str">
+        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
         <v/>
       </c>
       <c r="D122" s="48"/>
@@ -12499,11 +12483,11 @@
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="55"/>
       <c r="B123" s="48" t="str">
-        <f aca="false">Документи!A11</f>
-        <v>Серія та номер </v>
+        <f aca="false">Документи!A12</f>
+        <v>Ким виданий</v>
       </c>
       <c r="C123" s="48" t="str">
-        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
+        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
         <v/>
       </c>
       <c r="D123" s="48"/>
@@ -12511,34 +12495,34 @@
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="55"/>
       <c r="B124" s="48" t="str">
-        <f aca="false">Документи!A12</f>
-        <v>Ким виданий</v>
+        <f aca="false">Документи!A13</f>
+        <v>Дата видачі</v>
       </c>
       <c r="C124" s="48" t="str">
-        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
+        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
         <v/>
       </c>
       <c r="D124" s="48"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="55"/>
-      <c r="B125" s="48" t="str">
-        <f aca="false">Документи!A13</f>
-        <v>Дата видачі</v>
+      <c r="B125" s="48" t="s">
+        <v>161</v>
       </c>
       <c r="C125" s="48" t="str">
-        <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
+        <f aca="false">IF(D125 = 0, "", D125)</f>
         <v/>
       </c>
       <c r="D125" s="48"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="55"/>
-      <c r="B126" s="48" t="s">
-        <v>161</v>
-      </c>
-      <c r="C126" s="48" t="str">
-        <f aca="false">IF(D126 = 0, "", D126)</f>
+      <c r="B126" s="48" t="str">
+        <f aca="false">Документи!A16</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C126" s="56" t="str">
+        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
         <v/>
       </c>
       <c r="D126" s="48"/>
@@ -12546,11 +12530,11 @@
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="55"/>
       <c r="B127" s="48" t="str">
-        <f aca="false">Документи!A16</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C127" s="56" t="str">
-        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
+        <f aca="false">Документи!A17</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C127" s="48" t="str">
+        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
         <v/>
       </c>
       <c r="D127" s="48"/>
@@ -12558,26 +12542,20 @@
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="55"/>
       <c r="B128" s="48" t="str">
-        <f aca="false">Документи!A17</f>
-        <v>Ким виданий</v>
-      </c>
-      <c r="C128" s="48" t="str">
-        <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
-        <v/>
-      </c>
-      <c r="D128" s="48"/>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="55"/>
-      <c r="B129" s="48" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C129" s="48" t="str">
+      <c r="C128" s="48" t="str">
         <f aca="false">IF(Документи!B18 = 0, "", Документи!B18)</f>
         <v/>
       </c>
-      <c r="D129" s="48"/>
+      <c r="D128" s="48"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="0"/>
+      <c r="B129" s="0"/>
+      <c r="C129" s="0"/>
+      <c r="D129" s="0"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2"/>
@@ -12586,26 +12564,26 @@
   <mergeCells count="11">
     <mergeCell ref="G1:N1"/>
     <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="A2:A24"/>
+    <mergeCell ref="A2:A23"/>
     <mergeCell ref="O2:O16"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="O17:O28"/>
-    <mergeCell ref="A25:A37"/>
-    <mergeCell ref="A38:A87"/>
-    <mergeCell ref="A88:A117"/>
-    <mergeCell ref="A118:A129"/>
+    <mergeCell ref="A24:A36"/>
+    <mergeCell ref="A37:A86"/>
+    <mergeCell ref="A87:A116"/>
+    <mergeCell ref="A117:A128"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:K21" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D38:D42" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D37:D41" type="list">
       <formula1>'Системна інформація'!$Q$27:$ZA$27</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D44" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D43" type="list">
       <formula1>'Системна інформація'!$Q$11:$ZA$11</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat: new VIN field in MilitaryPerson
</commit_message>
<xml_diff>
--- a/docs/templates/update_form_p2.xlsx
+++ b/docs/templates/update_form_p2.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="164">
   <si>
     <t xml:space="preserve">Найменування підприємства (установи, організації)</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t xml:space="preserve">Список на основі БД (Voenkomat) із додаванням</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВІН</t>
   </si>
   <si>
     <t xml:space="preserve">АДРЕСИ ТА КОНТАКТИ</t>
@@ -521,10 +524,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -949,7 +951,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -965,7 +967,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1201,7 +1203,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:D35"/>
+  <dimension ref="A2:D36"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.37"/>
@@ -1368,6 +1370,10 @@
         <v>19</v>
       </c>
       <c r="B19" s="13"/>
+      <c r="C19" s="2" t="str">
+        <f aca="false">IF('Системна інформація'!D12 = 0, "", 'Системна інформація'!D12)</f>
+        <v/>
+      </c>
       <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1545,8 +1551,18 @@
         <v>42</v>
       </c>
     </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="12"/>
+      <c r="C36" s="2" t="str">
+        <f aca="false">IF('Системна інформація'!D25 = 0, "", 'Системна інформація'!D25)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="16">
+  <dataValidations count="17">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B14" type="list">
       <formula1>'Системна інформація'!$Q$2:$ZA$2</formula1>
       <formula2>0</formula2>
@@ -1611,6 +1627,10 @@
       <formula1>'Системна інформація'!$Q$4:$ZA$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="false" error="Перевірте наявність свого ТЦК в списку. У випадку його відсутності - введіть назву в це поле і натисніть ОК" errorStyle="warning" errorTitle="Такого ТЦК наразі не існує" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B36" type="none">
+      <formula1>'Системна інформація'!$Q$24:$ZA$24</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1638,12 +1658,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="19"/>
@@ -1651,105 +1671,102 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" s="21"/>
       <c r="C4" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D25 = 0, "", 'Системна інформація'!D25)</f>
+        <f aca="false">IF('Системна інформація'!D26 = 0, "", 'Системна інформація'!D26)</f>
         <v/>
       </c>
       <c r="D4" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="24"/>
       <c r="C5" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D26 = 0, "", 'Системна інформація'!D26)</f>
+        <f aca="false">IF('Системна інформація'!D27 = 0, "", 'Системна інформація'!D27)</f>
         <v/>
       </c>
       <c r="D5" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D27 = 0, "", 'Системна інформація'!D27)</f>
+        <f aca="false">IF('Системна інформація'!D28 = 0, "", 'Системна інформація'!D28)</f>
         <v/>
       </c>
       <c r="D6" s="17" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" s="22" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D28 = 0, "", 'Системна інформація'!D28)</f>
-        <v/>
-      </c>
-      <c r="D7" s="17"/>
-    </row>
-    <row r="8" s="22" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">IF('Системна інформація'!D29 = 0, "", 'Системна інформація'!D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="24"/>
       <c r="C8" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D29 = 0, "", 'Системна інформація'!D29)</f>
+        <f aca="false">IF('Системна інформація'!D30 = 0, "", 'Системна інформація'!D30)</f>
         <v/>
       </c>
       <c r="D8" s="17" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" s="22" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26"/>
       <c r="B9" s="27"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="17"/>
-    </row>
-    <row r="10" s="22" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B10" s="28"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11" s="24"/>
       <c r="C11" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D30 = 0, "", 'Системна інформація'!D30)</f>
+        <f aca="false">IF('Системна інформація'!D31 = 0, "", 'Системна інформація'!D31)</f>
         <v/>
       </c>
       <c r="D11" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B12" s="24"/>
       <c r="C12" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D31 = 0, "", 'Системна інформація'!D31)</f>
+        <f aca="false">IF('Системна інформація'!D32 = 0, "", 'Системна інформація'!D32)</f>
         <v/>
       </c>
       <c r="D12" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1758,7 +1775,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="29"/>
       <c r="C14" s="2"/>
@@ -1766,11 +1783,11 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D32 = 0, "", 'Системна інформація'!D32)</f>
+        <f aca="false">IF('Системна інформація'!D33 = 0, "", 'Системна інформація'!D33)</f>
         <v/>
       </c>
       <c r="D15" s="19" t="s">
@@ -1785,37 +1802,37 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D33 = 0, "", 'Системна інформація'!D33)</f>
+        <f aca="false">IF('Системна інформація'!D34 = 0, "", 'Системна інформація'!D34)</f>
         <v/>
       </c>
       <c r="D17" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D34 = 0, "", 'Системна інформація'!D34)</f>
+        <f aca="false">IF('Системна інформація'!D35 = 0, "", 'Системна інформація'!D35)</f>
         <v/>
       </c>
       <c r="D18" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="24"/>
       <c r="C19" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D35 = 0, "", 'Системна інформація'!D35)</f>
+        <f aca="false">IF('Системна інформація'!D36 = 0, "", 'Системна інформація'!D36)</f>
         <v/>
       </c>
       <c r="D19" s="17" t="s">
@@ -1824,25 +1841,25 @@
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B20" s="24"/>
       <c r="C20" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D36 = 0, "", 'Системна інформація'!D36)</f>
+        <f aca="false">IF('Системна інформація'!D37 = 0, "", 'Системна інформація'!D37)</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="24"/>
       <c r="C21" s="19" t="str">
-        <f aca="false">IF('Системна інформація'!D37 = 0, "", 'Системна інформація'!D37)</f>
+        <f aca="false">IF('Системна інформація'!D38 = 0, "", 'Системна інформація'!D38)</f>
         <v/>
       </c>
       <c r="D21" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,7 +1915,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -1918,7 +1935,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B3" s="33"/>
       <c r="C3" s="31"/>
@@ -1929,28 +1946,28 @@
     </row>
     <row r="4" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E4" s="34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H4" s="35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1997,7 +2014,7 @@
       <c r="A9" s="31"/>
       <c r="B9" s="31"/>
       <c r="D9" s="38" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E9" s="31"/>
       <c r="F9" s="31"/>
@@ -2019,7 +2036,7 @@
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="31"/>
       <c r="C11" s="31"/>
@@ -2030,13 +2047,13 @@
     </row>
     <row r="12" customFormat="false" ht="37.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2072,7 +2089,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="31"/>
       <c r="B19" s="38" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>12</v>
@@ -2127,21 +2144,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="40" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="41" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
       <c r="D3" s="41"/>
       <c r="E3" s="41"/>
     </row>
-    <row r="4" customFormat="false" ht="28.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>5</v>
@@ -2150,10 +2167,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,7 +2220,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2240,21 +2257,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="44" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D118 = 0, "", 'Системна інформація'!D118)</f>
+        <f aca="false">IF('Системна інформація'!D119 = 0, "", 'Системна інформація'!D119)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="s">
@@ -2263,37 +2280,37 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="45" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D119 = 0, "", 'Системна інформація'!D119)</f>
+        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
         <v/>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D120 = 0, "", 'Системна інформація'!D120)</f>
+        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
         <v/>
       </c>
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="45" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D121 = 0, "", 'Системна інформація'!D121)</f>
+        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
         <v/>
       </c>
       <c r="D7" s="2" t="s">
@@ -2305,17 +2322,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B9" s="31"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="44" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D122 = 0, "", 'Системна інформація'!D122)</f>
+        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="s">
@@ -2324,34 +2341,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="45" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D123 = 0, "", 'Системна інформація'!D123)</f>
+        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
         <v/>
       </c>
       <c r="D11" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D124 = 0, "", 'Системна інформація'!D124)</f>
+        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="45" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D125 = 0, "", 'Системна інформація'!D125)</f>
+        <f aca="false">IF('Системна інформація'!D126 = 0, "", 'Системна інформація'!D126)</f>
         <v/>
       </c>
       <c r="D13" s="2" t="s">
@@ -2363,43 +2380,43 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="40" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B15" s="31"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="45" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D127 = 0, "", 'Системна інформація'!D127)</f>
+        <f aca="false">IF('Системна інформація'!D128 = 0, "", 'Системна інформація'!D128)</f>
         <v/>
       </c>
       <c r="D16" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D128 = 0, "", 'Системна інформація'!D128)</f>
+        <f aca="false">IF('Системна інформація'!D129 = 0, "", 'Системна інформація'!D129)</f>
         <v/>
       </c>
       <c r="D17" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="45" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="2" t="str">
-        <f aca="false">IF('Системна інформація'!D129 = 0, "", 'Системна інформація'!D129)</f>
+        <f aca="false">IF('Системна інформація'!D130 = 0, "", 'Системна інформація'!D130)</f>
         <v/>
       </c>
       <c r="D18" s="2" t="s">
@@ -2445,20 +2462,20 @@
   <sheetData>
     <row r="1" s="48" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="47" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" s="48" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C1" s="48" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D1" s="48" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="49" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H1" s="49"/>
       <c r="I1" s="49"/>
@@ -2468,13 +2485,13 @@
       <c r="M1" s="49"/>
       <c r="N1" s="49"/>
       <c r="O1" s="50" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P1" s="51" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q1" s="50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="R1" s="50"/>
       <c r="S1" s="50"/>
@@ -2482,7 +2499,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="52" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B2" s="45" t="str">
         <f aca="false">Основна!A9</f>
@@ -2494,60 +2511,60 @@
       </c>
       <c r="D2" s="54"/>
       <c r="G2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="H2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="I2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="J2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="K2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="L2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="M2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="N2" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G2)),0)</f>
         <v>0</v>
       </c>
       <c r="O2" s="56" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="P2" s="9" t="s">
         <v>11</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2562,35 +2579,35 @@
       </c>
       <c r="D3" s="54"/>
       <c r="G3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="H3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="I3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="J3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="K3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="L3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="M3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="N3" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G3)),0)</f>
         <v>0</v>
       </c>
       <c r="O3" s="56"/>
@@ -2598,10 +2615,10 @@
         <v>13</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2616,35 +2633,35 @@
       </c>
       <c r="D4" s="54"/>
       <c r="G4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="H4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="I4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="J4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="K4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="L4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="M4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="N4" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G4)),0)</f>
         <v>0</v>
       </c>
       <c r="O4" s="56"/>
@@ -2652,28 +2669,28 @@
         <v>18</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2688,35 +2705,35 @@
       </c>
       <c r="D5" s="54"/>
       <c r="G5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(G$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(H$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="I5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(I$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(J$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="K5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(K$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="L5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(L$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="M5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(M$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="N5" s="55" t="n">
-        <f aca="true">OFFSET($D$38,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
+        <f aca="true">OFFSET($D$39,(ROW()-ROW(N$2))*8+(COLUMN()-COLUMN($G5)),0)</f>
         <v>0</v>
       </c>
       <c r="O5" s="56"/>
@@ -2724,10 +2741,10 @@
         <v>31</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2771,7 +2788,7 @@
       </c>
       <c r="D7" s="54"/>
       <c r="G7" s="57" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H7" s="57"/>
       <c r="I7" s="57"/>
@@ -2780,13 +2797,13 @@
         <v>39</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2801,23 +2818,23 @@
       </c>
       <c r="D8" s="54"/>
       <c r="G8" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="I8" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G8)),0)</f>
         <v>0</v>
       </c>
       <c r="O8" s="56"/>
       <c r="P8" s="58" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2832,26 +2849,26 @@
       </c>
       <c r="D9" s="54"/>
       <c r="G9" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="I9" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G9)),0)</f>
         <v>0</v>
       </c>
       <c r="O9" s="56"/>
       <c r="P9" s="30" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2866,29 +2883,29 @@
       </c>
       <c r="D10" s="54"/>
       <c r="G10" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="H10" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="I10" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G10)),0)</f>
         <v>0</v>
       </c>
       <c r="O10" s="56"/>
       <c r="P10" s="58" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2903,29 +2920,29 @@
       </c>
       <c r="D11" s="54"/>
       <c r="G11" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="H11" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="I11" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G11)),0)</f>
         <v>0</v>
       </c>
       <c r="O11" s="56"/>
       <c r="P11" s="58" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2940,35 +2957,35 @@
       </c>
       <c r="D12" s="54"/>
       <c r="G12" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="I12" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G12)),0)</f>
         <v>0</v>
       </c>
       <c r="O12" s="56"/>
       <c r="P12" s="58" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2983,29 +3000,29 @@
       </c>
       <c r="D13" s="54"/>
       <c r="G13" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(G$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="H13" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(H$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="I13" s="59" t="n">
-        <f aca="true">OFFSET($D$70,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
+        <f aca="true">OFFSET($D$71,(ROW()-ROW(I$8))*3+(COLUMN()-COLUMN($G13)),0)</f>
         <v>0</v>
       </c>
       <c r="O13" s="56"/>
       <c r="P13" s="58" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3028,25 +3045,25 @@
       <c r="M14" s="2"/>
       <c r="O14" s="56"/>
       <c r="P14" s="58" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="U14" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3061,7 +3078,7 @@
       </c>
       <c r="D15" s="54"/>
       <c r="G15" s="57" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H15" s="57"/>
       <c r="I15" s="57"/>
@@ -3071,13 +3088,13 @@
       <c r="M15" s="2"/>
       <c r="O15" s="56"/>
       <c r="P15" s="60" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="Q15" s="61" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="R15" s="61" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3092,36 +3109,36 @@
       </c>
       <c r="D16" s="54"/>
       <c r="G16" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="H16" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="I16" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="J16" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="K16" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G16)),0)</f>
         <v>0</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="O16" s="56"/>
       <c r="P16" s="60" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Q16" s="61" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="R16" s="61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3136,29 +3153,29 @@
       </c>
       <c r="D17" s="54"/>
       <c r="G17" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="H17" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="I17" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="K17" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G17)),0)</f>
         <v>0</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="O17" s="56" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>14</v>
@@ -3837,23 +3854,23 @@
       </c>
       <c r="D18" s="54"/>
       <c r="G18" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="H18" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="I18" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="J18" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="K18" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G18)),0)</f>
         <v>0</v>
       </c>
       <c r="L18" s="2"/>
@@ -4536,23 +4553,23 @@
       </c>
       <c r="D19" s="54"/>
       <c r="G19" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="H19" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="I19" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="J19" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="K19" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G19)),0)</f>
         <v>0</v>
       </c>
       <c r="L19" s="2"/>
@@ -5235,23 +5252,23 @@
       </c>
       <c r="D20" s="54"/>
       <c r="G20" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="H20" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="I20" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="J20" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="K20" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G20)),0)</f>
         <v>0</v>
       </c>
       <c r="L20" s="2"/>
@@ -5934,23 +5951,23 @@
       </c>
       <c r="D21" s="54"/>
       <c r="G21" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(G$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="H21" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(H$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="I21" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(I$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(J$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="K21" s="59" t="n">
-        <f aca="true">OFFSET($D$88,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
+        <f aca="true">OFFSET($D$89,(ROW()-ROW(K$16))*5+(COLUMN()-COLUMN($G21)),0)</f>
         <v>0</v>
       </c>
       <c r="L21" s="2"/>
@@ -7976,9 +7993,7 @@
       <c r="ZA23" s="62"/>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="52" t="s">
-        <v>156</v>
-      </c>
+      <c r="A24" s="52"/>
       <c r="B24" s="45" t="str">
         <f aca="false">Основна!A35</f>
         <v>Териториальний центр комплектування та соціальної підтримки</v>
@@ -8657,17 +8672,17 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="52"/>
       <c r="B25" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A4</f>
-        <v>Країна</v>
+        <f aca="false">Основна!A36</f>
+        <v>ВІН</v>
       </c>
       <c r="C25" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B4 = 0, "", 'Адреси Контакти'!B4)</f>
+        <f aca="false">IF(Основна!B36 = 0, "",  Основна!B36)</f>
         <v/>
       </c>
       <c r="D25" s="54"/>
       <c r="O25" s="56"/>
       <c r="P25" s="30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q25" s="62"/>
       <c r="R25" s="62"/>
@@ -9332,19 +9347,21 @@
       <c r="ZA25" s="62"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="52"/>
+      <c r="A26" s="52" t="s">
+        <v>157</v>
+      </c>
       <c r="B26" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A5</f>
-        <v>Область (України)</v>
+        <f aca="false">'Адреси Контакти'!A4</f>
+        <v>Країна</v>
       </c>
       <c r="C26" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B5 = 0, "", 'Адреси Контакти'!B5)</f>
+        <f aca="false">IF('Адреси Контакти'!B4 = 0, "", 'Адреси Контакти'!B4)</f>
         <v/>
       </c>
       <c r="D26" s="54"/>
       <c r="O26" s="56"/>
       <c r="P26" s="25" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Q26" s="62"/>
       <c r="R26" s="62"/>
@@ -10011,17 +10028,17 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="52"/>
       <c r="B27" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A6</f>
-        <v>Місто</v>
+        <f aca="false">'Адреси Контакти'!A5</f>
+        <v>Область (України)</v>
       </c>
       <c r="C27" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B6 = 0, "", 'Адреси Контакти'!B6)</f>
+        <f aca="false">IF('Адреси Контакти'!B5 = 0, "", 'Адреси Контакти'!B5)</f>
         <v/>
       </c>
       <c r="D27" s="54"/>
       <c r="O27" s="56"/>
       <c r="P27" s="25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q27" s="62"/>
       <c r="R27" s="62"/>
@@ -10688,17 +10705,17 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="52"/>
       <c r="B28" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A7</f>
-        <v>Адреса (вулиця, № будинку, квартири)</v>
+        <f aca="false">'Адреси Контакти'!A6</f>
+        <v>Місто</v>
       </c>
       <c r="C28" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B7 = 0, "", 'Адреси Контакти'!B7)</f>
+        <f aca="false">IF('Адреси Контакти'!B6 = 0, "", 'Адреси Контакти'!B6)</f>
         <v/>
       </c>
       <c r="D28" s="54"/>
       <c r="O28" s="56"/>
       <c r="P28" s="58" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q28" s="62"/>
       <c r="R28" s="62"/>
@@ -11365,11 +11382,11 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="52"/>
       <c r="B29" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A8</f>
-        <v>Індекс</v>
+        <f aca="false">'Адреси Контакти'!A7</f>
+        <v>Адреса (вулиця, № будинку, квартири)</v>
       </c>
       <c r="C29" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B8 = 0, "", 'Адреси Контакти'!B8)</f>
+        <f aca="false">IF('Адреси Контакти'!B7 = 0, "", 'Адреси Контакти'!B7)</f>
         <v/>
       </c>
       <c r="D29" s="54"/>
@@ -11377,11 +11394,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="52"/>
       <c r="B30" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A11</f>
-        <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
+        <f aca="false">'Адреси Контакти'!A8</f>
+        <v>Індекс</v>
       </c>
       <c r="C30" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B11 = 0, "", 'Адреси Контакти'!B11)</f>
+        <f aca="false">IF('Адреси Контакти'!B8 = 0, "", 'Адреси Контакти'!B8)</f>
         <v/>
       </c>
       <c r="D30" s="54"/>
@@ -11389,11 +11406,11 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="52"/>
       <c r="B31" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A12</f>
-        <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
+        <f aca="false">'Адреси Контакти'!A11</f>
+        <v>КОНТАКТНИЙ ТЕЛЕФОН (основний)</v>
       </c>
       <c r="C31" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B12 = 0, "", 'Адреси Контакти'!B12)</f>
+        <f aca="false">IF('Адреси Контакти'!B11 = 0, "", 'Адреси Контакти'!B11)</f>
         <v/>
       </c>
       <c r="D31" s="54"/>
@@ -11401,11 +11418,11 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="52"/>
       <c r="B32" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A15</f>
-        <v>Співпадає із адресою фактичного проживання</v>
+        <f aca="false">'Адреси Контакти'!A12</f>
+        <v>КОНТАКТНИЙ ТЕЛЕФОН (додатковий)</v>
       </c>
       <c r="C32" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B15 = 0, "", 'Адреси Контакти'!B15)</f>
+        <f aca="false">IF('Адреси Контакти'!B12 = 0, "", 'Адреси Контакти'!B12)</f>
         <v/>
       </c>
       <c r="D32" s="54"/>
@@ -11413,11 +11430,11 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="52"/>
       <c r="B33" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A17</f>
-        <v>Країна</v>
+        <f aca="false">'Адреси Контакти'!A15</f>
+        <v>Співпадає із адресою фактичного проживання</v>
       </c>
       <c r="C33" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B17 = 0, "", 'Адреси Контакти'!B17)</f>
+        <f aca="false">IF('Адреси Контакти'!B15 = 0, "", 'Адреси Контакти'!B15)</f>
         <v/>
       </c>
       <c r="D33" s="54"/>
@@ -11425,11 +11442,11 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="52"/>
       <c r="B34" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A18</f>
-        <v>Область (України)</v>
+        <f aca="false">'Адреси Контакти'!A17</f>
+        <v>Країна</v>
       </c>
       <c r="C34" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B18 = 0, "", 'Адреси Контакти'!B18)</f>
+        <f aca="false">IF('Адреси Контакти'!B17 = 0, "", 'Адреси Контакти'!B17)</f>
         <v/>
       </c>
       <c r="D34" s="54"/>
@@ -11437,11 +11454,11 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="52"/>
       <c r="B35" s="45" t="str">
-        <f aca="false">'Адреси Контакти'!A19</f>
-        <v>Місто</v>
+        <f aca="false">'Адреси Контакти'!A18</f>
+        <v>Область (України)</v>
       </c>
       <c r="C35" s="54" t="str">
-        <f aca="false">IF('Адреси Контакти'!B19 = 0, "", 'Адреси Контакти'!B19)</f>
+        <f aca="false">IF('Адреси Контакти'!B18 = 0, "", 'Адреси Контакти'!B18)</f>
         <v/>
       </c>
       <c r="D35" s="54"/>
@@ -11449,49 +11466,49 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="52"/>
       <c r="B36" s="45" t="str">
+        <f aca="false">'Адреси Контакти'!A19</f>
+        <v>Місто</v>
+      </c>
+      <c r="C36" s="54" t="str">
+        <f aca="false">IF('Адреси Контакти'!B19 = 0, "", 'Адреси Контакти'!B19)</f>
+        <v/>
+      </c>
+      <c r="D36" s="54"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="52"/>
+      <c r="B37" s="45" t="str">
         <f aca="false">'Адреси Контакти'!A20</f>
         <v>Адреса (вулиця, № будинку, квартири)</v>
       </c>
-      <c r="C36" s="54" t="str">
+      <c r="C37" s="54" t="str">
         <f aca="false">IF('Адреси Контакти'!B20 = 0, "", 'Адреси Контакти'!B20)</f>
         <v/>
       </c>
-      <c r="D36" s="54"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="52" t="s">
-        <v>159</v>
-      </c>
-      <c r="B37" s="45" t="str">
+      <c r="D37" s="54"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="52" t="s">
+        <v>160</v>
+      </c>
+      <c r="B38" s="45" t="str">
         <f aca="false">'Адреси Контакти'!A21</f>
         <v>Індекс</v>
       </c>
-      <c r="C37" s="54" t="str">
+      <c r="C38" s="54" t="str">
         <f aca="false">IF('Адреси Контакти'!B21 = 0, "", 'Адреси Контакти'!B21)</f>
         <v/>
       </c>
-      <c r="D37" s="54"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="52"/>
-      <c r="B38" s="45" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
-      </c>
-      <c r="C38" s="63" t="str">
-        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
-        <v/>
-      </c>
-      <c r="D38" s="64"/>
+      <c r="D38" s="54"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="52"/>
       <c r="B39" s="45" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C39" s="63" t="str">
-        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
+        <f aca="false">IF(Освіта!A5 = 0, "", Освіта!A5)</f>
         <v/>
       </c>
       <c r="D39" s="64"/>
@@ -11499,11 +11516,11 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="52"/>
       <c r="B40" s="45" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C40" s="63" t="str">
-        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
+        <f aca="false">IF(Освіта!B5 = 0, "", Освіта!B5)</f>
         <v/>
       </c>
       <c r="D40" s="64"/>
@@ -11511,11 +11528,11 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="52"/>
       <c r="B41" s="45" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C41" s="63" t="str">
-        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
+        <f aca="false">IF(Освіта!C5 = 0, "", Освіта!C5)</f>
         <v/>
       </c>
       <c r="D41" s="64"/>
@@ -11523,11 +11540,11 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="52"/>
       <c r="B42" s="45" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C42" s="63" t="str">
-        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
+        <f aca="false">IF(Освіта!D5 = 0, "", Освіта!D5)</f>
         <v/>
       </c>
       <c r="D42" s="64"/>
@@ -11535,11 +11552,11 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="52"/>
       <c r="B43" s="45" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C43" s="63" t="str">
-        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
+        <f aca="false">IF(Освіта!E5 = 0, "", Освіта!E5)</f>
         <v/>
       </c>
       <c r="D43" s="64"/>
@@ -11547,11 +11564,11 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="52"/>
       <c r="B44" s="45" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C44" s="63" t="str">
-        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
+        <f aca="false">IF(Освіта!F5 = 0, "", Освіта!F5)</f>
         <v/>
       </c>
       <c r="D44" s="64"/>
@@ -11559,11 +11576,11 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="52"/>
       <c r="B45" s="45" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C45" s="63" t="str">
-        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
+        <f aca="false">IF(Освіта!G5 = 0, "", Освіта!G5)</f>
         <v/>
       </c>
       <c r="D45" s="64"/>
@@ -11571,11 +11588,11 @@
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="52"/>
       <c r="B46" s="45" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C46" s="63" t="str">
-        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
+        <f aca="false">IF(Освіта!H5 = 0, "", Освіта!H5)</f>
         <v/>
       </c>
       <c r="D46" s="64"/>
@@ -11583,11 +11600,11 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="52"/>
       <c r="B47" s="45" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C47" s="63" t="str">
-        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
+        <f aca="false">IF(Освіта!A6 = 0, "", Освіта!A6)</f>
         <v/>
       </c>
       <c r="D47" s="64"/>
@@ -11595,11 +11612,11 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="52"/>
       <c r="B48" s="45" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C48" s="63" t="str">
-        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
+        <f aca="false">IF(Освіта!B6 = 0, "", Освіта!B6)</f>
         <v/>
       </c>
       <c r="D48" s="64"/>
@@ -11607,11 +11624,11 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="52"/>
       <c r="B49" s="45" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C49" s="63" t="str">
-        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
+        <f aca="false">IF(Освіта!C6 = 0, "", Освіта!C6)</f>
         <v/>
       </c>
       <c r="D49" s="64"/>
@@ -11619,11 +11636,11 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="52"/>
       <c r="B50" s="45" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C50" s="63" t="str">
-        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
+        <f aca="false">IF(Освіта!D6 = 0, "", Освіта!D6)</f>
         <v/>
       </c>
       <c r="D50" s="64"/>
@@ -11631,11 +11648,11 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="52"/>
       <c r="B51" s="45" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C51" s="63" t="str">
-        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
+        <f aca="false">IF(Освіта!E6 = 0, "", Освіта!E6)</f>
         <v/>
       </c>
       <c r="D51" s="64"/>
@@ -11643,11 +11660,11 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="52"/>
       <c r="B52" s="45" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C52" s="63" t="str">
-        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
+        <f aca="false">IF(Освіта!F6 = 0, "", Освіта!F6)</f>
         <v/>
       </c>
       <c r="D52" s="64"/>
@@ -11655,11 +11672,11 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="52"/>
       <c r="B53" s="45" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C53" s="63" t="str">
-        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
+        <f aca="false">IF(Освіта!G6 = 0, "", Освіта!G6)</f>
         <v/>
       </c>
       <c r="D53" s="64"/>
@@ -11667,11 +11684,11 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="52"/>
       <c r="B54" s="45" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C54" s="63" t="str">
-        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
+        <f aca="false">IF(Освіта!H6 = 0, "", Освіта!H6)</f>
         <v/>
       </c>
       <c r="D54" s="64"/>
@@ -11679,11 +11696,11 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="52"/>
       <c r="B55" s="45" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C55" s="63" t="str">
-        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
+        <f aca="false">IF(Освіта!A7 = 0, "", Освіта!A7)</f>
         <v/>
       </c>
       <c r="D55" s="64"/>
@@ -11691,11 +11708,11 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="52"/>
       <c r="B56" s="45" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C56" s="63" t="str">
-        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
+        <f aca="false">IF(Освіта!B7 = 0, "", Освіта!B7)</f>
         <v/>
       </c>
       <c r="D56" s="64"/>
@@ -11703,11 +11720,11 @@
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="52"/>
       <c r="B57" s="45" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C57" s="63" t="str">
-        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
+        <f aca="false">IF(Освіта!C7 = 0, "", Освіта!C7)</f>
         <v/>
       </c>
       <c r="D57" s="64"/>
@@ -11715,11 +11732,11 @@
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="52"/>
       <c r="B58" s="45" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C58" s="63" t="str">
-        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
+        <f aca="false">IF(Освіта!D7 = 0, "", Освіта!D7)</f>
         <v/>
       </c>
       <c r="D58" s="64"/>
@@ -11727,11 +11744,11 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="52"/>
       <c r="B59" s="45" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C59" s="63" t="str">
-        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
+        <f aca="false">IF(Освіта!E7 = 0, "", Освіта!E7)</f>
         <v/>
       </c>
       <c r="D59" s="64"/>
@@ -11739,11 +11756,11 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="52"/>
       <c r="B60" s="45" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C60" s="63" t="str">
-        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
+        <f aca="false">IF(Освіта!F7 = 0, "", Освіта!F7)</f>
         <v/>
       </c>
       <c r="D60" s="64"/>
@@ -11751,11 +11768,11 @@
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="52"/>
       <c r="B61" s="45" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C61" s="63" t="str">
-        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
+        <f aca="false">IF(Освіта!G7 = 0, "", Освіта!G7)</f>
         <v/>
       </c>
       <c r="D61" s="64"/>
@@ -11763,11 +11780,11 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="52"/>
       <c r="B62" s="45" t="str">
-        <f aca="false">Освіта!$A$4</f>
-        <v>Назва освітнього закладу</v>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
       </c>
       <c r="C62" s="63" t="str">
-        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
+        <f aca="false">IF(Освіта!H7 = 0, "", Освіта!H7)</f>
         <v/>
       </c>
       <c r="D62" s="64"/>
@@ -11775,11 +11792,11 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="52"/>
       <c r="B63" s="45" t="str">
-        <f aca="false">Освіта!$B$4</f>
-        <v>Серія дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$A$4</f>
+        <v>Назва освітнього закладу</v>
       </c>
       <c r="C63" s="63" t="str">
-        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
+        <f aca="false">IF(Освіта!A8 = 0, "", Освіта!A8)</f>
         <v/>
       </c>
       <c r="D63" s="64"/>
@@ -11787,11 +11804,11 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="52"/>
       <c r="B64" s="45" t="str">
-        <f aca="false">Освіта!$C$4</f>
-        <v>Номер дисплома (свідоцтва)</v>
+        <f aca="false">Освіта!$B$4</f>
+        <v>Серія дисплома (свідоцтва)</v>
       </c>
       <c r="C64" s="63" t="str">
-        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
+        <f aca="false">IF(Освіта!B8 = 0, "", Освіта!B8)</f>
         <v/>
       </c>
       <c r="D64" s="64"/>
@@ -11799,11 +11816,11 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="52"/>
       <c r="B65" s="45" t="str">
-        <f aca="false">Освіта!$D$4</f>
-        <v>Рік закінчення</v>
+        <f aca="false">Освіта!$C$4</f>
+        <v>Номер дисплома (свідоцтва)</v>
       </c>
       <c r="C65" s="63" t="str">
-        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
+        <f aca="false">IF(Освіта!C8 = 0, "", Освіта!C8)</f>
         <v/>
       </c>
       <c r="D65" s="64"/>
@@ -11811,11 +11828,11 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="52"/>
       <c r="B66" s="45" t="str">
-        <f aca="false">Освіта!$E$4</f>
-        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
+        <f aca="false">Освіта!$D$4</f>
+        <v>Рік закінчення</v>
       </c>
       <c r="C66" s="63" t="str">
-        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
+        <f aca="false">IF(Освіта!D8 = 0, "", Освіта!D8)</f>
         <v/>
       </c>
       <c r="D66" s="64"/>
@@ -11823,11 +11840,11 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="52"/>
       <c r="B67" s="45" t="str">
-        <f aca="false">Освіта!$F$4</f>
-        <v>Кваліфікація за дипломом (свідоцтвом)</v>
+        <f aca="false">Освіта!$E$4</f>
+        <v>Спеціальність (професія) за дипломом (свідоцтвом) </v>
       </c>
       <c r="C67" s="63" t="str">
-        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
+        <f aca="false">IF(Освіта!E8 = 0, "", Освіта!E8)</f>
         <v/>
       </c>
       <c r="D67" s="64"/>
@@ -11835,11 +11852,11 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="52"/>
       <c r="B68" s="45" t="str">
-        <f aca="false">Освіта!$G$4</f>
-        <v>Форма навчання (денна, вечірня, заочна)</v>
+        <f aca="false">Освіта!$F$4</f>
+        <v>Кваліфікація за дипломом (свідоцтвом)</v>
       </c>
       <c r="C68" s="63" t="str">
-        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
+        <f aca="false">IF(Освіта!F8 = 0, "", Освіта!F8)</f>
         <v/>
       </c>
       <c r="D68" s="64"/>
@@ -11847,11 +11864,11 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="52"/>
       <c r="B69" s="45" t="str">
-        <f aca="false">Освіта!$H$4</f>
-        <v>Рівень освіти</v>
+        <f aca="false">Освіта!$G$4</f>
+        <v>Форма навчання (денна, вечірня, заочна)</v>
       </c>
       <c r="C69" s="63" t="str">
-        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
+        <f aca="false">IF(Освіта!G8 = 0, "", Освіта!G8)</f>
         <v/>
       </c>
       <c r="D69" s="64"/>
@@ -11859,11 +11876,11 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="52"/>
       <c r="B70" s="45" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C70" s="65" t="str">
-        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
+        <f aca="false">Освіта!$H$4</f>
+        <v>Рівень освіти</v>
+      </c>
+      <c r="C70" s="63" t="str">
+        <f aca="false">IF(Освіта!H8 = 0, "", Освіта!H8)</f>
         <v/>
       </c>
       <c r="D70" s="64"/>
@@ -11871,35 +11888,35 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="52"/>
       <c r="B71" s="45" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C71" s="65" t="str">
+        <f aca="false">IF(Освіта!A13 = 0, "", Освіта!A13)</f>
+        <v/>
+      </c>
+      <c r="D71" s="64"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="52"/>
+      <c r="B72" s="45" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C71" s="65" t="str">
+      <c r="C72" s="65" t="str">
         <f aca="false">IF(Освіта!B13 = 0, "", Освіта!B13)</f>
         <v/>
       </c>
-      <c r="D71" s="64"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="52"/>
-      <c r="B72" s="2" t="str">
+      <c r="D72" s="64"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="52"/>
+      <c r="B73" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C72" s="65" t="str">
+      <c r="C73" s="65" t="str">
         <f aca="false">IF(Освіта!C13 = 0, "", Освіта!C13)</f>
-        <v/>
-      </c>
-      <c r="D72" s="64"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="52"/>
-      <c r="B73" s="45" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C73" s="65" t="str">
-        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
         <v/>
       </c>
       <c r="D73" s="64"/>
@@ -11907,35 +11924,35 @@
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="52"/>
       <c r="B74" s="45" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C74" s="65" t="str">
+        <f aca="false">IF(Освіта!A14 = 0, "", Освіта!A14)</f>
+        <v/>
+      </c>
+      <c r="D74" s="64"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="52"/>
+      <c r="B75" s="45" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C74" s="65" t="str">
+      <c r="C75" s="65" t="str">
         <f aca="false">IF(Освіта!B14 = 0, "", Освіта!B14)</f>
         <v/>
       </c>
-      <c r="D74" s="64"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="52"/>
-      <c r="B75" s="2" t="str">
+      <c r="D75" s="64"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="52"/>
+      <c r="B76" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C75" s="65" t="str">
+      <c r="C76" s="65" t="str">
         <f aca="false">IF(Освіта!C14 = 0, "", Освіта!C14)</f>
-        <v/>
-      </c>
-      <c r="D75" s="64"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="52"/>
-      <c r="B76" s="45" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C76" s="65" t="str">
-        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
         <v/>
       </c>
       <c r="D76" s="64"/>
@@ -11943,35 +11960,35 @@
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="52"/>
       <c r="B77" s="45" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C77" s="65" t="str">
+        <f aca="false">IF(Освіта!A15 = 0, "", Освіта!A15)</f>
+        <v/>
+      </c>
+      <c r="D77" s="64"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="52"/>
+      <c r="B78" s="45" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C77" s="65" t="str">
+      <c r="C78" s="65" t="str">
         <f aca="false">IF(Освіта!B15 = 0, "", Освіта!B15)</f>
         <v/>
       </c>
-      <c r="D77" s="64"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="52"/>
-      <c r="B78" s="2" t="str">
+      <c r="D78" s="64"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="52"/>
+      <c r="B79" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C78" s="65" t="str">
+      <c r="C79" s="65" t="str">
         <f aca="false">IF(Освіта!C15 = 0, "", Освіта!C15)</f>
-        <v/>
-      </c>
-      <c r="D78" s="64"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="52"/>
-      <c r="B79" s="45" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C79" s="65" t="str">
-        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
         <v/>
       </c>
       <c r="D79" s="64"/>
@@ -11979,35 +11996,35 @@
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="52"/>
       <c r="B80" s="45" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C80" s="65" t="str">
+        <f aca="false">IF(Освіта!A16 = 0, "", Освіта!A16)</f>
+        <v/>
+      </c>
+      <c r="D80" s="64"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="52"/>
+      <c r="B81" s="45" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C80" s="65" t="str">
+      <c r="C81" s="65" t="str">
         <f aca="false">IF(Освіта!B16 = 0, "", Освіта!B16)</f>
         <v/>
       </c>
-      <c r="D80" s="64"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="52"/>
-      <c r="B81" s="2" t="str">
+      <c r="D81" s="64"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="52"/>
+      <c r="B82" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C81" s="65" t="str">
+      <c r="C82" s="65" t="str">
         <f aca="false">IF(Освіта!C16 = 0, "", Освіта!C16)</f>
-        <v/>
-      </c>
-      <c r="D81" s="64"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="52"/>
-      <c r="B82" s="45" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C82" s="65" t="str">
-        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
         <v/>
       </c>
       <c r="D82" s="64"/>
@@ -12015,35 +12032,35 @@
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="52"/>
       <c r="B83" s="45" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C83" s="65" t="str">
+        <f aca="false">IF(Освіта!A17 = 0, "", Освіта!A17)</f>
+        <v/>
+      </c>
+      <c r="D83" s="64"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="52"/>
+      <c r="B84" s="45" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C83" s="65" t="str">
+      <c r="C84" s="65" t="str">
         <f aca="false">IF(Освіта!B17 = 0, "", Освіта!B17)</f>
         <v/>
       </c>
-      <c r="D83" s="64"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="52"/>
-      <c r="B84" s="2" t="str">
+      <c r="D84" s="64"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="52"/>
+      <c r="B85" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C84" s="65" t="str">
+      <c r="C85" s="65" t="str">
         <f aca="false">IF(Освіта!C17 = 0, "", Освіта!C17)</f>
-        <v/>
-      </c>
-      <c r="D84" s="64"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="52"/>
-      <c r="B85" s="45" t="str">
-        <f aca="false">Освіта!$A$12</f>
-        <v>Назва освітнього, наукового  закладу</v>
-      </c>
-      <c r="C85" s="65" t="str">
-        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
         <v/>
       </c>
       <c r="D85" s="64"/>
@@ -12051,73 +12068,73 @@
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="52"/>
       <c r="B86" s="45" t="str">
+        <f aca="false">Освіта!$A$12</f>
+        <v>Назва освітнього, наукового  закладу</v>
+      </c>
+      <c r="C86" s="65" t="str">
+        <f aca="false">IF(Освіта!A18 = 0, "", Освіта!A18)</f>
+        <v/>
+      </c>
+      <c r="D86" s="64"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="52"/>
+      <c r="B87" s="45" t="str">
         <f aca="false">Освіта!$B$12</f>
         <v>Рік закінчення</v>
       </c>
-      <c r="C86" s="65" t="str">
+      <c r="C87" s="65" t="str">
         <f aca="false">IF(Освіта!B18 = 0, "", Освіта!B18)</f>
         <v/>
       </c>
-      <c r="D86" s="64"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="52" t="s">
-        <v>160</v>
-      </c>
-      <c r="B87" s="2" t="str">
+      <c r="D87" s="64"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="52"/>
+      <c r="B88" s="2" t="str">
         <f aca="false">Освіта!$C$12</f>
         <v>Рівень підготовки</v>
       </c>
-      <c r="C87" s="65" t="str">
+      <c r="C88" s="65" t="str">
         <f aca="false">IF(Освіта!C18 = 0, "", Освіта!C18)</f>
         <v/>
       </c>
-      <c r="D87" s="64"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="52"/>
-      <c r="B88" s="45" t="str">
+      <c r="D88" s="64"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="52" t="s">
+        <v>161</v>
+      </c>
+      <c r="B89" s="45" t="str">
         <f aca="false">Родина!$A$4</f>
         <v>Ступінь родинного зв’язку (склад сім'ї)</v>
       </c>
-      <c r="C88" s="66" t="str">
+      <c r="C89" s="66" t="str">
         <f aca="false">IF(Родина!A5 = 0, "", Родина!A5)</f>
         <v/>
       </c>
-      <c r="D88" s="64"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="52"/>
-      <c r="B89" s="45" t="str">
+      <c r="D89" s="64"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="52"/>
+      <c r="B90" s="45" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C89" s="66" t="str">
+      <c r="C90" s="66" t="str">
         <f aca="false">IF(Родина!B5 = 0, "", Родина!B5)</f>
         <v/>
       </c>
-      <c r="D89" s="64"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="52"/>
-      <c r="B90" s="2" t="str">
+      <c r="D90" s="64"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="52"/>
+      <c r="B91" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C90" s="66" t="str">
+      <c r="C91" s="66" t="str">
         <f aca="false">IF(Родина!C5 = 0, "", Родина!C5)</f>
-        <v/>
-      </c>
-      <c r="D90" s="64"/>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="52"/>
-      <c r="B91" s="45" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C91" s="66" t="str">
-        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
         <v/>
       </c>
       <c r="D91" s="64"/>
@@ -12125,11 +12142,11 @@
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="52"/>
       <c r="B92" s="45" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C92" s="66" t="str">
-        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
+        <f aca="false">IF(Родина!D5 = 0, "", Родина!D5)</f>
         <v/>
       </c>
       <c r="D92" s="64"/>
@@ -12137,11 +12154,11 @@
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="52"/>
       <c r="B93" s="45" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C93" s="66" t="str">
-        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <f aca="false">IF(Родина!E5 = 0, "", Родина!E5)</f>
         <v/>
       </c>
       <c r="D93" s="64"/>
@@ -12149,35 +12166,35 @@
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="52"/>
       <c r="B94" s="45" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C94" s="66" t="str">
+        <f aca="false">IF(Родина!A6 = 0, "", Родина!A6)</f>
+        <v/>
+      </c>
+      <c r="D94" s="64"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="52"/>
+      <c r="B95" s="45" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C94" s="66" t="str">
+      <c r="C95" s="66" t="str">
         <f aca="false">IF(Родина!B6 = 0, "", Родина!B6)</f>
         <v/>
       </c>
-      <c r="D94" s="64"/>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="52"/>
-      <c r="B95" s="2" t="str">
+      <c r="D95" s="64"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="52"/>
+      <c r="B96" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C95" s="66" t="str">
+      <c r="C96" s="66" t="str">
         <f aca="false">IF(Родина!C6 = 0, "", Родина!C6)</f>
-        <v/>
-      </c>
-      <c r="D95" s="64"/>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="52"/>
-      <c r="B96" s="45" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C96" s="66" t="str">
-        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
         <v/>
       </c>
       <c r="D96" s="64"/>
@@ -12185,11 +12202,11 @@
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="52"/>
       <c r="B97" s="45" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C97" s="66" t="str">
-        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
+        <f aca="false">IF(Родина!D6 = 0, "", Родина!D6)</f>
         <v/>
       </c>
       <c r="D97" s="64"/>
@@ -12197,11 +12214,11 @@
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="52"/>
       <c r="B98" s="45" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C98" s="66" t="str">
-        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <f aca="false">IF(Родина!E6 = 0, "", Родина!E6)</f>
         <v/>
       </c>
       <c r="D98" s="64"/>
@@ -12209,35 +12226,35 @@
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="52"/>
       <c r="B99" s="45" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C99" s="66" t="str">
+        <f aca="false">IF(Родина!A7 = 0, "", Родина!A7)</f>
+        <v/>
+      </c>
+      <c r="D99" s="64"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="52"/>
+      <c r="B100" s="45" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C99" s="66" t="str">
+      <c r="C100" s="66" t="str">
         <f aca="false">IF(Родина!B7 = 0, "", Родина!B7)</f>
         <v/>
       </c>
-      <c r="D99" s="64"/>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="52"/>
-      <c r="B100" s="2" t="str">
+      <c r="D100" s="64"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="52"/>
+      <c r="B101" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C100" s="66" t="str">
+      <c r="C101" s="66" t="str">
         <f aca="false">IF(Родина!C7 = 0, "", Родина!C7)</f>
-        <v/>
-      </c>
-      <c r="D100" s="64"/>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="52"/>
-      <c r="B101" s="45" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C101" s="66" t="str">
-        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
         <v/>
       </c>
       <c r="D101" s="64"/>
@@ -12245,11 +12262,11 @@
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="52"/>
       <c r="B102" s="45" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C102" s="66" t="str">
-        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
+        <f aca="false">IF(Родина!D7 = 0, "", Родина!D7)</f>
         <v/>
       </c>
       <c r="D102" s="64"/>
@@ -12257,11 +12274,11 @@
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="52"/>
       <c r="B103" s="45" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C103" s="66" t="str">
-        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <f aca="false">IF(Родина!E7 = 0, "", Родина!E7)</f>
         <v/>
       </c>
       <c r="D103" s="64"/>
@@ -12269,35 +12286,35 @@
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="52"/>
       <c r="B104" s="45" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C104" s="66" t="str">
+        <f aca="false">IF(Родина!A8 = 0, "", Родина!A8)</f>
+        <v/>
+      </c>
+      <c r="D104" s="64"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="52"/>
+      <c r="B105" s="45" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C104" s="66" t="str">
+      <c r="C105" s="66" t="str">
         <f aca="false">IF(Родина!B8 = 0, "", Родина!B8)</f>
         <v/>
       </c>
-      <c r="D104" s="64"/>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="52"/>
-      <c r="B105" s="2" t="str">
+      <c r="D105" s="64"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="52"/>
+      <c r="B106" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C105" s="66" t="str">
+      <c r="C106" s="66" t="str">
         <f aca="false">IF(Родина!C8 = 0, "", Родина!C8)</f>
-        <v/>
-      </c>
-      <c r="D105" s="64"/>
-    </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="52"/>
-      <c r="B106" s="45" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C106" s="66" t="str">
-        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
         <v/>
       </c>
       <c r="D106" s="64"/>
@@ -12305,11 +12322,11 @@
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="52"/>
       <c r="B107" s="45" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C107" s="66" t="str">
-        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
+        <f aca="false">IF(Родина!D8 = 0, "", Родина!D8)</f>
         <v/>
       </c>
       <c r="D107" s="64"/>
@@ -12317,11 +12334,11 @@
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="52"/>
       <c r="B108" s="45" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C108" s="66" t="str">
-        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+        <f aca="false">IF(Родина!E8 = 0, "", Родина!E8)</f>
         <v/>
       </c>
       <c r="D108" s="64"/>
@@ -12329,35 +12346,35 @@
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="52"/>
       <c r="B109" s="45" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C109" s="66" t="str">
+        <f aca="false">IF(Родина!A9 = 0, "", Родина!A9)</f>
+        <v/>
+      </c>
+      <c r="D109" s="64"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="52"/>
+      <c r="B110" s="45" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C109" s="66" t="str">
+      <c r="C110" s="66" t="str">
         <f aca="false">IF(Родина!B9 = 0, "", Родина!B9)</f>
         <v/>
       </c>
-      <c r="D109" s="64"/>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="52"/>
-      <c r="B110" s="2" t="str">
+      <c r="D110" s="64"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="52"/>
+      <c r="B111" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C110" s="66" t="str">
+      <c r="C111" s="66" t="str">
         <f aca="false">IF(Родина!C9 = 0, "", Родина!C9)</f>
-        <v/>
-      </c>
-      <c r="D110" s="64"/>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="52"/>
-      <c r="B111" s="45" t="str">
-        <f aca="false">Родина!$D$4</f>
-        <v>По-батькові</v>
-      </c>
-      <c r="C111" s="66" t="str">
-        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
         <v/>
       </c>
       <c r="D111" s="64"/>
@@ -12365,11 +12382,11 @@
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="52"/>
       <c r="B112" s="45" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
+        <f aca="false">Родина!$D$4</f>
+        <v>По-батькові</v>
       </c>
       <c r="C112" s="66" t="str">
-        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
+        <f aca="false">IF(Родина!D9 = 0, "", Родина!D9)</f>
         <v/>
       </c>
       <c r="D112" s="64"/>
@@ -12377,11 +12394,11 @@
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="52"/>
       <c r="B113" s="45" t="str">
-        <f aca="false">Родина!$A$4</f>
-        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
       </c>
       <c r="C113" s="66" t="str">
-        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
+        <f aca="false">IF(Родина!E9 = 0, "", Родина!E9)</f>
         <v/>
       </c>
       <c r="D113" s="64"/>
@@ -12389,49 +12406,47 @@
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="52"/>
       <c r="B114" s="45" t="str">
+        <f aca="false">Родина!$A$4</f>
+        <v>Ступінь родинного зв’язку (склад сім'ї)</v>
+      </c>
+      <c r="C114" s="66" t="str">
+        <f aca="false">IF(Родина!A10 = 0, "", Родина!A10)</f>
+        <v/>
+      </c>
+      <c r="D114" s="64"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="52"/>
+      <c r="B115" s="45" t="str">
         <f aca="false">Родина!$B$4</f>
         <v>Прізвище</v>
       </c>
-      <c r="C114" s="66" t="str">
+      <c r="C115" s="66" t="str">
         <f aca="false">IF(Родина!B10 = 0, "", Родина!B10)</f>
         <v/>
       </c>
-      <c r="D114" s="64"/>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="52"/>
-      <c r="B115" s="2" t="str">
+      <c r="D115" s="64"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="52"/>
+      <c r="B116" s="2" t="str">
         <f aca="false">Родина!$C$4</f>
         <v>Ім’я</v>
       </c>
-      <c r="C115" s="66" t="str">
+      <c r="C116" s="66" t="str">
         <f aca="false">IF(Родина!C10 = 0, "", Родина!C10)</f>
         <v/>
       </c>
-      <c r="D115" s="64"/>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="52"/>
-      <c r="B116" s="45" t="str">
+      <c r="D116" s="64"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="52"/>
+      <c r="B117" s="45" t="str">
         <f aca="false">Родина!$D$4</f>
         <v>По-батькові</v>
       </c>
-      <c r="C116" s="66" t="str">
+      <c r="C117" s="66" t="str">
         <f aca="false">IF(Родина!D10 = 0, "", Родина!D10)</f>
-        <v/>
-      </c>
-      <c r="D116" s="64"/>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="52" t="s">
-        <v>161</v>
-      </c>
-      <c r="B117" s="45" t="str">
-        <f aca="false">Родина!$E$4</f>
-        <v>Рік народження</v>
-      </c>
-      <c r="C117" s="66" t="str">
-        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
         <v/>
       </c>
       <c r="D117" s="64"/>
@@ -12439,23 +12454,25 @@
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="52"/>
       <c r="B118" s="45" t="str">
+        <f aca="false">Родина!$E$4</f>
+        <v>Рік народження</v>
+      </c>
+      <c r="C118" s="66" t="str">
+        <f aca="false">IF(Родина!E10 = 0, "", Родина!E10)</f>
+        <v/>
+      </c>
+      <c r="D118" s="64"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="52" t="s">
+        <v>162</v>
+      </c>
+      <c r="B119" s="45" t="str">
         <f aca="false">Документи!A4</f>
         <v>Тип документу</v>
       </c>
-      <c r="C118" s="53" t="str">
+      <c r="C119" s="53" t="str">
         <f aca="false">IF(Документи!B4 = 0, "", Документи!B4)</f>
-        <v/>
-      </c>
-      <c r="D118" s="54"/>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="52"/>
-      <c r="B119" s="45" t="str">
-        <f aca="false">Документи!A5</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C119" s="54" t="str">
-        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
         <v/>
       </c>
       <c r="D119" s="54"/>
@@ -12463,11 +12480,11 @@
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="52"/>
       <c r="B120" s="45" t="str">
-        <f aca="false">Документи!A6</f>
-        <v>Ким виданий</v>
+        <f aca="false">Документи!A5</f>
+        <v>Серія та номер </v>
       </c>
       <c r="C120" s="54" t="str">
-        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
+        <f aca="false">IF(Документи!B5 = 0, "", Документи!B5)</f>
         <v/>
       </c>
       <c r="D120" s="54"/>
@@ -12475,11 +12492,11 @@
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="52"/>
       <c r="B121" s="45" t="str">
-        <f aca="false">Документи!A7</f>
-        <v>Дата видачі</v>
+        <f aca="false">Документи!A6</f>
+        <v>Ким виданий</v>
       </c>
       <c r="C121" s="54" t="str">
-        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
+        <f aca="false">IF(Документи!B6 = 0, "", Документи!B6)</f>
         <v/>
       </c>
       <c r="D121" s="54"/>
@@ -12487,11 +12504,11 @@
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="52"/>
       <c r="B122" s="45" t="str">
-        <f aca="false">Документи!A10</f>
-        <v>Тип документу</v>
-      </c>
-      <c r="C122" s="53" t="str">
-        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
+        <f aca="false">Документи!A7</f>
+        <v>Дата видачі</v>
+      </c>
+      <c r="C122" s="54" t="str">
+        <f aca="false">IF(Документи!B7 = 0, "", Документи!B7)</f>
         <v/>
       </c>
       <c r="D122" s="54"/>
@@ -12499,11 +12516,11 @@
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="52"/>
       <c r="B123" s="45" t="str">
-        <f aca="false">Документи!A11</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C123" s="54" t="str">
-        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
+        <f aca="false">Документи!A10</f>
+        <v>Тип документу</v>
+      </c>
+      <c r="C123" s="53" t="str">
+        <f aca="false">IF(Документи!B10 = 0, "", Документи!B10)</f>
         <v/>
       </c>
       <c r="D123" s="54"/>
@@ -12511,11 +12528,11 @@
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="52"/>
       <c r="B124" s="45" t="str">
-        <f aca="false">Документи!A12</f>
-        <v>Ким виданий</v>
+        <f aca="false">Документи!A11</f>
+        <v>Серія та номер </v>
       </c>
       <c r="C124" s="54" t="str">
-        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
+        <f aca="false">IF(Документи!B11 = 0, "", Документи!B11)</f>
         <v/>
       </c>
       <c r="D124" s="54"/>
@@ -12523,34 +12540,34 @@
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="52"/>
       <c r="B125" s="45" t="str">
+        <f aca="false">Документи!A12</f>
+        <v>Ким виданий</v>
+      </c>
+      <c r="C125" s="54" t="str">
+        <f aca="false">IF(Документи!B12 = 0, "", Документи!B12)</f>
+        <v/>
+      </c>
+      <c r="D125" s="54"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="52"/>
+      <c r="B126" s="45" t="str">
         <f aca="false">Документи!A13</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C125" s="54" t="str">
+      <c r="C126" s="54" t="str">
         <f aca="false">IF(Документи!B13 = 0, "", Документи!B13)</f>
-        <v/>
-      </c>
-      <c r="D125" s="54"/>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="52"/>
-      <c r="B126" s="45" t="s">
-        <v>162</v>
-      </c>
-      <c r="C126" s="54" t="str">
-        <f aca="false">IF(D126 = 0, "", D126)</f>
         <v/>
       </c>
       <c r="D126" s="54"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="52"/>
-      <c r="B127" s="45" t="str">
-        <f aca="false">Документи!A16</f>
-        <v>Серія та номер </v>
-      </c>
-      <c r="C127" s="53" t="str">
-        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
+      <c r="B127" s="45" t="s">
+        <v>163</v>
+      </c>
+      <c r="C127" s="54" t="str">
+        <f aca="false">IF(D127 = 0, "", D127)</f>
         <v/>
       </c>
       <c r="D127" s="54"/>
@@ -12558,54 +12575,63 @@
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="52"/>
       <c r="B128" s="45" t="str">
+        <f aca="false">Документи!A16</f>
+        <v>Серія та номер </v>
+      </c>
+      <c r="C128" s="53" t="str">
+        <f aca="false">IF(Документи!B16 = 0, "", Документи!B16)</f>
+        <v/>
+      </c>
+      <c r="D128" s="54"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="52"/>
+      <c r="B129" s="45" t="str">
         <f aca="false">Документи!A17</f>
         <v>Ким виданий</v>
       </c>
-      <c r="C128" s="54" t="str">
+      <c r="C129" s="54" t="str">
         <f aca="false">IF(Документи!B17 = 0, "", Документи!B17)</f>
         <v/>
       </c>
-      <c r="D128" s="54"/>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="2"/>
-      <c r="B129" s="45" t="str">
+      <c r="D129" s="54"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="52"/>
+      <c r="B130" s="45" t="str">
         <f aca="false">Документи!A18</f>
         <v>Дата видачі</v>
       </c>
-      <c r="C129" s="54" t="str">
+      <c r="C130" s="54" t="str">
         <f aca="false">IF(Документи!B18 = 0, "", Документи!B18)</f>
         <v/>
       </c>
-      <c r="D129" s="54"/>
-    </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="2"/>
+      <c r="D130" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="G1:N1"/>
     <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="A2:A23"/>
+    <mergeCell ref="A2:A25"/>
     <mergeCell ref="O2:O16"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="O17:O28"/>
-    <mergeCell ref="A24:A36"/>
-    <mergeCell ref="A37:A86"/>
-    <mergeCell ref="A87:A116"/>
-    <mergeCell ref="A117:A128"/>
+    <mergeCell ref="A26:A37"/>
+    <mergeCell ref="A38:A88"/>
+    <mergeCell ref="A89:A118"/>
+    <mergeCell ref="A119:A130"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G16:K21" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D38:D42" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D39:D43" type="list">
       <formula1>'Системна інформація'!$Q$27:$ZA$27</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D44" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D45" type="list">
       <formula1>'Системна інформація'!$Q$11:$ZA$11</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>